<commit_message>
Corrige le nombre de vacations de nuit par défaut (140/an)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1LRXK2yXR6W5viD25HWb5
</commit_message>
<xml_diff>
--- a/conges/conges_police_12h08.xlsx
+++ b/conges/conges_police_12h08.xlsx
@@ -707,7 +707,7 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>IF(Parametres!$B$13&gt;0,Parametres!$B$13,ROUND(365/4*2*Parametres!$B$8,0))*Parametres!$B$7*Parametres!$B$12</f>
+        <f>IF(Parametres!$B$13&gt;0,Parametres!$B$13,ROUND(140*Parametres!$B$8,0))*Parametres!$B$7*Parametres!$B$12</f>
         <v/>
       </c>
       <c r="C8" s="6">
@@ -728,7 +728,7 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Vacations nuit × heures nuit × coef. Cycle 2/2/3 ≈ 182 nuits/an.</t>
+          <t>Vacations nuit × heures nuit × coef. Défaut : 140 vacations/an (rapport Sénat 2019).</t>
         </is>
       </c>
     </row>
@@ -1264,7 +1264,7 @@
       </c>
       <c r="C6" s="16" t="inlineStr">
         <is>
-          <t>12h08 = 12,13 h.</t>
+          <t>12h08 = 12,13 h, dont 2 pauses de 20 min (rapport Sénat).</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>Laisse 0 pour estimer via le cycle (onglet Calcul).</t>
+          <t>Laisse 0 = 140 vacations/an (cycle binaire 12h08, rapport Sénat).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Récap congés : CA, CA HP, RTC, CET, CF, HS, RPS avec base, pris, reste
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1LRXK2yXR6W5viD25HWb5
</commit_message>
<xml_diff>
--- a/conges/conges_police_12h08.xlsx
+++ b/conges/conges_police_12h08.xlsx
@@ -128,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -138,10 +138,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="7" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,6 +150,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -520,16 +521,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G32"/>
+  <dimension ref="A1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="1" max="1"/>
     <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="62" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -543,7 +543,6 @@
       <c r="D1" s="2" t="n"/>
       <c r="E1" s="2" t="n"/>
       <c r="F1" s="2" t="n"/>
-      <c r="G1" s="2" t="n"/>
     </row>
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
@@ -556,7 +555,6 @@
       <c r="D2" s="2" t="n"/>
       <c r="E2" s="2" t="n"/>
       <c r="F2" s="2" t="n"/>
-      <c r="G2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n"/>
@@ -565,42 +563,36 @@
       <c r="D3" s="2" t="n"/>
       <c r="E3" s="2" t="n"/>
       <c r="F3" s="2" t="n"/>
-      <c r="G3" s="2" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>Droit</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Acquis (h)</t>
+          <t>De base (h)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Acquis (vacations)</t>
+          <t>Pris (h)</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Pris (h)</t>
+          <t>Reste (h)</t>
         </is>
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>Solde (h)</t>
+          <t>Reste (vacations)</t>
         </is>
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Solde (vacations)</t>
-        </is>
-      </c>
-      <c r="G4" s="4" t="inlineStr">
-        <is>
-          <t>Règle</t>
+          <t>Explication</t>
         </is>
       </c>
     </row>
@@ -615,22 +607,18 @@
         <v/>
       </c>
       <c r="C5" s="6">
-        <f>B5/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="D5" s="6">
         <f>SUMIF(Suivi!$C$5:$C$204,"CA",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
+      <c r="D5" s="7">
+        <f>B5-C5</f>
+        <v/>
+      </c>
       <c r="E5" s="6">
-        <f>B5-D5</f>
-        <v/>
-      </c>
-      <c r="F5" s="6">
-        <f>E5/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="G5" s="5" t="inlineStr">
+        <f>D5/Parametres!$B$6</f>
+        <v/>
+      </c>
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>25 j ouvrés × valeur horaire × quotité.</t>
         </is>
@@ -639,485 +627,464 @@
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>FRAC – Jours de fractionnement</t>
+          <t>CA HP – Hors période</t>
         </is>
       </c>
       <c r="B6" s="6">
-        <f>IF(Parametres!$B$16&gt;=8,2,IF(Parametres!$B$16&gt;=5,1,0))*Parametres!$B$10</f>
+        <f>IF(Parametres!$B$11&gt;=8,2,IF(Parametres!$B$11&gt;=5,1,0))*Parametres!$B$10</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>B6/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="D6" s="6">
-        <f>SUMIF(Suivi!$C$5:$C$204,"FRAC",Suivi!$E$5:$E$204)</f>
+        <f>SUMIF(Suivi!$C$5:$C$204,"CA HP",Suivi!$E$5:$E$204)</f>
+        <v/>
+      </c>
+      <c r="D6" s="7">
+        <f>B6-C6</f>
         <v/>
       </c>
       <c r="E6" s="6">
-        <f>B6-D6</f>
-        <v/>
-      </c>
-      <c r="F6" s="6">
-        <f>E6/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>1 j si 5-7 j CA hors mai-oct ; 2 j si ≥ 8.</t>
+        <f>D6/Parametres!$B$6</f>
+        <v/>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Bonus : 1 j si 5-7 j CA hors mai-oct ; 2 j si 8 et +.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>RTT / ARTT</t>
+          <t>RTC</t>
         </is>
       </c>
       <c r="B7" s="6">
-        <f>Parametres!$B$11</f>
+        <f>Parametres!$B$12</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>B7/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="D7" s="6">
-        <f>SUMIF(Suivi!$C$5:$C$204,"RTT",Suivi!$E$5:$E$204)</f>
+        <f>SUMIF(Suivi!$C$5:$C$204,"RTC",Suivi!$E$5:$E$204)</f>
+        <v/>
+      </c>
+      <c r="D7" s="7">
+        <f>B7-C7</f>
         <v/>
       </c>
       <c r="E7" s="6">
-        <f>B7-D7</f>
-        <v/>
-      </c>
-      <c r="F7" s="6">
-        <f>E7/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="G7" s="5" t="inlineStr">
-        <is>
-          <t>Selon cycle. Souvent 0 en 12h08.</t>
+        <f>D7/Parametres!$B$6</f>
+        <v/>
+      </c>
+      <c r="F7" s="5" t="inlineStr">
+        <is>
+          <t>Crédit saisi dans Parametres.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>RC Nuit – bonification nuit</t>
+          <t>CET – Compte épargne-temps</t>
         </is>
       </c>
       <c r="B8" s="6">
-        <f>IF(Parametres!$B$13&gt;0,Parametres!$B$13,ROUND(140*Parametres!$B$8,0))*Parametres!$B$7*Parametres!$B$12</f>
+        <f>(Parametres!$B$18+Parametres!$B$19)*Parametres!$B$10</f>
         <v/>
       </c>
       <c r="C8" s="6">
-        <f>B8/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="D8" s="6">
-        <f>SUMIF(Suivi!$C$5:$C$204,"RC Nuit",Suivi!$E$5:$E$204)</f>
+        <f>SUMIF(Suivi!$C$5:$C$204,"CET",Suivi!$E$5:$E$204)</f>
+        <v/>
+      </c>
+      <c r="D8" s="7">
+        <f>B8-C8</f>
         <v/>
       </c>
       <c r="E8" s="6">
-        <f>B8-D8</f>
-        <v/>
-      </c>
-      <c r="F8" s="6">
-        <f>E8/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>Vacations nuit × heures nuit × coef. Défaut : 140 vacations/an (rapport Sénat 2019).</t>
+        <f>D8/Parametres!$B$6</f>
+        <v/>
+      </c>
+      <c r="F8" s="5" t="inlineStr">
+        <is>
+          <t>Solde 1er janvier + jours versés.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>RC Férié – fériés travaillés</t>
+          <t>CF – Crédit férié</t>
         </is>
       </c>
       <c r="B9" s="6">
-        <f>Parametres!$B$14*Parametres!$B$15</f>
+        <f>Parametres!$B$13*Parametres!$B$14</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>B9/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="D9" s="6">
-        <f>SUMIF(Suivi!$C$5:$C$204,"RC Férié",Suivi!$E$5:$E$204)</f>
+        <f>SUMIF(Suivi!$C$5:$C$204,"CF",Suivi!$E$5:$E$204)</f>
+        <v/>
+      </c>
+      <c r="D9" s="7">
+        <f>B9-C9</f>
         <v/>
       </c>
       <c r="E9" s="6">
-        <f>B9-D9</f>
-        <v/>
-      </c>
-      <c r="F9" s="6">
-        <f>E9/Parametres!$B$6</f>
-        <v/>
-      </c>
-      <c r="G9" s="5" t="inlineStr">
-        <is>
-          <t>Récup des fériés travaillés.</t>
+        <f>D9/Parametres!$B$6</f>
+        <v/>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t>Nb fériés × heures par férié.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
-        <is>
-          <t>TOTAL droits annuels</t>
-        </is>
-      </c>
-      <c r="B10" s="8">
-        <f>SUM(B5:B9)</f>
-        <v/>
-      </c>
-      <c r="C10" s="8">
-        <f>SUM(C5:C9)</f>
-        <v/>
-      </c>
-      <c r="D10" s="8">
-        <f>SUM(D5:D9)</f>
-        <v/>
-      </c>
-      <c r="E10" s="8">
-        <f>SUM(E5:E9)</f>
-        <v/>
-      </c>
-      <c r="F10" s="8">
-        <f>SUM(F5:F9)</f>
-        <v/>
-      </c>
-      <c r="G10" s="7" t="inlineStr">
-        <is>
-          <t>Somme des droits ci-dessus.</t>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>HS – Heures supplémentaires</t>
+        </is>
+      </c>
+      <c r="B10" s="6">
+        <f>Parametres!$B$15</f>
+        <v/>
+      </c>
+      <c r="C10" s="6">
+        <f>SUMIF(Suivi!$C$5:$C$204,"HS",Suivi!$E$5:$E$204)</f>
+        <v/>
+      </c>
+      <c r="D10" s="7">
+        <f>B10-C10</f>
+        <v/>
+      </c>
+      <c r="E10" s="6">
+        <f>D10/Parametres!$B$6</f>
+        <v/>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t>Compteur HS récupérables.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
-      <c r="E11" s="2" t="n"/>
-      <c r="F11" s="2" t="n"/>
-      <c r="G11" s="2" t="n"/>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>RPS – Repos pénibilité nuit</t>
+        </is>
+      </c>
+      <c r="B11" s="6">
+        <f>IF(Parametres!$B$17&gt;0,Parametres!$B$17,ROUND(140*Parametres!$B$8,0))*Parametres!$B$7*Parametres!$B$16</f>
+        <v/>
+      </c>
+      <c r="C11" s="6">
+        <f>SUMIF(Suivi!$C$5:$C$204,"RPS",Suivi!$E$5:$E$204)</f>
+        <v/>
+      </c>
+      <c r="D11" s="7">
+        <f>B11-C11</f>
+        <v/>
+      </c>
+      <c r="E11" s="6">
+        <f>D11/Parametres!$B$6</f>
+        <v/>
+      </c>
+      <c r="F11" s="5" t="inlineStr">
+        <is>
+          <t>Vacations nuit × heures nuit × coef.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>CET – Compte épargne-temps</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="n"/>
-      <c r="C12" s="2" t="n"/>
-      <c r="D12" s="2" t="n"/>
-      <c r="E12" s="2" t="n"/>
-      <c r="F12" s="2" t="n"/>
-      <c r="G12" s="2" t="n"/>
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="B12" s="9">
+        <f>SUM(B5:B11)</f>
+        <v/>
+      </c>
+      <c r="C12" s="9">
+        <f>SUM(C5:C11)</f>
+        <v/>
+      </c>
+      <c r="D12" s="9">
+        <f>SUM(D5:D11)</f>
+        <v/>
+      </c>
+      <c r="E12" s="9">
+        <f>SUM(E5:E11)</f>
+        <v/>
+      </c>
+      <c r="F12" s="8" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
-        <is>
-          <t>Élément</t>
-        </is>
-      </c>
-      <c r="B13" s="4" t="inlineStr">
-        <is>
-          <t>Valeur</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr"/>
-      <c r="D13" s="4" t="inlineStr"/>
-      <c r="E13" s="4" t="inlineStr"/>
-      <c r="F13" s="4" t="inlineStr"/>
-      <c r="G13" s="4" t="inlineStr">
-        <is>
-          <t>Règle</t>
-        </is>
-      </c>
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+      <c r="F13" s="2" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
-        <is>
-          <t>Solde CET au 1er janvier (jours)</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="n">
-        <v>0</v>
-      </c>
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>CET – détail</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n"/>
       <c r="C14" s="2" t="n"/>
       <c r="D14" s="2" t="n"/>
       <c r="E14" s="2" t="n"/>
       <c r="F14" s="2" t="n"/>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Repris de ton relevé CET.</t>
-        </is>
-      </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
-        <is>
-          <t>Jours CA pris dans l'année</t>
-        </is>
-      </c>
-      <c r="B15" s="11">
-        <f>D5/Parametres!$B$10</f>
-        <v/>
-      </c>
-      <c r="C15" s="2" t="n"/>
-      <c r="D15" s="2" t="n"/>
-      <c r="E15" s="2" t="n"/>
-      <c r="F15" s="2" t="n"/>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Calculé depuis Suivi.</t>
+      <c r="A15" s="4" t="inlineStr">
+        <is>
+          <t>Élément</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Valeur</t>
+        </is>
+      </c>
+      <c r="C15" s="4" t="inlineStr"/>
+      <c r="D15" s="4" t="inlineStr"/>
+      <c r="E15" s="4" t="inlineStr"/>
+      <c r="F15" s="4" t="inlineStr">
+        <is>
+          <t>Règle</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Jours épargnables max</t>
+          <t>Jours CA pris dans l'année</t>
         </is>
       </c>
       <c r="B16" s="11">
-        <f>MAX(0,MIN((B5+B6)/Parametres!$B$10-B15,(B5+B6)/Parametres!$B$10-20))</f>
+        <f>C5/Parametres!$B$10</f>
         <v/>
       </c>
       <c r="C16" s="2" t="n"/>
       <c r="D16" s="2" t="n"/>
       <c r="E16" s="2" t="n"/>
-      <c r="F16" s="2" t="n"/>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>20 j de CA à prendre obligatoirement. Le reliquat (CA + frac.) est épargnable.</t>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Depuis Suivi.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Jours versés au CET cette année</t>
-        </is>
-      </c>
-      <c r="B17" s="10" t="n">
-        <v>0</v>
+          <t>Jours épargnables max</t>
+        </is>
+      </c>
+      <c r="B17" s="11">
+        <f>MAX(0,MIN((B5+B6-C5-C6)/Parametres!$B$10,(B5+B6)/Parametres!$B$10-20))</f>
+        <v/>
       </c>
       <c r="C17" s="2" t="n"/>
       <c r="D17" s="2" t="n"/>
       <c r="E17" s="2" t="n"/>
-      <c r="F17" s="2" t="n"/>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Ta demande (avant 31/01 N+1).</t>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>20 j de CA obligatoires. Le reliquat est épargnable.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Jours CET consommés (Suivi)</t>
+          <t>Solde CET restant (jours)</t>
         </is>
       </c>
       <c r="B18" s="11">
-        <f>SUMIF(Suivi!$C$5:$C$204,"CET",Suivi!$E$5:$E$204)/Parametres!$B$10</f>
+        <f>D8/Parametres!$B$10</f>
         <v/>
       </c>
       <c r="C18" s="2" t="n"/>
       <c r="D18" s="2" t="n"/>
       <c r="E18" s="2" t="n"/>
-      <c r="F18" s="2" t="n"/>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Absences type CET dans Suivi.</t>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Plafond 60 jours.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Solde CET fin d'année (jours)</t>
+          <t>Alerte plafond</t>
         </is>
       </c>
       <c r="B19" s="11">
-        <f>B14+MIN(B17,B16)-B18</f>
+        <f>IF(B18&gt;60,"Plafond 60 j dépassé","OK")</f>
         <v/>
       </c>
       <c r="C19" s="2" t="n"/>
       <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="n"/>
-      <c r="F19" s="2" t="n"/>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Plafond 60 jours.</t>
-        </is>
-      </c>
+      <c r="F19" s="2" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Alerte plafond</t>
+          <t>Jours indemnisables (au-delà de 15)</t>
         </is>
       </c>
       <c r="B20" s="11">
-        <f>IF(B19&gt;60,"Plafond 60 j dépassé","OK")</f>
+        <f>MAX(0,MIN(B18,60)-15)</f>
         <v/>
       </c>
       <c r="C20" s="2" t="n"/>
       <c r="D20" s="2" t="n"/>
       <c r="E20" s="2" t="n"/>
-      <c r="F20" s="2" t="n"/>
-      <c r="G20" s="2" t="inlineStr"/>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Option possible au-delà de 15 j.</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Jours indemnisables (au-delà de 15)</t>
-        </is>
-      </c>
-      <c r="B21" s="11">
-        <f>MAX(0,MIN(B19,60)-15)</f>
+          <t>Valeur si indemnisés (€)</t>
+        </is>
+      </c>
+      <c r="B21" s="12">
+        <f>B20*IF(Parametres!$B$20="A",Parametres!$B$23,IF(Parametres!$B$20="B",Parametres!$B$22,Parametres!$B$21))</f>
         <v/>
       </c>
       <c r="C21" s="2" t="n"/>
       <c r="D21" s="2" t="n"/>
       <c r="E21" s="2" t="n"/>
-      <c r="F21" s="2" t="n"/>
-      <c r="G21" s="2" t="inlineStr">
-        <is>
-          <t>Option possible au-delà de 15 j.</t>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Montant brut selon catégorie.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
-        <is>
-          <t>Valeur si indemnisés (€)</t>
-        </is>
-      </c>
-      <c r="B22" s="12">
-        <f>B21*IF(Parametres!$B$17="A",Parametres!$B$20,IF(Parametres!$B$17="B",Parametres!$B$19,Parametres!$B$18))</f>
-        <v/>
-      </c>
+      <c r="A22" s="2" t="n"/>
+      <c r="B22" s="2" t="n"/>
       <c r="C22" s="2" t="n"/>
       <c r="D22" s="2" t="n"/>
       <c r="E22" s="2" t="n"/>
       <c r="F22" s="2" t="n"/>
-      <c r="G22" s="2" t="inlineStr">
-        <is>
-          <t>Montant brut selon catégorie.</t>
-        </is>
-      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n"/>
+      <c r="A23" s="10" t="inlineStr">
+        <is>
+          <t>ASA – Autorisations spéciales d'absence (hors compteur)</t>
+        </is>
+      </c>
       <c r="B23" s="2" t="n"/>
       <c r="C23" s="2" t="n"/>
       <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="n"/>
       <c r="F23" s="2" t="n"/>
-      <c r="G23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>ASA – Autorisations spéciales d'absence (hors compteur)</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="n"/>
-      <c r="C24" s="2" t="n"/>
-      <c r="D24" s="2" t="n"/>
-      <c r="E24" s="2" t="n"/>
-      <c r="F24" s="2" t="n"/>
-      <c r="G24" s="2" t="n"/>
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>Motif</t>
+        </is>
+      </c>
+      <c r="B24" s="4" t="inlineStr">
+        <is>
+          <t>Jours</t>
+        </is>
+      </c>
+      <c r="C24" s="4" t="inlineStr"/>
+      <c r="D24" s="4" t="inlineStr"/>
+      <c r="E24" s="4" t="inlineStr"/>
+      <c r="F24" s="4" t="inlineStr">
+        <is>
+          <t>Règle</t>
+        </is>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
-        <is>
-          <t>Motif</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Jours</t>
-        </is>
-      </c>
-      <c r="C25" s="4" t="inlineStr"/>
-      <c r="D25" s="4" t="inlineStr"/>
-      <c r="E25" s="4" t="inlineStr"/>
-      <c r="F25" s="4" t="inlineStr"/>
-      <c r="G25" s="4" t="inlineStr">
-        <is>
-          <t>Règle</t>
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>Garde d'enfant malade</t>
+        </is>
+      </c>
+      <c r="B25" s="13">
+        <f>IF(Parametres!$B$24="O",IF(Parametres!$B$25="O",12,6)*Parametres!$B$8,0)</f>
+        <v/>
+      </c>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>6 j/an ; 12 j si seul ou conjoint sans droit. À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>Garde d'enfant malade</t>
-        </is>
-      </c>
-      <c r="B26" s="13">
-        <f>IF(Parametres!$B$21="O",IF(Parametres!$B$22="O",12,6)*Parametres!$B$8,0)</f>
-        <v/>
+          <t>Mariage / PACS de l'agent</t>
+        </is>
+      </c>
+      <c r="B26" s="13" t="n">
+        <v>5</v>
       </c>
       <c r="C26" s="2" t="n"/>
       <c r="D26" s="2" t="n"/>
       <c r="E26" s="2" t="n"/>
-      <c r="F26" s="2" t="n"/>
-      <c r="G26" s="2" t="inlineStr">
-        <is>
-          <t>6 j/an ; 12 j si seul ou conjoint sans droit. À vérifier.</t>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>Barème FP. À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Mariage / PACS de l'agent</t>
+          <t>Décès conjoint / parent / enfant</t>
         </is>
       </c>
       <c r="B27" s="13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="C27" s="2" t="n"/>
       <c r="D27" s="2" t="n"/>
       <c r="E27" s="2" t="n"/>
-      <c r="F27" s="2" t="n"/>
-      <c r="G27" s="2" t="inlineStr">
-        <is>
-          <t>Barème FP. À vérifier.</t>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>Barème FP. Enfant : régime renforcé.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>Décès conjoint / parent / enfant</t>
-        </is>
-      </c>
-      <c r="B28" s="13" t="n">
-        <v>3</v>
+          <t>Naissance / adoption</t>
+        </is>
+      </c>
+      <c r="B28" s="13" t="inlineStr">
+        <is>
+          <t>Voir RH</t>
+        </is>
       </c>
       <c r="C28" s="2" t="n"/>
       <c r="D28" s="2" t="n"/>
       <c r="E28" s="2" t="n"/>
-      <c r="F28" s="2" t="n"/>
-      <c r="G28" s="2" t="inlineStr">
-        <is>
-          <t>Barème FP. Enfant : régime renforcé.</t>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>Congé naissance 3 j + paternité 25 j.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>Naissance / adoption</t>
+          <t>Déménagement</t>
         </is>
       </c>
       <c r="B29" s="13" t="inlineStr">
@@ -1128,55 +1095,31 @@
       <c r="C29" s="2" t="n"/>
       <c r="D29" s="2" t="n"/>
       <c r="E29" s="2" t="n"/>
-      <c r="F29" s="2" t="n"/>
-      <c r="G29" s="2" t="inlineStr">
-        <is>
-          <t>Congé naissance 3 j + paternité 25 j.</t>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>Selon note de service.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="5" t="inlineStr">
-        <is>
-          <t>Déménagement</t>
-        </is>
-      </c>
-      <c r="B30" s="13" t="inlineStr">
-        <is>
-          <t>Voir RH</t>
-        </is>
-      </c>
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
       <c r="C30" s="2" t="n"/>
       <c r="D30" s="2" t="n"/>
       <c r="E30" s="2" t="n"/>
       <c r="F30" s="2" t="n"/>
-      <c r="G30" s="2" t="inlineStr">
-        <is>
-          <t>Selon note de service.</t>
-        </is>
-      </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Les montants et barèmes sont indicatifs. Vérifie avec ton secrétariat / Géopol et ta note de service locale.</t>
+        </is>
+      </c>
       <c r="B31" s="2" t="n"/>
       <c r="C31" s="2" t="n"/>
       <c r="D31" s="2" t="n"/>
       <c r="E31" s="2" t="n"/>
       <c r="F31" s="2" t="n"/>
-      <c r="G31" s="2" t="n"/>
-    </row>
-    <row r="32">
-      <c r="A32" s="14" t="inlineStr">
-        <is>
-          <t>Les montants et barèmes sont indicatifs. Vérifie avec ton secrétariat / Géopol et ta note de service locale.</t>
-        </is>
-      </c>
-      <c r="B32" s="2" t="n"/>
-      <c r="C32" s="2" t="n"/>
-      <c r="D32" s="2" t="n"/>
-      <c r="E32" s="2" t="n"/>
-      <c r="F32" s="2" t="n"/>
-      <c r="G32" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1189,7 +1132,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1274,7 +1217,7 @@
           <t>Heures de nuit par vacation</t>
         </is>
       </c>
-      <c r="B7" s="10" t="n">
+      <c r="B7" s="17" t="n">
         <v>8</v>
       </c>
       <c r="C7" s="16" t="inlineStr">
@@ -1289,7 +1232,7 @@
           <t>Quotité de travail</t>
         </is>
       </c>
-      <c r="B8" s="17" t="n">
+      <c r="B8" s="18" t="n">
         <v>1</v>
       </c>
       <c r="C8" s="16" t="inlineStr">
@@ -1309,7 +1252,7 @@
       </c>
       <c r="C9" s="16" t="inlineStr">
         <is>
-          <t>Décret 84-972 : 5 × obligations hebdo = 25 jours.</t>
+          <t>Décret 84-972 : 25 jours ouvrés.</t>
         </is>
       </c>
     </row>
@@ -1319,34 +1262,34 @@
           <t>Valeur horaire d'1 jour de CA (h)</t>
         </is>
       </c>
-      <c r="B10" s="10" t="n">
+      <c r="B10" s="17" t="n">
         <v>7</v>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>À vérifier avec ton service RH / Géopol. Souvent 7h ou 7h12.</t>
+          <t>À vérifier avec ton secrétariat / Géopol.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>RTT / ARTT annuels (heures)</t>
-        </is>
-      </c>
-      <c r="B11" s="10" t="n">
+          <t>CA HP – jours CA pris hors 1/05–31/10</t>
+        </is>
+      </c>
+      <c r="B11" s="15" t="n">
         <v>0</v>
       </c>
       <c r="C11" s="16" t="inlineStr">
         <is>
-          <t>En 12h08 : souvent 0. Saisis le crédit si ton cycle en génère.</t>
+          <t>5 à 7 j = 1 j bonus ; 8 j et + = 2 j bonus.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>Bonification nuit (coef. sur heures de nuit)</t>
+          <t>RTC – crédit annuel (heures)</t>
         </is>
       </c>
       <c r="B12" s="17" t="n">
@@ -1354,14 +1297,14 @@
       </c>
       <c r="C12" s="16" t="inlineStr">
         <is>
-          <t>Saisis le % de ta note de service (ex. 10 %). 0 si aucune.</t>
+          <t>Repris de ton relevé Géopol.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Nombre de vacations de nuit / an</t>
+          <t>CF – nombre de fériés crédités</t>
         </is>
       </c>
       <c r="B13" s="15" t="n">
@@ -1369,147 +1312,192 @@
       </c>
       <c r="C13" s="16" t="inlineStr">
         <is>
-          <t>Laisse 0 = 140 vacations/an (cycle binaire 12h08, rapport Sénat).</t>
+          <t>Fériés ouvrant un crédit férié. Voir relevé.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>Jours fériés travaillés (vacations)</t>
-        </is>
-      </c>
-      <c r="B14" s="15" t="n">
-        <v>0</v>
+          <t>CF – heures par férié</t>
+        </is>
+      </c>
+      <c r="B14" s="11">
+        <f>B6</f>
+        <v/>
       </c>
       <c r="C14" s="16" t="inlineStr">
         <is>
-          <t>Fériés tombant sur une vacation travaillée.</t>
+          <t>Par défaut = 1 vacation. Modifiable.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Récup par férié travaillé (heures)</t>
-        </is>
-      </c>
-      <c r="B15" s="11">
-        <f>B6</f>
-        <v/>
+          <t>HS – heures sup. au compteur (heures)</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="n">
+        <v>0</v>
       </c>
       <c r="C15" s="16" t="inlineStr">
         <is>
-          <t>Par défaut = 1 vacation. Modifiable.</t>
+          <t>Solde HS récupérables. Voir relevé.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>Jours CA pris hors période 1/05–31/10</t>
-        </is>
-      </c>
-      <c r="B16" s="15" t="n">
+          <t>RPS – coef. sur heures de nuit</t>
+        </is>
+      </c>
+      <c r="B16" s="18" t="n">
         <v>0</v>
       </c>
       <c r="C16" s="16" t="inlineStr">
         <is>
-          <t>Sert au calcul du fractionnement.</t>
+          <t>Taux de ta note de service. 0 si inconnu.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Catégorie (C, B, A)</t>
-        </is>
-      </c>
-      <c r="B17" s="18" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
+          <t>RPS – vacations de nuit / an</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="n">
+        <v>0</v>
       </c>
       <c r="C17" s="16" t="inlineStr">
         <is>
-          <t>Pour l'indemnisation CET.</t>
+          <t>0 = 140 vacations/an (cycle binaire, rapport Sénat).</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>Taux CET catégorie C (€/jour)</t>
-        </is>
-      </c>
-      <c r="B18" s="19" t="n">
-        <v>83</v>
+          <t>CET – solde au 1er janvier (jours)</t>
+        </is>
+      </c>
+      <c r="B18" s="17" t="n">
+        <v>0</v>
       </c>
       <c r="C18" s="16" t="inlineStr">
         <is>
-          <t>Arrêté 2024 – à vérifier.</t>
+          <t>Repris de ton relevé CET.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>Taux CET catégorie B (€/jour)</t>
-        </is>
-      </c>
-      <c r="B19" s="19" t="n">
-        <v>100</v>
+          <t>CET – jours versés cette année</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="n">
+        <v>0</v>
       </c>
       <c r="C19" s="16" t="inlineStr">
         <is>
-          <t>Arrêté 2024 – à vérifier.</t>
+          <t>Ta demande d'alimentation.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>Taux CET catégorie A (€/jour)</t>
-        </is>
-      </c>
-      <c r="B20" s="19" t="n">
-        <v>150</v>
+          <t>Catégorie (C, B, A)</t>
+        </is>
+      </c>
+      <c r="B20" s="19" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
       <c r="C20" s="16" t="inlineStr">
         <is>
-          <t>Arrêté 2024 – à vérifier.</t>
+          <t>Pour l'indemnisation CET.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>Enfants à charge &lt; 16 ans (O/N)</t>
-        </is>
-      </c>
-      <c r="B21" s="18" t="inlineStr">
-        <is>
-          <t>O</t>
-        </is>
+          <t>Taux CET catégorie C (€/jour)</t>
+        </is>
+      </c>
+      <c r="B21" s="20" t="n">
+        <v>83</v>
       </c>
       <c r="C21" s="16" t="inlineStr">
         <is>
-          <t>Pour ASA garde d'enfant.</t>
+          <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
+          <t>Taux CET catégorie B (€/jour)</t>
+        </is>
+      </c>
+      <c r="B22" s="20" t="n">
+        <v>100</v>
+      </c>
+      <c r="C22" s="16" t="inlineStr">
+        <is>
+          <t>À vérifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Taux CET catégorie A (€/jour)</t>
+        </is>
+      </c>
+      <c r="B23" s="20" t="n">
+        <v>150</v>
+      </c>
+      <c r="C23" s="16" t="inlineStr">
+        <is>
+          <t>À vérifier.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Enfants à charge &lt; 16 ans (O/N)</t>
+        </is>
+      </c>
+      <c r="B24" s="19" t="inlineStr">
+        <is>
+          <t>O</t>
+        </is>
+      </c>
+      <c r="C24" s="16" t="inlineStr">
+        <is>
+          <t>Pour ASA garde d'enfant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
           <t>Élève seul l'enfant ou conjoint sans droit (O/N)</t>
         </is>
       </c>
-      <c r="B22" s="18" t="inlineStr">
+      <c r="B25" s="19" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C22" s="16" t="inlineStr">
+      <c r="C25" s="16" t="inlineStr">
         <is>
           <t>Doublement ASA garde d'enfant.</t>
         </is>
@@ -1517,10 +1505,10 @@
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation sqref="B17" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"C,B,A"</formula1>
     </dataValidation>
-    <dataValidation sqref="B21 B22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+    <dataValidation sqref="B24 B25" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
       <formula1>"O,N"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1610,2223 +1598,2223 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="20" t="n">
+      <c r="A5" s="21" t="n">
         <v>46063</v>
       </c>
-      <c r="B5" s="20" t="n">
+      <c r="B5" s="21" t="n">
         <v>46066</v>
       </c>
-      <c r="C5" s="21" t="inlineStr">
+      <c r="C5" s="22" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="22" t="n">
         <v>2</v>
       </c>
       <c r="E5" s="11">
         <f>IF(D5="","",D5*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F5" s="21" t="inlineStr">
+      <c r="F5" s="22" t="inlineStr">
         <is>
           <t>Exemple – à effacer</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="20" t="n"/>
-      <c r="B6" s="20" t="n"/>
-      <c r="C6" s="21" t="n"/>
-      <c r="D6" s="21" t="n"/>
+      <c r="A6" s="21" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
       <c r="E6" s="11">
         <f>IF(D6="","",D6*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F6" s="21" t="n"/>
+      <c r="F6" s="22" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="20" t="n"/>
-      <c r="B7" s="20" t="n"/>
-      <c r="C7" s="21" t="n"/>
-      <c r="D7" s="21" t="n"/>
+      <c r="A7" s="21" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="22" t="n"/>
       <c r="E7" s="11">
         <f>IF(D7="","",D7*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F7" s="21" t="n"/>
+      <c r="F7" s="22" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="20" t="n"/>
-      <c r="B8" s="20" t="n"/>
-      <c r="C8" s="21" t="n"/>
-      <c r="D8" s="21" t="n"/>
+      <c r="A8" s="21" t="n"/>
+      <c r="B8" s="21" t="n"/>
+      <c r="C8" s="22" t="n"/>
+      <c r="D8" s="22" t="n"/>
       <c r="E8" s="11">
         <f>IF(D8="","",D8*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F8" s="21" t="n"/>
+      <c r="F8" s="22" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="20" t="n"/>
-      <c r="B9" s="20" t="n"/>
-      <c r="C9" s="21" t="n"/>
-      <c r="D9" s="21" t="n"/>
+      <c r="A9" s="21" t="n"/>
+      <c r="B9" s="21" t="n"/>
+      <c r="C9" s="22" t="n"/>
+      <c r="D9" s="22" t="n"/>
       <c r="E9" s="11">
         <f>IF(D9="","",D9*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F9" s="21" t="n"/>
+      <c r="F9" s="22" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="20" t="n"/>
-      <c r="B10" s="20" t="n"/>
-      <c r="C10" s="21" t="n"/>
-      <c r="D10" s="21" t="n"/>
+      <c r="A10" s="21" t="n"/>
+      <c r="B10" s="21" t="n"/>
+      <c r="C10" s="22" t="n"/>
+      <c r="D10" s="22" t="n"/>
       <c r="E10" s="11">
         <f>IF(D10="","",D10*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F10" s="21" t="n"/>
+      <c r="F10" s="22" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="20" t="n"/>
-      <c r="B11" s="20" t="n"/>
-      <c r="C11" s="21" t="n"/>
-      <c r="D11" s="21" t="n"/>
+      <c r="A11" s="21" t="n"/>
+      <c r="B11" s="21" t="n"/>
+      <c r="C11" s="22" t="n"/>
+      <c r="D11" s="22" t="n"/>
       <c r="E11" s="11">
         <f>IF(D11="","",D11*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F11" s="21" t="n"/>
+      <c r="F11" s="22" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="20" t="n"/>
-      <c r="B12" s="20" t="n"/>
-      <c r="C12" s="21" t="n"/>
-      <c r="D12" s="21" t="n"/>
+      <c r="A12" s="21" t="n"/>
+      <c r="B12" s="21" t="n"/>
+      <c r="C12" s="22" t="n"/>
+      <c r="D12" s="22" t="n"/>
       <c r="E12" s="11">
         <f>IF(D12="","",D12*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F12" s="21" t="n"/>
+      <c r="F12" s="22" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="20" t="n"/>
-      <c r="B13" s="20" t="n"/>
-      <c r="C13" s="21" t="n"/>
-      <c r="D13" s="21" t="n"/>
+      <c r="A13" s="21" t="n"/>
+      <c r="B13" s="21" t="n"/>
+      <c r="C13" s="22" t="n"/>
+      <c r="D13" s="22" t="n"/>
       <c r="E13" s="11">
         <f>IF(D13="","",D13*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F13" s="21" t="n"/>
+      <c r="F13" s="22" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="20" t="n"/>
-      <c r="B14" s="20" t="n"/>
-      <c r="C14" s="21" t="n"/>
-      <c r="D14" s="21" t="n"/>
+      <c r="A14" s="21" t="n"/>
+      <c r="B14" s="21" t="n"/>
+      <c r="C14" s="22" t="n"/>
+      <c r="D14" s="22" t="n"/>
       <c r="E14" s="11">
         <f>IF(D14="","",D14*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F14" s="21" t="n"/>
+      <c r="F14" s="22" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="20" t="n"/>
-      <c r="B15" s="20" t="n"/>
-      <c r="C15" s="21" t="n"/>
-      <c r="D15" s="21" t="n"/>
+      <c r="A15" s="21" t="n"/>
+      <c r="B15" s="21" t="n"/>
+      <c r="C15" s="22" t="n"/>
+      <c r="D15" s="22" t="n"/>
       <c r="E15" s="11">
         <f>IF(D15="","",D15*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F15" s="21" t="n"/>
+      <c r="F15" s="22" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="20" t="n"/>
-      <c r="B16" s="20" t="n"/>
-      <c r="C16" s="21" t="n"/>
-      <c r="D16" s="21" t="n"/>
+      <c r="A16" s="21" t="n"/>
+      <c r="B16" s="21" t="n"/>
+      <c r="C16" s="22" t="n"/>
+      <c r="D16" s="22" t="n"/>
       <c r="E16" s="11">
         <f>IF(D16="","",D16*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F16" s="21" t="n"/>
+      <c r="F16" s="22" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="20" t="n"/>
-      <c r="B17" s="20" t="n"/>
-      <c r="C17" s="21" t="n"/>
-      <c r="D17" s="21" t="n"/>
+      <c r="A17" s="21" t="n"/>
+      <c r="B17" s="21" t="n"/>
+      <c r="C17" s="22" t="n"/>
+      <c r="D17" s="22" t="n"/>
       <c r="E17" s="11">
         <f>IF(D17="","",D17*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F17" s="21" t="n"/>
+      <c r="F17" s="22" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="20" t="n"/>
-      <c r="B18" s="20" t="n"/>
-      <c r="C18" s="21" t="n"/>
-      <c r="D18" s="21" t="n"/>
+      <c r="A18" s="21" t="n"/>
+      <c r="B18" s="21" t="n"/>
+      <c r="C18" s="22" t="n"/>
+      <c r="D18" s="22" t="n"/>
       <c r="E18" s="11">
         <f>IF(D18="","",D18*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F18" s="21" t="n"/>
+      <c r="F18" s="22" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="20" t="n"/>
-      <c r="B19" s="20" t="n"/>
-      <c r="C19" s="21" t="n"/>
-      <c r="D19" s="21" t="n"/>
+      <c r="A19" s="21" t="n"/>
+      <c r="B19" s="21" t="n"/>
+      <c r="C19" s="22" t="n"/>
+      <c r="D19" s="22" t="n"/>
       <c r="E19" s="11">
         <f>IF(D19="","",D19*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F19" s="21" t="n"/>
+      <c r="F19" s="22" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="20" t="n"/>
-      <c r="B20" s="20" t="n"/>
-      <c r="C20" s="21" t="n"/>
-      <c r="D20" s="21" t="n"/>
+      <c r="A20" s="21" t="n"/>
+      <c r="B20" s="21" t="n"/>
+      <c r="C20" s="22" t="n"/>
+      <c r="D20" s="22" t="n"/>
       <c r="E20" s="11">
         <f>IF(D20="","",D20*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F20" s="21" t="n"/>
+      <c r="F20" s="22" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="20" t="n"/>
-      <c r="B21" s="20" t="n"/>
-      <c r="C21" s="21" t="n"/>
-      <c r="D21" s="21" t="n"/>
+      <c r="A21" s="21" t="n"/>
+      <c r="B21" s="21" t="n"/>
+      <c r="C21" s="22" t="n"/>
+      <c r="D21" s="22" t="n"/>
       <c r="E21" s="11">
         <f>IF(D21="","",D21*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F21" s="21" t="n"/>
+      <c r="F21" s="22" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="n"/>
-      <c r="B22" s="20" t="n"/>
-      <c r="C22" s="21" t="n"/>
-      <c r="D22" s="21" t="n"/>
+      <c r="A22" s="21" t="n"/>
+      <c r="B22" s="21" t="n"/>
+      <c r="C22" s="22" t="n"/>
+      <c r="D22" s="22" t="n"/>
       <c r="E22" s="11">
         <f>IF(D22="","",D22*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F22" s="21" t="n"/>
+      <c r="F22" s="22" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="20" t="n"/>
-      <c r="B23" s="20" t="n"/>
-      <c r="C23" s="21" t="n"/>
-      <c r="D23" s="21" t="n"/>
+      <c r="A23" s="21" t="n"/>
+      <c r="B23" s="21" t="n"/>
+      <c r="C23" s="22" t="n"/>
+      <c r="D23" s="22" t="n"/>
       <c r="E23" s="11">
         <f>IF(D23="","",D23*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F23" s="21" t="n"/>
+      <c r="F23" s="22" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="20" t="n"/>
-      <c r="B24" s="20" t="n"/>
-      <c r="C24" s="21" t="n"/>
-      <c r="D24" s="21" t="n"/>
+      <c r="A24" s="21" t="n"/>
+      <c r="B24" s="21" t="n"/>
+      <c r="C24" s="22" t="n"/>
+      <c r="D24" s="22" t="n"/>
       <c r="E24" s="11">
         <f>IF(D24="","",D24*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F24" s="21" t="n"/>
+      <c r="F24" s="22" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="20" t="n"/>
-      <c r="B25" s="20" t="n"/>
-      <c r="C25" s="21" t="n"/>
-      <c r="D25" s="21" t="n"/>
+      <c r="A25" s="21" t="n"/>
+      <c r="B25" s="21" t="n"/>
+      <c r="C25" s="22" t="n"/>
+      <c r="D25" s="22" t="n"/>
       <c r="E25" s="11">
         <f>IF(D25="","",D25*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F25" s="21" t="n"/>
+      <c r="F25" s="22" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="20" t="n"/>
-      <c r="B26" s="20" t="n"/>
-      <c r="C26" s="21" t="n"/>
-      <c r="D26" s="21" t="n"/>
+      <c r="A26" s="21" t="n"/>
+      <c r="B26" s="21" t="n"/>
+      <c r="C26" s="22" t="n"/>
+      <c r="D26" s="22" t="n"/>
       <c r="E26" s="11">
         <f>IF(D26="","",D26*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F26" s="21" t="n"/>
+      <c r="F26" s="22" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="20" t="n"/>
-      <c r="B27" s="20" t="n"/>
-      <c r="C27" s="21" t="n"/>
-      <c r="D27" s="21" t="n"/>
+      <c r="A27" s="21" t="n"/>
+      <c r="B27" s="21" t="n"/>
+      <c r="C27" s="22" t="n"/>
+      <c r="D27" s="22" t="n"/>
       <c r="E27" s="11">
         <f>IF(D27="","",D27*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F27" s="21" t="n"/>
+      <c r="F27" s="22" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="20" t="n"/>
-      <c r="B28" s="20" t="n"/>
-      <c r="C28" s="21" t="n"/>
-      <c r="D28" s="21" t="n"/>
+      <c r="A28" s="21" t="n"/>
+      <c r="B28" s="21" t="n"/>
+      <c r="C28" s="22" t="n"/>
+      <c r="D28" s="22" t="n"/>
       <c r="E28" s="11">
         <f>IF(D28="","",D28*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F28" s="21" t="n"/>
+      <c r="F28" s="22" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="20" t="n"/>
-      <c r="B29" s="20" t="n"/>
-      <c r="C29" s="21" t="n"/>
-      <c r="D29" s="21" t="n"/>
+      <c r="A29" s="21" t="n"/>
+      <c r="B29" s="21" t="n"/>
+      <c r="C29" s="22" t="n"/>
+      <c r="D29" s="22" t="n"/>
       <c r="E29" s="11">
         <f>IF(D29="","",D29*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F29" s="21" t="n"/>
+      <c r="F29" s="22" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="20" t="n"/>
-      <c r="B30" s="20" t="n"/>
-      <c r="C30" s="21" t="n"/>
-      <c r="D30" s="21" t="n"/>
+      <c r="A30" s="21" t="n"/>
+      <c r="B30" s="21" t="n"/>
+      <c r="C30" s="22" t="n"/>
+      <c r="D30" s="22" t="n"/>
       <c r="E30" s="11">
         <f>IF(D30="","",D30*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F30" s="21" t="n"/>
+      <c r="F30" s="22" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="n"/>
-      <c r="B31" s="20" t="n"/>
-      <c r="C31" s="21" t="n"/>
-      <c r="D31" s="21" t="n"/>
+      <c r="A31" s="21" t="n"/>
+      <c r="B31" s="21" t="n"/>
+      <c r="C31" s="22" t="n"/>
+      <c r="D31" s="22" t="n"/>
       <c r="E31" s="11">
         <f>IF(D31="","",D31*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F31" s="21" t="n"/>
+      <c r="F31" s="22" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="20" t="n"/>
-      <c r="B32" s="20" t="n"/>
-      <c r="C32" s="21" t="n"/>
-      <c r="D32" s="21" t="n"/>
+      <c r="A32" s="21" t="n"/>
+      <c r="B32" s="21" t="n"/>
+      <c r="C32" s="22" t="n"/>
+      <c r="D32" s="22" t="n"/>
       <c r="E32" s="11">
         <f>IF(D32="","",D32*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F32" s="21" t="n"/>
+      <c r="F32" s="22" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="20" t="n"/>
-      <c r="B33" s="20" t="n"/>
-      <c r="C33" s="21" t="n"/>
-      <c r="D33" s="21" t="n"/>
+      <c r="A33" s="21" t="n"/>
+      <c r="B33" s="21" t="n"/>
+      <c r="C33" s="22" t="n"/>
+      <c r="D33" s="22" t="n"/>
       <c r="E33" s="11">
         <f>IF(D33="","",D33*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F33" s="21" t="n"/>
+      <c r="F33" s="22" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="20" t="n"/>
-      <c r="B34" s="20" t="n"/>
-      <c r="C34" s="21" t="n"/>
-      <c r="D34" s="21" t="n"/>
+      <c r="A34" s="21" t="n"/>
+      <c r="B34" s="21" t="n"/>
+      <c r="C34" s="22" t="n"/>
+      <c r="D34" s="22" t="n"/>
       <c r="E34" s="11">
         <f>IF(D34="","",D34*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F34" s="21" t="n"/>
+      <c r="F34" s="22" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="20" t="n"/>
-      <c r="B35" s="20" t="n"/>
-      <c r="C35" s="21" t="n"/>
-      <c r="D35" s="21" t="n"/>
+      <c r="A35" s="21" t="n"/>
+      <c r="B35" s="21" t="n"/>
+      <c r="C35" s="22" t="n"/>
+      <c r="D35" s="22" t="n"/>
       <c r="E35" s="11">
         <f>IF(D35="","",D35*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F35" s="21" t="n"/>
+      <c r="F35" s="22" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="20" t="n"/>
-      <c r="B36" s="20" t="n"/>
-      <c r="C36" s="21" t="n"/>
-      <c r="D36" s="21" t="n"/>
+      <c r="A36" s="21" t="n"/>
+      <c r="B36" s="21" t="n"/>
+      <c r="C36" s="22" t="n"/>
+      <c r="D36" s="22" t="n"/>
       <c r="E36" s="11">
         <f>IF(D36="","",D36*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F36" s="21" t="n"/>
+      <c r="F36" s="22" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="20" t="n"/>
-      <c r="B37" s="20" t="n"/>
-      <c r="C37" s="21" t="n"/>
-      <c r="D37" s="21" t="n"/>
+      <c r="A37" s="21" t="n"/>
+      <c r="B37" s="21" t="n"/>
+      <c r="C37" s="22" t="n"/>
+      <c r="D37" s="22" t="n"/>
       <c r="E37" s="11">
         <f>IF(D37="","",D37*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F37" s="21" t="n"/>
+      <c r="F37" s="22" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="20" t="n"/>
-      <c r="B38" s="20" t="n"/>
-      <c r="C38" s="21" t="n"/>
-      <c r="D38" s="21" t="n"/>
+      <c r="A38" s="21" t="n"/>
+      <c r="B38" s="21" t="n"/>
+      <c r="C38" s="22" t="n"/>
+      <c r="D38" s="22" t="n"/>
       <c r="E38" s="11">
         <f>IF(D38="","",D38*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F38" s="21" t="n"/>
+      <c r="F38" s="22" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="20" t="n"/>
-      <c r="B39" s="20" t="n"/>
-      <c r="C39" s="21" t="n"/>
-      <c r="D39" s="21" t="n"/>
+      <c r="A39" s="21" t="n"/>
+      <c r="B39" s="21" t="n"/>
+      <c r="C39" s="22" t="n"/>
+      <c r="D39" s="22" t="n"/>
       <c r="E39" s="11">
         <f>IF(D39="","",D39*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F39" s="21" t="n"/>
+      <c r="F39" s="22" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="20" t="n"/>
-      <c r="B40" s="20" t="n"/>
-      <c r="C40" s="21" t="n"/>
-      <c r="D40" s="21" t="n"/>
+      <c r="A40" s="21" t="n"/>
+      <c r="B40" s="21" t="n"/>
+      <c r="C40" s="22" t="n"/>
+      <c r="D40" s="22" t="n"/>
       <c r="E40" s="11">
         <f>IF(D40="","",D40*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F40" s="21" t="n"/>
+      <c r="F40" s="22" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="20" t="n"/>
-      <c r="B41" s="20" t="n"/>
-      <c r="C41" s="21" t="n"/>
-      <c r="D41" s="21" t="n"/>
+      <c r="A41" s="21" t="n"/>
+      <c r="B41" s="21" t="n"/>
+      <c r="C41" s="22" t="n"/>
+      <c r="D41" s="22" t="n"/>
       <c r="E41" s="11">
         <f>IF(D41="","",D41*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F41" s="21" t="n"/>
+      <c r="F41" s="22" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="20" t="n"/>
-      <c r="B42" s="20" t="n"/>
-      <c r="C42" s="21" t="n"/>
-      <c r="D42" s="21" t="n"/>
+      <c r="A42" s="21" t="n"/>
+      <c r="B42" s="21" t="n"/>
+      <c r="C42" s="22" t="n"/>
+      <c r="D42" s="22" t="n"/>
       <c r="E42" s="11">
         <f>IF(D42="","",D42*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F42" s="21" t="n"/>
+      <c r="F42" s="22" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="20" t="n"/>
-      <c r="B43" s="20" t="n"/>
-      <c r="C43" s="21" t="n"/>
-      <c r="D43" s="21" t="n"/>
+      <c r="A43" s="21" t="n"/>
+      <c r="B43" s="21" t="n"/>
+      <c r="C43" s="22" t="n"/>
+      <c r="D43" s="22" t="n"/>
       <c r="E43" s="11">
         <f>IF(D43="","",D43*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F43" s="21" t="n"/>
+      <c r="F43" s="22" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="20" t="n"/>
-      <c r="B44" s="20" t="n"/>
-      <c r="C44" s="21" t="n"/>
-      <c r="D44" s="21" t="n"/>
+      <c r="A44" s="21" t="n"/>
+      <c r="B44" s="21" t="n"/>
+      <c r="C44" s="22" t="n"/>
+      <c r="D44" s="22" t="n"/>
       <c r="E44" s="11">
         <f>IF(D44="","",D44*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F44" s="21" t="n"/>
+      <c r="F44" s="22" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="20" t="n"/>
-      <c r="B45" s="20" t="n"/>
-      <c r="C45" s="21" t="n"/>
-      <c r="D45" s="21" t="n"/>
+      <c r="A45" s="21" t="n"/>
+      <c r="B45" s="21" t="n"/>
+      <c r="C45" s="22" t="n"/>
+      <c r="D45" s="22" t="n"/>
       <c r="E45" s="11">
         <f>IF(D45="","",D45*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F45" s="21" t="n"/>
+      <c r="F45" s="22" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="20" t="n"/>
-      <c r="B46" s="20" t="n"/>
-      <c r="C46" s="21" t="n"/>
-      <c r="D46" s="21" t="n"/>
+      <c r="A46" s="21" t="n"/>
+      <c r="B46" s="21" t="n"/>
+      <c r="C46" s="22" t="n"/>
+      <c r="D46" s="22" t="n"/>
       <c r="E46" s="11">
         <f>IF(D46="","",D46*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F46" s="21" t="n"/>
+      <c r="F46" s="22" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="20" t="n"/>
-      <c r="B47" s="20" t="n"/>
-      <c r="C47" s="21" t="n"/>
-      <c r="D47" s="21" t="n"/>
+      <c r="A47" s="21" t="n"/>
+      <c r="B47" s="21" t="n"/>
+      <c r="C47" s="22" t="n"/>
+      <c r="D47" s="22" t="n"/>
       <c r="E47" s="11">
         <f>IF(D47="","",D47*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F47" s="21" t="n"/>
+      <c r="F47" s="22" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="20" t="n"/>
-      <c r="B48" s="20" t="n"/>
-      <c r="C48" s="21" t="n"/>
-      <c r="D48" s="21" t="n"/>
+      <c r="A48" s="21" t="n"/>
+      <c r="B48" s="21" t="n"/>
+      <c r="C48" s="22" t="n"/>
+      <c r="D48" s="22" t="n"/>
       <c r="E48" s="11">
         <f>IF(D48="","",D48*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F48" s="21" t="n"/>
+      <c r="F48" s="22" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="20" t="n"/>
-      <c r="B49" s="20" t="n"/>
-      <c r="C49" s="21" t="n"/>
-      <c r="D49" s="21" t="n"/>
+      <c r="A49" s="21" t="n"/>
+      <c r="B49" s="21" t="n"/>
+      <c r="C49" s="22" t="n"/>
+      <c r="D49" s="22" t="n"/>
       <c r="E49" s="11">
         <f>IF(D49="","",D49*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F49" s="21" t="n"/>
+      <c r="F49" s="22" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="20" t="n"/>
-      <c r="B50" s="20" t="n"/>
-      <c r="C50" s="21" t="n"/>
-      <c r="D50" s="21" t="n"/>
+      <c r="A50" s="21" t="n"/>
+      <c r="B50" s="21" t="n"/>
+      <c r="C50" s="22" t="n"/>
+      <c r="D50" s="22" t="n"/>
       <c r="E50" s="11">
         <f>IF(D50="","",D50*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F50" s="21" t="n"/>
+      <c r="F50" s="22" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="20" t="n"/>
-      <c r="B51" s="20" t="n"/>
-      <c r="C51" s="21" t="n"/>
-      <c r="D51" s="21" t="n"/>
+      <c r="A51" s="21" t="n"/>
+      <c r="B51" s="21" t="n"/>
+      <c r="C51" s="22" t="n"/>
+      <c r="D51" s="22" t="n"/>
       <c r="E51" s="11">
         <f>IF(D51="","",D51*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F51" s="21" t="n"/>
+      <c r="F51" s="22" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="20" t="n"/>
-      <c r="B52" s="20" t="n"/>
-      <c r="C52" s="21" t="n"/>
-      <c r="D52" s="21" t="n"/>
+      <c r="A52" s="21" t="n"/>
+      <c r="B52" s="21" t="n"/>
+      <c r="C52" s="22" t="n"/>
+      <c r="D52" s="22" t="n"/>
       <c r="E52" s="11">
         <f>IF(D52="","",D52*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F52" s="21" t="n"/>
+      <c r="F52" s="22" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="20" t="n"/>
-      <c r="B53" s="20" t="n"/>
-      <c r="C53" s="21" t="n"/>
-      <c r="D53" s="21" t="n"/>
+      <c r="A53" s="21" t="n"/>
+      <c r="B53" s="21" t="n"/>
+      <c r="C53" s="22" t="n"/>
+      <c r="D53" s="22" t="n"/>
       <c r="E53" s="11">
         <f>IF(D53="","",D53*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F53" s="21" t="n"/>
+      <c r="F53" s="22" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="20" t="n"/>
-      <c r="B54" s="20" t="n"/>
-      <c r="C54" s="21" t="n"/>
-      <c r="D54" s="21" t="n"/>
+      <c r="A54" s="21" t="n"/>
+      <c r="B54" s="21" t="n"/>
+      <c r="C54" s="22" t="n"/>
+      <c r="D54" s="22" t="n"/>
       <c r="E54" s="11">
         <f>IF(D54="","",D54*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F54" s="21" t="n"/>
+      <c r="F54" s="22" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="20" t="n"/>
-      <c r="B55" s="20" t="n"/>
-      <c r="C55" s="21" t="n"/>
-      <c r="D55" s="21" t="n"/>
+      <c r="A55" s="21" t="n"/>
+      <c r="B55" s="21" t="n"/>
+      <c r="C55" s="22" t="n"/>
+      <c r="D55" s="22" t="n"/>
       <c r="E55" s="11">
         <f>IF(D55="","",D55*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F55" s="21" t="n"/>
+      <c r="F55" s="22" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="20" t="n"/>
-      <c r="B56" s="20" t="n"/>
-      <c r="C56" s="21" t="n"/>
-      <c r="D56" s="21" t="n"/>
+      <c r="A56" s="21" t="n"/>
+      <c r="B56" s="21" t="n"/>
+      <c r="C56" s="22" t="n"/>
+      <c r="D56" s="22" t="n"/>
       <c r="E56" s="11">
         <f>IF(D56="","",D56*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F56" s="21" t="n"/>
+      <c r="F56" s="22" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="20" t="n"/>
-      <c r="B57" s="20" t="n"/>
-      <c r="C57" s="21" t="n"/>
-      <c r="D57" s="21" t="n"/>
+      <c r="A57" s="21" t="n"/>
+      <c r="B57" s="21" t="n"/>
+      <c r="C57" s="22" t="n"/>
+      <c r="D57" s="22" t="n"/>
       <c r="E57" s="11">
         <f>IF(D57="","",D57*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F57" s="21" t="n"/>
+      <c r="F57" s="22" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="20" t="n"/>
-      <c r="B58" s="20" t="n"/>
-      <c r="C58" s="21" t="n"/>
-      <c r="D58" s="21" t="n"/>
+      <c r="A58" s="21" t="n"/>
+      <c r="B58" s="21" t="n"/>
+      <c r="C58" s="22" t="n"/>
+      <c r="D58" s="22" t="n"/>
       <c r="E58" s="11">
         <f>IF(D58="","",D58*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F58" s="21" t="n"/>
+      <c r="F58" s="22" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="20" t="n"/>
-      <c r="B59" s="20" t="n"/>
-      <c r="C59" s="21" t="n"/>
-      <c r="D59" s="21" t="n"/>
+      <c r="A59" s="21" t="n"/>
+      <c r="B59" s="21" t="n"/>
+      <c r="C59" s="22" t="n"/>
+      <c r="D59" s="22" t="n"/>
       <c r="E59" s="11">
         <f>IF(D59="","",D59*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F59" s="21" t="n"/>
+      <c r="F59" s="22" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="20" t="n"/>
-      <c r="B60" s="20" t="n"/>
-      <c r="C60" s="21" t="n"/>
-      <c r="D60" s="21" t="n"/>
+      <c r="A60" s="21" t="n"/>
+      <c r="B60" s="21" t="n"/>
+      <c r="C60" s="22" t="n"/>
+      <c r="D60" s="22" t="n"/>
       <c r="E60" s="11">
         <f>IF(D60="","",D60*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F60" s="21" t="n"/>
+      <c r="F60" s="22" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="20" t="n"/>
-      <c r="B61" s="20" t="n"/>
-      <c r="C61" s="21" t="n"/>
-      <c r="D61" s="21" t="n"/>
+      <c r="A61" s="21" t="n"/>
+      <c r="B61" s="21" t="n"/>
+      <c r="C61" s="22" t="n"/>
+      <c r="D61" s="22" t="n"/>
       <c r="E61" s="11">
         <f>IF(D61="","",D61*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F61" s="21" t="n"/>
+      <c r="F61" s="22" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="20" t="n"/>
-      <c r="B62" s="20" t="n"/>
-      <c r="C62" s="21" t="n"/>
-      <c r="D62" s="21" t="n"/>
+      <c r="A62" s="21" t="n"/>
+      <c r="B62" s="21" t="n"/>
+      <c r="C62" s="22" t="n"/>
+      <c r="D62" s="22" t="n"/>
       <c r="E62" s="11">
         <f>IF(D62="","",D62*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F62" s="21" t="n"/>
+      <c r="F62" s="22" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="20" t="n"/>
-      <c r="B63" s="20" t="n"/>
-      <c r="C63" s="21" t="n"/>
-      <c r="D63" s="21" t="n"/>
+      <c r="A63" s="21" t="n"/>
+      <c r="B63" s="21" t="n"/>
+      <c r="C63" s="22" t="n"/>
+      <c r="D63" s="22" t="n"/>
       <c r="E63" s="11">
         <f>IF(D63="","",D63*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F63" s="21" t="n"/>
+      <c r="F63" s="22" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="20" t="n"/>
-      <c r="B64" s="20" t="n"/>
-      <c r="C64" s="21" t="n"/>
-      <c r="D64" s="21" t="n"/>
+      <c r="A64" s="21" t="n"/>
+      <c r="B64" s="21" t="n"/>
+      <c r="C64" s="22" t="n"/>
+      <c r="D64" s="22" t="n"/>
       <c r="E64" s="11">
         <f>IF(D64="","",D64*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F64" s="21" t="n"/>
+      <c r="F64" s="22" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="20" t="n"/>
-      <c r="B65" s="20" t="n"/>
-      <c r="C65" s="21" t="n"/>
-      <c r="D65" s="21" t="n"/>
+      <c r="A65" s="21" t="n"/>
+      <c r="B65" s="21" t="n"/>
+      <c r="C65" s="22" t="n"/>
+      <c r="D65" s="22" t="n"/>
       <c r="E65" s="11">
         <f>IF(D65="","",D65*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F65" s="21" t="n"/>
+      <c r="F65" s="22" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="20" t="n"/>
-      <c r="B66" s="20" t="n"/>
-      <c r="C66" s="21" t="n"/>
-      <c r="D66" s="21" t="n"/>
+      <c r="A66" s="21" t="n"/>
+      <c r="B66" s="21" t="n"/>
+      <c r="C66" s="22" t="n"/>
+      <c r="D66" s="22" t="n"/>
       <c r="E66" s="11">
         <f>IF(D66="","",D66*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F66" s="21" t="n"/>
+      <c r="F66" s="22" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="20" t="n"/>
-      <c r="B67" s="20" t="n"/>
-      <c r="C67" s="21" t="n"/>
-      <c r="D67" s="21" t="n"/>
+      <c r="A67" s="21" t="n"/>
+      <c r="B67" s="21" t="n"/>
+      <c r="C67" s="22" t="n"/>
+      <c r="D67" s="22" t="n"/>
       <c r="E67" s="11">
         <f>IF(D67="","",D67*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F67" s="21" t="n"/>
+      <c r="F67" s="22" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="20" t="n"/>
-      <c r="B68" s="20" t="n"/>
-      <c r="C68" s="21" t="n"/>
-      <c r="D68" s="21" t="n"/>
+      <c r="A68" s="21" t="n"/>
+      <c r="B68" s="21" t="n"/>
+      <c r="C68" s="22" t="n"/>
+      <c r="D68" s="22" t="n"/>
       <c r="E68" s="11">
         <f>IF(D68="","",D68*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F68" s="21" t="n"/>
+      <c r="F68" s="22" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="20" t="n"/>
-      <c r="B69" s="20" t="n"/>
-      <c r="C69" s="21" t="n"/>
-      <c r="D69" s="21" t="n"/>
+      <c r="A69" s="21" t="n"/>
+      <c r="B69" s="21" t="n"/>
+      <c r="C69" s="22" t="n"/>
+      <c r="D69" s="22" t="n"/>
       <c r="E69" s="11">
         <f>IF(D69="","",D69*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F69" s="21" t="n"/>
+      <c r="F69" s="22" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="20" t="n"/>
-      <c r="B70" s="20" t="n"/>
-      <c r="C70" s="21" t="n"/>
-      <c r="D70" s="21" t="n"/>
+      <c r="A70" s="21" t="n"/>
+      <c r="B70" s="21" t="n"/>
+      <c r="C70" s="22" t="n"/>
+      <c r="D70" s="22" t="n"/>
       <c r="E70" s="11">
         <f>IF(D70="","",D70*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F70" s="21" t="n"/>
+      <c r="F70" s="22" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="20" t="n"/>
-      <c r="B71" s="20" t="n"/>
-      <c r="C71" s="21" t="n"/>
-      <c r="D71" s="21" t="n"/>
+      <c r="A71" s="21" t="n"/>
+      <c r="B71" s="21" t="n"/>
+      <c r="C71" s="22" t="n"/>
+      <c r="D71" s="22" t="n"/>
       <c r="E71" s="11">
         <f>IF(D71="","",D71*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F71" s="21" t="n"/>
+      <c r="F71" s="22" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="20" t="n"/>
-      <c r="B72" s="20" t="n"/>
-      <c r="C72" s="21" t="n"/>
-      <c r="D72" s="21" t="n"/>
+      <c r="A72" s="21" t="n"/>
+      <c r="B72" s="21" t="n"/>
+      <c r="C72" s="22" t="n"/>
+      <c r="D72" s="22" t="n"/>
       <c r="E72" s="11">
         <f>IF(D72="","",D72*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F72" s="21" t="n"/>
+      <c r="F72" s="22" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="20" t="n"/>
-      <c r="B73" s="20" t="n"/>
-      <c r="C73" s="21" t="n"/>
-      <c r="D73" s="21" t="n"/>
+      <c r="A73" s="21" t="n"/>
+      <c r="B73" s="21" t="n"/>
+      <c r="C73" s="22" t="n"/>
+      <c r="D73" s="22" t="n"/>
       <c r="E73" s="11">
         <f>IF(D73="","",D73*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F73" s="21" t="n"/>
+      <c r="F73" s="22" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="20" t="n"/>
-      <c r="B74" s="20" t="n"/>
-      <c r="C74" s="21" t="n"/>
-      <c r="D74" s="21" t="n"/>
+      <c r="A74" s="21" t="n"/>
+      <c r="B74" s="21" t="n"/>
+      <c r="C74" s="22" t="n"/>
+      <c r="D74" s="22" t="n"/>
       <c r="E74" s="11">
         <f>IF(D74="","",D74*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F74" s="21" t="n"/>
+      <c r="F74" s="22" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="20" t="n"/>
-      <c r="B75" s="20" t="n"/>
-      <c r="C75" s="21" t="n"/>
-      <c r="D75" s="21" t="n"/>
+      <c r="A75" s="21" t="n"/>
+      <c r="B75" s="21" t="n"/>
+      <c r="C75" s="22" t="n"/>
+      <c r="D75" s="22" t="n"/>
       <c r="E75" s="11">
         <f>IF(D75="","",D75*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F75" s="21" t="n"/>
+      <c r="F75" s="22" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="20" t="n"/>
-      <c r="B76" s="20" t="n"/>
-      <c r="C76" s="21" t="n"/>
-      <c r="D76" s="21" t="n"/>
+      <c r="A76" s="21" t="n"/>
+      <c r="B76" s="21" t="n"/>
+      <c r="C76" s="22" t="n"/>
+      <c r="D76" s="22" t="n"/>
       <c r="E76" s="11">
         <f>IF(D76="","",D76*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F76" s="21" t="n"/>
+      <c r="F76" s="22" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="20" t="n"/>
-      <c r="B77" s="20" t="n"/>
-      <c r="C77" s="21" t="n"/>
-      <c r="D77" s="21" t="n"/>
+      <c r="A77" s="21" t="n"/>
+      <c r="B77" s="21" t="n"/>
+      <c r="C77" s="22" t="n"/>
+      <c r="D77" s="22" t="n"/>
       <c r="E77" s="11">
         <f>IF(D77="","",D77*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F77" s="21" t="n"/>
+      <c r="F77" s="22" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="20" t="n"/>
-      <c r="B78" s="20" t="n"/>
-      <c r="C78" s="21" t="n"/>
-      <c r="D78" s="21" t="n"/>
+      <c r="A78" s="21" t="n"/>
+      <c r="B78" s="21" t="n"/>
+      <c r="C78" s="22" t="n"/>
+      <c r="D78" s="22" t="n"/>
       <c r="E78" s="11">
         <f>IF(D78="","",D78*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F78" s="21" t="n"/>
+      <c r="F78" s="22" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="20" t="n"/>
-      <c r="B79" s="20" t="n"/>
-      <c r="C79" s="21" t="n"/>
-      <c r="D79" s="21" t="n"/>
+      <c r="A79" s="21" t="n"/>
+      <c r="B79" s="21" t="n"/>
+      <c r="C79" s="22" t="n"/>
+      <c r="D79" s="22" t="n"/>
       <c r="E79" s="11">
         <f>IF(D79="","",D79*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F79" s="21" t="n"/>
+      <c r="F79" s="22" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="20" t="n"/>
-      <c r="B80" s="20" t="n"/>
-      <c r="C80" s="21" t="n"/>
-      <c r="D80" s="21" t="n"/>
+      <c r="A80" s="21" t="n"/>
+      <c r="B80" s="21" t="n"/>
+      <c r="C80" s="22" t="n"/>
+      <c r="D80" s="22" t="n"/>
       <c r="E80" s="11">
         <f>IF(D80="","",D80*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F80" s="21" t="n"/>
+      <c r="F80" s="22" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="20" t="n"/>
-      <c r="B81" s="20" t="n"/>
-      <c r="C81" s="21" t="n"/>
-      <c r="D81" s="21" t="n"/>
+      <c r="A81" s="21" t="n"/>
+      <c r="B81" s="21" t="n"/>
+      <c r="C81" s="22" t="n"/>
+      <c r="D81" s="22" t="n"/>
       <c r="E81" s="11">
         <f>IF(D81="","",D81*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F81" s="21" t="n"/>
+      <c r="F81" s="22" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="20" t="n"/>
-      <c r="B82" s="20" t="n"/>
-      <c r="C82" s="21" t="n"/>
-      <c r="D82" s="21" t="n"/>
+      <c r="A82" s="21" t="n"/>
+      <c r="B82" s="21" t="n"/>
+      <c r="C82" s="22" t="n"/>
+      <c r="D82" s="22" t="n"/>
       <c r="E82" s="11">
         <f>IF(D82="","",D82*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F82" s="21" t="n"/>
+      <c r="F82" s="22" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="20" t="n"/>
-      <c r="B83" s="20" t="n"/>
-      <c r="C83" s="21" t="n"/>
-      <c r="D83" s="21" t="n"/>
+      <c r="A83" s="21" t="n"/>
+      <c r="B83" s="21" t="n"/>
+      <c r="C83" s="22" t="n"/>
+      <c r="D83" s="22" t="n"/>
       <c r="E83" s="11">
         <f>IF(D83="","",D83*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F83" s="21" t="n"/>
+      <c r="F83" s="22" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="20" t="n"/>
-      <c r="B84" s="20" t="n"/>
-      <c r="C84" s="21" t="n"/>
-      <c r="D84" s="21" t="n"/>
+      <c r="A84" s="21" t="n"/>
+      <c r="B84" s="21" t="n"/>
+      <c r="C84" s="22" t="n"/>
+      <c r="D84" s="22" t="n"/>
       <c r="E84" s="11">
         <f>IF(D84="","",D84*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F84" s="21" t="n"/>
+      <c r="F84" s="22" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="20" t="n"/>
-      <c r="B85" s="20" t="n"/>
-      <c r="C85" s="21" t="n"/>
-      <c r="D85" s="21" t="n"/>
+      <c r="A85" s="21" t="n"/>
+      <c r="B85" s="21" t="n"/>
+      <c r="C85" s="22" t="n"/>
+      <c r="D85" s="22" t="n"/>
       <c r="E85" s="11">
         <f>IF(D85="","",D85*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F85" s="21" t="n"/>
+      <c r="F85" s="22" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="20" t="n"/>
-      <c r="B86" s="20" t="n"/>
-      <c r="C86" s="21" t="n"/>
-      <c r="D86" s="21" t="n"/>
+      <c r="A86" s="21" t="n"/>
+      <c r="B86" s="21" t="n"/>
+      <c r="C86" s="22" t="n"/>
+      <c r="D86" s="22" t="n"/>
       <c r="E86" s="11">
         <f>IF(D86="","",D86*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F86" s="21" t="n"/>
+      <c r="F86" s="22" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="20" t="n"/>
-      <c r="B87" s="20" t="n"/>
-      <c r="C87" s="21" t="n"/>
-      <c r="D87" s="21" t="n"/>
+      <c r="A87" s="21" t="n"/>
+      <c r="B87" s="21" t="n"/>
+      <c r="C87" s="22" t="n"/>
+      <c r="D87" s="22" t="n"/>
       <c r="E87" s="11">
         <f>IF(D87="","",D87*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F87" s="21" t="n"/>
+      <c r="F87" s="22" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="20" t="n"/>
-      <c r="B88" s="20" t="n"/>
-      <c r="C88" s="21" t="n"/>
-      <c r="D88" s="21" t="n"/>
+      <c r="A88" s="21" t="n"/>
+      <c r="B88" s="21" t="n"/>
+      <c r="C88" s="22" t="n"/>
+      <c r="D88" s="22" t="n"/>
       <c r="E88" s="11">
         <f>IF(D88="","",D88*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F88" s="21" t="n"/>
+      <c r="F88" s="22" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="20" t="n"/>
-      <c r="B89" s="20" t="n"/>
-      <c r="C89" s="21" t="n"/>
-      <c r="D89" s="21" t="n"/>
+      <c r="A89" s="21" t="n"/>
+      <c r="B89" s="21" t="n"/>
+      <c r="C89" s="22" t="n"/>
+      <c r="D89" s="22" t="n"/>
       <c r="E89" s="11">
         <f>IF(D89="","",D89*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F89" s="21" t="n"/>
+      <c r="F89" s="22" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="20" t="n"/>
-      <c r="B90" s="20" t="n"/>
-      <c r="C90" s="21" t="n"/>
-      <c r="D90" s="21" t="n"/>
+      <c r="A90" s="21" t="n"/>
+      <c r="B90" s="21" t="n"/>
+      <c r="C90" s="22" t="n"/>
+      <c r="D90" s="22" t="n"/>
       <c r="E90" s="11">
         <f>IF(D90="","",D90*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F90" s="21" t="n"/>
+      <c r="F90" s="22" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="20" t="n"/>
-      <c r="B91" s="20" t="n"/>
-      <c r="C91" s="21" t="n"/>
-      <c r="D91" s="21" t="n"/>
+      <c r="A91" s="21" t="n"/>
+      <c r="B91" s="21" t="n"/>
+      <c r="C91" s="22" t="n"/>
+      <c r="D91" s="22" t="n"/>
       <c r="E91" s="11">
         <f>IF(D91="","",D91*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F91" s="21" t="n"/>
+      <c r="F91" s="22" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="20" t="n"/>
-      <c r="B92" s="20" t="n"/>
-      <c r="C92" s="21" t="n"/>
-      <c r="D92" s="21" t="n"/>
+      <c r="A92" s="21" t="n"/>
+      <c r="B92" s="21" t="n"/>
+      <c r="C92" s="22" t="n"/>
+      <c r="D92" s="22" t="n"/>
       <c r="E92" s="11">
         <f>IF(D92="","",D92*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F92" s="21" t="n"/>
+      <c r="F92" s="22" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="20" t="n"/>
-      <c r="B93" s="20" t="n"/>
-      <c r="C93" s="21" t="n"/>
-      <c r="D93" s="21" t="n"/>
+      <c r="A93" s="21" t="n"/>
+      <c r="B93" s="21" t="n"/>
+      <c r="C93" s="22" t="n"/>
+      <c r="D93" s="22" t="n"/>
       <c r="E93" s="11">
         <f>IF(D93="","",D93*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F93" s="21" t="n"/>
+      <c r="F93" s="22" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="20" t="n"/>
-      <c r="B94" s="20" t="n"/>
-      <c r="C94" s="21" t="n"/>
-      <c r="D94" s="21" t="n"/>
+      <c r="A94" s="21" t="n"/>
+      <c r="B94" s="21" t="n"/>
+      <c r="C94" s="22" t="n"/>
+      <c r="D94" s="22" t="n"/>
       <c r="E94" s="11">
         <f>IF(D94="","",D94*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F94" s="21" t="n"/>
+      <c r="F94" s="22" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="20" t="n"/>
-      <c r="B95" s="20" t="n"/>
-      <c r="C95" s="21" t="n"/>
-      <c r="D95" s="21" t="n"/>
+      <c r="A95" s="21" t="n"/>
+      <c r="B95" s="21" t="n"/>
+      <c r="C95" s="22" t="n"/>
+      <c r="D95" s="22" t="n"/>
       <c r="E95" s="11">
         <f>IF(D95="","",D95*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F95" s="21" t="n"/>
+      <c r="F95" s="22" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="20" t="n"/>
-      <c r="B96" s="20" t="n"/>
-      <c r="C96" s="21" t="n"/>
-      <c r="D96" s="21" t="n"/>
+      <c r="A96" s="21" t="n"/>
+      <c r="B96" s="21" t="n"/>
+      <c r="C96" s="22" t="n"/>
+      <c r="D96" s="22" t="n"/>
       <c r="E96" s="11">
         <f>IF(D96="","",D96*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F96" s="21" t="n"/>
+      <c r="F96" s="22" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="20" t="n"/>
-      <c r="B97" s="20" t="n"/>
-      <c r="C97" s="21" t="n"/>
-      <c r="D97" s="21" t="n"/>
+      <c r="A97" s="21" t="n"/>
+      <c r="B97" s="21" t="n"/>
+      <c r="C97" s="22" t="n"/>
+      <c r="D97" s="22" t="n"/>
       <c r="E97" s="11">
         <f>IF(D97="","",D97*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F97" s="21" t="n"/>
+      <c r="F97" s="22" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="20" t="n"/>
-      <c r="B98" s="20" t="n"/>
-      <c r="C98" s="21" t="n"/>
-      <c r="D98" s="21" t="n"/>
+      <c r="A98" s="21" t="n"/>
+      <c r="B98" s="21" t="n"/>
+      <c r="C98" s="22" t="n"/>
+      <c r="D98" s="22" t="n"/>
       <c r="E98" s="11">
         <f>IF(D98="","",D98*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F98" s="21" t="n"/>
+      <c r="F98" s="22" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="20" t="n"/>
-      <c r="B99" s="20" t="n"/>
-      <c r="C99" s="21" t="n"/>
-      <c r="D99" s="21" t="n"/>
+      <c r="A99" s="21" t="n"/>
+      <c r="B99" s="21" t="n"/>
+      <c r="C99" s="22" t="n"/>
+      <c r="D99" s="22" t="n"/>
       <c r="E99" s="11">
         <f>IF(D99="","",D99*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F99" s="21" t="n"/>
+      <c r="F99" s="22" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="20" t="n"/>
-      <c r="B100" s="20" t="n"/>
-      <c r="C100" s="21" t="n"/>
-      <c r="D100" s="21" t="n"/>
+      <c r="A100" s="21" t="n"/>
+      <c r="B100" s="21" t="n"/>
+      <c r="C100" s="22" t="n"/>
+      <c r="D100" s="22" t="n"/>
       <c r="E100" s="11">
         <f>IF(D100="","",D100*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F100" s="21" t="n"/>
+      <c r="F100" s="22" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="20" t="n"/>
-      <c r="B101" s="20" t="n"/>
-      <c r="C101" s="21" t="n"/>
-      <c r="D101" s="21" t="n"/>
+      <c r="A101" s="21" t="n"/>
+      <c r="B101" s="21" t="n"/>
+      <c r="C101" s="22" t="n"/>
+      <c r="D101" s="22" t="n"/>
       <c r="E101" s="11">
         <f>IF(D101="","",D101*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F101" s="21" t="n"/>
+      <c r="F101" s="22" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="20" t="n"/>
-      <c r="B102" s="20" t="n"/>
-      <c r="C102" s="21" t="n"/>
-      <c r="D102" s="21" t="n"/>
+      <c r="A102" s="21" t="n"/>
+      <c r="B102" s="21" t="n"/>
+      <c r="C102" s="22" t="n"/>
+      <c r="D102" s="22" t="n"/>
       <c r="E102" s="11">
         <f>IF(D102="","",D102*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F102" s="21" t="n"/>
+      <c r="F102" s="22" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="20" t="n"/>
-      <c r="B103" s="20" t="n"/>
-      <c r="C103" s="21" t="n"/>
-      <c r="D103" s="21" t="n"/>
+      <c r="A103" s="21" t="n"/>
+      <c r="B103" s="21" t="n"/>
+      <c r="C103" s="22" t="n"/>
+      <c r="D103" s="22" t="n"/>
       <c r="E103" s="11">
         <f>IF(D103="","",D103*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F103" s="21" t="n"/>
+      <c r="F103" s="22" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="20" t="n"/>
-      <c r="B104" s="20" t="n"/>
-      <c r="C104" s="21" t="n"/>
-      <c r="D104" s="21" t="n"/>
+      <c r="A104" s="21" t="n"/>
+      <c r="B104" s="21" t="n"/>
+      <c r="C104" s="22" t="n"/>
+      <c r="D104" s="22" t="n"/>
       <c r="E104" s="11">
         <f>IF(D104="","",D104*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F104" s="21" t="n"/>
+      <c r="F104" s="22" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="20" t="n"/>
-      <c r="B105" s="20" t="n"/>
-      <c r="C105" s="21" t="n"/>
-      <c r="D105" s="21" t="n"/>
+      <c r="A105" s="21" t="n"/>
+      <c r="B105" s="21" t="n"/>
+      <c r="C105" s="22" t="n"/>
+      <c r="D105" s="22" t="n"/>
       <c r="E105" s="11">
         <f>IF(D105="","",D105*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F105" s="21" t="n"/>
+      <c r="F105" s="22" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="20" t="n"/>
-      <c r="B106" s="20" t="n"/>
-      <c r="C106" s="21" t="n"/>
-      <c r="D106" s="21" t="n"/>
+      <c r="A106" s="21" t="n"/>
+      <c r="B106" s="21" t="n"/>
+      <c r="C106" s="22" t="n"/>
+      <c r="D106" s="22" t="n"/>
       <c r="E106" s="11">
         <f>IF(D106="","",D106*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F106" s="21" t="n"/>
+      <c r="F106" s="22" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="20" t="n"/>
-      <c r="B107" s="20" t="n"/>
-      <c r="C107" s="21" t="n"/>
-      <c r="D107" s="21" t="n"/>
+      <c r="A107" s="21" t="n"/>
+      <c r="B107" s="21" t="n"/>
+      <c r="C107" s="22" t="n"/>
+      <c r="D107" s="22" t="n"/>
       <c r="E107" s="11">
         <f>IF(D107="","",D107*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F107" s="21" t="n"/>
+      <c r="F107" s="22" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="20" t="n"/>
-      <c r="B108" s="20" t="n"/>
-      <c r="C108" s="21" t="n"/>
-      <c r="D108" s="21" t="n"/>
+      <c r="A108" s="21" t="n"/>
+      <c r="B108" s="21" t="n"/>
+      <c r="C108" s="22" t="n"/>
+      <c r="D108" s="22" t="n"/>
       <c r="E108" s="11">
         <f>IF(D108="","",D108*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F108" s="21" t="n"/>
+      <c r="F108" s="22" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="20" t="n"/>
-      <c r="B109" s="20" t="n"/>
-      <c r="C109" s="21" t="n"/>
-      <c r="D109" s="21" t="n"/>
+      <c r="A109" s="21" t="n"/>
+      <c r="B109" s="21" t="n"/>
+      <c r="C109" s="22" t="n"/>
+      <c r="D109" s="22" t="n"/>
       <c r="E109" s="11">
         <f>IF(D109="","",D109*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F109" s="21" t="n"/>
+      <c r="F109" s="22" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="20" t="n"/>
-      <c r="B110" s="20" t="n"/>
-      <c r="C110" s="21" t="n"/>
-      <c r="D110" s="21" t="n"/>
+      <c r="A110" s="21" t="n"/>
+      <c r="B110" s="21" t="n"/>
+      <c r="C110" s="22" t="n"/>
+      <c r="D110" s="22" t="n"/>
       <c r="E110" s="11">
         <f>IF(D110="","",D110*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F110" s="21" t="n"/>
+      <c r="F110" s="22" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="20" t="n"/>
-      <c r="B111" s="20" t="n"/>
-      <c r="C111" s="21" t="n"/>
-      <c r="D111" s="21" t="n"/>
+      <c r="A111" s="21" t="n"/>
+      <c r="B111" s="21" t="n"/>
+      <c r="C111" s="22" t="n"/>
+      <c r="D111" s="22" t="n"/>
       <c r="E111" s="11">
         <f>IF(D111="","",D111*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F111" s="21" t="n"/>
+      <c r="F111" s="22" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="20" t="n"/>
-      <c r="B112" s="20" t="n"/>
-      <c r="C112" s="21" t="n"/>
-      <c r="D112" s="21" t="n"/>
+      <c r="A112" s="21" t="n"/>
+      <c r="B112" s="21" t="n"/>
+      <c r="C112" s="22" t="n"/>
+      <c r="D112" s="22" t="n"/>
       <c r="E112" s="11">
         <f>IF(D112="","",D112*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F112" s="21" t="n"/>
+      <c r="F112" s="22" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="20" t="n"/>
-      <c r="B113" s="20" t="n"/>
-      <c r="C113" s="21" t="n"/>
-      <c r="D113" s="21" t="n"/>
+      <c r="A113" s="21" t="n"/>
+      <c r="B113" s="21" t="n"/>
+      <c r="C113" s="22" t="n"/>
+      <c r="D113" s="22" t="n"/>
       <c r="E113" s="11">
         <f>IF(D113="","",D113*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F113" s="21" t="n"/>
+      <c r="F113" s="22" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="20" t="n"/>
-      <c r="B114" s="20" t="n"/>
-      <c r="C114" s="21" t="n"/>
-      <c r="D114" s="21" t="n"/>
+      <c r="A114" s="21" t="n"/>
+      <c r="B114" s="21" t="n"/>
+      <c r="C114" s="22" t="n"/>
+      <c r="D114" s="22" t="n"/>
       <c r="E114" s="11">
         <f>IF(D114="","",D114*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F114" s="21" t="n"/>
+      <c r="F114" s="22" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="20" t="n"/>
-      <c r="B115" s="20" t="n"/>
-      <c r="C115" s="21" t="n"/>
-      <c r="D115" s="21" t="n"/>
+      <c r="A115" s="21" t="n"/>
+      <c r="B115" s="21" t="n"/>
+      <c r="C115" s="22" t="n"/>
+      <c r="D115" s="22" t="n"/>
       <c r="E115" s="11">
         <f>IF(D115="","",D115*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F115" s="21" t="n"/>
+      <c r="F115" s="22" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="20" t="n"/>
-      <c r="B116" s="20" t="n"/>
-      <c r="C116" s="21" t="n"/>
-      <c r="D116" s="21" t="n"/>
+      <c r="A116" s="21" t="n"/>
+      <c r="B116" s="21" t="n"/>
+      <c r="C116" s="22" t="n"/>
+      <c r="D116" s="22" t="n"/>
       <c r="E116" s="11">
         <f>IF(D116="","",D116*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F116" s="21" t="n"/>
+      <c r="F116" s="22" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="20" t="n"/>
-      <c r="B117" s="20" t="n"/>
-      <c r="C117" s="21" t="n"/>
-      <c r="D117" s="21" t="n"/>
+      <c r="A117" s="21" t="n"/>
+      <c r="B117" s="21" t="n"/>
+      <c r="C117" s="22" t="n"/>
+      <c r="D117" s="22" t="n"/>
       <c r="E117" s="11">
         <f>IF(D117="","",D117*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F117" s="21" t="n"/>
+      <c r="F117" s="22" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="20" t="n"/>
-      <c r="B118" s="20" t="n"/>
-      <c r="C118" s="21" t="n"/>
-      <c r="D118" s="21" t="n"/>
+      <c r="A118" s="21" t="n"/>
+      <c r="B118" s="21" t="n"/>
+      <c r="C118" s="22" t="n"/>
+      <c r="D118" s="22" t="n"/>
       <c r="E118" s="11">
         <f>IF(D118="","",D118*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F118" s="21" t="n"/>
+      <c r="F118" s="22" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="20" t="n"/>
-      <c r="B119" s="20" t="n"/>
-      <c r="C119" s="21" t="n"/>
-      <c r="D119" s="21" t="n"/>
+      <c r="A119" s="21" t="n"/>
+      <c r="B119" s="21" t="n"/>
+      <c r="C119" s="22" t="n"/>
+      <c r="D119" s="22" t="n"/>
       <c r="E119" s="11">
         <f>IF(D119="","",D119*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F119" s="21" t="n"/>
+      <c r="F119" s="22" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="20" t="n"/>
-      <c r="B120" s="20" t="n"/>
-      <c r="C120" s="21" t="n"/>
-      <c r="D120" s="21" t="n"/>
+      <c r="A120" s="21" t="n"/>
+      <c r="B120" s="21" t="n"/>
+      <c r="C120" s="22" t="n"/>
+      <c r="D120" s="22" t="n"/>
       <c r="E120" s="11">
         <f>IF(D120="","",D120*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F120" s="21" t="n"/>
+      <c r="F120" s="22" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="20" t="n"/>
-      <c r="B121" s="20" t="n"/>
-      <c r="C121" s="21" t="n"/>
-      <c r="D121" s="21" t="n"/>
+      <c r="A121" s="21" t="n"/>
+      <c r="B121" s="21" t="n"/>
+      <c r="C121" s="22" t="n"/>
+      <c r="D121" s="22" t="n"/>
       <c r="E121" s="11">
         <f>IF(D121="","",D121*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F121" s="21" t="n"/>
+      <c r="F121" s="22" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="20" t="n"/>
-      <c r="B122" s="20" t="n"/>
-      <c r="C122" s="21" t="n"/>
-      <c r="D122" s="21" t="n"/>
+      <c r="A122" s="21" t="n"/>
+      <c r="B122" s="21" t="n"/>
+      <c r="C122" s="22" t="n"/>
+      <c r="D122" s="22" t="n"/>
       <c r="E122" s="11">
         <f>IF(D122="","",D122*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F122" s="21" t="n"/>
+      <c r="F122" s="22" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="20" t="n"/>
-      <c r="B123" s="20" t="n"/>
-      <c r="C123" s="21" t="n"/>
-      <c r="D123" s="21" t="n"/>
+      <c r="A123" s="21" t="n"/>
+      <c r="B123" s="21" t="n"/>
+      <c r="C123" s="22" t="n"/>
+      <c r="D123" s="22" t="n"/>
       <c r="E123" s="11">
         <f>IF(D123="","",D123*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F123" s="21" t="n"/>
+      <c r="F123" s="22" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="20" t="n"/>
-      <c r="B124" s="20" t="n"/>
-      <c r="C124" s="21" t="n"/>
-      <c r="D124" s="21" t="n"/>
+      <c r="A124" s="21" t="n"/>
+      <c r="B124" s="21" t="n"/>
+      <c r="C124" s="22" t="n"/>
+      <c r="D124" s="22" t="n"/>
       <c r="E124" s="11">
         <f>IF(D124="","",D124*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F124" s="21" t="n"/>
+      <c r="F124" s="22" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="20" t="n"/>
-      <c r="B125" s="20" t="n"/>
-      <c r="C125" s="21" t="n"/>
-      <c r="D125" s="21" t="n"/>
+      <c r="A125" s="21" t="n"/>
+      <c r="B125" s="21" t="n"/>
+      <c r="C125" s="22" t="n"/>
+      <c r="D125" s="22" t="n"/>
       <c r="E125" s="11">
         <f>IF(D125="","",D125*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F125" s="21" t="n"/>
+      <c r="F125" s="22" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="20" t="n"/>
-      <c r="B126" s="20" t="n"/>
-      <c r="C126" s="21" t="n"/>
-      <c r="D126" s="21" t="n"/>
+      <c r="A126" s="21" t="n"/>
+      <c r="B126" s="21" t="n"/>
+      <c r="C126" s="22" t="n"/>
+      <c r="D126" s="22" t="n"/>
       <c r="E126" s="11">
         <f>IF(D126="","",D126*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F126" s="21" t="n"/>
+      <c r="F126" s="22" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="20" t="n"/>
-      <c r="B127" s="20" t="n"/>
-      <c r="C127" s="21" t="n"/>
-      <c r="D127" s="21" t="n"/>
+      <c r="A127" s="21" t="n"/>
+      <c r="B127" s="21" t="n"/>
+      <c r="C127" s="22" t="n"/>
+      <c r="D127" s="22" t="n"/>
       <c r="E127" s="11">
         <f>IF(D127="","",D127*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F127" s="21" t="n"/>
+      <c r="F127" s="22" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="20" t="n"/>
-      <c r="B128" s="20" t="n"/>
-      <c r="C128" s="21" t="n"/>
-      <c r="D128" s="21" t="n"/>
+      <c r="A128" s="21" t="n"/>
+      <c r="B128" s="21" t="n"/>
+      <c r="C128" s="22" t="n"/>
+      <c r="D128" s="22" t="n"/>
       <c r="E128" s="11">
         <f>IF(D128="","",D128*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F128" s="21" t="n"/>
+      <c r="F128" s="22" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="20" t="n"/>
-      <c r="B129" s="20" t="n"/>
-      <c r="C129" s="21" t="n"/>
-      <c r="D129" s="21" t="n"/>
+      <c r="A129" s="21" t="n"/>
+      <c r="B129" s="21" t="n"/>
+      <c r="C129" s="22" t="n"/>
+      <c r="D129" s="22" t="n"/>
       <c r="E129" s="11">
         <f>IF(D129="","",D129*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F129" s="21" t="n"/>
+      <c r="F129" s="22" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="20" t="n"/>
-      <c r="B130" s="20" t="n"/>
-      <c r="C130" s="21" t="n"/>
-      <c r="D130" s="21" t="n"/>
+      <c r="A130" s="21" t="n"/>
+      <c r="B130" s="21" t="n"/>
+      <c r="C130" s="22" t="n"/>
+      <c r="D130" s="22" t="n"/>
       <c r="E130" s="11">
         <f>IF(D130="","",D130*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F130" s="21" t="n"/>
+      <c r="F130" s="22" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="20" t="n"/>
-      <c r="B131" s="20" t="n"/>
-      <c r="C131" s="21" t="n"/>
-      <c r="D131" s="21" t="n"/>
+      <c r="A131" s="21" t="n"/>
+      <c r="B131" s="21" t="n"/>
+      <c r="C131" s="22" t="n"/>
+      <c r="D131" s="22" t="n"/>
       <c r="E131" s="11">
         <f>IF(D131="","",D131*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F131" s="21" t="n"/>
+      <c r="F131" s="22" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="20" t="n"/>
-      <c r="B132" s="20" t="n"/>
-      <c r="C132" s="21" t="n"/>
-      <c r="D132" s="21" t="n"/>
+      <c r="A132" s="21" t="n"/>
+      <c r="B132" s="21" t="n"/>
+      <c r="C132" s="22" t="n"/>
+      <c r="D132" s="22" t="n"/>
       <c r="E132" s="11">
         <f>IF(D132="","",D132*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F132" s="21" t="n"/>
+      <c r="F132" s="22" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="20" t="n"/>
-      <c r="B133" s="20" t="n"/>
-      <c r="C133" s="21" t="n"/>
-      <c r="D133" s="21" t="n"/>
+      <c r="A133" s="21" t="n"/>
+      <c r="B133" s="21" t="n"/>
+      <c r="C133" s="22" t="n"/>
+      <c r="D133" s="22" t="n"/>
       <c r="E133" s="11">
         <f>IF(D133="","",D133*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F133" s="21" t="n"/>
+      <c r="F133" s="22" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="20" t="n"/>
-      <c r="B134" s="20" t="n"/>
-      <c r="C134" s="21" t="n"/>
-      <c r="D134" s="21" t="n"/>
+      <c r="A134" s="21" t="n"/>
+      <c r="B134" s="21" t="n"/>
+      <c r="C134" s="22" t="n"/>
+      <c r="D134" s="22" t="n"/>
       <c r="E134" s="11">
         <f>IF(D134="","",D134*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F134" s="21" t="n"/>
+      <c r="F134" s="22" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="20" t="n"/>
-      <c r="B135" s="20" t="n"/>
-      <c r="C135" s="21" t="n"/>
-      <c r="D135" s="21" t="n"/>
+      <c r="A135" s="21" t="n"/>
+      <c r="B135" s="21" t="n"/>
+      <c r="C135" s="22" t="n"/>
+      <c r="D135" s="22" t="n"/>
       <c r="E135" s="11">
         <f>IF(D135="","",D135*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F135" s="21" t="n"/>
+      <c r="F135" s="22" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="20" t="n"/>
-      <c r="B136" s="20" t="n"/>
-      <c r="C136" s="21" t="n"/>
-      <c r="D136" s="21" t="n"/>
+      <c r="A136" s="21" t="n"/>
+      <c r="B136" s="21" t="n"/>
+      <c r="C136" s="22" t="n"/>
+      <c r="D136" s="22" t="n"/>
       <c r="E136" s="11">
         <f>IF(D136="","",D136*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F136" s="21" t="n"/>
+      <c r="F136" s="22" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="20" t="n"/>
-      <c r="B137" s="20" t="n"/>
-      <c r="C137" s="21" t="n"/>
-      <c r="D137" s="21" t="n"/>
+      <c r="A137" s="21" t="n"/>
+      <c r="B137" s="21" t="n"/>
+      <c r="C137" s="22" t="n"/>
+      <c r="D137" s="22" t="n"/>
       <c r="E137" s="11">
         <f>IF(D137="","",D137*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F137" s="21" t="n"/>
+      <c r="F137" s="22" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="20" t="n"/>
-      <c r="B138" s="20" t="n"/>
-      <c r="C138" s="21" t="n"/>
-      <c r="D138" s="21" t="n"/>
+      <c r="A138" s="21" t="n"/>
+      <c r="B138" s="21" t="n"/>
+      <c r="C138" s="22" t="n"/>
+      <c r="D138" s="22" t="n"/>
       <c r="E138" s="11">
         <f>IF(D138="","",D138*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F138" s="21" t="n"/>
+      <c r="F138" s="22" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="20" t="n"/>
-      <c r="B139" s="20" t="n"/>
-      <c r="C139" s="21" t="n"/>
-      <c r="D139" s="21" t="n"/>
+      <c r="A139" s="21" t="n"/>
+      <c r="B139" s="21" t="n"/>
+      <c r="C139" s="22" t="n"/>
+      <c r="D139" s="22" t="n"/>
       <c r="E139" s="11">
         <f>IF(D139="","",D139*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F139" s="21" t="n"/>
+      <c r="F139" s="22" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="20" t="n"/>
-      <c r="B140" s="20" t="n"/>
-      <c r="C140" s="21" t="n"/>
-      <c r="D140" s="21" t="n"/>
+      <c r="A140" s="21" t="n"/>
+      <c r="B140" s="21" t="n"/>
+      <c r="C140" s="22" t="n"/>
+      <c r="D140" s="22" t="n"/>
       <c r="E140" s="11">
         <f>IF(D140="","",D140*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F140" s="21" t="n"/>
+      <c r="F140" s="22" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="20" t="n"/>
-      <c r="B141" s="20" t="n"/>
-      <c r="C141" s="21" t="n"/>
-      <c r="D141" s="21" t="n"/>
+      <c r="A141" s="21" t="n"/>
+      <c r="B141" s="21" t="n"/>
+      <c r="C141" s="22" t="n"/>
+      <c r="D141" s="22" t="n"/>
       <c r="E141" s="11">
         <f>IF(D141="","",D141*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F141" s="21" t="n"/>
+      <c r="F141" s="22" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="20" t="n"/>
-      <c r="B142" s="20" t="n"/>
-      <c r="C142" s="21" t="n"/>
-      <c r="D142" s="21" t="n"/>
+      <c r="A142" s="21" t="n"/>
+      <c r="B142" s="21" t="n"/>
+      <c r="C142" s="22" t="n"/>
+      <c r="D142" s="22" t="n"/>
       <c r="E142" s="11">
         <f>IF(D142="","",D142*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F142" s="21" t="n"/>
+      <c r="F142" s="22" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="20" t="n"/>
-      <c r="B143" s="20" t="n"/>
-      <c r="C143" s="21" t="n"/>
-      <c r="D143" s="21" t="n"/>
+      <c r="A143" s="21" t="n"/>
+      <c r="B143" s="21" t="n"/>
+      <c r="C143" s="22" t="n"/>
+      <c r="D143" s="22" t="n"/>
       <c r="E143" s="11">
         <f>IF(D143="","",D143*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F143" s="21" t="n"/>
+      <c r="F143" s="22" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="20" t="n"/>
-      <c r="B144" s="20" t="n"/>
-      <c r="C144" s="21" t="n"/>
-      <c r="D144" s="21" t="n"/>
+      <c r="A144" s="21" t="n"/>
+      <c r="B144" s="21" t="n"/>
+      <c r="C144" s="22" t="n"/>
+      <c r="D144" s="22" t="n"/>
       <c r="E144" s="11">
         <f>IF(D144="","",D144*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F144" s="21" t="n"/>
+      <c r="F144" s="22" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="20" t="n"/>
-      <c r="B145" s="20" t="n"/>
-      <c r="C145" s="21" t="n"/>
-      <c r="D145" s="21" t="n"/>
+      <c r="A145" s="21" t="n"/>
+      <c r="B145" s="21" t="n"/>
+      <c r="C145" s="22" t="n"/>
+      <c r="D145" s="22" t="n"/>
       <c r="E145" s="11">
         <f>IF(D145="","",D145*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F145" s="21" t="n"/>
+      <c r="F145" s="22" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="20" t="n"/>
-      <c r="B146" s="20" t="n"/>
-      <c r="C146" s="21" t="n"/>
-      <c r="D146" s="21" t="n"/>
+      <c r="A146" s="21" t="n"/>
+      <c r="B146" s="21" t="n"/>
+      <c r="C146" s="22" t="n"/>
+      <c r="D146" s="22" t="n"/>
       <c r="E146" s="11">
         <f>IF(D146="","",D146*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F146" s="21" t="n"/>
+      <c r="F146" s="22" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="20" t="n"/>
-      <c r="B147" s="20" t="n"/>
-      <c r="C147" s="21" t="n"/>
-      <c r="D147" s="21" t="n"/>
+      <c r="A147" s="21" t="n"/>
+      <c r="B147" s="21" t="n"/>
+      <c r="C147" s="22" t="n"/>
+      <c r="D147" s="22" t="n"/>
       <c r="E147" s="11">
         <f>IF(D147="","",D147*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F147" s="21" t="n"/>
+      <c r="F147" s="22" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="20" t="n"/>
-      <c r="B148" s="20" t="n"/>
-      <c r="C148" s="21" t="n"/>
-      <c r="D148" s="21" t="n"/>
+      <c r="A148" s="21" t="n"/>
+      <c r="B148" s="21" t="n"/>
+      <c r="C148" s="22" t="n"/>
+      <c r="D148" s="22" t="n"/>
       <c r="E148" s="11">
         <f>IF(D148="","",D148*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F148" s="21" t="n"/>
+      <c r="F148" s="22" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="20" t="n"/>
-      <c r="B149" s="20" t="n"/>
-      <c r="C149" s="21" t="n"/>
-      <c r="D149" s="21" t="n"/>
+      <c r="A149" s="21" t="n"/>
+      <c r="B149" s="21" t="n"/>
+      <c r="C149" s="22" t="n"/>
+      <c r="D149" s="22" t="n"/>
       <c r="E149" s="11">
         <f>IF(D149="","",D149*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F149" s="21" t="n"/>
+      <c r="F149" s="22" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="20" t="n"/>
-      <c r="B150" s="20" t="n"/>
-      <c r="C150" s="21" t="n"/>
-      <c r="D150" s="21" t="n"/>
+      <c r="A150" s="21" t="n"/>
+      <c r="B150" s="21" t="n"/>
+      <c r="C150" s="22" t="n"/>
+      <c r="D150" s="22" t="n"/>
       <c r="E150" s="11">
         <f>IF(D150="","",D150*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F150" s="21" t="n"/>
+      <c r="F150" s="22" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="20" t="n"/>
-      <c r="B151" s="20" t="n"/>
-      <c r="C151" s="21" t="n"/>
-      <c r="D151" s="21" t="n"/>
+      <c r="A151" s="21" t="n"/>
+      <c r="B151" s="21" t="n"/>
+      <c r="C151" s="22" t="n"/>
+      <c r="D151" s="22" t="n"/>
       <c r="E151" s="11">
         <f>IF(D151="","",D151*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F151" s="21" t="n"/>
+      <c r="F151" s="22" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="20" t="n"/>
-      <c r="B152" s="20" t="n"/>
-      <c r="C152" s="21" t="n"/>
-      <c r="D152" s="21" t="n"/>
+      <c r="A152" s="21" t="n"/>
+      <c r="B152" s="21" t="n"/>
+      <c r="C152" s="22" t="n"/>
+      <c r="D152" s="22" t="n"/>
       <c r="E152" s="11">
         <f>IF(D152="","",D152*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F152" s="21" t="n"/>
+      <c r="F152" s="22" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="20" t="n"/>
-      <c r="B153" s="20" t="n"/>
-      <c r="C153" s="21" t="n"/>
-      <c r="D153" s="21" t="n"/>
+      <c r="A153" s="21" t="n"/>
+      <c r="B153" s="21" t="n"/>
+      <c r="C153" s="22" t="n"/>
+      <c r="D153" s="22" t="n"/>
       <c r="E153" s="11">
         <f>IF(D153="","",D153*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F153" s="21" t="n"/>
+      <c r="F153" s="22" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="20" t="n"/>
-      <c r="B154" s="20" t="n"/>
-      <c r="C154" s="21" t="n"/>
-      <c r="D154" s="21" t="n"/>
+      <c r="A154" s="21" t="n"/>
+      <c r="B154" s="21" t="n"/>
+      <c r="C154" s="22" t="n"/>
+      <c r="D154" s="22" t="n"/>
       <c r="E154" s="11">
         <f>IF(D154="","",D154*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F154" s="21" t="n"/>
+      <c r="F154" s="22" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="20" t="n"/>
-      <c r="B155" s="20" t="n"/>
-      <c r="C155" s="21" t="n"/>
-      <c r="D155" s="21" t="n"/>
+      <c r="A155" s="21" t="n"/>
+      <c r="B155" s="21" t="n"/>
+      <c r="C155" s="22" t="n"/>
+      <c r="D155" s="22" t="n"/>
       <c r="E155" s="11">
         <f>IF(D155="","",D155*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F155" s="21" t="n"/>
+      <c r="F155" s="22" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="20" t="n"/>
-      <c r="B156" s="20" t="n"/>
-      <c r="C156" s="21" t="n"/>
-      <c r="D156" s="21" t="n"/>
+      <c r="A156" s="21" t="n"/>
+      <c r="B156" s="21" t="n"/>
+      <c r="C156" s="22" t="n"/>
+      <c r="D156" s="22" t="n"/>
       <c r="E156" s="11">
         <f>IF(D156="","",D156*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F156" s="21" t="n"/>
+      <c r="F156" s="22" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="20" t="n"/>
-      <c r="B157" s="20" t="n"/>
-      <c r="C157" s="21" t="n"/>
-      <c r="D157" s="21" t="n"/>
+      <c r="A157" s="21" t="n"/>
+      <c r="B157" s="21" t="n"/>
+      <c r="C157" s="22" t="n"/>
+      <c r="D157" s="22" t="n"/>
       <c r="E157" s="11">
         <f>IF(D157="","",D157*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F157" s="21" t="n"/>
+      <c r="F157" s="22" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="20" t="n"/>
-      <c r="B158" s="20" t="n"/>
-      <c r="C158" s="21" t="n"/>
-      <c r="D158" s="21" t="n"/>
+      <c r="A158" s="21" t="n"/>
+      <c r="B158" s="21" t="n"/>
+      <c r="C158" s="22" t="n"/>
+      <c r="D158" s="22" t="n"/>
       <c r="E158" s="11">
         <f>IF(D158="","",D158*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F158" s="21" t="n"/>
+      <c r="F158" s="22" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="20" t="n"/>
-      <c r="B159" s="20" t="n"/>
-      <c r="C159" s="21" t="n"/>
-      <c r="D159" s="21" t="n"/>
+      <c r="A159" s="21" t="n"/>
+      <c r="B159" s="21" t="n"/>
+      <c r="C159" s="22" t="n"/>
+      <c r="D159" s="22" t="n"/>
       <c r="E159" s="11">
         <f>IF(D159="","",D159*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F159" s="21" t="n"/>
+      <c r="F159" s="22" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="20" t="n"/>
-      <c r="B160" s="20" t="n"/>
-      <c r="C160" s="21" t="n"/>
-      <c r="D160" s="21" t="n"/>
+      <c r="A160" s="21" t="n"/>
+      <c r="B160" s="21" t="n"/>
+      <c r="C160" s="22" t="n"/>
+      <c r="D160" s="22" t="n"/>
       <c r="E160" s="11">
         <f>IF(D160="","",D160*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F160" s="21" t="n"/>
+      <c r="F160" s="22" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="20" t="n"/>
-      <c r="B161" s="20" t="n"/>
-      <c r="C161" s="21" t="n"/>
-      <c r="D161" s="21" t="n"/>
+      <c r="A161" s="21" t="n"/>
+      <c r="B161" s="21" t="n"/>
+      <c r="C161" s="22" t="n"/>
+      <c r="D161" s="22" t="n"/>
       <c r="E161" s="11">
         <f>IF(D161="","",D161*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F161" s="21" t="n"/>
+      <c r="F161" s="22" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="20" t="n"/>
-      <c r="B162" s="20" t="n"/>
-      <c r="C162" s="21" t="n"/>
-      <c r="D162" s="21" t="n"/>
+      <c r="A162" s="21" t="n"/>
+      <c r="B162" s="21" t="n"/>
+      <c r="C162" s="22" t="n"/>
+      <c r="D162" s="22" t="n"/>
       <c r="E162" s="11">
         <f>IF(D162="","",D162*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F162" s="21" t="n"/>
+      <c r="F162" s="22" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="20" t="n"/>
-      <c r="B163" s="20" t="n"/>
-      <c r="C163" s="21" t="n"/>
-      <c r="D163" s="21" t="n"/>
+      <c r="A163" s="21" t="n"/>
+      <c r="B163" s="21" t="n"/>
+      <c r="C163" s="22" t="n"/>
+      <c r="D163" s="22" t="n"/>
       <c r="E163" s="11">
         <f>IF(D163="","",D163*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F163" s="21" t="n"/>
+      <c r="F163" s="22" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="20" t="n"/>
-      <c r="B164" s="20" t="n"/>
-      <c r="C164" s="21" t="n"/>
-      <c r="D164" s="21" t="n"/>
+      <c r="A164" s="21" t="n"/>
+      <c r="B164" s="21" t="n"/>
+      <c r="C164" s="22" t="n"/>
+      <c r="D164" s="22" t="n"/>
       <c r="E164" s="11">
         <f>IF(D164="","",D164*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F164" s="21" t="n"/>
+      <c r="F164" s="22" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="20" t="n"/>
-      <c r="B165" s="20" t="n"/>
-      <c r="C165" s="21" t="n"/>
-      <c r="D165" s="21" t="n"/>
+      <c r="A165" s="21" t="n"/>
+      <c r="B165" s="21" t="n"/>
+      <c r="C165" s="22" t="n"/>
+      <c r="D165" s="22" t="n"/>
       <c r="E165" s="11">
         <f>IF(D165="","",D165*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F165" s="21" t="n"/>
+      <c r="F165" s="22" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="20" t="n"/>
-      <c r="B166" s="20" t="n"/>
-      <c r="C166" s="21" t="n"/>
-      <c r="D166" s="21" t="n"/>
+      <c r="A166" s="21" t="n"/>
+      <c r="B166" s="21" t="n"/>
+      <c r="C166" s="22" t="n"/>
+      <c r="D166" s="22" t="n"/>
       <c r="E166" s="11">
         <f>IF(D166="","",D166*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F166" s="21" t="n"/>
+      <c r="F166" s="22" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="20" t="n"/>
-      <c r="B167" s="20" t="n"/>
-      <c r="C167" s="21" t="n"/>
-      <c r="D167" s="21" t="n"/>
+      <c r="A167" s="21" t="n"/>
+      <c r="B167" s="21" t="n"/>
+      <c r="C167" s="22" t="n"/>
+      <c r="D167" s="22" t="n"/>
       <c r="E167" s="11">
         <f>IF(D167="","",D167*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F167" s="21" t="n"/>
+      <c r="F167" s="22" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="20" t="n"/>
-      <c r="B168" s="20" t="n"/>
-      <c r="C168" s="21" t="n"/>
-      <c r="D168" s="21" t="n"/>
+      <c r="A168" s="21" t="n"/>
+      <c r="B168" s="21" t="n"/>
+      <c r="C168" s="22" t="n"/>
+      <c r="D168" s="22" t="n"/>
       <c r="E168" s="11">
         <f>IF(D168="","",D168*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F168" s="21" t="n"/>
+      <c r="F168" s="22" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" s="20" t="n"/>
-      <c r="B169" s="20" t="n"/>
-      <c r="C169" s="21" t="n"/>
-      <c r="D169" s="21" t="n"/>
+      <c r="A169" s="21" t="n"/>
+      <c r="B169" s="21" t="n"/>
+      <c r="C169" s="22" t="n"/>
+      <c r="D169" s="22" t="n"/>
       <c r="E169" s="11">
         <f>IF(D169="","",D169*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F169" s="21" t="n"/>
+      <c r="F169" s="22" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="20" t="n"/>
-      <c r="B170" s="20" t="n"/>
-      <c r="C170" s="21" t="n"/>
-      <c r="D170" s="21" t="n"/>
+      <c r="A170" s="21" t="n"/>
+      <c r="B170" s="21" t="n"/>
+      <c r="C170" s="22" t="n"/>
+      <c r="D170" s="22" t="n"/>
       <c r="E170" s="11">
         <f>IF(D170="","",D170*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F170" s="21" t="n"/>
+      <c r="F170" s="22" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="20" t="n"/>
-      <c r="B171" s="20" t="n"/>
-      <c r="C171" s="21" t="n"/>
-      <c r="D171" s="21" t="n"/>
+      <c r="A171" s="21" t="n"/>
+      <c r="B171" s="21" t="n"/>
+      <c r="C171" s="22" t="n"/>
+      <c r="D171" s="22" t="n"/>
       <c r="E171" s="11">
         <f>IF(D171="","",D171*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F171" s="21" t="n"/>
+      <c r="F171" s="22" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="20" t="n"/>
-      <c r="B172" s="20" t="n"/>
-      <c r="C172" s="21" t="n"/>
-      <c r="D172" s="21" t="n"/>
+      <c r="A172" s="21" t="n"/>
+      <c r="B172" s="21" t="n"/>
+      <c r="C172" s="22" t="n"/>
+      <c r="D172" s="22" t="n"/>
       <c r="E172" s="11">
         <f>IF(D172="","",D172*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F172" s="21" t="n"/>
+      <c r="F172" s="22" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" s="20" t="n"/>
-      <c r="B173" s="20" t="n"/>
-      <c r="C173" s="21" t="n"/>
-      <c r="D173" s="21" t="n"/>
+      <c r="A173" s="21" t="n"/>
+      <c r="B173" s="21" t="n"/>
+      <c r="C173" s="22" t="n"/>
+      <c r="D173" s="22" t="n"/>
       <c r="E173" s="11">
         <f>IF(D173="","",D173*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F173" s="21" t="n"/>
+      <c r="F173" s="22" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="20" t="n"/>
-      <c r="B174" s="20" t="n"/>
-      <c r="C174" s="21" t="n"/>
-      <c r="D174" s="21" t="n"/>
+      <c r="A174" s="21" t="n"/>
+      <c r="B174" s="21" t="n"/>
+      <c r="C174" s="22" t="n"/>
+      <c r="D174" s="22" t="n"/>
       <c r="E174" s="11">
         <f>IF(D174="","",D174*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F174" s="21" t="n"/>
+      <c r="F174" s="22" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="20" t="n"/>
-      <c r="B175" s="20" t="n"/>
-      <c r="C175" s="21" t="n"/>
-      <c r="D175" s="21" t="n"/>
+      <c r="A175" s="21" t="n"/>
+      <c r="B175" s="21" t="n"/>
+      <c r="C175" s="22" t="n"/>
+      <c r="D175" s="22" t="n"/>
       <c r="E175" s="11">
         <f>IF(D175="","",D175*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F175" s="21" t="n"/>
+      <c r="F175" s="22" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" s="20" t="n"/>
-      <c r="B176" s="20" t="n"/>
-      <c r="C176" s="21" t="n"/>
-      <c r="D176" s="21" t="n"/>
+      <c r="A176" s="21" t="n"/>
+      <c r="B176" s="21" t="n"/>
+      <c r="C176" s="22" t="n"/>
+      <c r="D176" s="22" t="n"/>
       <c r="E176" s="11">
         <f>IF(D176="","",D176*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F176" s="21" t="n"/>
+      <c r="F176" s="22" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="20" t="n"/>
-      <c r="B177" s="20" t="n"/>
-      <c r="C177" s="21" t="n"/>
-      <c r="D177" s="21" t="n"/>
+      <c r="A177" s="21" t="n"/>
+      <c r="B177" s="21" t="n"/>
+      <c r="C177" s="22" t="n"/>
+      <c r="D177" s="22" t="n"/>
       <c r="E177" s="11">
         <f>IF(D177="","",D177*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F177" s="21" t="n"/>
+      <c r="F177" s="22" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="20" t="n"/>
-      <c r="B178" s="20" t="n"/>
-      <c r="C178" s="21" t="n"/>
-      <c r="D178" s="21" t="n"/>
+      <c r="A178" s="21" t="n"/>
+      <c r="B178" s="21" t="n"/>
+      <c r="C178" s="22" t="n"/>
+      <c r="D178" s="22" t="n"/>
       <c r="E178" s="11">
         <f>IF(D178="","",D178*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F178" s="21" t="n"/>
+      <c r="F178" s="22" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" s="20" t="n"/>
-      <c r="B179" s="20" t="n"/>
-      <c r="C179" s="21" t="n"/>
-      <c r="D179" s="21" t="n"/>
+      <c r="A179" s="21" t="n"/>
+      <c r="B179" s="21" t="n"/>
+      <c r="C179" s="22" t="n"/>
+      <c r="D179" s="22" t="n"/>
       <c r="E179" s="11">
         <f>IF(D179="","",D179*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F179" s="21" t="n"/>
+      <c r="F179" s="22" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" s="20" t="n"/>
-      <c r="B180" s="20" t="n"/>
-      <c r="C180" s="21" t="n"/>
-      <c r="D180" s="21" t="n"/>
+      <c r="A180" s="21" t="n"/>
+      <c r="B180" s="21" t="n"/>
+      <c r="C180" s="22" t="n"/>
+      <c r="D180" s="22" t="n"/>
       <c r="E180" s="11">
         <f>IF(D180="","",D180*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F180" s="21" t="n"/>
+      <c r="F180" s="22" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="20" t="n"/>
-      <c r="B181" s="20" t="n"/>
-      <c r="C181" s="21" t="n"/>
-      <c r="D181" s="21" t="n"/>
+      <c r="A181" s="21" t="n"/>
+      <c r="B181" s="21" t="n"/>
+      <c r="C181" s="22" t="n"/>
+      <c r="D181" s="22" t="n"/>
       <c r="E181" s="11">
         <f>IF(D181="","",D181*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F181" s="21" t="n"/>
+      <c r="F181" s="22" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="20" t="n"/>
-      <c r="B182" s="20" t="n"/>
-      <c r="C182" s="21" t="n"/>
-      <c r="D182" s="21" t="n"/>
+      <c r="A182" s="21" t="n"/>
+      <c r="B182" s="21" t="n"/>
+      <c r="C182" s="22" t="n"/>
+      <c r="D182" s="22" t="n"/>
       <c r="E182" s="11">
         <f>IF(D182="","",D182*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F182" s="21" t="n"/>
+      <c r="F182" s="22" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="20" t="n"/>
-      <c r="B183" s="20" t="n"/>
-      <c r="C183" s="21" t="n"/>
-      <c r="D183" s="21" t="n"/>
+      <c r="A183" s="21" t="n"/>
+      <c r="B183" s="21" t="n"/>
+      <c r="C183" s="22" t="n"/>
+      <c r="D183" s="22" t="n"/>
       <c r="E183" s="11">
         <f>IF(D183="","",D183*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F183" s="21" t="n"/>
+      <c r="F183" s="22" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="20" t="n"/>
-      <c r="B184" s="20" t="n"/>
-      <c r="C184" s="21" t="n"/>
-      <c r="D184" s="21" t="n"/>
+      <c r="A184" s="21" t="n"/>
+      <c r="B184" s="21" t="n"/>
+      <c r="C184" s="22" t="n"/>
+      <c r="D184" s="22" t="n"/>
       <c r="E184" s="11">
         <f>IF(D184="","",D184*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F184" s="21" t="n"/>
+      <c r="F184" s="22" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="20" t="n"/>
-      <c r="B185" s="20" t="n"/>
-      <c r="C185" s="21" t="n"/>
-      <c r="D185" s="21" t="n"/>
+      <c r="A185" s="21" t="n"/>
+      <c r="B185" s="21" t="n"/>
+      <c r="C185" s="22" t="n"/>
+      <c r="D185" s="22" t="n"/>
       <c r="E185" s="11">
         <f>IF(D185="","",D185*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F185" s="21" t="n"/>
+      <c r="F185" s="22" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="20" t="n"/>
-      <c r="B186" s="20" t="n"/>
-      <c r="C186" s="21" t="n"/>
-      <c r="D186" s="21" t="n"/>
+      <c r="A186" s="21" t="n"/>
+      <c r="B186" s="21" t="n"/>
+      <c r="C186" s="22" t="n"/>
+      <c r="D186" s="22" t="n"/>
       <c r="E186" s="11">
         <f>IF(D186="","",D186*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F186" s="21" t="n"/>
+      <c r="F186" s="22" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" s="20" t="n"/>
-      <c r="B187" s="20" t="n"/>
-      <c r="C187" s="21" t="n"/>
-      <c r="D187" s="21" t="n"/>
+      <c r="A187" s="21" t="n"/>
+      <c r="B187" s="21" t="n"/>
+      <c r="C187" s="22" t="n"/>
+      <c r="D187" s="22" t="n"/>
       <c r="E187" s="11">
         <f>IF(D187="","",D187*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F187" s="21" t="n"/>
+      <c r="F187" s="22" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" s="20" t="n"/>
-      <c r="B188" s="20" t="n"/>
-      <c r="C188" s="21" t="n"/>
-      <c r="D188" s="21" t="n"/>
+      <c r="A188" s="21" t="n"/>
+      <c r="B188" s="21" t="n"/>
+      <c r="C188" s="22" t="n"/>
+      <c r="D188" s="22" t="n"/>
       <c r="E188" s="11">
         <f>IF(D188="","",D188*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F188" s="21" t="n"/>
+      <c r="F188" s="22" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" s="20" t="n"/>
-      <c r="B189" s="20" t="n"/>
-      <c r="C189" s="21" t="n"/>
-      <c r="D189" s="21" t="n"/>
+      <c r="A189" s="21" t="n"/>
+      <c r="B189" s="21" t="n"/>
+      <c r="C189" s="22" t="n"/>
+      <c r="D189" s="22" t="n"/>
       <c r="E189" s="11">
         <f>IF(D189="","",D189*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F189" s="21" t="n"/>
+      <c r="F189" s="22" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" s="20" t="n"/>
-      <c r="B190" s="20" t="n"/>
-      <c r="C190" s="21" t="n"/>
-      <c r="D190" s="21" t="n"/>
+      <c r="A190" s="21" t="n"/>
+      <c r="B190" s="21" t="n"/>
+      <c r="C190" s="22" t="n"/>
+      <c r="D190" s="22" t="n"/>
       <c r="E190" s="11">
         <f>IF(D190="","",D190*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F190" s="21" t="n"/>
+      <c r="F190" s="22" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="20" t="n"/>
-      <c r="B191" s="20" t="n"/>
-      <c r="C191" s="21" t="n"/>
-      <c r="D191" s="21" t="n"/>
+      <c r="A191" s="21" t="n"/>
+      <c r="B191" s="21" t="n"/>
+      <c r="C191" s="22" t="n"/>
+      <c r="D191" s="22" t="n"/>
       <c r="E191" s="11">
         <f>IF(D191="","",D191*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F191" s="21" t="n"/>
+      <c r="F191" s="22" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="20" t="n"/>
-      <c r="B192" s="20" t="n"/>
-      <c r="C192" s="21" t="n"/>
-      <c r="D192" s="21" t="n"/>
+      <c r="A192" s="21" t="n"/>
+      <c r="B192" s="21" t="n"/>
+      <c r="C192" s="22" t="n"/>
+      <c r="D192" s="22" t="n"/>
       <c r="E192" s="11">
         <f>IF(D192="","",D192*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F192" s="21" t="n"/>
+      <c r="F192" s="22" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="20" t="n"/>
-      <c r="B193" s="20" t="n"/>
-      <c r="C193" s="21" t="n"/>
-      <c r="D193" s="21" t="n"/>
+      <c r="A193" s="21" t="n"/>
+      <c r="B193" s="21" t="n"/>
+      <c r="C193" s="22" t="n"/>
+      <c r="D193" s="22" t="n"/>
       <c r="E193" s="11">
         <f>IF(D193="","",D193*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F193" s="21" t="n"/>
+      <c r="F193" s="22" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="20" t="n"/>
-      <c r="B194" s="20" t="n"/>
-      <c r="C194" s="21" t="n"/>
-      <c r="D194" s="21" t="n"/>
+      <c r="A194" s="21" t="n"/>
+      <c r="B194" s="21" t="n"/>
+      <c r="C194" s="22" t="n"/>
+      <c r="D194" s="22" t="n"/>
       <c r="E194" s="11">
         <f>IF(D194="","",D194*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F194" s="21" t="n"/>
+      <c r="F194" s="22" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="20" t="n"/>
-      <c r="B195" s="20" t="n"/>
-      <c r="C195" s="21" t="n"/>
-      <c r="D195" s="21" t="n"/>
+      <c r="A195" s="21" t="n"/>
+      <c r="B195" s="21" t="n"/>
+      <c r="C195" s="22" t="n"/>
+      <c r="D195" s="22" t="n"/>
       <c r="E195" s="11">
         <f>IF(D195="","",D195*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F195" s="21" t="n"/>
+      <c r="F195" s="22" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="20" t="n"/>
-      <c r="B196" s="20" t="n"/>
-      <c r="C196" s="21" t="n"/>
-      <c r="D196" s="21" t="n"/>
+      <c r="A196" s="21" t="n"/>
+      <c r="B196" s="21" t="n"/>
+      <c r="C196" s="22" t="n"/>
+      <c r="D196" s="22" t="n"/>
       <c r="E196" s="11">
         <f>IF(D196="","",D196*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F196" s="21" t="n"/>
+      <c r="F196" s="22" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="20" t="n"/>
-      <c r="B197" s="20" t="n"/>
-      <c r="C197" s="21" t="n"/>
-      <c r="D197" s="21" t="n"/>
+      <c r="A197" s="21" t="n"/>
+      <c r="B197" s="21" t="n"/>
+      <c r="C197" s="22" t="n"/>
+      <c r="D197" s="22" t="n"/>
       <c r="E197" s="11">
         <f>IF(D197="","",D197*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F197" s="21" t="n"/>
+      <c r="F197" s="22" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="20" t="n"/>
-      <c r="B198" s="20" t="n"/>
-      <c r="C198" s="21" t="n"/>
-      <c r="D198" s="21" t="n"/>
+      <c r="A198" s="21" t="n"/>
+      <c r="B198" s="21" t="n"/>
+      <c r="C198" s="22" t="n"/>
+      <c r="D198" s="22" t="n"/>
       <c r="E198" s="11">
         <f>IF(D198="","",D198*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F198" s="21" t="n"/>
+      <c r="F198" s="22" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" s="20" t="n"/>
-      <c r="B199" s="20" t="n"/>
-      <c r="C199" s="21" t="n"/>
-      <c r="D199" s="21" t="n"/>
+      <c r="A199" s="21" t="n"/>
+      <c r="B199" s="21" t="n"/>
+      <c r="C199" s="22" t="n"/>
+      <c r="D199" s="22" t="n"/>
       <c r="E199" s="11">
         <f>IF(D199="","",D199*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F199" s="21" t="n"/>
+      <c r="F199" s="22" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="20" t="n"/>
-      <c r="B200" s="20" t="n"/>
-      <c r="C200" s="21" t="n"/>
-      <c r="D200" s="21" t="n"/>
+      <c r="A200" s="21" t="n"/>
+      <c r="B200" s="21" t="n"/>
+      <c r="C200" s="22" t="n"/>
+      <c r="D200" s="22" t="n"/>
       <c r="E200" s="11">
         <f>IF(D200="","",D200*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F200" s="21" t="n"/>
+      <c r="F200" s="22" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" s="20" t="n"/>
-      <c r="B201" s="20" t="n"/>
-      <c r="C201" s="21" t="n"/>
-      <c r="D201" s="21" t="n"/>
+      <c r="A201" s="21" t="n"/>
+      <c r="B201" s="21" t="n"/>
+      <c r="C201" s="22" t="n"/>
+      <c r="D201" s="22" t="n"/>
       <c r="E201" s="11">
         <f>IF(D201="","",D201*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F201" s="21" t="n"/>
+      <c r="F201" s="22" t="n"/>
     </row>
     <row r="202">
-      <c r="A202" s="20" t="n"/>
-      <c r="B202" s="20" t="n"/>
-      <c r="C202" s="21" t="n"/>
-      <c r="D202" s="21" t="n"/>
+      <c r="A202" s="21" t="n"/>
+      <c r="B202" s="21" t="n"/>
+      <c r="C202" s="22" t="n"/>
+      <c r="D202" s="22" t="n"/>
       <c r="E202" s="11">
         <f>IF(D202="","",D202*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F202" s="21" t="n"/>
+      <c r="F202" s="22" t="n"/>
     </row>
     <row r="203">
-      <c r="A203" s="20" t="n"/>
-      <c r="B203" s="20" t="n"/>
-      <c r="C203" s="21" t="n"/>
-      <c r="D203" s="21" t="n"/>
+      <c r="A203" s="21" t="n"/>
+      <c r="B203" s="21" t="n"/>
+      <c r="C203" s="22" t="n"/>
+      <c r="D203" s="22" t="n"/>
       <c r="E203" s="11">
         <f>IF(D203="","",D203*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F203" s="21" t="n"/>
+      <c r="F203" s="22" t="n"/>
     </row>
     <row r="204">
-      <c r="A204" s="20" t="n"/>
-      <c r="B204" s="20" t="n"/>
-      <c r="C204" s="21" t="n"/>
-      <c r="D204" s="21" t="n"/>
+      <c r="A204" s="21" t="n"/>
+      <c r="B204" s="21" t="n"/>
+      <c r="C204" s="22" t="n"/>
+      <c r="D204" s="22" t="n"/>
       <c r="E204" s="11">
         <f>IF(D204="","",D204*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F204" s="21" t="n"/>
+      <c r="F204" s="22" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="C5:C204" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"CA,FRAC,RTT,RC Nuit,RC Férié,CET,ASA,HS"</formula1>
+      <formula1>"CA,CA HP,RTC,CET,CF,HS,RPS,ASA"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Tableau simple : valeurs affichées en jours
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1LRXK2yXR6W5viD25HWb5
</commit_message>
<xml_diff>
--- a/conges/conges_police_12h08.xlsx
+++ b/conges/conges_police_12h08.xlsx
@@ -19,10 +19,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="#,##0 €"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="0.00;[Red]-0.00"/>
+    <numFmt numFmtId="167" formatCode="0.0;[Red]-0.0"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -146,11 +147,11 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -590,15 +591,15 @@
         </is>
       </c>
       <c r="B4" s="5">
-        <f>Calcul!B5</f>
+        <f>Calcul!B5/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="C4" s="5">
-        <f>Calcul!C5</f>
+        <f>Calcul!C5/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="D4" s="5">
-        <f>Calcul!D5</f>
+        <f>Calcul!D5/Parametres!$B$26</f>
         <v/>
       </c>
     </row>
@@ -609,15 +610,15 @@
         </is>
       </c>
       <c r="B5" s="5">
-        <f>Calcul!B6</f>
+        <f>Calcul!B6/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="C5" s="5">
-        <f>Calcul!C6</f>
+        <f>Calcul!C6/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="D5" s="5">
-        <f>Calcul!D6</f>
+        <f>Calcul!D6/Parametres!$B$26</f>
         <v/>
       </c>
     </row>
@@ -628,15 +629,15 @@
         </is>
       </c>
       <c r="B6" s="5">
-        <f>Calcul!B7</f>
+        <f>Calcul!B7/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="C6" s="5">
-        <f>Calcul!C7</f>
+        <f>Calcul!C7/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="D6" s="5">
-        <f>Calcul!D7</f>
+        <f>Calcul!D7/Parametres!$B$26</f>
         <v/>
       </c>
     </row>
@@ -647,15 +648,15 @@
         </is>
       </c>
       <c r="B7" s="5">
-        <f>Calcul!B8</f>
+        <f>Calcul!B8/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="C7" s="5">
-        <f>Calcul!C8</f>
+        <f>Calcul!C8/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="D7" s="5">
-        <f>Calcul!D8</f>
+        <f>Calcul!D8/Parametres!$B$26</f>
         <v/>
       </c>
     </row>
@@ -666,15 +667,15 @@
         </is>
       </c>
       <c r="B8" s="5">
-        <f>Calcul!B9</f>
+        <f>Calcul!B9/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="C8" s="5">
-        <f>Calcul!C9</f>
+        <f>Calcul!C9/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="D8" s="5">
-        <f>Calcul!D9</f>
+        <f>Calcul!D9/Parametres!$B$26</f>
         <v/>
       </c>
     </row>
@@ -685,15 +686,15 @@
         </is>
       </c>
       <c r="B9" s="5">
-        <f>Calcul!B10</f>
+        <f>Calcul!B10/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="C9" s="5">
-        <f>Calcul!C10</f>
+        <f>Calcul!C10/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="D9" s="5">
-        <f>Calcul!D10</f>
+        <f>Calcul!D10/Parametres!$B$26</f>
         <v/>
       </c>
     </row>
@@ -704,15 +705,15 @@
         </is>
       </c>
       <c r="B10" s="5">
-        <f>Calcul!B11</f>
+        <f>Calcul!B11/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="C10" s="5">
-        <f>Calcul!C11</f>
+        <f>Calcul!C11/Parametres!$B$26</f>
         <v/>
       </c>
       <c r="D10" s="5">
-        <f>Calcul!D11</f>
+        <f>Calcul!D11/Parametres!$B$26</f>
         <v/>
       </c>
     </row>
@@ -738,7 +739,7 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Valeurs en heures.</t>
+          <t>Valeurs en jours (1 jour = 1 vacation de 12h08, modifiable dans Parametres B26).</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1365,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -1732,6 +1733,22 @@
       <c r="C25" s="22" t="inlineStr">
         <is>
           <t>Doublement ASA garde d'enfant.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
+          <t>Durée d'un jour dans le Tableau (h)</t>
+        </is>
+      </c>
+      <c r="B26" s="17">
+        <f>B6</f>
+        <v/>
+      </c>
+      <c r="C26" s="22" t="inlineStr">
+        <is>
+          <t>Par défaut 1 jour = 1 vacation de 12h08. Mets 7 pour des jours ouvrés.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tableau simple : saisie directe actuel et pris
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1LRXK2yXR6W5viD25HWb5
</commit_message>
<xml_diff>
--- a/conges/conges_police_12h08.xlsx
+++ b/conges/conges_police_12h08.xlsx
@@ -25,7 +25,7 @@
     <numFmt numFmtId="166" formatCode="0.00;[Red]-0.00"/>
     <numFmt numFmtId="167" formatCode="0.0;[Red]-0.0"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -89,6 +89,11 @@
       <name val="Arial"/>
       <sz val="12"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="000000FF"/>
+      <sz val="12"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -139,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -147,6 +152,9 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="167" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
@@ -542,7 +550,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -590,16 +598,14 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="B4" s="5">
-        <f>Calcul!B5/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="C4" s="5">
-        <f>Calcul!C5/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="D4" s="5">
-        <f>Calcul!D5/Parametres!$B$26</f>
+      <c r="B4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C4" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="6">
+        <f>B4-C4</f>
         <v/>
       </c>
     </row>
@@ -609,16 +615,14 @@
           <t>CA HP</t>
         </is>
       </c>
-      <c r="B5" s="5">
-        <f>Calcul!B6/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="C5" s="5">
-        <f>Calcul!C6/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="D5" s="5">
-        <f>Calcul!D6/Parametres!$B$26</f>
+      <c r="B5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="6">
+        <f>B5-C5</f>
         <v/>
       </c>
     </row>
@@ -628,16 +632,14 @@
           <t>RTC</t>
         </is>
       </c>
-      <c r="B6" s="5">
-        <f>Calcul!B7/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="C6" s="5">
-        <f>Calcul!C7/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="D6" s="5">
-        <f>Calcul!D7/Parametres!$B$26</f>
+      <c r="B6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="6">
+        <f>B6-C6</f>
         <v/>
       </c>
     </row>
@@ -647,16 +649,14 @@
           <t>CET</t>
         </is>
       </c>
-      <c r="B7" s="5">
-        <f>Calcul!B8/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="C7" s="5">
-        <f>Calcul!C8/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="D7" s="5">
-        <f>Calcul!D8/Parametres!$B$26</f>
+      <c r="B7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="6">
+        <f>B7-C7</f>
         <v/>
       </c>
     </row>
@@ -666,16 +666,14 @@
           <t>CF</t>
         </is>
       </c>
-      <c r="B8" s="5">
-        <f>Calcul!B9/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="C8" s="5">
-        <f>Calcul!C9/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="D8" s="5">
-        <f>Calcul!D9/Parametres!$B$26</f>
+      <c r="B8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="6">
+        <f>B8-C8</f>
         <v/>
       </c>
     </row>
@@ -685,16 +683,14 @@
           <t>HS</t>
         </is>
       </c>
-      <c r="B9" s="5">
-        <f>Calcul!B10/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="C9" s="5">
-        <f>Calcul!C10/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="D9" s="5">
-        <f>Calcul!D10/Parametres!$B$26</f>
+      <c r="B9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="6">
+        <f>B9-C9</f>
         <v/>
       </c>
     </row>
@@ -704,42 +700,47 @@
           <t>RPS</t>
         </is>
       </c>
-      <c r="B10" s="5">
-        <f>Calcul!B11/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="C10" s="5">
-        <f>Calcul!C11/Parametres!$B$26</f>
-        <v/>
-      </c>
-      <c r="D10" s="5">
-        <f>Calcul!D11/Parametres!$B$26</f>
+      <c r="B10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="6">
+        <f>B10-C10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="6" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="7">
+      <c r="B11" s="8">
         <f>SUM(B4:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="7">
+      <c r="C11" s="8">
         <f>SUM(C4:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="7">
+      <c r="D11" s="8">
         <f>SUM(D4:D10)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
-        <is>
-          <t>Valeurs en jours (1 jour = 1 vacation de 12h08, modifiable dans Parametres B26).</t>
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>Cases jaunes : tape tes chiffres en jours. Restant et Total se calculent seuls.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
+        <is>
+          <t>Les autres onglets sont une aide au calcul, facultative.</t>
         </is>
       </c>
     </row>
@@ -771,31 +772,31 @@
           <t>Mes droits à congés – récapitulatif</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
-      <c r="C1" s="9" t="n"/>
-      <c r="D1" s="9" t="n"/>
-      <c r="E1" s="9" t="n"/>
-      <c r="F1" s="9" t="n"/>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="10" t="n"/>
+      <c r="F1" s="10" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Tout se calcule depuis Parametres et Suivi. Ne rien saisir ici.</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="10" t="n"/>
+      <c r="D2" s="10" t="n"/>
+      <c r="E2" s="10" t="n"/>
+      <c r="F2" s="10" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="9" t="n"/>
+      <c r="A3" s="10" t="n"/>
+      <c r="B3" s="10" t="n"/>
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="10" t="n"/>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -830,244 +831,244 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>CA – Congés annuels</t>
         </is>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="13">
         <f>Parametres!$B$9*Parametres!$B$10*Parametres!$B$8</f>
         <v/>
       </c>
-      <c r="C5" s="12">
+      <c r="C5" s="13">
         <f>SUMIF(Suivi!$C$5:$C$204,"CA",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D5" s="13">
+      <c r="D5" s="14">
         <f>B5-C5</f>
         <v/>
       </c>
-      <c r="E5" s="12">
+      <c r="E5" s="13">
         <f>D5/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="12" t="inlineStr">
         <is>
           <t>25 j ouvrés × valeur horaire × quotité.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>CA HP – Hors période</t>
         </is>
       </c>
-      <c r="B6" s="12">
+      <c r="B6" s="13">
         <f>IF(Parametres!$B$11&gt;=8,2,IF(Parametres!$B$11&gt;=5,1,0))*Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C6" s="12">
+      <c r="C6" s="13">
         <f>SUMIF(Suivi!$C$5:$C$204,"CA HP",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D6" s="13">
+      <c r="D6" s="14">
         <f>B6-C6</f>
         <v/>
       </c>
-      <c r="E6" s="12">
+      <c r="E6" s="13">
         <f>D6/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F6" s="12" t="inlineStr">
         <is>
           <t>Bonus : 1 j si 5-7 j CA hors mai-oct ; 2 j si 8 et +.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>RTC</t>
         </is>
       </c>
-      <c r="B7" s="12">
+      <c r="B7" s="13">
         <f>Parametres!$B$12</f>
         <v/>
       </c>
-      <c r="C7" s="12">
+      <c r="C7" s="13">
         <f>SUMIF(Suivi!$C$5:$C$204,"RTC",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D7" s="13">
+      <c r="D7" s="14">
         <f>B7-C7</f>
         <v/>
       </c>
-      <c r="E7" s="12">
+      <c r="E7" s="13">
         <f>D7/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="12" t="inlineStr">
         <is>
           <t>Crédit saisi dans Parametres.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>CET – Compte épargne-temps</t>
         </is>
       </c>
-      <c r="B8" s="12">
+      <c r="B8" s="13">
         <f>(Parametres!$B$18+Parametres!$B$19)*Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C8" s="12">
+      <c r="C8" s="13">
         <f>SUMIF(Suivi!$C$5:$C$204,"CET",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D8" s="13">
+      <c r="D8" s="14">
         <f>B8-C8</f>
         <v/>
       </c>
-      <c r="E8" s="12">
+      <c r="E8" s="13">
         <f>D8/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="F8" s="12" t="inlineStr">
         <is>
           <t>Solde 1er janvier + jours versés.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>CF – Crédit férié</t>
         </is>
       </c>
-      <c r="B9" s="12">
+      <c r="B9" s="13">
         <f>Parametres!$B$13*Parametres!$B$14</f>
         <v/>
       </c>
-      <c r="C9" s="12">
+      <c r="C9" s="13">
         <f>SUMIF(Suivi!$C$5:$C$204,"CF",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D9" s="13">
+      <c r="D9" s="14">
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="12">
+      <c r="E9" s="13">
         <f>D9/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F9" s="12" t="inlineStr">
         <is>
           <t>Nb fériés × heures par férié.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>HS – Heures supplémentaires</t>
         </is>
       </c>
-      <c r="B10" s="12">
+      <c r="B10" s="13">
         <f>Parametres!$B$15</f>
         <v/>
       </c>
-      <c r="C10" s="12">
+      <c r="C10" s="13">
         <f>SUMIF(Suivi!$C$5:$C$204,"HS",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D10" s="13">
+      <c r="D10" s="14">
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="12">
+      <c r="E10" s="13">
         <f>D10/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F10" s="12" t="inlineStr">
         <is>
           <t>Compteur HS récupérables.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>RPS – Repos pénibilité nuit</t>
         </is>
       </c>
-      <c r="B11" s="12">
+      <c r="B11" s="13">
         <f>IF(Parametres!$B$17&gt;0,Parametres!$B$17,ROUND(140*Parametres!$B$8,0))*Parametres!$B$7*Parametres!$B$16</f>
         <v/>
       </c>
-      <c r="C11" s="12">
+      <c r="C11" s="13">
         <f>SUMIF(Suivi!$C$5:$C$204,"RPS",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D11" s="13">
+      <c r="D11" s="14">
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="12">
+      <c r="E11" s="13">
         <f>D11/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F11" s="12" t="inlineStr">
         <is>
           <t>Vacations nuit × heures nuit × coef.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="15" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="15">
+      <c r="B12" s="16">
         <f>SUM(B5:B11)</f>
         <v/>
       </c>
-      <c r="C12" s="15">
+      <c r="C12" s="16">
         <f>SUM(C5:C11)</f>
         <v/>
       </c>
-      <c r="D12" s="15">
+      <c r="D12" s="16">
         <f>SUM(D5:D11)</f>
         <v/>
       </c>
-      <c r="E12" s="15">
+      <c r="E12" s="16">
         <f>SUM(E5:E11)</f>
         <v/>
       </c>
-      <c r="F12" s="14" t="n"/>
+      <c r="F12" s="15" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="n"/>
-      <c r="B13" s="9" t="n"/>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
-      <c r="E13" s="9" t="n"/>
-      <c r="F13" s="9" t="n"/>
+      <c r="A13" s="10" t="n"/>
+      <c r="B13" s="10" t="n"/>
+      <c r="C13" s="10" t="n"/>
+      <c r="D13" s="10" t="n"/>
+      <c r="E13" s="10" t="n"/>
+      <c r="F13" s="10" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>CET – détail</t>
         </is>
       </c>
-      <c r="B14" s="9" t="n"/>
-      <c r="C14" s="9" t="n"/>
-      <c r="D14" s="9" t="n"/>
-      <c r="E14" s="9" t="n"/>
-      <c r="F14" s="9" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="10" t="n"/>
+      <c r="D14" s="10" t="n"/>
+      <c r="E14" s="10" t="n"/>
+      <c r="F14" s="10" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1090,134 +1091,134 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Jours CA pris dans l'année</t>
         </is>
       </c>
-      <c r="B16" s="17">
+      <c r="B16" s="18">
         <f>C5/Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C16" s="9" t="n"/>
-      <c r="D16" s="9" t="n"/>
-      <c r="E16" s="9" t="n"/>
-      <c r="F16" s="9" t="inlineStr">
+      <c r="C16" s="10" t="n"/>
+      <c r="D16" s="10" t="n"/>
+      <c r="E16" s="10" t="n"/>
+      <c r="F16" s="10" t="inlineStr">
         <is>
           <t>Depuis Suivi.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Jours épargnables max</t>
         </is>
       </c>
-      <c r="B17" s="17">
+      <c r="B17" s="18">
         <f>MAX(0,MIN((B5+B6-C5-C6)/Parametres!$B$10,(B5+B6)/Parametres!$B$10-20))</f>
         <v/>
       </c>
-      <c r="C17" s="9" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="9" t="n"/>
-      <c r="F17" s="9" t="inlineStr">
+      <c r="C17" s="10" t="n"/>
+      <c r="D17" s="10" t="n"/>
+      <c r="E17" s="10" t="n"/>
+      <c r="F17" s="10" t="inlineStr">
         <is>
           <t>20 j de CA obligatoires. Le reliquat est épargnable.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>Solde CET restant (jours)</t>
         </is>
       </c>
-      <c r="B18" s="17">
+      <c r="B18" s="18">
         <f>D8/Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C18" s="9" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="9" t="n"/>
-      <c r="F18" s="9" t="inlineStr">
+      <c r="C18" s="10" t="n"/>
+      <c r="D18" s="10" t="n"/>
+      <c r="E18" s="10" t="n"/>
+      <c r="F18" s="10" t="inlineStr">
         <is>
           <t>Plafond 60 jours.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Alerte plafond</t>
         </is>
       </c>
-      <c r="B19" s="17">
+      <c r="B19" s="18">
         <f>IF(B18&gt;60,"Plafond 60 j dépassé","OK")</f>
         <v/>
       </c>
-      <c r="C19" s="9" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="9" t="n"/>
-      <c r="F19" s="9" t="inlineStr"/>
+      <c r="C19" s="10" t="n"/>
+      <c r="D19" s="10" t="n"/>
+      <c r="E19" s="10" t="n"/>
+      <c r="F19" s="10" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Jours indemnisables (au-delà de 15)</t>
         </is>
       </c>
-      <c r="B20" s="17">
+      <c r="B20" s="18">
         <f>MAX(0,MIN(B18,60)-15)</f>
         <v/>
       </c>
-      <c r="C20" s="9" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="9" t="n"/>
-      <c r="F20" s="9" t="inlineStr">
+      <c r="C20" s="10" t="n"/>
+      <c r="D20" s="10" t="n"/>
+      <c r="E20" s="10" t="n"/>
+      <c r="F20" s="10" t="inlineStr">
         <is>
           <t>Option possible au-delà de 15 j.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Valeur si indemnisés (€)</t>
         </is>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="19">
         <f>B20*IF(Parametres!$B$20="A",Parametres!$B$23,IF(Parametres!$B$20="B",Parametres!$B$22,Parametres!$B$21))</f>
         <v/>
       </c>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="9" t="inlineStr">
+      <c r="C21" s="10" t="n"/>
+      <c r="D21" s="10" t="n"/>
+      <c r="E21" s="10" t="n"/>
+      <c r="F21" s="10" t="inlineStr">
         <is>
           <t>Montant brut selon catégorie.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="9" t="n"/>
-      <c r="B22" s="9" t="n"/>
-      <c r="C22" s="9" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="9" t="n"/>
-      <c r="F22" s="9" t="n"/>
+      <c r="A22" s="10" t="n"/>
+      <c r="B22" s="10" t="n"/>
+      <c r="C22" s="10" t="n"/>
+      <c r="D22" s="10" t="n"/>
+      <c r="E22" s="10" t="n"/>
+      <c r="F22" s="10" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>ASA – Autorisations spéciales d'absence (hors compteur)</t>
         </is>
       </c>
-      <c r="B23" s="9" t="n"/>
-      <c r="C23" s="9" t="n"/>
-      <c r="D23" s="9" t="n"/>
-      <c r="E23" s="9" t="n"/>
-      <c r="F23" s="9" t="n"/>
+      <c r="B23" s="10" t="n"/>
+      <c r="C23" s="10" t="n"/>
+      <c r="D23" s="10" t="n"/>
+      <c r="E23" s="10" t="n"/>
+      <c r="F23" s="10" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1240,119 +1241,119 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Garde d'enfant malade</t>
         </is>
       </c>
-      <c r="B25" s="19">
+      <c r="B25" s="20">
         <f>IF(Parametres!$B$24="O",IF(Parametres!$B$25="O",12,6)*Parametres!$B$8,0)</f>
         <v/>
       </c>
-      <c r="C25" s="9" t="n"/>
-      <c r="D25" s="9" t="n"/>
-      <c r="E25" s="9" t="n"/>
-      <c r="F25" s="9" t="inlineStr">
+      <c r="C25" s="10" t="n"/>
+      <c r="D25" s="10" t="n"/>
+      <c r="E25" s="10" t="n"/>
+      <c r="F25" s="10" t="inlineStr">
         <is>
           <t>6 j/an ; 12 j si seul ou conjoint sans droit. À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Mariage / PACS de l'agent</t>
         </is>
       </c>
-      <c r="B26" s="19" t="n">
+      <c r="B26" s="20" t="n">
         <v>5</v>
       </c>
-      <c r="C26" s="9" t="n"/>
-      <c r="D26" s="9" t="n"/>
-      <c r="E26" s="9" t="n"/>
-      <c r="F26" s="9" t="inlineStr">
+      <c r="C26" s="10" t="n"/>
+      <c r="D26" s="10" t="n"/>
+      <c r="E26" s="10" t="n"/>
+      <c r="F26" s="10" t="inlineStr">
         <is>
           <t>Barème FP. À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="11" t="inlineStr">
+      <c r="A27" s="12" t="inlineStr">
         <is>
           <t>Décès conjoint / parent / enfant</t>
         </is>
       </c>
-      <c r="B27" s="19" t="n">
+      <c r="B27" s="20" t="n">
         <v>3</v>
       </c>
-      <c r="C27" s="9" t="n"/>
-      <c r="D27" s="9" t="n"/>
-      <c r="E27" s="9" t="n"/>
-      <c r="F27" s="9" t="inlineStr">
+      <c r="C27" s="10" t="n"/>
+      <c r="D27" s="10" t="n"/>
+      <c r="E27" s="10" t="n"/>
+      <c r="F27" s="10" t="inlineStr">
         <is>
           <t>Barème FP. Enfant : régime renforcé.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="11" t="inlineStr">
+      <c r="A28" s="12" t="inlineStr">
         <is>
           <t>Naissance / adoption</t>
         </is>
       </c>
-      <c r="B28" s="19" t="inlineStr">
+      <c r="B28" s="20" t="inlineStr">
         <is>
           <t>Voir RH</t>
         </is>
       </c>
-      <c r="C28" s="9" t="n"/>
-      <c r="D28" s="9" t="n"/>
-      <c r="E28" s="9" t="n"/>
-      <c r="F28" s="9" t="inlineStr">
+      <c r="C28" s="10" t="n"/>
+      <c r="D28" s="10" t="n"/>
+      <c r="E28" s="10" t="n"/>
+      <c r="F28" s="10" t="inlineStr">
         <is>
           <t>Congé naissance 3 j + paternité 25 j.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="11" t="inlineStr">
+      <c r="A29" s="12" t="inlineStr">
         <is>
           <t>Déménagement</t>
         </is>
       </c>
-      <c r="B29" s="19" t="inlineStr">
+      <c r="B29" s="20" t="inlineStr">
         <is>
           <t>Voir RH</t>
         </is>
       </c>
-      <c r="C29" s="9" t="n"/>
-      <c r="D29" s="9" t="n"/>
-      <c r="E29" s="9" t="n"/>
-      <c r="F29" s="9" t="inlineStr">
+      <c r="C29" s="10" t="n"/>
+      <c r="D29" s="10" t="n"/>
+      <c r="E29" s="10" t="n"/>
+      <c r="F29" s="10" t="inlineStr">
         <is>
           <t>Selon note de service.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="9" t="n"/>
-      <c r="B30" s="9" t="n"/>
-      <c r="C30" s="9" t="n"/>
-      <c r="D30" s="9" t="n"/>
-      <c r="E30" s="9" t="n"/>
-      <c r="F30" s="9" t="n"/>
+      <c r="A30" s="10" t="n"/>
+      <c r="B30" s="10" t="n"/>
+      <c r="C30" s="10" t="n"/>
+      <c r="D30" s="10" t="n"/>
+      <c r="E30" s="10" t="n"/>
+      <c r="F30" s="10" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="20" t="inlineStr">
+      <c r="A31" s="21" t="inlineStr">
         <is>
           <t>Les montants et barèmes sont indicatifs. Vérifie avec ton secrétariat / Géopol et ta note de service locale.</t>
         </is>
       </c>
-      <c r="B31" s="9" t="n"/>
-      <c r="C31" s="9" t="n"/>
-      <c r="D31" s="9" t="n"/>
-      <c r="E31" s="9" t="n"/>
-      <c r="F31" s="9" t="n"/>
+      <c r="B31" s="10" t="n"/>
+      <c r="C31" s="10" t="n"/>
+      <c r="D31" s="10" t="n"/>
+      <c r="E31" s="10" t="n"/>
+      <c r="F31" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1379,22 +1380,22 @@
           <t>Paramètres – Police nationale, cycle 12h08 de nuit</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
-      <c r="C1" s="9" t="n"/>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Cellules jaunes / texte bleu = à saisir. Le reste se calcule seul.</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="n"/>
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="10" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="n"/>
+      <c r="A3" s="10" t="n"/>
+      <c r="B3" s="10" t="n"/>
+      <c r="C3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1414,339 +1415,339 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="12" t="inlineStr">
         <is>
           <t>Année de référence</t>
         </is>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="22" t="n">
         <v>2026</v>
       </c>
-      <c r="C5" s="22" t="inlineStr">
+      <c r="C5" s="23" t="inlineStr">
         <is>
           <t>Année civile des droits.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="11" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Durée d'une vacation (heures)</t>
         </is>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="18">
         <f>12+8/60</f>
         <v/>
       </c>
-      <c r="C6" s="22" t="inlineStr">
+      <c r="C6" s="23" t="inlineStr">
         <is>
           <t>12h08 = 12,13 h, dont 2 pauses de 20 min (rapport Sénat).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="11" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Heures de nuit par vacation</t>
         </is>
       </c>
-      <c r="B7" s="23" t="n">
+      <c r="B7" s="24" t="n">
         <v>9</v>
       </c>
-      <c r="C7" s="22" t="inlineStr">
+      <c r="C7" s="23" t="inlineStr">
         <is>
           <t>Heures entre 21h et 6h (RGEMPN). 9h si vacation couvre toute la plage.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="11" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Quotité de travail</t>
         </is>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="25" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="22" t="inlineStr">
+      <c r="C8" s="23" t="inlineStr">
         <is>
           <t>100 % = temps plein.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="11" t="inlineStr">
+      <c r="A9" s="12" t="inlineStr">
         <is>
           <t>CA – jours ouvrés réglementaires</t>
         </is>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B9" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="C9" s="22" t="inlineStr">
+      <c r="C9" s="23" t="inlineStr">
         <is>
           <t>Décret 84-972 : 25 jours ouvrés.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Valeur horaire d'1 jour de CA (h)</t>
         </is>
       </c>
-      <c r="B10" s="23" t="n">
+      <c r="B10" s="24" t="n">
         <v>7</v>
       </c>
-      <c r="C10" s="22" t="inlineStr">
+      <c r="C10" s="23" t="inlineStr">
         <is>
           <t>À vérifier avec ton secrétariat / Géopol.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>CA HP – jours CA pris hors 1/05–31/10</t>
         </is>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="22" t="inlineStr">
+      <c r="C11" s="23" t="inlineStr">
         <is>
           <t>5 à 7 j = 1 j bonus ; 8 j et + = 2 j bonus.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>RTC – crédit annuel (heures)</t>
         </is>
       </c>
-      <c r="B12" s="23" t="n">
+      <c r="B12" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="22" t="inlineStr">
+      <c r="C12" s="23" t="inlineStr">
         <is>
           <t>Crédit annuel horaire d'ARTT en régime cyclique (RGEMPN art. 39). Voir Géopol.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>CF – nombre de fériés crédités</t>
         </is>
       </c>
-      <c r="B13" s="21" t="n">
+      <c r="B13" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="22" t="inlineStr">
+      <c r="C13" s="23" t="inlineStr">
         <is>
           <t>Crédit férié annuel, en heures, pour régime cyclique. Voir Géopol.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="11" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>CF – heures par férié</t>
         </is>
       </c>
-      <c r="B14" s="17">
+      <c r="B14" s="18">
         <f>B6</f>
         <v/>
       </c>
-      <c r="C14" s="22" t="inlineStr">
+      <c r="C14" s="23" t="inlineStr">
         <is>
           <t>Par défaut = 1 vacation. Modifiable.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>HS – heures sup. au compteur (heures)</t>
         </is>
       </c>
-      <c r="B15" s="23" t="n">
+      <c r="B15" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="22" t="inlineStr">
+      <c r="C15" s="23" t="inlineStr">
         <is>
           <t>Solde HS récupérables. Voir relevé.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>RPS – coef. sur heures de nuit</t>
         </is>
       </c>
-      <c r="B16" s="24" t="n">
+      <c r="B16" s="25" t="n">
         <v>0.1</v>
       </c>
-      <c r="C16" s="22" t="inlineStr">
+      <c r="C16" s="23" t="inlineStr">
         <is>
           <t>0,1 par heure de nuit 21h-6h (0,4 dimanche, non cumulable). Source : RGEMPN.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="11" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>RPS – vacations de nuit / an</t>
         </is>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="22" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="22" t="inlineStr">
+      <c r="C17" s="23" t="inlineStr">
         <is>
           <t>0 = 140 vacations/an (cycle binaire, rapport Sénat).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t>CET – solde au 1er janvier (jours)</t>
         </is>
       </c>
-      <c r="B18" s="23" t="n">
+      <c r="B18" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="22" t="inlineStr">
+      <c r="C18" s="23" t="inlineStr">
         <is>
           <t>Repris de ton relevé CET.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="11" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>CET – jours versés cette année</t>
         </is>
       </c>
-      <c r="B19" s="23" t="n">
+      <c r="B19" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="C19" s="22" t="inlineStr">
+      <c r="C19" s="23" t="inlineStr">
         <is>
           <t>Ta demande d'alimentation.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="11" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Catégorie (C, B, A)</t>
         </is>
       </c>
-      <c r="B20" s="25" t="inlineStr">
+      <c r="B20" s="26" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C20" s="22" t="inlineStr">
+      <c r="C20" s="23" t="inlineStr">
         <is>
           <t>Pour l'indemnisation CET.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Taux CET catégorie C (€/jour)</t>
         </is>
       </c>
-      <c r="B21" s="26" t="n">
+      <c r="B21" s="27" t="n">
         <v>83</v>
       </c>
-      <c r="C21" s="22" t="inlineStr">
+      <c r="C21" s="23" t="inlineStr">
         <is>
           <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Taux CET catégorie B (€/jour)</t>
         </is>
       </c>
-      <c r="B22" s="26" t="n">
+      <c r="B22" s="27" t="n">
         <v>100</v>
       </c>
-      <c r="C22" s="22" t="inlineStr">
+      <c r="C22" s="23" t="inlineStr">
         <is>
           <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="11" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Taux CET catégorie A (€/jour)</t>
         </is>
       </c>
-      <c r="B23" s="26" t="n">
+      <c r="B23" s="27" t="n">
         <v>150</v>
       </c>
-      <c r="C23" s="22" t="inlineStr">
+      <c r="C23" s="23" t="inlineStr">
         <is>
           <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="11" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Enfants à charge &lt; 16 ans (O/N)</t>
         </is>
       </c>
-      <c r="B24" s="25" t="inlineStr">
+      <c r="B24" s="26" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="C24" s="22" t="inlineStr">
+      <c r="C24" s="23" t="inlineStr">
         <is>
           <t>Pour ASA garde d'enfant.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="11" t="inlineStr">
+      <c r="A25" s="12" t="inlineStr">
         <is>
           <t>Élève seul l'enfant ou conjoint sans droit (O/N)</t>
         </is>
       </c>
-      <c r="B25" s="25" t="inlineStr">
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C25" s="22" t="inlineStr">
+      <c r="C25" s="23" t="inlineStr">
         <is>
           <t>Doublement ASA garde d'enfant.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="11" t="inlineStr">
+      <c r="A26" s="12" t="inlineStr">
         <is>
           <t>Durée d'un jour dans le Tableau (h)</t>
         </is>
       </c>
-      <c r="B26" s="17">
+      <c r="B26" s="18">
         <f>B6</f>
         <v/>
       </c>
-      <c r="C26" s="22" t="inlineStr">
+      <c r="C26" s="23" t="inlineStr">
         <is>
           <t>Par défaut 1 jour = 1 vacation de 12h08. Mets 7 pour des jours ouvrés.</t>
         </is>
@@ -1788,31 +1789,31 @@
           <t>Journal des absences posées</t>
         </is>
       </c>
-      <c r="B1" s="9" t="n"/>
-      <c r="C1" s="9" t="n"/>
-      <c r="D1" s="9" t="n"/>
-      <c r="E1" s="9" t="n"/>
-      <c r="F1" s="9" t="n"/>
+      <c r="B1" s="10" t="n"/>
+      <c r="C1" s="10" t="n"/>
+      <c r="D1" s="10" t="n"/>
+      <c r="E1" s="10" t="n"/>
+      <c r="F1" s="10" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="10" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>Une ligne par absence. Choisis le type dans la liste. Heures calculées seules.</t>
         </is>
       </c>
-      <c r="B2" s="9" t="n"/>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
-      <c r="E2" s="9" t="n"/>
-      <c r="F2" s="9" t="n"/>
+      <c r="B2" s="10" t="n"/>
+      <c r="C2" s="10" t="n"/>
+      <c r="D2" s="10" t="n"/>
+      <c r="E2" s="10" t="n"/>
+      <c r="F2" s="10" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="9" t="n"/>
-      <c r="B3" s="9" t="n"/>
-      <c r="C3" s="9" t="n"/>
-      <c r="D3" s="9" t="n"/>
-      <c r="E3" s="9" t="n"/>
-      <c r="F3" s="9" t="n"/>
+      <c r="A3" s="10" t="n"/>
+      <c r="B3" s="10" t="n"/>
+      <c r="C3" s="10" t="n"/>
+      <c r="D3" s="10" t="n"/>
+      <c r="E3" s="10" t="n"/>
+      <c r="F3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1847,2218 +1848,2218 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="27" t="n">
+      <c r="A5" s="28" t="n">
         <v>46063</v>
       </c>
-      <c r="B5" s="27" t="n">
+      <c r="B5" s="28" t="n">
         <v>46066</v>
       </c>
-      <c r="C5" s="28" t="inlineStr">
+      <c r="C5" s="29" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D5" s="28" t="n">
+      <c r="D5" s="29" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="17">
+      <c r="E5" s="18">
         <f>IF(D5="","",D5*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F5" s="28" t="inlineStr">
+      <c r="F5" s="29" t="inlineStr">
         <is>
           <t>Exemple – à effacer</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="27" t="n"/>
-      <c r="B6" s="27" t="n"/>
-      <c r="C6" s="28" t="n"/>
-      <c r="D6" s="28" t="n"/>
-      <c r="E6" s="17">
+      <c r="A6" s="28" t="n"/>
+      <c r="B6" s="28" t="n"/>
+      <c r="C6" s="29" t="n"/>
+      <c r="D6" s="29" t="n"/>
+      <c r="E6" s="18">
         <f>IF(D6="","",D6*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F6" s="28" t="n"/>
+      <c r="F6" s="29" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="27" t="n"/>
-      <c r="B7" s="27" t="n"/>
-      <c r="C7" s="28" t="n"/>
-      <c r="D7" s="28" t="n"/>
-      <c r="E7" s="17">
+      <c r="A7" s="28" t="n"/>
+      <c r="B7" s="28" t="n"/>
+      <c r="C7" s="29" t="n"/>
+      <c r="D7" s="29" t="n"/>
+      <c r="E7" s="18">
         <f>IF(D7="","",D7*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F7" s="28" t="n"/>
+      <c r="F7" s="29" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="27" t="n"/>
-      <c r="B8" s="27" t="n"/>
-      <c r="C8" s="28" t="n"/>
-      <c r="D8" s="28" t="n"/>
-      <c r="E8" s="17">
+      <c r="A8" s="28" t="n"/>
+      <c r="B8" s="28" t="n"/>
+      <c r="C8" s="29" t="n"/>
+      <c r="D8" s="29" t="n"/>
+      <c r="E8" s="18">
         <f>IF(D8="","",D8*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F8" s="28" t="n"/>
+      <c r="F8" s="29" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="27" t="n"/>
-      <c r="B9" s="27" t="n"/>
-      <c r="C9" s="28" t="n"/>
-      <c r="D9" s="28" t="n"/>
-      <c r="E9" s="17">
+      <c r="A9" s="28" t="n"/>
+      <c r="B9" s="28" t="n"/>
+      <c r="C9" s="29" t="n"/>
+      <c r="D9" s="29" t="n"/>
+      <c r="E9" s="18">
         <f>IF(D9="","",D9*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F9" s="28" t="n"/>
+      <c r="F9" s="29" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="27" t="n"/>
-      <c r="B10" s="27" t="n"/>
-      <c r="C10" s="28" t="n"/>
-      <c r="D10" s="28" t="n"/>
-      <c r="E10" s="17">
+      <c r="A10" s="28" t="n"/>
+      <c r="B10" s="28" t="n"/>
+      <c r="C10" s="29" t="n"/>
+      <c r="D10" s="29" t="n"/>
+      <c r="E10" s="18">
         <f>IF(D10="","",D10*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F10" s="28" t="n"/>
+      <c r="F10" s="29" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="27" t="n"/>
-      <c r="B11" s="27" t="n"/>
-      <c r="C11" s="28" t="n"/>
-      <c r="D11" s="28" t="n"/>
-      <c r="E11" s="17">
+      <c r="A11" s="28" t="n"/>
+      <c r="B11" s="28" t="n"/>
+      <c r="C11" s="29" t="n"/>
+      <c r="D11" s="29" t="n"/>
+      <c r="E11" s="18">
         <f>IF(D11="","",D11*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F11" s="28" t="n"/>
+      <c r="F11" s="29" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="27" t="n"/>
-      <c r="B12" s="27" t="n"/>
-      <c r="C12" s="28" t="n"/>
-      <c r="D12" s="28" t="n"/>
-      <c r="E12" s="17">
+      <c r="A12" s="28" t="n"/>
+      <c r="B12" s="28" t="n"/>
+      <c r="C12" s="29" t="n"/>
+      <c r="D12" s="29" t="n"/>
+      <c r="E12" s="18">
         <f>IF(D12="","",D12*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F12" s="28" t="n"/>
+      <c r="F12" s="29" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="27" t="n"/>
-      <c r="B13" s="27" t="n"/>
-      <c r="C13" s="28" t="n"/>
-      <c r="D13" s="28" t="n"/>
-      <c r="E13" s="17">
+      <c r="A13" s="28" t="n"/>
+      <c r="B13" s="28" t="n"/>
+      <c r="C13" s="29" t="n"/>
+      <c r="D13" s="29" t="n"/>
+      <c r="E13" s="18">
         <f>IF(D13="","",D13*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F13" s="28" t="n"/>
+      <c r="F13" s="29" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="27" t="n"/>
-      <c r="B14" s="27" t="n"/>
-      <c r="C14" s="28" t="n"/>
-      <c r="D14" s="28" t="n"/>
-      <c r="E14" s="17">
+      <c r="A14" s="28" t="n"/>
+      <c r="B14" s="28" t="n"/>
+      <c r="C14" s="29" t="n"/>
+      <c r="D14" s="29" t="n"/>
+      <c r="E14" s="18">
         <f>IF(D14="","",D14*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F14" s="28" t="n"/>
+      <c r="F14" s="29" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="27" t="n"/>
-      <c r="B15" s="27" t="n"/>
-      <c r="C15" s="28" t="n"/>
-      <c r="D15" s="28" t="n"/>
-      <c r="E15" s="17">
+      <c r="A15" s="28" t="n"/>
+      <c r="B15" s="28" t="n"/>
+      <c r="C15" s="29" t="n"/>
+      <c r="D15" s="29" t="n"/>
+      <c r="E15" s="18">
         <f>IF(D15="","",D15*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F15" s="28" t="n"/>
+      <c r="F15" s="29" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="27" t="n"/>
-      <c r="B16" s="27" t="n"/>
-      <c r="C16" s="28" t="n"/>
-      <c r="D16" s="28" t="n"/>
-      <c r="E16" s="17">
+      <c r="A16" s="28" t="n"/>
+      <c r="B16" s="28" t="n"/>
+      <c r="C16" s="29" t="n"/>
+      <c r="D16" s="29" t="n"/>
+      <c r="E16" s="18">
         <f>IF(D16="","",D16*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F16" s="28" t="n"/>
+      <c r="F16" s="29" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="27" t="n"/>
-      <c r="B17" s="27" t="n"/>
-      <c r="C17" s="28" t="n"/>
-      <c r="D17" s="28" t="n"/>
-      <c r="E17" s="17">
+      <c r="A17" s="28" t="n"/>
+      <c r="B17" s="28" t="n"/>
+      <c r="C17" s="29" t="n"/>
+      <c r="D17" s="29" t="n"/>
+      <c r="E17" s="18">
         <f>IF(D17="","",D17*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F17" s="28" t="n"/>
+      <c r="F17" s="29" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="27" t="n"/>
-      <c r="B18" s="27" t="n"/>
-      <c r="C18" s="28" t="n"/>
-      <c r="D18" s="28" t="n"/>
-      <c r="E18" s="17">
+      <c r="A18" s="28" t="n"/>
+      <c r="B18" s="28" t="n"/>
+      <c r="C18" s="29" t="n"/>
+      <c r="D18" s="29" t="n"/>
+      <c r="E18" s="18">
         <f>IF(D18="","",D18*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F18" s="28" t="n"/>
+      <c r="F18" s="29" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="27" t="n"/>
-      <c r="B19" s="27" t="n"/>
-      <c r="C19" s="28" t="n"/>
-      <c r="D19" s="28" t="n"/>
-      <c r="E19" s="17">
+      <c r="A19" s="28" t="n"/>
+      <c r="B19" s="28" t="n"/>
+      <c r="C19" s="29" t="n"/>
+      <c r="D19" s="29" t="n"/>
+      <c r="E19" s="18">
         <f>IF(D19="","",D19*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F19" s="28" t="n"/>
+      <c r="F19" s="29" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="27" t="n"/>
-      <c r="B20" s="27" t="n"/>
-      <c r="C20" s="28" t="n"/>
-      <c r="D20" s="28" t="n"/>
-      <c r="E20" s="17">
+      <c r="A20" s="28" t="n"/>
+      <c r="B20" s="28" t="n"/>
+      <c r="C20" s="29" t="n"/>
+      <c r="D20" s="29" t="n"/>
+      <c r="E20" s="18">
         <f>IF(D20="","",D20*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F20" s="28" t="n"/>
+      <c r="F20" s="29" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="27" t="n"/>
-      <c r="B21" s="27" t="n"/>
-      <c r="C21" s="28" t="n"/>
-      <c r="D21" s="28" t="n"/>
-      <c r="E21" s="17">
+      <c r="A21" s="28" t="n"/>
+      <c r="B21" s="28" t="n"/>
+      <c r="C21" s="29" t="n"/>
+      <c r="D21" s="29" t="n"/>
+      <c r="E21" s="18">
         <f>IF(D21="","",D21*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F21" s="28" t="n"/>
+      <c r="F21" s="29" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="27" t="n"/>
-      <c r="B22" s="27" t="n"/>
-      <c r="C22" s="28" t="n"/>
-      <c r="D22" s="28" t="n"/>
-      <c r="E22" s="17">
+      <c r="A22" s="28" t="n"/>
+      <c r="B22" s="28" t="n"/>
+      <c r="C22" s="29" t="n"/>
+      <c r="D22" s="29" t="n"/>
+      <c r="E22" s="18">
         <f>IF(D22="","",D22*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F22" s="28" t="n"/>
+      <c r="F22" s="29" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="27" t="n"/>
-      <c r="B23" s="27" t="n"/>
-      <c r="C23" s="28" t="n"/>
-      <c r="D23" s="28" t="n"/>
-      <c r="E23" s="17">
+      <c r="A23" s="28" t="n"/>
+      <c r="B23" s="28" t="n"/>
+      <c r="C23" s="29" t="n"/>
+      <c r="D23" s="29" t="n"/>
+      <c r="E23" s="18">
         <f>IF(D23="","",D23*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F23" s="28" t="n"/>
+      <c r="F23" s="29" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="27" t="n"/>
-      <c r="B24" s="27" t="n"/>
-      <c r="C24" s="28" t="n"/>
-      <c r="D24" s="28" t="n"/>
-      <c r="E24" s="17">
+      <c r="A24" s="28" t="n"/>
+      <c r="B24" s="28" t="n"/>
+      <c r="C24" s="29" t="n"/>
+      <c r="D24" s="29" t="n"/>
+      <c r="E24" s="18">
         <f>IF(D24="","",D24*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F24" s="28" t="n"/>
+      <c r="F24" s="29" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="27" t="n"/>
-      <c r="B25" s="27" t="n"/>
-      <c r="C25" s="28" t="n"/>
-      <c r="D25" s="28" t="n"/>
-      <c r="E25" s="17">
+      <c r="A25" s="28" t="n"/>
+      <c r="B25" s="28" t="n"/>
+      <c r="C25" s="29" t="n"/>
+      <c r="D25" s="29" t="n"/>
+      <c r="E25" s="18">
         <f>IF(D25="","",D25*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F25" s="28" t="n"/>
+      <c r="F25" s="29" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="27" t="n"/>
-      <c r="B26" s="27" t="n"/>
-      <c r="C26" s="28" t="n"/>
-      <c r="D26" s="28" t="n"/>
-      <c r="E26" s="17">
+      <c r="A26" s="28" t="n"/>
+      <c r="B26" s="28" t="n"/>
+      <c r="C26" s="29" t="n"/>
+      <c r="D26" s="29" t="n"/>
+      <c r="E26" s="18">
         <f>IF(D26="","",D26*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F26" s="28" t="n"/>
+      <c r="F26" s="29" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="27" t="n"/>
-      <c r="B27" s="27" t="n"/>
-      <c r="C27" s="28" t="n"/>
-      <c r="D27" s="28" t="n"/>
-      <c r="E27" s="17">
+      <c r="A27" s="28" t="n"/>
+      <c r="B27" s="28" t="n"/>
+      <c r="C27" s="29" t="n"/>
+      <c r="D27" s="29" t="n"/>
+      <c r="E27" s="18">
         <f>IF(D27="","",D27*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F27" s="28" t="n"/>
+      <c r="F27" s="29" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="27" t="n"/>
-      <c r="B28" s="27" t="n"/>
-      <c r="C28" s="28" t="n"/>
-      <c r="D28" s="28" t="n"/>
-      <c r="E28" s="17">
+      <c r="A28" s="28" t="n"/>
+      <c r="B28" s="28" t="n"/>
+      <c r="C28" s="29" t="n"/>
+      <c r="D28" s="29" t="n"/>
+      <c r="E28" s="18">
         <f>IF(D28="","",D28*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F28" s="28" t="n"/>
+      <c r="F28" s="29" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="27" t="n"/>
-      <c r="B29" s="27" t="n"/>
-      <c r="C29" s="28" t="n"/>
-      <c r="D29" s="28" t="n"/>
-      <c r="E29" s="17">
+      <c r="A29" s="28" t="n"/>
+      <c r="B29" s="28" t="n"/>
+      <c r="C29" s="29" t="n"/>
+      <c r="D29" s="29" t="n"/>
+      <c r="E29" s="18">
         <f>IF(D29="","",D29*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F29" s="28" t="n"/>
+      <c r="F29" s="29" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="27" t="n"/>
-      <c r="B30" s="27" t="n"/>
-      <c r="C30" s="28" t="n"/>
-      <c r="D30" s="28" t="n"/>
-      <c r="E30" s="17">
+      <c r="A30" s="28" t="n"/>
+      <c r="B30" s="28" t="n"/>
+      <c r="C30" s="29" t="n"/>
+      <c r="D30" s="29" t="n"/>
+      <c r="E30" s="18">
         <f>IF(D30="","",D30*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F30" s="28" t="n"/>
+      <c r="F30" s="29" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="27" t="n"/>
-      <c r="B31" s="27" t="n"/>
-      <c r="C31" s="28" t="n"/>
-      <c r="D31" s="28" t="n"/>
-      <c r="E31" s="17">
+      <c r="A31" s="28" t="n"/>
+      <c r="B31" s="28" t="n"/>
+      <c r="C31" s="29" t="n"/>
+      <c r="D31" s="29" t="n"/>
+      <c r="E31" s="18">
         <f>IF(D31="","",D31*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F31" s="28" t="n"/>
+      <c r="F31" s="29" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="27" t="n"/>
-      <c r="B32" s="27" t="n"/>
-      <c r="C32" s="28" t="n"/>
-      <c r="D32" s="28" t="n"/>
-      <c r="E32" s="17">
+      <c r="A32" s="28" t="n"/>
+      <c r="B32" s="28" t="n"/>
+      <c r="C32" s="29" t="n"/>
+      <c r="D32" s="29" t="n"/>
+      <c r="E32" s="18">
         <f>IF(D32="","",D32*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F32" s="28" t="n"/>
+      <c r="F32" s="29" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="27" t="n"/>
-      <c r="B33" s="27" t="n"/>
-      <c r="C33" s="28" t="n"/>
-      <c r="D33" s="28" t="n"/>
-      <c r="E33" s="17">
+      <c r="A33" s="28" t="n"/>
+      <c r="B33" s="28" t="n"/>
+      <c r="C33" s="29" t="n"/>
+      <c r="D33" s="29" t="n"/>
+      <c r="E33" s="18">
         <f>IF(D33="","",D33*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F33" s="28" t="n"/>
+      <c r="F33" s="29" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="27" t="n"/>
-      <c r="B34" s="27" t="n"/>
-      <c r="C34" s="28" t="n"/>
-      <c r="D34" s="28" t="n"/>
-      <c r="E34" s="17">
+      <c r="A34" s="28" t="n"/>
+      <c r="B34" s="28" t="n"/>
+      <c r="C34" s="29" t="n"/>
+      <c r="D34" s="29" t="n"/>
+      <c r="E34" s="18">
         <f>IF(D34="","",D34*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F34" s="28" t="n"/>
+      <c r="F34" s="29" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="27" t="n"/>
-      <c r="B35" s="27" t="n"/>
-      <c r="C35" s="28" t="n"/>
-      <c r="D35" s="28" t="n"/>
-      <c r="E35" s="17">
+      <c r="A35" s="28" t="n"/>
+      <c r="B35" s="28" t="n"/>
+      <c r="C35" s="29" t="n"/>
+      <c r="D35" s="29" t="n"/>
+      <c r="E35" s="18">
         <f>IF(D35="","",D35*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F35" s="28" t="n"/>
+      <c r="F35" s="29" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="27" t="n"/>
-      <c r="B36" s="27" t="n"/>
-      <c r="C36" s="28" t="n"/>
-      <c r="D36" s="28" t="n"/>
-      <c r="E36" s="17">
+      <c r="A36" s="28" t="n"/>
+      <c r="B36" s="28" t="n"/>
+      <c r="C36" s="29" t="n"/>
+      <c r="D36" s="29" t="n"/>
+      <c r="E36" s="18">
         <f>IF(D36="","",D36*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F36" s="28" t="n"/>
+      <c r="F36" s="29" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="27" t="n"/>
-      <c r="B37" s="27" t="n"/>
-      <c r="C37" s="28" t="n"/>
-      <c r="D37" s="28" t="n"/>
-      <c r="E37" s="17">
+      <c r="A37" s="28" t="n"/>
+      <c r="B37" s="28" t="n"/>
+      <c r="C37" s="29" t="n"/>
+      <c r="D37" s="29" t="n"/>
+      <c r="E37" s="18">
         <f>IF(D37="","",D37*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F37" s="28" t="n"/>
+      <c r="F37" s="29" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="27" t="n"/>
-      <c r="B38" s="27" t="n"/>
-      <c r="C38" s="28" t="n"/>
-      <c r="D38" s="28" t="n"/>
-      <c r="E38" s="17">
+      <c r="A38" s="28" t="n"/>
+      <c r="B38" s="28" t="n"/>
+      <c r="C38" s="29" t="n"/>
+      <c r="D38" s="29" t="n"/>
+      <c r="E38" s="18">
         <f>IF(D38="","",D38*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F38" s="28" t="n"/>
+      <c r="F38" s="29" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="27" t="n"/>
-      <c r="B39" s="27" t="n"/>
-      <c r="C39" s="28" t="n"/>
-      <c r="D39" s="28" t="n"/>
-      <c r="E39" s="17">
+      <c r="A39" s="28" t="n"/>
+      <c r="B39" s="28" t="n"/>
+      <c r="C39" s="29" t="n"/>
+      <c r="D39" s="29" t="n"/>
+      <c r="E39" s="18">
         <f>IF(D39="","",D39*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F39" s="28" t="n"/>
+      <c r="F39" s="29" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="27" t="n"/>
-      <c r="B40" s="27" t="n"/>
-      <c r="C40" s="28" t="n"/>
-      <c r="D40" s="28" t="n"/>
-      <c r="E40" s="17">
+      <c r="A40" s="28" t="n"/>
+      <c r="B40" s="28" t="n"/>
+      <c r="C40" s="29" t="n"/>
+      <c r="D40" s="29" t="n"/>
+      <c r="E40" s="18">
         <f>IF(D40="","",D40*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F40" s="28" t="n"/>
+      <c r="F40" s="29" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="27" t="n"/>
-      <c r="B41" s="27" t="n"/>
-      <c r="C41" s="28" t="n"/>
-      <c r="D41" s="28" t="n"/>
-      <c r="E41" s="17">
+      <c r="A41" s="28" t="n"/>
+      <c r="B41" s="28" t="n"/>
+      <c r="C41" s="29" t="n"/>
+      <c r="D41" s="29" t="n"/>
+      <c r="E41" s="18">
         <f>IF(D41="","",D41*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F41" s="28" t="n"/>
+      <c r="F41" s="29" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="27" t="n"/>
-      <c r="B42" s="27" t="n"/>
-      <c r="C42" s="28" t="n"/>
-      <c r="D42" s="28" t="n"/>
-      <c r="E42" s="17">
+      <c r="A42" s="28" t="n"/>
+      <c r="B42" s="28" t="n"/>
+      <c r="C42" s="29" t="n"/>
+      <c r="D42" s="29" t="n"/>
+      <c r="E42" s="18">
         <f>IF(D42="","",D42*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F42" s="28" t="n"/>
+      <c r="F42" s="29" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="27" t="n"/>
-      <c r="B43" s="27" t="n"/>
-      <c r="C43" s="28" t="n"/>
-      <c r="D43" s="28" t="n"/>
-      <c r="E43" s="17">
+      <c r="A43" s="28" t="n"/>
+      <c r="B43" s="28" t="n"/>
+      <c r="C43" s="29" t="n"/>
+      <c r="D43" s="29" t="n"/>
+      <c r="E43" s="18">
         <f>IF(D43="","",D43*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F43" s="28" t="n"/>
+      <c r="F43" s="29" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="27" t="n"/>
-      <c r="B44" s="27" t="n"/>
-      <c r="C44" s="28" t="n"/>
-      <c r="D44" s="28" t="n"/>
-      <c r="E44" s="17">
+      <c r="A44" s="28" t="n"/>
+      <c r="B44" s="28" t="n"/>
+      <c r="C44" s="29" t="n"/>
+      <c r="D44" s="29" t="n"/>
+      <c r="E44" s="18">
         <f>IF(D44="","",D44*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F44" s="28" t="n"/>
+      <c r="F44" s="29" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="27" t="n"/>
-      <c r="B45" s="27" t="n"/>
-      <c r="C45" s="28" t="n"/>
-      <c r="D45" s="28" t="n"/>
-      <c r="E45" s="17">
+      <c r="A45" s="28" t="n"/>
+      <c r="B45" s="28" t="n"/>
+      <c r="C45" s="29" t="n"/>
+      <c r="D45" s="29" t="n"/>
+      <c r="E45" s="18">
         <f>IF(D45="","",D45*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F45" s="28" t="n"/>
+      <c r="F45" s="29" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="27" t="n"/>
-      <c r="B46" s="27" t="n"/>
-      <c r="C46" s="28" t="n"/>
-      <c r="D46" s="28" t="n"/>
-      <c r="E46" s="17">
+      <c r="A46" s="28" t="n"/>
+      <c r="B46" s="28" t="n"/>
+      <c r="C46" s="29" t="n"/>
+      <c r="D46" s="29" t="n"/>
+      <c r="E46" s="18">
         <f>IF(D46="","",D46*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F46" s="28" t="n"/>
+      <c r="F46" s="29" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="27" t="n"/>
-      <c r="B47" s="27" t="n"/>
-      <c r="C47" s="28" t="n"/>
-      <c r="D47" s="28" t="n"/>
-      <c r="E47" s="17">
+      <c r="A47" s="28" t="n"/>
+      <c r="B47" s="28" t="n"/>
+      <c r="C47" s="29" t="n"/>
+      <c r="D47" s="29" t="n"/>
+      <c r="E47" s="18">
         <f>IF(D47="","",D47*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F47" s="28" t="n"/>
+      <c r="F47" s="29" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="27" t="n"/>
-      <c r="B48" s="27" t="n"/>
-      <c r="C48" s="28" t="n"/>
-      <c r="D48" s="28" t="n"/>
-      <c r="E48" s="17">
+      <c r="A48" s="28" t="n"/>
+      <c r="B48" s="28" t="n"/>
+      <c r="C48" s="29" t="n"/>
+      <c r="D48" s="29" t="n"/>
+      <c r="E48" s="18">
         <f>IF(D48="","",D48*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F48" s="28" t="n"/>
+      <c r="F48" s="29" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="27" t="n"/>
-      <c r="B49" s="27" t="n"/>
-      <c r="C49" s="28" t="n"/>
-      <c r="D49" s="28" t="n"/>
-      <c r="E49" s="17">
+      <c r="A49" s="28" t="n"/>
+      <c r="B49" s="28" t="n"/>
+      <c r="C49" s="29" t="n"/>
+      <c r="D49" s="29" t="n"/>
+      <c r="E49" s="18">
         <f>IF(D49="","",D49*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F49" s="28" t="n"/>
+      <c r="F49" s="29" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="27" t="n"/>
-      <c r="B50" s="27" t="n"/>
-      <c r="C50" s="28" t="n"/>
-      <c r="D50" s="28" t="n"/>
-      <c r="E50" s="17">
+      <c r="A50" s="28" t="n"/>
+      <c r="B50" s="28" t="n"/>
+      <c r="C50" s="29" t="n"/>
+      <c r="D50" s="29" t="n"/>
+      <c r="E50" s="18">
         <f>IF(D50="","",D50*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F50" s="28" t="n"/>
+      <c r="F50" s="29" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="27" t="n"/>
-      <c r="B51" s="27" t="n"/>
-      <c r="C51" s="28" t="n"/>
-      <c r="D51" s="28" t="n"/>
-      <c r="E51" s="17">
+      <c r="A51" s="28" t="n"/>
+      <c r="B51" s="28" t="n"/>
+      <c r="C51" s="29" t="n"/>
+      <c r="D51" s="29" t="n"/>
+      <c r="E51" s="18">
         <f>IF(D51="","",D51*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F51" s="28" t="n"/>
+      <c r="F51" s="29" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="27" t="n"/>
-      <c r="B52" s="27" t="n"/>
-      <c r="C52" s="28" t="n"/>
-      <c r="D52" s="28" t="n"/>
-      <c r="E52" s="17">
+      <c r="A52" s="28" t="n"/>
+      <c r="B52" s="28" t="n"/>
+      <c r="C52" s="29" t="n"/>
+      <c r="D52" s="29" t="n"/>
+      <c r="E52" s="18">
         <f>IF(D52="","",D52*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F52" s="28" t="n"/>
+      <c r="F52" s="29" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="27" t="n"/>
-      <c r="B53" s="27" t="n"/>
-      <c r="C53" s="28" t="n"/>
-      <c r="D53" s="28" t="n"/>
-      <c r="E53" s="17">
+      <c r="A53" s="28" t="n"/>
+      <c r="B53" s="28" t="n"/>
+      <c r="C53" s="29" t="n"/>
+      <c r="D53" s="29" t="n"/>
+      <c r="E53" s="18">
         <f>IF(D53="","",D53*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F53" s="28" t="n"/>
+      <c r="F53" s="29" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="27" t="n"/>
-      <c r="B54" s="27" t="n"/>
-      <c r="C54" s="28" t="n"/>
-      <c r="D54" s="28" t="n"/>
-      <c r="E54" s="17">
+      <c r="A54" s="28" t="n"/>
+      <c r="B54" s="28" t="n"/>
+      <c r="C54" s="29" t="n"/>
+      <c r="D54" s="29" t="n"/>
+      <c r="E54" s="18">
         <f>IF(D54="","",D54*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F54" s="28" t="n"/>
+      <c r="F54" s="29" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="27" t="n"/>
-      <c r="B55" s="27" t="n"/>
-      <c r="C55" s="28" t="n"/>
-      <c r="D55" s="28" t="n"/>
-      <c r="E55" s="17">
+      <c r="A55" s="28" t="n"/>
+      <c r="B55" s="28" t="n"/>
+      <c r="C55" s="29" t="n"/>
+      <c r="D55" s="29" t="n"/>
+      <c r="E55" s="18">
         <f>IF(D55="","",D55*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F55" s="28" t="n"/>
+      <c r="F55" s="29" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="27" t="n"/>
-      <c r="B56" s="27" t="n"/>
-      <c r="C56" s="28" t="n"/>
-      <c r="D56" s="28" t="n"/>
-      <c r="E56" s="17">
+      <c r="A56" s="28" t="n"/>
+      <c r="B56" s="28" t="n"/>
+      <c r="C56" s="29" t="n"/>
+      <c r="D56" s="29" t="n"/>
+      <c r="E56" s="18">
         <f>IF(D56="","",D56*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F56" s="28" t="n"/>
+      <c r="F56" s="29" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="27" t="n"/>
-      <c r="B57" s="27" t="n"/>
-      <c r="C57" s="28" t="n"/>
-      <c r="D57" s="28" t="n"/>
-      <c r="E57" s="17">
+      <c r="A57" s="28" t="n"/>
+      <c r="B57" s="28" t="n"/>
+      <c r="C57" s="29" t="n"/>
+      <c r="D57" s="29" t="n"/>
+      <c r="E57" s="18">
         <f>IF(D57="","",D57*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F57" s="28" t="n"/>
+      <c r="F57" s="29" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="27" t="n"/>
-      <c r="B58" s="27" t="n"/>
-      <c r="C58" s="28" t="n"/>
-      <c r="D58" s="28" t="n"/>
-      <c r="E58" s="17">
+      <c r="A58" s="28" t="n"/>
+      <c r="B58" s="28" t="n"/>
+      <c r="C58" s="29" t="n"/>
+      <c r="D58" s="29" t="n"/>
+      <c r="E58" s="18">
         <f>IF(D58="","",D58*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F58" s="28" t="n"/>
+      <c r="F58" s="29" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="27" t="n"/>
-      <c r="B59" s="27" t="n"/>
-      <c r="C59" s="28" t="n"/>
-      <c r="D59" s="28" t="n"/>
-      <c r="E59" s="17">
+      <c r="A59" s="28" t="n"/>
+      <c r="B59" s="28" t="n"/>
+      <c r="C59" s="29" t="n"/>
+      <c r="D59" s="29" t="n"/>
+      <c r="E59" s="18">
         <f>IF(D59="","",D59*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F59" s="28" t="n"/>
+      <c r="F59" s="29" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="27" t="n"/>
-      <c r="B60" s="27" t="n"/>
-      <c r="C60" s="28" t="n"/>
-      <c r="D60" s="28" t="n"/>
-      <c r="E60" s="17">
+      <c r="A60" s="28" t="n"/>
+      <c r="B60" s="28" t="n"/>
+      <c r="C60" s="29" t="n"/>
+      <c r="D60" s="29" t="n"/>
+      <c r="E60" s="18">
         <f>IF(D60="","",D60*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F60" s="28" t="n"/>
+      <c r="F60" s="29" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="27" t="n"/>
-      <c r="B61" s="27" t="n"/>
-      <c r="C61" s="28" t="n"/>
-      <c r="D61" s="28" t="n"/>
-      <c r="E61" s="17">
+      <c r="A61" s="28" t="n"/>
+      <c r="B61" s="28" t="n"/>
+      <c r="C61" s="29" t="n"/>
+      <c r="D61" s="29" t="n"/>
+      <c r="E61" s="18">
         <f>IF(D61="","",D61*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F61" s="28" t="n"/>
+      <c r="F61" s="29" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="27" t="n"/>
-      <c r="B62" s="27" t="n"/>
-      <c r="C62" s="28" t="n"/>
-      <c r="D62" s="28" t="n"/>
-      <c r="E62" s="17">
+      <c r="A62" s="28" t="n"/>
+      <c r="B62" s="28" t="n"/>
+      <c r="C62" s="29" t="n"/>
+      <c r="D62" s="29" t="n"/>
+      <c r="E62" s="18">
         <f>IF(D62="","",D62*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F62" s="28" t="n"/>
+      <c r="F62" s="29" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="27" t="n"/>
-      <c r="B63" s="27" t="n"/>
-      <c r="C63" s="28" t="n"/>
-      <c r="D63" s="28" t="n"/>
-      <c r="E63" s="17">
+      <c r="A63" s="28" t="n"/>
+      <c r="B63" s="28" t="n"/>
+      <c r="C63" s="29" t="n"/>
+      <c r="D63" s="29" t="n"/>
+      <c r="E63" s="18">
         <f>IF(D63="","",D63*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F63" s="28" t="n"/>
+      <c r="F63" s="29" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="27" t="n"/>
-      <c r="B64" s="27" t="n"/>
-      <c r="C64" s="28" t="n"/>
-      <c r="D64" s="28" t="n"/>
-      <c r="E64" s="17">
+      <c r="A64" s="28" t="n"/>
+      <c r="B64" s="28" t="n"/>
+      <c r="C64" s="29" t="n"/>
+      <c r="D64" s="29" t="n"/>
+      <c r="E64" s="18">
         <f>IF(D64="","",D64*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F64" s="28" t="n"/>
+      <c r="F64" s="29" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="27" t="n"/>
-      <c r="B65" s="27" t="n"/>
-      <c r="C65" s="28" t="n"/>
-      <c r="D65" s="28" t="n"/>
-      <c r="E65" s="17">
+      <c r="A65" s="28" t="n"/>
+      <c r="B65" s="28" t="n"/>
+      <c r="C65" s="29" t="n"/>
+      <c r="D65" s="29" t="n"/>
+      <c r="E65" s="18">
         <f>IF(D65="","",D65*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F65" s="28" t="n"/>
+      <c r="F65" s="29" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="27" t="n"/>
-      <c r="B66" s="27" t="n"/>
-      <c r="C66" s="28" t="n"/>
-      <c r="D66" s="28" t="n"/>
-      <c r="E66" s="17">
+      <c r="A66" s="28" t="n"/>
+      <c r="B66" s="28" t="n"/>
+      <c r="C66" s="29" t="n"/>
+      <c r="D66" s="29" t="n"/>
+      <c r="E66" s="18">
         <f>IF(D66="","",D66*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F66" s="28" t="n"/>
+      <c r="F66" s="29" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="27" t="n"/>
-      <c r="B67" s="27" t="n"/>
-      <c r="C67" s="28" t="n"/>
-      <c r="D67" s="28" t="n"/>
-      <c r="E67" s="17">
+      <c r="A67" s="28" t="n"/>
+      <c r="B67" s="28" t="n"/>
+      <c r="C67" s="29" t="n"/>
+      <c r="D67" s="29" t="n"/>
+      <c r="E67" s="18">
         <f>IF(D67="","",D67*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F67" s="28" t="n"/>
+      <c r="F67" s="29" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="27" t="n"/>
-      <c r="B68" s="27" t="n"/>
-      <c r="C68" s="28" t="n"/>
-      <c r="D68" s="28" t="n"/>
-      <c r="E68" s="17">
+      <c r="A68" s="28" t="n"/>
+      <c r="B68" s="28" t="n"/>
+      <c r="C68" s="29" t="n"/>
+      <c r="D68" s="29" t="n"/>
+      <c r="E68" s="18">
         <f>IF(D68="","",D68*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F68" s="28" t="n"/>
+      <c r="F68" s="29" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="27" t="n"/>
-      <c r="B69" s="27" t="n"/>
-      <c r="C69" s="28" t="n"/>
-      <c r="D69" s="28" t="n"/>
-      <c r="E69" s="17">
+      <c r="A69" s="28" t="n"/>
+      <c r="B69" s="28" t="n"/>
+      <c r="C69" s="29" t="n"/>
+      <c r="D69" s="29" t="n"/>
+      <c r="E69" s="18">
         <f>IF(D69="","",D69*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F69" s="28" t="n"/>
+      <c r="F69" s="29" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="27" t="n"/>
-      <c r="B70" s="27" t="n"/>
-      <c r="C70" s="28" t="n"/>
-      <c r="D70" s="28" t="n"/>
-      <c r="E70" s="17">
+      <c r="A70" s="28" t="n"/>
+      <c r="B70" s="28" t="n"/>
+      <c r="C70" s="29" t="n"/>
+      <c r="D70" s="29" t="n"/>
+      <c r="E70" s="18">
         <f>IF(D70="","",D70*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F70" s="28" t="n"/>
+      <c r="F70" s="29" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="27" t="n"/>
-      <c r="B71" s="27" t="n"/>
-      <c r="C71" s="28" t="n"/>
-      <c r="D71" s="28" t="n"/>
-      <c r="E71" s="17">
+      <c r="A71" s="28" t="n"/>
+      <c r="B71" s="28" t="n"/>
+      <c r="C71" s="29" t="n"/>
+      <c r="D71" s="29" t="n"/>
+      <c r="E71" s="18">
         <f>IF(D71="","",D71*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F71" s="28" t="n"/>
+      <c r="F71" s="29" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="27" t="n"/>
-      <c r="B72" s="27" t="n"/>
-      <c r="C72" s="28" t="n"/>
-      <c r="D72" s="28" t="n"/>
-      <c r="E72" s="17">
+      <c r="A72" s="28" t="n"/>
+      <c r="B72" s="28" t="n"/>
+      <c r="C72" s="29" t="n"/>
+      <c r="D72" s="29" t="n"/>
+      <c r="E72" s="18">
         <f>IF(D72="","",D72*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F72" s="28" t="n"/>
+      <c r="F72" s="29" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="27" t="n"/>
-      <c r="B73" s="27" t="n"/>
-      <c r="C73" s="28" t="n"/>
-      <c r="D73" s="28" t="n"/>
-      <c r="E73" s="17">
+      <c r="A73" s="28" t="n"/>
+      <c r="B73" s="28" t="n"/>
+      <c r="C73" s="29" t="n"/>
+      <c r="D73" s="29" t="n"/>
+      <c r="E73" s="18">
         <f>IF(D73="","",D73*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F73" s="28" t="n"/>
+      <c r="F73" s="29" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="27" t="n"/>
-      <c r="B74" s="27" t="n"/>
-      <c r="C74" s="28" t="n"/>
-      <c r="D74" s="28" t="n"/>
-      <c r="E74" s="17">
+      <c r="A74" s="28" t="n"/>
+      <c r="B74" s="28" t="n"/>
+      <c r="C74" s="29" t="n"/>
+      <c r="D74" s="29" t="n"/>
+      <c r="E74" s="18">
         <f>IF(D74="","",D74*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F74" s="28" t="n"/>
+      <c r="F74" s="29" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="27" t="n"/>
-      <c r="B75" s="27" t="n"/>
-      <c r="C75" s="28" t="n"/>
-      <c r="D75" s="28" t="n"/>
-      <c r="E75" s="17">
+      <c r="A75" s="28" t="n"/>
+      <c r="B75" s="28" t="n"/>
+      <c r="C75" s="29" t="n"/>
+      <c r="D75" s="29" t="n"/>
+      <c r="E75" s="18">
         <f>IF(D75="","",D75*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F75" s="28" t="n"/>
+      <c r="F75" s="29" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="27" t="n"/>
-      <c r="B76" s="27" t="n"/>
-      <c r="C76" s="28" t="n"/>
-      <c r="D76" s="28" t="n"/>
-      <c r="E76" s="17">
+      <c r="A76" s="28" t="n"/>
+      <c r="B76" s="28" t="n"/>
+      <c r="C76" s="29" t="n"/>
+      <c r="D76" s="29" t="n"/>
+      <c r="E76" s="18">
         <f>IF(D76="","",D76*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F76" s="28" t="n"/>
+      <c r="F76" s="29" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="27" t="n"/>
-      <c r="B77" s="27" t="n"/>
-      <c r="C77" s="28" t="n"/>
-      <c r="D77" s="28" t="n"/>
-      <c r="E77" s="17">
+      <c r="A77" s="28" t="n"/>
+      <c r="B77" s="28" t="n"/>
+      <c r="C77" s="29" t="n"/>
+      <c r="D77" s="29" t="n"/>
+      <c r="E77" s="18">
         <f>IF(D77="","",D77*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F77" s="28" t="n"/>
+      <c r="F77" s="29" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="27" t="n"/>
-      <c r="B78" s="27" t="n"/>
-      <c r="C78" s="28" t="n"/>
-      <c r="D78" s="28" t="n"/>
-      <c r="E78" s="17">
+      <c r="A78" s="28" t="n"/>
+      <c r="B78" s="28" t="n"/>
+      <c r="C78" s="29" t="n"/>
+      <c r="D78" s="29" t="n"/>
+      <c r="E78" s="18">
         <f>IF(D78="","",D78*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F78" s="28" t="n"/>
+      <c r="F78" s="29" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="27" t="n"/>
-      <c r="B79" s="27" t="n"/>
-      <c r="C79" s="28" t="n"/>
-      <c r="D79" s="28" t="n"/>
-      <c r="E79" s="17">
+      <c r="A79" s="28" t="n"/>
+      <c r="B79" s="28" t="n"/>
+      <c r="C79" s="29" t="n"/>
+      <c r="D79" s="29" t="n"/>
+      <c r="E79" s="18">
         <f>IF(D79="","",D79*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F79" s="28" t="n"/>
+      <c r="F79" s="29" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="27" t="n"/>
-      <c r="B80" s="27" t="n"/>
-      <c r="C80" s="28" t="n"/>
-      <c r="D80" s="28" t="n"/>
-      <c r="E80" s="17">
+      <c r="A80" s="28" t="n"/>
+      <c r="B80" s="28" t="n"/>
+      <c r="C80" s="29" t="n"/>
+      <c r="D80" s="29" t="n"/>
+      <c r="E80" s="18">
         <f>IF(D80="","",D80*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F80" s="28" t="n"/>
+      <c r="F80" s="29" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="27" t="n"/>
-      <c r="B81" s="27" t="n"/>
-      <c r="C81" s="28" t="n"/>
-      <c r="D81" s="28" t="n"/>
-      <c r="E81" s="17">
+      <c r="A81" s="28" t="n"/>
+      <c r="B81" s="28" t="n"/>
+      <c r="C81" s="29" t="n"/>
+      <c r="D81" s="29" t="n"/>
+      <c r="E81" s="18">
         <f>IF(D81="","",D81*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F81" s="28" t="n"/>
+      <c r="F81" s="29" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="27" t="n"/>
-      <c r="B82" s="27" t="n"/>
-      <c r="C82" s="28" t="n"/>
-      <c r="D82" s="28" t="n"/>
-      <c r="E82" s="17">
+      <c r="A82" s="28" t="n"/>
+      <c r="B82" s="28" t="n"/>
+      <c r="C82" s="29" t="n"/>
+      <c r="D82" s="29" t="n"/>
+      <c r="E82" s="18">
         <f>IF(D82="","",D82*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F82" s="28" t="n"/>
+      <c r="F82" s="29" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="27" t="n"/>
-      <c r="B83" s="27" t="n"/>
-      <c r="C83" s="28" t="n"/>
-      <c r="D83" s="28" t="n"/>
-      <c r="E83" s="17">
+      <c r="A83" s="28" t="n"/>
+      <c r="B83" s="28" t="n"/>
+      <c r="C83" s="29" t="n"/>
+      <c r="D83" s="29" t="n"/>
+      <c r="E83" s="18">
         <f>IF(D83="","",D83*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F83" s="28" t="n"/>
+      <c r="F83" s="29" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="27" t="n"/>
-      <c r="B84" s="27" t="n"/>
-      <c r="C84" s="28" t="n"/>
-      <c r="D84" s="28" t="n"/>
-      <c r="E84" s="17">
+      <c r="A84" s="28" t="n"/>
+      <c r="B84" s="28" t="n"/>
+      <c r="C84" s="29" t="n"/>
+      <c r="D84" s="29" t="n"/>
+      <c r="E84" s="18">
         <f>IF(D84="","",D84*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F84" s="28" t="n"/>
+      <c r="F84" s="29" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="27" t="n"/>
-      <c r="B85" s="27" t="n"/>
-      <c r="C85" s="28" t="n"/>
-      <c r="D85" s="28" t="n"/>
-      <c r="E85" s="17">
+      <c r="A85" s="28" t="n"/>
+      <c r="B85" s="28" t="n"/>
+      <c r="C85" s="29" t="n"/>
+      <c r="D85" s="29" t="n"/>
+      <c r="E85" s="18">
         <f>IF(D85="","",D85*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F85" s="28" t="n"/>
+      <c r="F85" s="29" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="27" t="n"/>
-      <c r="B86" s="27" t="n"/>
-      <c r="C86" s="28" t="n"/>
-      <c r="D86" s="28" t="n"/>
-      <c r="E86" s="17">
+      <c r="A86" s="28" t="n"/>
+      <c r="B86" s="28" t="n"/>
+      <c r="C86" s="29" t="n"/>
+      <c r="D86" s="29" t="n"/>
+      <c r="E86" s="18">
         <f>IF(D86="","",D86*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F86" s="28" t="n"/>
+      <c r="F86" s="29" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="27" t="n"/>
-      <c r="B87" s="27" t="n"/>
-      <c r="C87" s="28" t="n"/>
-      <c r="D87" s="28" t="n"/>
-      <c r="E87" s="17">
+      <c r="A87" s="28" t="n"/>
+      <c r="B87" s="28" t="n"/>
+      <c r="C87" s="29" t="n"/>
+      <c r="D87" s="29" t="n"/>
+      <c r="E87" s="18">
         <f>IF(D87="","",D87*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F87" s="28" t="n"/>
+      <c r="F87" s="29" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="27" t="n"/>
-      <c r="B88" s="27" t="n"/>
-      <c r="C88" s="28" t="n"/>
-      <c r="D88" s="28" t="n"/>
-      <c r="E88" s="17">
+      <c r="A88" s="28" t="n"/>
+      <c r="B88" s="28" t="n"/>
+      <c r="C88" s="29" t="n"/>
+      <c r="D88" s="29" t="n"/>
+      <c r="E88" s="18">
         <f>IF(D88="","",D88*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F88" s="28" t="n"/>
+      <c r="F88" s="29" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="27" t="n"/>
-      <c r="B89" s="27" t="n"/>
-      <c r="C89" s="28" t="n"/>
-      <c r="D89" s="28" t="n"/>
-      <c r="E89" s="17">
+      <c r="A89" s="28" t="n"/>
+      <c r="B89" s="28" t="n"/>
+      <c r="C89" s="29" t="n"/>
+      <c r="D89" s="29" t="n"/>
+      <c r="E89" s="18">
         <f>IF(D89="","",D89*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F89" s="28" t="n"/>
+      <c r="F89" s="29" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="27" t="n"/>
-      <c r="B90" s="27" t="n"/>
-      <c r="C90" s="28" t="n"/>
-      <c r="D90" s="28" t="n"/>
-      <c r="E90" s="17">
+      <c r="A90" s="28" t="n"/>
+      <c r="B90" s="28" t="n"/>
+      <c r="C90" s="29" t="n"/>
+      <c r="D90" s="29" t="n"/>
+      <c r="E90" s="18">
         <f>IF(D90="","",D90*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F90" s="28" t="n"/>
+      <c r="F90" s="29" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="27" t="n"/>
-      <c r="B91" s="27" t="n"/>
-      <c r="C91" s="28" t="n"/>
-      <c r="D91" s="28" t="n"/>
-      <c r="E91" s="17">
+      <c r="A91" s="28" t="n"/>
+      <c r="B91" s="28" t="n"/>
+      <c r="C91" s="29" t="n"/>
+      <c r="D91" s="29" t="n"/>
+      <c r="E91" s="18">
         <f>IF(D91="","",D91*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F91" s="28" t="n"/>
+      <c r="F91" s="29" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="27" t="n"/>
-      <c r="B92" s="27" t="n"/>
-      <c r="C92" s="28" t="n"/>
-      <c r="D92" s="28" t="n"/>
-      <c r="E92" s="17">
+      <c r="A92" s="28" t="n"/>
+      <c r="B92" s="28" t="n"/>
+      <c r="C92" s="29" t="n"/>
+      <c r="D92" s="29" t="n"/>
+      <c r="E92" s="18">
         <f>IF(D92="","",D92*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F92" s="28" t="n"/>
+      <c r="F92" s="29" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="27" t="n"/>
-      <c r="B93" s="27" t="n"/>
-      <c r="C93" s="28" t="n"/>
-      <c r="D93" s="28" t="n"/>
-      <c r="E93" s="17">
+      <c r="A93" s="28" t="n"/>
+      <c r="B93" s="28" t="n"/>
+      <c r="C93" s="29" t="n"/>
+      <c r="D93" s="29" t="n"/>
+      <c r="E93" s="18">
         <f>IF(D93="","",D93*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F93" s="28" t="n"/>
+      <c r="F93" s="29" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="27" t="n"/>
-      <c r="B94" s="27" t="n"/>
-      <c r="C94" s="28" t="n"/>
-      <c r="D94" s="28" t="n"/>
-      <c r="E94" s="17">
+      <c r="A94" s="28" t="n"/>
+      <c r="B94" s="28" t="n"/>
+      <c r="C94" s="29" t="n"/>
+      <c r="D94" s="29" t="n"/>
+      <c r="E94" s="18">
         <f>IF(D94="","",D94*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F94" s="28" t="n"/>
+      <c r="F94" s="29" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="27" t="n"/>
-      <c r="B95" s="27" t="n"/>
-      <c r="C95" s="28" t="n"/>
-      <c r="D95" s="28" t="n"/>
-      <c r="E95" s="17">
+      <c r="A95" s="28" t="n"/>
+      <c r="B95" s="28" t="n"/>
+      <c r="C95" s="29" t="n"/>
+      <c r="D95" s="29" t="n"/>
+      <c r="E95" s="18">
         <f>IF(D95="","",D95*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F95" s="28" t="n"/>
+      <c r="F95" s="29" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="27" t="n"/>
-      <c r="B96" s="27" t="n"/>
-      <c r="C96" s="28" t="n"/>
-      <c r="D96" s="28" t="n"/>
-      <c r="E96" s="17">
+      <c r="A96" s="28" t="n"/>
+      <c r="B96" s="28" t="n"/>
+      <c r="C96" s="29" t="n"/>
+      <c r="D96" s="29" t="n"/>
+      <c r="E96" s="18">
         <f>IF(D96="","",D96*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F96" s="28" t="n"/>
+      <c r="F96" s="29" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="27" t="n"/>
-      <c r="B97" s="27" t="n"/>
-      <c r="C97" s="28" t="n"/>
-      <c r="D97" s="28" t="n"/>
-      <c r="E97" s="17">
+      <c r="A97" s="28" t="n"/>
+      <c r="B97" s="28" t="n"/>
+      <c r="C97" s="29" t="n"/>
+      <c r="D97" s="29" t="n"/>
+      <c r="E97" s="18">
         <f>IF(D97="","",D97*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F97" s="28" t="n"/>
+      <c r="F97" s="29" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="27" t="n"/>
-      <c r="B98" s="27" t="n"/>
-      <c r="C98" s="28" t="n"/>
-      <c r="D98" s="28" t="n"/>
-      <c r="E98" s="17">
+      <c r="A98" s="28" t="n"/>
+      <c r="B98" s="28" t="n"/>
+      <c r="C98" s="29" t="n"/>
+      <c r="D98" s="29" t="n"/>
+      <c r="E98" s="18">
         <f>IF(D98="","",D98*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F98" s="28" t="n"/>
+      <c r="F98" s="29" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="27" t="n"/>
-      <c r="B99" s="27" t="n"/>
-      <c r="C99" s="28" t="n"/>
-      <c r="D99" s="28" t="n"/>
-      <c r="E99" s="17">
+      <c r="A99" s="28" t="n"/>
+      <c r="B99" s="28" t="n"/>
+      <c r="C99" s="29" t="n"/>
+      <c r="D99" s="29" t="n"/>
+      <c r="E99" s="18">
         <f>IF(D99="","",D99*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F99" s="28" t="n"/>
+      <c r="F99" s="29" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="27" t="n"/>
-      <c r="B100" s="27" t="n"/>
-      <c r="C100" s="28" t="n"/>
-      <c r="D100" s="28" t="n"/>
-      <c r="E100" s="17">
+      <c r="A100" s="28" t="n"/>
+      <c r="B100" s="28" t="n"/>
+      <c r="C100" s="29" t="n"/>
+      <c r="D100" s="29" t="n"/>
+      <c r="E100" s="18">
         <f>IF(D100="","",D100*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F100" s="28" t="n"/>
+      <c r="F100" s="29" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="27" t="n"/>
-      <c r="B101" s="27" t="n"/>
-      <c r="C101" s="28" t="n"/>
-      <c r="D101" s="28" t="n"/>
-      <c r="E101" s="17">
+      <c r="A101" s="28" t="n"/>
+      <c r="B101" s="28" t="n"/>
+      <c r="C101" s="29" t="n"/>
+      <c r="D101" s="29" t="n"/>
+      <c r="E101" s="18">
         <f>IF(D101="","",D101*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F101" s="28" t="n"/>
+      <c r="F101" s="29" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="27" t="n"/>
-      <c r="B102" s="27" t="n"/>
-      <c r="C102" s="28" t="n"/>
-      <c r="D102" s="28" t="n"/>
-      <c r="E102" s="17">
+      <c r="A102" s="28" t="n"/>
+      <c r="B102" s="28" t="n"/>
+      <c r="C102" s="29" t="n"/>
+      <c r="D102" s="29" t="n"/>
+      <c r="E102" s="18">
         <f>IF(D102="","",D102*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F102" s="28" t="n"/>
+      <c r="F102" s="29" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="27" t="n"/>
-      <c r="B103" s="27" t="n"/>
-      <c r="C103" s="28" t="n"/>
-      <c r="D103" s="28" t="n"/>
-      <c r="E103" s="17">
+      <c r="A103" s="28" t="n"/>
+      <c r="B103" s="28" t="n"/>
+      <c r="C103" s="29" t="n"/>
+      <c r="D103" s="29" t="n"/>
+      <c r="E103" s="18">
         <f>IF(D103="","",D103*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F103" s="28" t="n"/>
+      <c r="F103" s="29" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="27" t="n"/>
-      <c r="B104" s="27" t="n"/>
-      <c r="C104" s="28" t="n"/>
-      <c r="D104" s="28" t="n"/>
-      <c r="E104" s="17">
+      <c r="A104" s="28" t="n"/>
+      <c r="B104" s="28" t="n"/>
+      <c r="C104" s="29" t="n"/>
+      <c r="D104" s="29" t="n"/>
+      <c r="E104" s="18">
         <f>IF(D104="","",D104*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F104" s="28" t="n"/>
+      <c r="F104" s="29" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="27" t="n"/>
-      <c r="B105" s="27" t="n"/>
-      <c r="C105" s="28" t="n"/>
-      <c r="D105" s="28" t="n"/>
-      <c r="E105" s="17">
+      <c r="A105" s="28" t="n"/>
+      <c r="B105" s="28" t="n"/>
+      <c r="C105" s="29" t="n"/>
+      <c r="D105" s="29" t="n"/>
+      <c r="E105" s="18">
         <f>IF(D105="","",D105*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F105" s="28" t="n"/>
+      <c r="F105" s="29" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="27" t="n"/>
-      <c r="B106" s="27" t="n"/>
-      <c r="C106" s="28" t="n"/>
-      <c r="D106" s="28" t="n"/>
-      <c r="E106" s="17">
+      <c r="A106" s="28" t="n"/>
+      <c r="B106" s="28" t="n"/>
+      <c r="C106" s="29" t="n"/>
+      <c r="D106" s="29" t="n"/>
+      <c r="E106" s="18">
         <f>IF(D106="","",D106*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F106" s="28" t="n"/>
+      <c r="F106" s="29" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="27" t="n"/>
-      <c r="B107" s="27" t="n"/>
-      <c r="C107" s="28" t="n"/>
-      <c r="D107" s="28" t="n"/>
-      <c r="E107" s="17">
+      <c r="A107" s="28" t="n"/>
+      <c r="B107" s="28" t="n"/>
+      <c r="C107" s="29" t="n"/>
+      <c r="D107" s="29" t="n"/>
+      <c r="E107" s="18">
         <f>IF(D107="","",D107*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F107" s="28" t="n"/>
+      <c r="F107" s="29" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="27" t="n"/>
-      <c r="B108" s="27" t="n"/>
-      <c r="C108" s="28" t="n"/>
-      <c r="D108" s="28" t="n"/>
-      <c r="E108" s="17">
+      <c r="A108" s="28" t="n"/>
+      <c r="B108" s="28" t="n"/>
+      <c r="C108" s="29" t="n"/>
+      <c r="D108" s="29" t="n"/>
+      <c r="E108" s="18">
         <f>IF(D108="","",D108*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F108" s="28" t="n"/>
+      <c r="F108" s="29" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="27" t="n"/>
-      <c r="B109" s="27" t="n"/>
-      <c r="C109" s="28" t="n"/>
-      <c r="D109" s="28" t="n"/>
-      <c r="E109" s="17">
+      <c r="A109" s="28" t="n"/>
+      <c r="B109" s="28" t="n"/>
+      <c r="C109" s="29" t="n"/>
+      <c r="D109" s="29" t="n"/>
+      <c r="E109" s="18">
         <f>IF(D109="","",D109*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F109" s="28" t="n"/>
+      <c r="F109" s="29" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="27" t="n"/>
-      <c r="B110" s="27" t="n"/>
-      <c r="C110" s="28" t="n"/>
-      <c r="D110" s="28" t="n"/>
-      <c r="E110" s="17">
+      <c r="A110" s="28" t="n"/>
+      <c r="B110" s="28" t="n"/>
+      <c r="C110" s="29" t="n"/>
+      <c r="D110" s="29" t="n"/>
+      <c r="E110" s="18">
         <f>IF(D110="","",D110*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F110" s="28" t="n"/>
+      <c r="F110" s="29" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="27" t="n"/>
-      <c r="B111" s="27" t="n"/>
-      <c r="C111" s="28" t="n"/>
-      <c r="D111" s="28" t="n"/>
-      <c r="E111" s="17">
+      <c r="A111" s="28" t="n"/>
+      <c r="B111" s="28" t="n"/>
+      <c r="C111" s="29" t="n"/>
+      <c r="D111" s="29" t="n"/>
+      <c r="E111" s="18">
         <f>IF(D111="","",D111*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F111" s="28" t="n"/>
+      <c r="F111" s="29" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="27" t="n"/>
-      <c r="B112" s="27" t="n"/>
-      <c r="C112" s="28" t="n"/>
-      <c r="D112" s="28" t="n"/>
-      <c r="E112" s="17">
+      <c r="A112" s="28" t="n"/>
+      <c r="B112" s="28" t="n"/>
+      <c r="C112" s="29" t="n"/>
+      <c r="D112" s="29" t="n"/>
+      <c r="E112" s="18">
         <f>IF(D112="","",D112*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F112" s="28" t="n"/>
+      <c r="F112" s="29" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="27" t="n"/>
-      <c r="B113" s="27" t="n"/>
-      <c r="C113" s="28" t="n"/>
-      <c r="D113" s="28" t="n"/>
-      <c r="E113" s="17">
+      <c r="A113" s="28" t="n"/>
+      <c r="B113" s="28" t="n"/>
+      <c r="C113" s="29" t="n"/>
+      <c r="D113" s="29" t="n"/>
+      <c r="E113" s="18">
         <f>IF(D113="","",D113*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F113" s="28" t="n"/>
+      <c r="F113" s="29" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="27" t="n"/>
-      <c r="B114" s="27" t="n"/>
-      <c r="C114" s="28" t="n"/>
-      <c r="D114" s="28" t="n"/>
-      <c r="E114" s="17">
+      <c r="A114" s="28" t="n"/>
+      <c r="B114" s="28" t="n"/>
+      <c r="C114" s="29" t="n"/>
+      <c r="D114" s="29" t="n"/>
+      <c r="E114" s="18">
         <f>IF(D114="","",D114*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F114" s="28" t="n"/>
+      <c r="F114" s="29" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="27" t="n"/>
-      <c r="B115" s="27" t="n"/>
-      <c r="C115" s="28" t="n"/>
-      <c r="D115" s="28" t="n"/>
-      <c r="E115" s="17">
+      <c r="A115" s="28" t="n"/>
+      <c r="B115" s="28" t="n"/>
+      <c r="C115" s="29" t="n"/>
+      <c r="D115" s="29" t="n"/>
+      <c r="E115" s="18">
         <f>IF(D115="","",D115*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F115" s="28" t="n"/>
+      <c r="F115" s="29" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="27" t="n"/>
-      <c r="B116" s="27" t="n"/>
-      <c r="C116" s="28" t="n"/>
-      <c r="D116" s="28" t="n"/>
-      <c r="E116" s="17">
+      <c r="A116" s="28" t="n"/>
+      <c r="B116" s="28" t="n"/>
+      <c r="C116" s="29" t="n"/>
+      <c r="D116" s="29" t="n"/>
+      <c r="E116" s="18">
         <f>IF(D116="","",D116*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F116" s="28" t="n"/>
+      <c r="F116" s="29" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="27" t="n"/>
-      <c r="B117" s="27" t="n"/>
-      <c r="C117" s="28" t="n"/>
-      <c r="D117" s="28" t="n"/>
-      <c r="E117" s="17">
+      <c r="A117" s="28" t="n"/>
+      <c r="B117" s="28" t="n"/>
+      <c r="C117" s="29" t="n"/>
+      <c r="D117" s="29" t="n"/>
+      <c r="E117" s="18">
         <f>IF(D117="","",D117*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F117" s="28" t="n"/>
+      <c r="F117" s="29" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="27" t="n"/>
-      <c r="B118" s="27" t="n"/>
-      <c r="C118" s="28" t="n"/>
-      <c r="D118" s="28" t="n"/>
-      <c r="E118" s="17">
+      <c r="A118" s="28" t="n"/>
+      <c r="B118" s="28" t="n"/>
+      <c r="C118" s="29" t="n"/>
+      <c r="D118" s="29" t="n"/>
+      <c r="E118" s="18">
         <f>IF(D118="","",D118*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F118" s="28" t="n"/>
+      <c r="F118" s="29" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="27" t="n"/>
-      <c r="B119" s="27" t="n"/>
-      <c r="C119" s="28" t="n"/>
-      <c r="D119" s="28" t="n"/>
-      <c r="E119" s="17">
+      <c r="A119" s="28" t="n"/>
+      <c r="B119" s="28" t="n"/>
+      <c r="C119" s="29" t="n"/>
+      <c r="D119" s="29" t="n"/>
+      <c r="E119" s="18">
         <f>IF(D119="","",D119*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F119" s="28" t="n"/>
+      <c r="F119" s="29" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="27" t="n"/>
-      <c r="B120" s="27" t="n"/>
-      <c r="C120" s="28" t="n"/>
-      <c r="D120" s="28" t="n"/>
-      <c r="E120" s="17">
+      <c r="A120" s="28" t="n"/>
+      <c r="B120" s="28" t="n"/>
+      <c r="C120" s="29" t="n"/>
+      <c r="D120" s="29" t="n"/>
+      <c r="E120" s="18">
         <f>IF(D120="","",D120*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F120" s="28" t="n"/>
+      <c r="F120" s="29" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="27" t="n"/>
-      <c r="B121" s="27" t="n"/>
-      <c r="C121" s="28" t="n"/>
-      <c r="D121" s="28" t="n"/>
-      <c r="E121" s="17">
+      <c r="A121" s="28" t="n"/>
+      <c r="B121" s="28" t="n"/>
+      <c r="C121" s="29" t="n"/>
+      <c r="D121" s="29" t="n"/>
+      <c r="E121" s="18">
         <f>IF(D121="","",D121*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F121" s="28" t="n"/>
+      <c r="F121" s="29" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="27" t="n"/>
-      <c r="B122" s="27" t="n"/>
-      <c r="C122" s="28" t="n"/>
-      <c r="D122" s="28" t="n"/>
-      <c r="E122" s="17">
+      <c r="A122" s="28" t="n"/>
+      <c r="B122" s="28" t="n"/>
+      <c r="C122" s="29" t="n"/>
+      <c r="D122" s="29" t="n"/>
+      <c r="E122" s="18">
         <f>IF(D122="","",D122*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F122" s="28" t="n"/>
+      <c r="F122" s="29" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="27" t="n"/>
-      <c r="B123" s="27" t="n"/>
-      <c r="C123" s="28" t="n"/>
-      <c r="D123" s="28" t="n"/>
-      <c r="E123" s="17">
+      <c r="A123" s="28" t="n"/>
+      <c r="B123" s="28" t="n"/>
+      <c r="C123" s="29" t="n"/>
+      <c r="D123" s="29" t="n"/>
+      <c r="E123" s="18">
         <f>IF(D123="","",D123*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F123" s="28" t="n"/>
+      <c r="F123" s="29" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="27" t="n"/>
-      <c r="B124" s="27" t="n"/>
-      <c r="C124" s="28" t="n"/>
-      <c r="D124" s="28" t="n"/>
-      <c r="E124" s="17">
+      <c r="A124" s="28" t="n"/>
+      <c r="B124" s="28" t="n"/>
+      <c r="C124" s="29" t="n"/>
+      <c r="D124" s="29" t="n"/>
+      <c r="E124" s="18">
         <f>IF(D124="","",D124*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F124" s="28" t="n"/>
+      <c r="F124" s="29" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="27" t="n"/>
-      <c r="B125" s="27" t="n"/>
-      <c r="C125" s="28" t="n"/>
-      <c r="D125" s="28" t="n"/>
-      <c r="E125" s="17">
+      <c r="A125" s="28" t="n"/>
+      <c r="B125" s="28" t="n"/>
+      <c r="C125" s="29" t="n"/>
+      <c r="D125" s="29" t="n"/>
+      <c r="E125" s="18">
         <f>IF(D125="","",D125*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F125" s="28" t="n"/>
+      <c r="F125" s="29" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="27" t="n"/>
-      <c r="B126" s="27" t="n"/>
-      <c r="C126" s="28" t="n"/>
-      <c r="D126" s="28" t="n"/>
-      <c r="E126" s="17">
+      <c r="A126" s="28" t="n"/>
+      <c r="B126" s="28" t="n"/>
+      <c r="C126" s="29" t="n"/>
+      <c r="D126" s="29" t="n"/>
+      <c r="E126" s="18">
         <f>IF(D126="","",D126*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F126" s="28" t="n"/>
+      <c r="F126" s="29" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="27" t="n"/>
-      <c r="B127" s="27" t="n"/>
-      <c r="C127" s="28" t="n"/>
-      <c r="D127" s="28" t="n"/>
-      <c r="E127" s="17">
+      <c r="A127" s="28" t="n"/>
+      <c r="B127" s="28" t="n"/>
+      <c r="C127" s="29" t="n"/>
+      <c r="D127" s="29" t="n"/>
+      <c r="E127" s="18">
         <f>IF(D127="","",D127*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F127" s="28" t="n"/>
+      <c r="F127" s="29" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="27" t="n"/>
-      <c r="B128" s="27" t="n"/>
-      <c r="C128" s="28" t="n"/>
-      <c r="D128" s="28" t="n"/>
-      <c r="E128" s="17">
+      <c r="A128" s="28" t="n"/>
+      <c r="B128" s="28" t="n"/>
+      <c r="C128" s="29" t="n"/>
+      <c r="D128" s="29" t="n"/>
+      <c r="E128" s="18">
         <f>IF(D128="","",D128*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F128" s="28" t="n"/>
+      <c r="F128" s="29" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="27" t="n"/>
-      <c r="B129" s="27" t="n"/>
-      <c r="C129" s="28" t="n"/>
-      <c r="D129" s="28" t="n"/>
-      <c r="E129" s="17">
+      <c r="A129" s="28" t="n"/>
+      <c r="B129" s="28" t="n"/>
+      <c r="C129" s="29" t="n"/>
+      <c r="D129" s="29" t="n"/>
+      <c r="E129" s="18">
         <f>IF(D129="","",D129*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F129" s="28" t="n"/>
+      <c r="F129" s="29" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="27" t="n"/>
-      <c r="B130" s="27" t="n"/>
-      <c r="C130" s="28" t="n"/>
-      <c r="D130" s="28" t="n"/>
-      <c r="E130" s="17">
+      <c r="A130" s="28" t="n"/>
+      <c r="B130" s="28" t="n"/>
+      <c r="C130" s="29" t="n"/>
+      <c r="D130" s="29" t="n"/>
+      <c r="E130" s="18">
         <f>IF(D130="","",D130*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F130" s="28" t="n"/>
+      <c r="F130" s="29" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="27" t="n"/>
-      <c r="B131" s="27" t="n"/>
-      <c r="C131" s="28" t="n"/>
-      <c r="D131" s="28" t="n"/>
-      <c r="E131" s="17">
+      <c r="A131" s="28" t="n"/>
+      <c r="B131" s="28" t="n"/>
+      <c r="C131" s="29" t="n"/>
+      <c r="D131" s="29" t="n"/>
+      <c r="E131" s="18">
         <f>IF(D131="","",D131*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F131" s="28" t="n"/>
+      <c r="F131" s="29" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="27" t="n"/>
-      <c r="B132" s="27" t="n"/>
-      <c r="C132" s="28" t="n"/>
-      <c r="D132" s="28" t="n"/>
-      <c r="E132" s="17">
+      <c r="A132" s="28" t="n"/>
+      <c r="B132" s="28" t="n"/>
+      <c r="C132" s="29" t="n"/>
+      <c r="D132" s="29" t="n"/>
+      <c r="E132" s="18">
         <f>IF(D132="","",D132*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F132" s="28" t="n"/>
+      <c r="F132" s="29" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="27" t="n"/>
-      <c r="B133" s="27" t="n"/>
-      <c r="C133" s="28" t="n"/>
-      <c r="D133" s="28" t="n"/>
-      <c r="E133" s="17">
+      <c r="A133" s="28" t="n"/>
+      <c r="B133" s="28" t="n"/>
+      <c r="C133" s="29" t="n"/>
+      <c r="D133" s="29" t="n"/>
+      <c r="E133" s="18">
         <f>IF(D133="","",D133*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F133" s="28" t="n"/>
+      <c r="F133" s="29" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="27" t="n"/>
-      <c r="B134" s="27" t="n"/>
-      <c r="C134" s="28" t="n"/>
-      <c r="D134" s="28" t="n"/>
-      <c r="E134" s="17">
+      <c r="A134" s="28" t="n"/>
+      <c r="B134" s="28" t="n"/>
+      <c r="C134" s="29" t="n"/>
+      <c r="D134" s="29" t="n"/>
+      <c r="E134" s="18">
         <f>IF(D134="","",D134*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F134" s="28" t="n"/>
+      <c r="F134" s="29" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="27" t="n"/>
-      <c r="B135" s="27" t="n"/>
-      <c r="C135" s="28" t="n"/>
-      <c r="D135" s="28" t="n"/>
-      <c r="E135" s="17">
+      <c r="A135" s="28" t="n"/>
+      <c r="B135" s="28" t="n"/>
+      <c r="C135" s="29" t="n"/>
+      <c r="D135" s="29" t="n"/>
+      <c r="E135" s="18">
         <f>IF(D135="","",D135*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F135" s="28" t="n"/>
+      <c r="F135" s="29" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="27" t="n"/>
-      <c r="B136" s="27" t="n"/>
-      <c r="C136" s="28" t="n"/>
-      <c r="D136" s="28" t="n"/>
-      <c r="E136" s="17">
+      <c r="A136" s="28" t="n"/>
+      <c r="B136" s="28" t="n"/>
+      <c r="C136" s="29" t="n"/>
+      <c r="D136" s="29" t="n"/>
+      <c r="E136" s="18">
         <f>IF(D136="","",D136*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F136" s="28" t="n"/>
+      <c r="F136" s="29" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="27" t="n"/>
-      <c r="B137" s="27" t="n"/>
-      <c r="C137" s="28" t="n"/>
-      <c r="D137" s="28" t="n"/>
-      <c r="E137" s="17">
+      <c r="A137" s="28" t="n"/>
+      <c r="B137" s="28" t="n"/>
+      <c r="C137" s="29" t="n"/>
+      <c r="D137" s="29" t="n"/>
+      <c r="E137" s="18">
         <f>IF(D137="","",D137*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F137" s="28" t="n"/>
+      <c r="F137" s="29" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="27" t="n"/>
-      <c r="B138" s="27" t="n"/>
-      <c r="C138" s="28" t="n"/>
-      <c r="D138" s="28" t="n"/>
-      <c r="E138" s="17">
+      <c r="A138" s="28" t="n"/>
+      <c r="B138" s="28" t="n"/>
+      <c r="C138" s="29" t="n"/>
+      <c r="D138" s="29" t="n"/>
+      <c r="E138" s="18">
         <f>IF(D138="","",D138*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F138" s="28" t="n"/>
+      <c r="F138" s="29" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="27" t="n"/>
-      <c r="B139" s="27" t="n"/>
-      <c r="C139" s="28" t="n"/>
-      <c r="D139" s="28" t="n"/>
-      <c r="E139" s="17">
+      <c r="A139" s="28" t="n"/>
+      <c r="B139" s="28" t="n"/>
+      <c r="C139" s="29" t="n"/>
+      <c r="D139" s="29" t="n"/>
+      <c r="E139" s="18">
         <f>IF(D139="","",D139*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F139" s="28" t="n"/>
+      <c r="F139" s="29" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="27" t="n"/>
-      <c r="B140" s="27" t="n"/>
-      <c r="C140" s="28" t="n"/>
-      <c r="D140" s="28" t="n"/>
-      <c r="E140" s="17">
+      <c r="A140" s="28" t="n"/>
+      <c r="B140" s="28" t="n"/>
+      <c r="C140" s="29" t="n"/>
+      <c r="D140" s="29" t="n"/>
+      <c r="E140" s="18">
         <f>IF(D140="","",D140*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F140" s="28" t="n"/>
+      <c r="F140" s="29" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="27" t="n"/>
-      <c r="B141" s="27" t="n"/>
-      <c r="C141" s="28" t="n"/>
-      <c r="D141" s="28" t="n"/>
-      <c r="E141" s="17">
+      <c r="A141" s="28" t="n"/>
+      <c r="B141" s="28" t="n"/>
+      <c r="C141" s="29" t="n"/>
+      <c r="D141" s="29" t="n"/>
+      <c r="E141" s="18">
         <f>IF(D141="","",D141*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F141" s="28" t="n"/>
+      <c r="F141" s="29" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="27" t="n"/>
-      <c r="B142" s="27" t="n"/>
-      <c r="C142" s="28" t="n"/>
-      <c r="D142" s="28" t="n"/>
-      <c r="E142" s="17">
+      <c r="A142" s="28" t="n"/>
+      <c r="B142" s="28" t="n"/>
+      <c r="C142" s="29" t="n"/>
+      <c r="D142" s="29" t="n"/>
+      <c r="E142" s="18">
         <f>IF(D142="","",D142*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F142" s="28" t="n"/>
+      <c r="F142" s="29" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="27" t="n"/>
-      <c r="B143" s="27" t="n"/>
-      <c r="C143" s="28" t="n"/>
-      <c r="D143" s="28" t="n"/>
-      <c r="E143" s="17">
+      <c r="A143" s="28" t="n"/>
+      <c r="B143" s="28" t="n"/>
+      <c r="C143" s="29" t="n"/>
+      <c r="D143" s="29" t="n"/>
+      <c r="E143" s="18">
         <f>IF(D143="","",D143*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F143" s="28" t="n"/>
+      <c r="F143" s="29" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="27" t="n"/>
-      <c r="B144" s="27" t="n"/>
-      <c r="C144" s="28" t="n"/>
-      <c r="D144" s="28" t="n"/>
-      <c r="E144" s="17">
+      <c r="A144" s="28" t="n"/>
+      <c r="B144" s="28" t="n"/>
+      <c r="C144" s="29" t="n"/>
+      <c r="D144" s="29" t="n"/>
+      <c r="E144" s="18">
         <f>IF(D144="","",D144*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F144" s="28" t="n"/>
+      <c r="F144" s="29" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="27" t="n"/>
-      <c r="B145" s="27" t="n"/>
-      <c r="C145" s="28" t="n"/>
-      <c r="D145" s="28" t="n"/>
-      <c r="E145" s="17">
+      <c r="A145" s="28" t="n"/>
+      <c r="B145" s="28" t="n"/>
+      <c r="C145" s="29" t="n"/>
+      <c r="D145" s="29" t="n"/>
+      <c r="E145" s="18">
         <f>IF(D145="","",D145*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F145" s="28" t="n"/>
+      <c r="F145" s="29" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="27" t="n"/>
-      <c r="B146" s="27" t="n"/>
-      <c r="C146" s="28" t="n"/>
-      <c r="D146" s="28" t="n"/>
-      <c r="E146" s="17">
+      <c r="A146" s="28" t="n"/>
+      <c r="B146" s="28" t="n"/>
+      <c r="C146" s="29" t="n"/>
+      <c r="D146" s="29" t="n"/>
+      <c r="E146" s="18">
         <f>IF(D146="","",D146*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F146" s="28" t="n"/>
+      <c r="F146" s="29" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="27" t="n"/>
-      <c r="B147" s="27" t="n"/>
-      <c r="C147" s="28" t="n"/>
-      <c r="D147" s="28" t="n"/>
-      <c r="E147" s="17">
+      <c r="A147" s="28" t="n"/>
+      <c r="B147" s="28" t="n"/>
+      <c r="C147" s="29" t="n"/>
+      <c r="D147" s="29" t="n"/>
+      <c r="E147" s="18">
         <f>IF(D147="","",D147*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F147" s="28" t="n"/>
+      <c r="F147" s="29" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="27" t="n"/>
-      <c r="B148" s="27" t="n"/>
-      <c r="C148" s="28" t="n"/>
-      <c r="D148" s="28" t="n"/>
-      <c r="E148" s="17">
+      <c r="A148" s="28" t="n"/>
+      <c r="B148" s="28" t="n"/>
+      <c r="C148" s="29" t="n"/>
+      <c r="D148" s="29" t="n"/>
+      <c r="E148" s="18">
         <f>IF(D148="","",D148*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F148" s="28" t="n"/>
+      <c r="F148" s="29" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="27" t="n"/>
-      <c r="B149" s="27" t="n"/>
-      <c r="C149" s="28" t="n"/>
-      <c r="D149" s="28" t="n"/>
-      <c r="E149" s="17">
+      <c r="A149" s="28" t="n"/>
+      <c r="B149" s="28" t="n"/>
+      <c r="C149" s="29" t="n"/>
+      <c r="D149" s="29" t="n"/>
+      <c r="E149" s="18">
         <f>IF(D149="","",D149*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F149" s="28" t="n"/>
+      <c r="F149" s="29" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="27" t="n"/>
-      <c r="B150" s="27" t="n"/>
-      <c r="C150" s="28" t="n"/>
-      <c r="D150" s="28" t="n"/>
-      <c r="E150" s="17">
+      <c r="A150" s="28" t="n"/>
+      <c r="B150" s="28" t="n"/>
+      <c r="C150" s="29" t="n"/>
+      <c r="D150" s="29" t="n"/>
+      <c r="E150" s="18">
         <f>IF(D150="","",D150*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F150" s="28" t="n"/>
+      <c r="F150" s="29" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="27" t="n"/>
-      <c r="B151" s="27" t="n"/>
-      <c r="C151" s="28" t="n"/>
-      <c r="D151" s="28" t="n"/>
-      <c r="E151" s="17">
+      <c r="A151" s="28" t="n"/>
+      <c r="B151" s="28" t="n"/>
+      <c r="C151" s="29" t="n"/>
+      <c r="D151" s="29" t="n"/>
+      <c r="E151" s="18">
         <f>IF(D151="","",D151*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F151" s="28" t="n"/>
+      <c r="F151" s="29" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="27" t="n"/>
-      <c r="B152" s="27" t="n"/>
-      <c r="C152" s="28" t="n"/>
-      <c r="D152" s="28" t="n"/>
-      <c r="E152" s="17">
+      <c r="A152" s="28" t="n"/>
+      <c r="B152" s="28" t="n"/>
+      <c r="C152" s="29" t="n"/>
+      <c r="D152" s="29" t="n"/>
+      <c r="E152" s="18">
         <f>IF(D152="","",D152*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F152" s="28" t="n"/>
+      <c r="F152" s="29" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="27" t="n"/>
-      <c r="B153" s="27" t="n"/>
-      <c r="C153" s="28" t="n"/>
-      <c r="D153" s="28" t="n"/>
-      <c r="E153" s="17">
+      <c r="A153" s="28" t="n"/>
+      <c r="B153" s="28" t="n"/>
+      <c r="C153" s="29" t="n"/>
+      <c r="D153" s="29" t="n"/>
+      <c r="E153" s="18">
         <f>IF(D153="","",D153*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F153" s="28" t="n"/>
+      <c r="F153" s="29" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="27" t="n"/>
-      <c r="B154" s="27" t="n"/>
-      <c r="C154" s="28" t="n"/>
-      <c r="D154" s="28" t="n"/>
-      <c r="E154" s="17">
+      <c r="A154" s="28" t="n"/>
+      <c r="B154" s="28" t="n"/>
+      <c r="C154" s="29" t="n"/>
+      <c r="D154" s="29" t="n"/>
+      <c r="E154" s="18">
         <f>IF(D154="","",D154*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F154" s="28" t="n"/>
+      <c r="F154" s="29" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="27" t="n"/>
-      <c r="B155" s="27" t="n"/>
-      <c r="C155" s="28" t="n"/>
-      <c r="D155" s="28" t="n"/>
-      <c r="E155" s="17">
+      <c r="A155" s="28" t="n"/>
+      <c r="B155" s="28" t="n"/>
+      <c r="C155" s="29" t="n"/>
+      <c r="D155" s="29" t="n"/>
+      <c r="E155" s="18">
         <f>IF(D155="","",D155*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F155" s="28" t="n"/>
+      <c r="F155" s="29" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="27" t="n"/>
-      <c r="B156" s="27" t="n"/>
-      <c r="C156" s="28" t="n"/>
-      <c r="D156" s="28" t="n"/>
-      <c r="E156" s="17">
+      <c r="A156" s="28" t="n"/>
+      <c r="B156" s="28" t="n"/>
+      <c r="C156" s="29" t="n"/>
+      <c r="D156" s="29" t="n"/>
+      <c r="E156" s="18">
         <f>IF(D156="","",D156*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F156" s="28" t="n"/>
+      <c r="F156" s="29" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="27" t="n"/>
-      <c r="B157" s="27" t="n"/>
-      <c r="C157" s="28" t="n"/>
-      <c r="D157" s="28" t="n"/>
-      <c r="E157" s="17">
+      <c r="A157" s="28" t="n"/>
+      <c r="B157" s="28" t="n"/>
+      <c r="C157" s="29" t="n"/>
+      <c r="D157" s="29" t="n"/>
+      <c r="E157" s="18">
         <f>IF(D157="","",D157*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F157" s="28" t="n"/>
+      <c r="F157" s="29" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="27" t="n"/>
-      <c r="B158" s="27" t="n"/>
-      <c r="C158" s="28" t="n"/>
-      <c r="D158" s="28" t="n"/>
-      <c r="E158" s="17">
+      <c r="A158" s="28" t="n"/>
+      <c r="B158" s="28" t="n"/>
+      <c r="C158" s="29" t="n"/>
+      <c r="D158" s="29" t="n"/>
+      <c r="E158" s="18">
         <f>IF(D158="","",D158*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F158" s="28" t="n"/>
+      <c r="F158" s="29" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="27" t="n"/>
-      <c r="B159" s="27" t="n"/>
-      <c r="C159" s="28" t="n"/>
-      <c r="D159" s="28" t="n"/>
-      <c r="E159" s="17">
+      <c r="A159" s="28" t="n"/>
+      <c r="B159" s="28" t="n"/>
+      <c r="C159" s="29" t="n"/>
+      <c r="D159" s="29" t="n"/>
+      <c r="E159" s="18">
         <f>IF(D159="","",D159*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F159" s="28" t="n"/>
+      <c r="F159" s="29" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="27" t="n"/>
-      <c r="B160" s="27" t="n"/>
-      <c r="C160" s="28" t="n"/>
-      <c r="D160" s="28" t="n"/>
-      <c r="E160" s="17">
+      <c r="A160" s="28" t="n"/>
+      <c r="B160" s="28" t="n"/>
+      <c r="C160" s="29" t="n"/>
+      <c r="D160" s="29" t="n"/>
+      <c r="E160" s="18">
         <f>IF(D160="","",D160*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F160" s="28" t="n"/>
+      <c r="F160" s="29" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="27" t="n"/>
-      <c r="B161" s="27" t="n"/>
-      <c r="C161" s="28" t="n"/>
-      <c r="D161" s="28" t="n"/>
-      <c r="E161" s="17">
+      <c r="A161" s="28" t="n"/>
+      <c r="B161" s="28" t="n"/>
+      <c r="C161" s="29" t="n"/>
+      <c r="D161" s="29" t="n"/>
+      <c r="E161" s="18">
         <f>IF(D161="","",D161*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F161" s="28" t="n"/>
+      <c r="F161" s="29" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="27" t="n"/>
-      <c r="B162" s="27" t="n"/>
-      <c r="C162" s="28" t="n"/>
-      <c r="D162" s="28" t="n"/>
-      <c r="E162" s="17">
+      <c r="A162" s="28" t="n"/>
+      <c r="B162" s="28" t="n"/>
+      <c r="C162" s="29" t="n"/>
+      <c r="D162" s="29" t="n"/>
+      <c r="E162" s="18">
         <f>IF(D162="","",D162*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F162" s="28" t="n"/>
+      <c r="F162" s="29" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="27" t="n"/>
-      <c r="B163" s="27" t="n"/>
-      <c r="C163" s="28" t="n"/>
-      <c r="D163" s="28" t="n"/>
-      <c r="E163" s="17">
+      <c r="A163" s="28" t="n"/>
+      <c r="B163" s="28" t="n"/>
+      <c r="C163" s="29" t="n"/>
+      <c r="D163" s="29" t="n"/>
+      <c r="E163" s="18">
         <f>IF(D163="","",D163*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F163" s="28" t="n"/>
+      <c r="F163" s="29" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="27" t="n"/>
-      <c r="B164" s="27" t="n"/>
-      <c r="C164" s="28" t="n"/>
-      <c r="D164" s="28" t="n"/>
-      <c r="E164" s="17">
+      <c r="A164" s="28" t="n"/>
+      <c r="B164" s="28" t="n"/>
+      <c r="C164" s="29" t="n"/>
+      <c r="D164" s="29" t="n"/>
+      <c r="E164" s="18">
         <f>IF(D164="","",D164*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F164" s="28" t="n"/>
+      <c r="F164" s="29" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="27" t="n"/>
-      <c r="B165" s="27" t="n"/>
-      <c r="C165" s="28" t="n"/>
-      <c r="D165" s="28" t="n"/>
-      <c r="E165" s="17">
+      <c r="A165" s="28" t="n"/>
+      <c r="B165" s="28" t="n"/>
+      <c r="C165" s="29" t="n"/>
+      <c r="D165" s="29" t="n"/>
+      <c r="E165" s="18">
         <f>IF(D165="","",D165*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F165" s="28" t="n"/>
+      <c r="F165" s="29" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="27" t="n"/>
-      <c r="B166" s="27" t="n"/>
-      <c r="C166" s="28" t="n"/>
-      <c r="D166" s="28" t="n"/>
-      <c r="E166" s="17">
+      <c r="A166" s="28" t="n"/>
+      <c r="B166" s="28" t="n"/>
+      <c r="C166" s="29" t="n"/>
+      <c r="D166" s="29" t="n"/>
+      <c r="E166" s="18">
         <f>IF(D166="","",D166*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F166" s="28" t="n"/>
+      <c r="F166" s="29" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="27" t="n"/>
-      <c r="B167" s="27" t="n"/>
-      <c r="C167" s="28" t="n"/>
-      <c r="D167" s="28" t="n"/>
-      <c r="E167" s="17">
+      <c r="A167" s="28" t="n"/>
+      <c r="B167" s="28" t="n"/>
+      <c r="C167" s="29" t="n"/>
+      <c r="D167" s="29" t="n"/>
+      <c r="E167" s="18">
         <f>IF(D167="","",D167*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F167" s="28" t="n"/>
+      <c r="F167" s="29" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="27" t="n"/>
-      <c r="B168" s="27" t="n"/>
-      <c r="C168" s="28" t="n"/>
-      <c r="D168" s="28" t="n"/>
-      <c r="E168" s="17">
+      <c r="A168" s="28" t="n"/>
+      <c r="B168" s="28" t="n"/>
+      <c r="C168" s="29" t="n"/>
+      <c r="D168" s="29" t="n"/>
+      <c r="E168" s="18">
         <f>IF(D168="","",D168*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F168" s="28" t="n"/>
+      <c r="F168" s="29" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" s="27" t="n"/>
-      <c r="B169" s="27" t="n"/>
-      <c r="C169" s="28" t="n"/>
-      <c r="D169" s="28" t="n"/>
-      <c r="E169" s="17">
+      <c r="A169" s="28" t="n"/>
+      <c r="B169" s="28" t="n"/>
+      <c r="C169" s="29" t="n"/>
+      <c r="D169" s="29" t="n"/>
+      <c r="E169" s="18">
         <f>IF(D169="","",D169*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F169" s="28" t="n"/>
+      <c r="F169" s="29" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="27" t="n"/>
-      <c r="B170" s="27" t="n"/>
-      <c r="C170" s="28" t="n"/>
-      <c r="D170" s="28" t="n"/>
-      <c r="E170" s="17">
+      <c r="A170" s="28" t="n"/>
+      <c r="B170" s="28" t="n"/>
+      <c r="C170" s="29" t="n"/>
+      <c r="D170" s="29" t="n"/>
+      <c r="E170" s="18">
         <f>IF(D170="","",D170*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F170" s="28" t="n"/>
+      <c r="F170" s="29" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="27" t="n"/>
-      <c r="B171" s="27" t="n"/>
-      <c r="C171" s="28" t="n"/>
-      <c r="D171" s="28" t="n"/>
-      <c r="E171" s="17">
+      <c r="A171" s="28" t="n"/>
+      <c r="B171" s="28" t="n"/>
+      <c r="C171" s="29" t="n"/>
+      <c r="D171" s="29" t="n"/>
+      <c r="E171" s="18">
         <f>IF(D171="","",D171*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F171" s="28" t="n"/>
+      <c r="F171" s="29" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="27" t="n"/>
-      <c r="B172" s="27" t="n"/>
-      <c r="C172" s="28" t="n"/>
-      <c r="D172" s="28" t="n"/>
-      <c r="E172" s="17">
+      <c r="A172" s="28" t="n"/>
+      <c r="B172" s="28" t="n"/>
+      <c r="C172" s="29" t="n"/>
+      <c r="D172" s="29" t="n"/>
+      <c r="E172" s="18">
         <f>IF(D172="","",D172*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F172" s="28" t="n"/>
+      <c r="F172" s="29" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" s="27" t="n"/>
-      <c r="B173" s="27" t="n"/>
-      <c r="C173" s="28" t="n"/>
-      <c r="D173" s="28" t="n"/>
-      <c r="E173" s="17">
+      <c r="A173" s="28" t="n"/>
+      <c r="B173" s="28" t="n"/>
+      <c r="C173" s="29" t="n"/>
+      <c r="D173" s="29" t="n"/>
+      <c r="E173" s="18">
         <f>IF(D173="","",D173*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F173" s="28" t="n"/>
+      <c r="F173" s="29" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="27" t="n"/>
-      <c r="B174" s="27" t="n"/>
-      <c r="C174" s="28" t="n"/>
-      <c r="D174" s="28" t="n"/>
-      <c r="E174" s="17">
+      <c r="A174" s="28" t="n"/>
+      <c r="B174" s="28" t="n"/>
+      <c r="C174" s="29" t="n"/>
+      <c r="D174" s="29" t="n"/>
+      <c r="E174" s="18">
         <f>IF(D174="","",D174*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F174" s="28" t="n"/>
+      <c r="F174" s="29" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="27" t="n"/>
-      <c r="B175" s="27" t="n"/>
-      <c r="C175" s="28" t="n"/>
-      <c r="D175" s="28" t="n"/>
-      <c r="E175" s="17">
+      <c r="A175" s="28" t="n"/>
+      <c r="B175" s="28" t="n"/>
+      <c r="C175" s="29" t="n"/>
+      <c r="D175" s="29" t="n"/>
+      <c r="E175" s="18">
         <f>IF(D175="","",D175*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F175" s="28" t="n"/>
+      <c r="F175" s="29" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" s="27" t="n"/>
-      <c r="B176" s="27" t="n"/>
-      <c r="C176" s="28" t="n"/>
-      <c r="D176" s="28" t="n"/>
-      <c r="E176" s="17">
+      <c r="A176" s="28" t="n"/>
+      <c r="B176" s="28" t="n"/>
+      <c r="C176" s="29" t="n"/>
+      <c r="D176" s="29" t="n"/>
+      <c r="E176" s="18">
         <f>IF(D176="","",D176*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F176" s="28" t="n"/>
+      <c r="F176" s="29" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="27" t="n"/>
-      <c r="B177" s="27" t="n"/>
-      <c r="C177" s="28" t="n"/>
-      <c r="D177" s="28" t="n"/>
-      <c r="E177" s="17">
+      <c r="A177" s="28" t="n"/>
+      <c r="B177" s="28" t="n"/>
+      <c r="C177" s="29" t="n"/>
+      <c r="D177" s="29" t="n"/>
+      <c r="E177" s="18">
         <f>IF(D177="","",D177*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F177" s="28" t="n"/>
+      <c r="F177" s="29" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="27" t="n"/>
-      <c r="B178" s="27" t="n"/>
-      <c r="C178" s="28" t="n"/>
-      <c r="D178" s="28" t="n"/>
-      <c r="E178" s="17">
+      <c r="A178" s="28" t="n"/>
+      <c r="B178" s="28" t="n"/>
+      <c r="C178" s="29" t="n"/>
+      <c r="D178" s="29" t="n"/>
+      <c r="E178" s="18">
         <f>IF(D178="","",D178*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F178" s="28" t="n"/>
+      <c r="F178" s="29" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" s="27" t="n"/>
-      <c r="B179" s="27" t="n"/>
-      <c r="C179" s="28" t="n"/>
-      <c r="D179" s="28" t="n"/>
-      <c r="E179" s="17">
+      <c r="A179" s="28" t="n"/>
+      <c r="B179" s="28" t="n"/>
+      <c r="C179" s="29" t="n"/>
+      <c r="D179" s="29" t="n"/>
+      <c r="E179" s="18">
         <f>IF(D179="","",D179*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F179" s="28" t="n"/>
+      <c r="F179" s="29" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" s="27" t="n"/>
-      <c r="B180" s="27" t="n"/>
-      <c r="C180" s="28" t="n"/>
-      <c r="D180" s="28" t="n"/>
-      <c r="E180" s="17">
+      <c r="A180" s="28" t="n"/>
+      <c r="B180" s="28" t="n"/>
+      <c r="C180" s="29" t="n"/>
+      <c r="D180" s="29" t="n"/>
+      <c r="E180" s="18">
         <f>IF(D180="","",D180*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F180" s="28" t="n"/>
+      <c r="F180" s="29" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="27" t="n"/>
-      <c r="B181" s="27" t="n"/>
-      <c r="C181" s="28" t="n"/>
-      <c r="D181" s="28" t="n"/>
-      <c r="E181" s="17">
+      <c r="A181" s="28" t="n"/>
+      <c r="B181" s="28" t="n"/>
+      <c r="C181" s="29" t="n"/>
+      <c r="D181" s="29" t="n"/>
+      <c r="E181" s="18">
         <f>IF(D181="","",D181*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F181" s="28" t="n"/>
+      <c r="F181" s="29" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="27" t="n"/>
-      <c r="B182" s="27" t="n"/>
-      <c r="C182" s="28" t="n"/>
-      <c r="D182" s="28" t="n"/>
-      <c r="E182" s="17">
+      <c r="A182" s="28" t="n"/>
+      <c r="B182" s="28" t="n"/>
+      <c r="C182" s="29" t="n"/>
+      <c r="D182" s="29" t="n"/>
+      <c r="E182" s="18">
         <f>IF(D182="","",D182*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F182" s="28" t="n"/>
+      <c r="F182" s="29" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="27" t="n"/>
-      <c r="B183" s="27" t="n"/>
-      <c r="C183" s="28" t="n"/>
-      <c r="D183" s="28" t="n"/>
-      <c r="E183" s="17">
+      <c r="A183" s="28" t="n"/>
+      <c r="B183" s="28" t="n"/>
+      <c r="C183" s="29" t="n"/>
+      <c r="D183" s="29" t="n"/>
+      <c r="E183" s="18">
         <f>IF(D183="","",D183*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F183" s="28" t="n"/>
+      <c r="F183" s="29" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="27" t="n"/>
-      <c r="B184" s="27" t="n"/>
-      <c r="C184" s="28" t="n"/>
-      <c r="D184" s="28" t="n"/>
-      <c r="E184" s="17">
+      <c r="A184" s="28" t="n"/>
+      <c r="B184" s="28" t="n"/>
+      <c r="C184" s="29" t="n"/>
+      <c r="D184" s="29" t="n"/>
+      <c r="E184" s="18">
         <f>IF(D184="","",D184*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F184" s="28" t="n"/>
+      <c r="F184" s="29" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="27" t="n"/>
-      <c r="B185" s="27" t="n"/>
-      <c r="C185" s="28" t="n"/>
-      <c r="D185" s="28" t="n"/>
-      <c r="E185" s="17">
+      <c r="A185" s="28" t="n"/>
+      <c r="B185" s="28" t="n"/>
+      <c r="C185" s="29" t="n"/>
+      <c r="D185" s="29" t="n"/>
+      <c r="E185" s="18">
         <f>IF(D185="","",D185*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F185" s="28" t="n"/>
+      <c r="F185" s="29" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="27" t="n"/>
-      <c r="B186" s="27" t="n"/>
-      <c r="C186" s="28" t="n"/>
-      <c r="D186" s="28" t="n"/>
-      <c r="E186" s="17">
+      <c r="A186" s="28" t="n"/>
+      <c r="B186" s="28" t="n"/>
+      <c r="C186" s="29" t="n"/>
+      <c r="D186" s="29" t="n"/>
+      <c r="E186" s="18">
         <f>IF(D186="","",D186*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F186" s="28" t="n"/>
+      <c r="F186" s="29" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" s="27" t="n"/>
-      <c r="B187" s="27" t="n"/>
-      <c r="C187" s="28" t="n"/>
-      <c r="D187" s="28" t="n"/>
-      <c r="E187" s="17">
+      <c r="A187" s="28" t="n"/>
+      <c r="B187" s="28" t="n"/>
+      <c r="C187" s="29" t="n"/>
+      <c r="D187" s="29" t="n"/>
+      <c r="E187" s="18">
         <f>IF(D187="","",D187*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F187" s="28" t="n"/>
+      <c r="F187" s="29" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" s="27" t="n"/>
-      <c r="B188" s="27" t="n"/>
-      <c r="C188" s="28" t="n"/>
-      <c r="D188" s="28" t="n"/>
-      <c r="E188" s="17">
+      <c r="A188" s="28" t="n"/>
+      <c r="B188" s="28" t="n"/>
+      <c r="C188" s="29" t="n"/>
+      <c r="D188" s="29" t="n"/>
+      <c r="E188" s="18">
         <f>IF(D188="","",D188*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F188" s="28" t="n"/>
+      <c r="F188" s="29" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" s="27" t="n"/>
-      <c r="B189" s="27" t="n"/>
-      <c r="C189" s="28" t="n"/>
-      <c r="D189" s="28" t="n"/>
-      <c r="E189" s="17">
+      <c r="A189" s="28" t="n"/>
+      <c r="B189" s="28" t="n"/>
+      <c r="C189" s="29" t="n"/>
+      <c r="D189" s="29" t="n"/>
+      <c r="E189" s="18">
         <f>IF(D189="","",D189*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F189" s="28" t="n"/>
+      <c r="F189" s="29" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" s="27" t="n"/>
-      <c r="B190" s="27" t="n"/>
-      <c r="C190" s="28" t="n"/>
-      <c r="D190" s="28" t="n"/>
-      <c r="E190" s="17">
+      <c r="A190" s="28" t="n"/>
+      <c r="B190" s="28" t="n"/>
+      <c r="C190" s="29" t="n"/>
+      <c r="D190" s="29" t="n"/>
+      <c r="E190" s="18">
         <f>IF(D190="","",D190*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F190" s="28" t="n"/>
+      <c r="F190" s="29" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="27" t="n"/>
-      <c r="B191" s="27" t="n"/>
-      <c r="C191" s="28" t="n"/>
-      <c r="D191" s="28" t="n"/>
-      <c r="E191" s="17">
+      <c r="A191" s="28" t="n"/>
+      <c r="B191" s="28" t="n"/>
+      <c r="C191" s="29" t="n"/>
+      <c r="D191" s="29" t="n"/>
+      <c r="E191" s="18">
         <f>IF(D191="","",D191*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F191" s="28" t="n"/>
+      <c r="F191" s="29" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="27" t="n"/>
-      <c r="B192" s="27" t="n"/>
-      <c r="C192" s="28" t="n"/>
-      <c r="D192" s="28" t="n"/>
-      <c r="E192" s="17">
+      <c r="A192" s="28" t="n"/>
+      <c r="B192" s="28" t="n"/>
+      <c r="C192" s="29" t="n"/>
+      <c r="D192" s="29" t="n"/>
+      <c r="E192" s="18">
         <f>IF(D192="","",D192*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F192" s="28" t="n"/>
+      <c r="F192" s="29" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="27" t="n"/>
-      <c r="B193" s="27" t="n"/>
-      <c r="C193" s="28" t="n"/>
-      <c r="D193" s="28" t="n"/>
-      <c r="E193" s="17">
+      <c r="A193" s="28" t="n"/>
+      <c r="B193" s="28" t="n"/>
+      <c r="C193" s="29" t="n"/>
+      <c r="D193" s="29" t="n"/>
+      <c r="E193" s="18">
         <f>IF(D193="","",D193*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F193" s="28" t="n"/>
+      <c r="F193" s="29" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="27" t="n"/>
-      <c r="B194" s="27" t="n"/>
-      <c r="C194" s="28" t="n"/>
-      <c r="D194" s="28" t="n"/>
-      <c r="E194" s="17">
+      <c r="A194" s="28" t="n"/>
+      <c r="B194" s="28" t="n"/>
+      <c r="C194" s="29" t="n"/>
+      <c r="D194" s="29" t="n"/>
+      <c r="E194" s="18">
         <f>IF(D194="","",D194*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F194" s="28" t="n"/>
+      <c r="F194" s="29" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="27" t="n"/>
-      <c r="B195" s="27" t="n"/>
-      <c r="C195" s="28" t="n"/>
-      <c r="D195" s="28" t="n"/>
-      <c r="E195" s="17">
+      <c r="A195" s="28" t="n"/>
+      <c r="B195" s="28" t="n"/>
+      <c r="C195" s="29" t="n"/>
+      <c r="D195" s="29" t="n"/>
+      <c r="E195" s="18">
         <f>IF(D195="","",D195*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F195" s="28" t="n"/>
+      <c r="F195" s="29" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="27" t="n"/>
-      <c r="B196" s="27" t="n"/>
-      <c r="C196" s="28" t="n"/>
-      <c r="D196" s="28" t="n"/>
-      <c r="E196" s="17">
+      <c r="A196" s="28" t="n"/>
+      <c r="B196" s="28" t="n"/>
+      <c r="C196" s="29" t="n"/>
+      <c r="D196" s="29" t="n"/>
+      <c r="E196" s="18">
         <f>IF(D196="","",D196*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F196" s="28" t="n"/>
+      <c r="F196" s="29" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="27" t="n"/>
-      <c r="B197" s="27" t="n"/>
-      <c r="C197" s="28" t="n"/>
-      <c r="D197" s="28" t="n"/>
-      <c r="E197" s="17">
+      <c r="A197" s="28" t="n"/>
+      <c r="B197" s="28" t="n"/>
+      <c r="C197" s="29" t="n"/>
+      <c r="D197" s="29" t="n"/>
+      <c r="E197" s="18">
         <f>IF(D197="","",D197*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F197" s="28" t="n"/>
+      <c r="F197" s="29" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="27" t="n"/>
-      <c r="B198" s="27" t="n"/>
-      <c r="C198" s="28" t="n"/>
-      <c r="D198" s="28" t="n"/>
-      <c r="E198" s="17">
+      <c r="A198" s="28" t="n"/>
+      <c r="B198" s="28" t="n"/>
+      <c r="C198" s="29" t="n"/>
+      <c r="D198" s="29" t="n"/>
+      <c r="E198" s="18">
         <f>IF(D198="","",D198*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F198" s="28" t="n"/>
+      <c r="F198" s="29" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" s="27" t="n"/>
-      <c r="B199" s="27" t="n"/>
-      <c r="C199" s="28" t="n"/>
-      <c r="D199" s="28" t="n"/>
-      <c r="E199" s="17">
+      <c r="A199" s="28" t="n"/>
+      <c r="B199" s="28" t="n"/>
+      <c r="C199" s="29" t="n"/>
+      <c r="D199" s="29" t="n"/>
+      <c r="E199" s="18">
         <f>IF(D199="","",D199*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F199" s="28" t="n"/>
+      <c r="F199" s="29" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="27" t="n"/>
-      <c r="B200" s="27" t="n"/>
-      <c r="C200" s="28" t="n"/>
-      <c r="D200" s="28" t="n"/>
-      <c r="E200" s="17">
+      <c r="A200" s="28" t="n"/>
+      <c r="B200" s="28" t="n"/>
+      <c r="C200" s="29" t="n"/>
+      <c r="D200" s="29" t="n"/>
+      <c r="E200" s="18">
         <f>IF(D200="","",D200*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F200" s="28" t="n"/>
+      <c r="F200" s="29" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" s="27" t="n"/>
-      <c r="B201" s="27" t="n"/>
-      <c r="C201" s="28" t="n"/>
-      <c r="D201" s="28" t="n"/>
-      <c r="E201" s="17">
+      <c r="A201" s="28" t="n"/>
+      <c r="B201" s="28" t="n"/>
+      <c r="C201" s="29" t="n"/>
+      <c r="D201" s="29" t="n"/>
+      <c r="E201" s="18">
         <f>IF(D201="","",D201*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F201" s="28" t="n"/>
+      <c r="F201" s="29" t="n"/>
     </row>
     <row r="202">
-      <c r="A202" s="27" t="n"/>
-      <c r="B202" s="27" t="n"/>
-      <c r="C202" s="28" t="n"/>
-      <c r="D202" s="28" t="n"/>
-      <c r="E202" s="17">
+      <c r="A202" s="28" t="n"/>
+      <c r="B202" s="28" t="n"/>
+      <c r="C202" s="29" t="n"/>
+      <c r="D202" s="29" t="n"/>
+      <c r="E202" s="18">
         <f>IF(D202="","",D202*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F202" s="28" t="n"/>
+      <c r="F202" s="29" t="n"/>
     </row>
     <row r="203">
-      <c r="A203" s="27" t="n"/>
-      <c r="B203" s="27" t="n"/>
-      <c r="C203" s="28" t="n"/>
-      <c r="D203" s="28" t="n"/>
-      <c r="E203" s="17">
+      <c r="A203" s="28" t="n"/>
+      <c r="B203" s="28" t="n"/>
+      <c r="C203" s="29" t="n"/>
+      <c r="D203" s="29" t="n"/>
+      <c r="E203" s="18">
         <f>IF(D203="","",D203*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F203" s="28" t="n"/>
+      <c r="F203" s="29" t="n"/>
     </row>
     <row r="204">
-      <c r="A204" s="27" t="n"/>
-      <c r="B204" s="27" t="n"/>
-      <c r="C204" s="28" t="n"/>
-      <c r="D204" s="28" t="n"/>
-      <c r="E204" s="17">
+      <c r="A204" s="28" t="n"/>
+      <c r="B204" s="28" t="n"/>
+      <c r="C204" s="29" t="n"/>
+      <c r="D204" s="29" t="n"/>
+      <c r="E204" s="18">
         <f>IF(D204="","",D204*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F204" s="28" t="n"/>
+      <c r="F204" s="29" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Tableau simple : actuel en heures et en jours, total des deux
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1LRXK2yXR6W5viD25HWb5
</commit_message>
<xml_diff>
--- a/conges/conges_police_12h08.xlsx
+++ b/conges/conges_police_12h08.xlsx
@@ -144,7 +144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -152,17 +152,25 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="167" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="167" fontId="11" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -179,7 +187,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="9" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="5" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -550,13 +557,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D14"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,17 +586,22 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Actuel</t>
+          <t>Actuel (heures)</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Pris</t>
+          <t>Actuel (jours)</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
         <is>
-          <t>Restant</t>
+          <t>Pris (jours)</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Restant (jours)</t>
         </is>
       </c>
     </row>
@@ -601,11 +614,15 @@
       <c r="B4" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="6">
+        <f>B4/$B$15</f>
+        <v/>
+      </c>
+      <c r="D4" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D4" s="6">
-        <f>B4-C4</f>
+      <c r="E4" s="6">
+        <f>C4-D4</f>
         <v/>
       </c>
     </row>
@@ -618,11 +635,15 @@
       <c r="B5" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="6">
+        <f>B5/$B$15</f>
+        <v/>
+      </c>
+      <c r="D5" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D5" s="6">
-        <f>B5-C5</f>
+      <c r="E5" s="6">
+        <f>C5-D5</f>
         <v/>
       </c>
     </row>
@@ -635,11 +656,15 @@
       <c r="B6" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="6">
+        <f>B6/$B$15</f>
+        <v/>
+      </c>
+      <c r="D6" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D6" s="6">
-        <f>B6-C6</f>
+      <c r="E6" s="6">
+        <f>C6-D6</f>
         <v/>
       </c>
     </row>
@@ -652,11 +677,15 @@
       <c r="B7" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="6">
+        <f>B7/$B$15</f>
+        <v/>
+      </c>
+      <c r="D7" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D7" s="6">
-        <f>B7-C7</f>
+      <c r="E7" s="6">
+        <f>C7-D7</f>
         <v/>
       </c>
     </row>
@@ -669,11 +698,15 @@
       <c r="B8" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="6">
+        <f>B8/$B$15</f>
+        <v/>
+      </c>
+      <c r="D8" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D8" s="6">
-        <f>B8-C8</f>
+      <c r="E8" s="6">
+        <f>C8-D8</f>
         <v/>
       </c>
     </row>
@@ -686,11 +719,15 @@
       <c r="B9" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="6">
+        <f>B9/$B$15</f>
+        <v/>
+      </c>
+      <c r="D9" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D9" s="6">
-        <f>B9-C9</f>
+      <c r="E9" s="6">
+        <f>C9-D9</f>
         <v/>
       </c>
     </row>
@@ -703,42 +740,66 @@
       <c r="B10" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6">
+        <f>B10/$B$15</f>
+        <v/>
+      </c>
+      <c r="D10" s="7" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="6">
-        <f>B10-C10</f>
+      <c r="E10" s="6">
+        <f>C10-D10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="8">
+      <c r="B11" s="9">
         <f>SUM(B4:B10)</f>
         <v/>
       </c>
-      <c r="C11" s="8">
+      <c r="C11" s="10">
         <f>SUM(C4:C10)</f>
         <v/>
       </c>
-      <c r="D11" s="8">
+      <c r="D11" s="10">
         <f>SUM(D4:D10)</f>
         <v/>
       </c>
+      <c r="E11" s="10">
+        <f>SUM(E4:E10)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Cases jaunes : tape tes chiffres en jours. Restant et Total se calculent seuls.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
+        <is>
+          <t>Cases jaunes : tape l'actuel en heures et le pris en jours. Le reste se calcule seul.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="12" t="inlineStr">
+        <is>
+          <t>1 jour =</t>
+        </is>
+      </c>
+      <c r="B15" s="13">
+        <f>12+8/60</f>
+        <v/>
+      </c>
+      <c r="C15" s="11" t="inlineStr">
+        <is>
+          <t>heures (12h08). Mets 7 pour un jour ouvré.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>Les autres onglets sont une aide au calcul, facultative.</t>
         </is>
@@ -772,31 +833,31 @@
           <t>Mes droits à congés – récapitulatif</t>
         </is>
       </c>
-      <c r="B1" s="10" t="n"/>
-      <c r="C1" s="10" t="n"/>
-      <c r="D1" s="10" t="n"/>
-      <c r="E1" s="10" t="n"/>
-      <c r="F1" s="10" t="n"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Tout se calcule depuis Parametres et Suivi. Ne rien saisir ici.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="14" t="n"/>
+      <c r="E2" s="14" t="n"/>
+      <c r="F2" s="14" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="n"/>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
+      <c r="A3" s="14" t="n"/>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -831,244 +892,244 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>CA – Congés annuels</t>
         </is>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="17">
         <f>Parametres!$B$9*Parametres!$B$10*Parametres!$B$8</f>
         <v/>
       </c>
-      <c r="C5" s="13">
+      <c r="C5" s="17">
         <f>SUMIF(Suivi!$C$5:$C$204,"CA",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="18">
         <f>B5-C5</f>
         <v/>
       </c>
-      <c r="E5" s="13">
+      <c r="E5" s="17">
         <f>D5/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F5" s="12" t="inlineStr">
+      <c r="F5" s="16" t="inlineStr">
         <is>
           <t>25 j ouvrés × valeur horaire × quotité.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>CA HP – Hors période</t>
         </is>
       </c>
-      <c r="B6" s="13">
+      <c r="B6" s="17">
         <f>IF(Parametres!$B$11&gt;=8,2,IF(Parametres!$B$11&gt;=5,1,0))*Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C6" s="13">
+      <c r="C6" s="17">
         <f>SUMIF(Suivi!$C$5:$C$204,"CA HP",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D6" s="14">
+      <c r="D6" s="18">
         <f>B6-C6</f>
         <v/>
       </c>
-      <c r="E6" s="13">
+      <c r="E6" s="17">
         <f>D6/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F6" s="12" t="inlineStr">
+      <c r="F6" s="16" t="inlineStr">
         <is>
           <t>Bonus : 1 j si 5-7 j CA hors mai-oct ; 2 j si 8 et +.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>RTC</t>
         </is>
       </c>
-      <c r="B7" s="13">
+      <c r="B7" s="17">
         <f>Parametres!$B$12</f>
         <v/>
       </c>
-      <c r="C7" s="13">
+      <c r="C7" s="17">
         <f>SUMIF(Suivi!$C$5:$C$204,"RTC",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D7" s="14">
+      <c r="D7" s="18">
         <f>B7-C7</f>
         <v/>
       </c>
-      <c r="E7" s="13">
+      <c r="E7" s="17">
         <f>D7/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F7" s="12" t="inlineStr">
+      <c r="F7" s="16" t="inlineStr">
         <is>
           <t>Crédit saisi dans Parametres.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>CET – Compte épargne-temps</t>
         </is>
       </c>
-      <c r="B8" s="13">
+      <c r="B8" s="17">
         <f>(Parametres!$B$18+Parametres!$B$19)*Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C8" s="13">
+      <c r="C8" s="17">
         <f>SUMIF(Suivi!$C$5:$C$204,"CET",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D8" s="14">
+      <c r="D8" s="18">
         <f>B8-C8</f>
         <v/>
       </c>
-      <c r="E8" s="13">
+      <c r="E8" s="17">
         <f>D8/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F8" s="12" t="inlineStr">
+      <c r="F8" s="16" t="inlineStr">
         <is>
           <t>Solde 1er janvier + jours versés.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>CF – Crédit férié</t>
         </is>
       </c>
-      <c r="B9" s="13">
+      <c r="B9" s="17">
         <f>Parametres!$B$13*Parametres!$B$14</f>
         <v/>
       </c>
-      <c r="C9" s="13">
+      <c r="C9" s="17">
         <f>SUMIF(Suivi!$C$5:$C$204,"CF",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D9" s="14">
+      <c r="D9" s="18">
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="13">
+      <c r="E9" s="17">
         <f>D9/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F9" s="12" t="inlineStr">
+      <c r="F9" s="16" t="inlineStr">
         <is>
           <t>Nb fériés × heures par férié.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>HS – Heures supplémentaires</t>
         </is>
       </c>
-      <c r="B10" s="13">
+      <c r="B10" s="17">
         <f>Parametres!$B$15</f>
         <v/>
       </c>
-      <c r="C10" s="13">
+      <c r="C10" s="17">
         <f>SUMIF(Suivi!$C$5:$C$204,"HS",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D10" s="14">
+      <c r="D10" s="18">
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="13">
+      <c r="E10" s="17">
         <f>D10/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F10" s="12" t="inlineStr">
+      <c r="F10" s="16" t="inlineStr">
         <is>
           <t>Compteur HS récupérables.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>RPS – Repos pénibilité nuit</t>
         </is>
       </c>
-      <c r="B11" s="13">
+      <c r="B11" s="17">
         <f>IF(Parametres!$B$17&gt;0,Parametres!$B$17,ROUND(140*Parametres!$B$8,0))*Parametres!$B$7*Parametres!$B$16</f>
         <v/>
       </c>
-      <c r="C11" s="13">
+      <c r="C11" s="17">
         <f>SUMIF(Suivi!$C$5:$C$204,"RPS",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D11" s="14">
+      <c r="D11" s="18">
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="13">
+      <c r="E11" s="17">
         <f>D11/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F11" s="12" t="inlineStr">
+      <c r="F11" s="16" t="inlineStr">
         <is>
           <t>Vacations nuit × heures nuit × coef.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="15" t="inlineStr">
+      <c r="A12" s="19" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="16">
+      <c r="B12" s="20">
         <f>SUM(B5:B11)</f>
         <v/>
       </c>
-      <c r="C12" s="16">
+      <c r="C12" s="20">
         <f>SUM(C5:C11)</f>
         <v/>
       </c>
-      <c r="D12" s="16">
+      <c r="D12" s="20">
         <f>SUM(D5:D11)</f>
         <v/>
       </c>
-      <c r="E12" s="16">
+      <c r="E12" s="20">
         <f>SUM(E5:E11)</f>
         <v/>
       </c>
-      <c r="F12" s="15" t="n"/>
+      <c r="F12" s="19" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="10" t="n"/>
-      <c r="B13" s="10" t="n"/>
-      <c r="C13" s="10" t="n"/>
-      <c r="D13" s="10" t="n"/>
-      <c r="E13" s="10" t="n"/>
-      <c r="F13" s="10" t="n"/>
+      <c r="A13" s="14" t="n"/>
+      <c r="B13" s="14" t="n"/>
+      <c r="C13" s="14" t="n"/>
+      <c r="D13" s="14" t="n"/>
+      <c r="E13" s="14" t="n"/>
+      <c r="F13" s="14" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>CET – détail</t>
         </is>
       </c>
-      <c r="B14" s="10" t="n"/>
-      <c r="C14" s="10" t="n"/>
-      <c r="D14" s="10" t="n"/>
-      <c r="E14" s="10" t="n"/>
-      <c r="F14" s="10" t="n"/>
+      <c r="B14" s="14" t="n"/>
+      <c r="C14" s="14" t="n"/>
+      <c r="D14" s="14" t="n"/>
+      <c r="E14" s="14" t="n"/>
+      <c r="F14" s="14" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1091,134 +1152,134 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>Jours CA pris dans l'année</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="22">
         <f>C5/Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C16" s="10" t="n"/>
-      <c r="D16" s="10" t="n"/>
-      <c r="E16" s="10" t="n"/>
-      <c r="F16" s="10" t="inlineStr">
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="14" t="n"/>
+      <c r="E16" s="14" t="n"/>
+      <c r="F16" s="14" t="inlineStr">
         <is>
           <t>Depuis Suivi.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>Jours épargnables max</t>
         </is>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="22">
         <f>MAX(0,MIN((B5+B6-C5-C6)/Parametres!$B$10,(B5+B6)/Parametres!$B$10-20))</f>
         <v/>
       </c>
-      <c r="C17" s="10" t="n"/>
-      <c r="D17" s="10" t="n"/>
-      <c r="E17" s="10" t="n"/>
-      <c r="F17" s="10" t="inlineStr">
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="14" t="n"/>
+      <c r="E17" s="14" t="n"/>
+      <c r="F17" s="14" t="inlineStr">
         <is>
           <t>20 j de CA obligatoires. Le reliquat est épargnable.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>Solde CET restant (jours)</t>
         </is>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="22">
         <f>D8/Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C18" s="10" t="n"/>
-      <c r="D18" s="10" t="n"/>
-      <c r="E18" s="10" t="n"/>
-      <c r="F18" s="10" t="inlineStr">
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="14" t="n"/>
+      <c r="E18" s="14" t="n"/>
+      <c r="F18" s="14" t="inlineStr">
         <is>
           <t>Plafond 60 jours.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>Alerte plafond</t>
         </is>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="22">
         <f>IF(B18&gt;60,"Plafond 60 j dépassé","OK")</f>
         <v/>
       </c>
-      <c r="C19" s="10" t="n"/>
-      <c r="D19" s="10" t="n"/>
-      <c r="E19" s="10" t="n"/>
-      <c r="F19" s="10" t="inlineStr"/>
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="14" t="n"/>
+      <c r="E19" s="14" t="n"/>
+      <c r="F19" s="14" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Jours indemnisables (au-delà de 15)</t>
         </is>
       </c>
-      <c r="B20" s="18">
+      <c r="B20" s="22">
         <f>MAX(0,MIN(B18,60)-15)</f>
         <v/>
       </c>
-      <c r="C20" s="10" t="n"/>
-      <c r="D20" s="10" t="n"/>
-      <c r="E20" s="10" t="n"/>
-      <c r="F20" s="10" t="inlineStr">
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="14" t="n"/>
+      <c r="E20" s="14" t="n"/>
+      <c r="F20" s="14" t="inlineStr">
         <is>
           <t>Option possible au-delà de 15 j.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Valeur si indemnisés (€)</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="23">
         <f>B20*IF(Parametres!$B$20="A",Parametres!$B$23,IF(Parametres!$B$20="B",Parametres!$B$22,Parametres!$B$21))</f>
         <v/>
       </c>
-      <c r="C21" s="10" t="n"/>
-      <c r="D21" s="10" t="n"/>
-      <c r="E21" s="10" t="n"/>
-      <c r="F21" s="10" t="inlineStr">
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="14" t="n"/>
+      <c r="E21" s="14" t="n"/>
+      <c r="F21" s="14" t="inlineStr">
         <is>
           <t>Montant brut selon catégorie.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="10" t="n"/>
-      <c r="B22" s="10" t="n"/>
-      <c r="C22" s="10" t="n"/>
-      <c r="D22" s="10" t="n"/>
-      <c r="E22" s="10" t="n"/>
-      <c r="F22" s="10" t="n"/>
+      <c r="A22" s="14" t="n"/>
+      <c r="B22" s="14" t="n"/>
+      <c r="C22" s="14" t="n"/>
+      <c r="D22" s="14" t="n"/>
+      <c r="E22" s="14" t="n"/>
+      <c r="F22" s="14" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="17" t="inlineStr">
+      <c r="A23" s="21" t="inlineStr">
         <is>
           <t>ASA – Autorisations spéciales d'absence (hors compteur)</t>
         </is>
       </c>
-      <c r="B23" s="10" t="n"/>
-      <c r="C23" s="10" t="n"/>
-      <c r="D23" s="10" t="n"/>
-      <c r="E23" s="10" t="n"/>
-      <c r="F23" s="10" t="n"/>
+      <c r="B23" s="14" t="n"/>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="14" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1241,119 +1302,119 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Garde d'enfant malade</t>
         </is>
       </c>
-      <c r="B25" s="20">
+      <c r="B25" s="24">
         <f>IF(Parametres!$B$24="O",IF(Parametres!$B$25="O",12,6)*Parametres!$B$8,0)</f>
         <v/>
       </c>
-      <c r="C25" s="10" t="n"/>
-      <c r="D25" s="10" t="n"/>
-      <c r="E25" s="10" t="n"/>
-      <c r="F25" s="10" t="inlineStr">
+      <c r="C25" s="14" t="n"/>
+      <c r="D25" s="14" t="n"/>
+      <c r="E25" s="14" t="n"/>
+      <c r="F25" s="14" t="inlineStr">
         <is>
           <t>6 j/an ; 12 j si seul ou conjoint sans droit. À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>Mariage / PACS de l'agent</t>
         </is>
       </c>
-      <c r="B26" s="20" t="n">
+      <c r="B26" s="24" t="n">
         <v>5</v>
       </c>
-      <c r="C26" s="10" t="n"/>
-      <c r="D26" s="10" t="n"/>
-      <c r="E26" s="10" t="n"/>
-      <c r="F26" s="10" t="inlineStr">
+      <c r="C26" s="14" t="n"/>
+      <c r="D26" s="14" t="n"/>
+      <c r="E26" s="14" t="n"/>
+      <c r="F26" s="14" t="inlineStr">
         <is>
           <t>Barème FP. À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="16" t="inlineStr">
         <is>
           <t>Décès conjoint / parent / enfant</t>
         </is>
       </c>
-      <c r="B27" s="20" t="n">
+      <c r="B27" s="24" t="n">
         <v>3</v>
       </c>
-      <c r="C27" s="10" t="n"/>
-      <c r="D27" s="10" t="n"/>
-      <c r="E27" s="10" t="n"/>
-      <c r="F27" s="10" t="inlineStr">
+      <c r="C27" s="14" t="n"/>
+      <c r="D27" s="14" t="n"/>
+      <c r="E27" s="14" t="n"/>
+      <c r="F27" s="14" t="inlineStr">
         <is>
           <t>Barème FP. Enfant : régime renforcé.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="A28" s="16" t="inlineStr">
         <is>
           <t>Naissance / adoption</t>
         </is>
       </c>
-      <c r="B28" s="20" t="inlineStr">
+      <c r="B28" s="24" t="inlineStr">
         <is>
           <t>Voir RH</t>
         </is>
       </c>
-      <c r="C28" s="10" t="n"/>
-      <c r="D28" s="10" t="n"/>
-      <c r="E28" s="10" t="n"/>
-      <c r="F28" s="10" t="inlineStr">
+      <c r="C28" s="14" t="n"/>
+      <c r="D28" s="14" t="n"/>
+      <c r="E28" s="14" t="n"/>
+      <c r="F28" s="14" t="inlineStr">
         <is>
           <t>Congé naissance 3 j + paternité 25 j.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="A29" s="16" t="inlineStr">
         <is>
           <t>Déménagement</t>
         </is>
       </c>
-      <c r="B29" s="20" t="inlineStr">
+      <c r="B29" s="24" t="inlineStr">
         <is>
           <t>Voir RH</t>
         </is>
       </c>
-      <c r="C29" s="10" t="n"/>
-      <c r="D29" s="10" t="n"/>
-      <c r="E29" s="10" t="n"/>
-      <c r="F29" s="10" t="inlineStr">
+      <c r="C29" s="14" t="n"/>
+      <c r="D29" s="14" t="n"/>
+      <c r="E29" s="14" t="n"/>
+      <c r="F29" s="14" t="inlineStr">
         <is>
           <t>Selon note de service.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="10" t="n"/>
-      <c r="B30" s="10" t="n"/>
-      <c r="C30" s="10" t="n"/>
-      <c r="D30" s="10" t="n"/>
-      <c r="E30" s="10" t="n"/>
-      <c r="F30" s="10" t="n"/>
+      <c r="A30" s="14" t="n"/>
+      <c r="B30" s="14" t="n"/>
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14" t="n"/>
+      <c r="F30" s="14" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="21" t="inlineStr">
+      <c r="A31" s="25" t="inlineStr">
         <is>
           <t>Les montants et barèmes sont indicatifs. Vérifie avec ton secrétariat / Géopol et ta note de service locale.</t>
         </is>
       </c>
-      <c r="B31" s="10" t="n"/>
-      <c r="C31" s="10" t="n"/>
-      <c r="D31" s="10" t="n"/>
-      <c r="E31" s="10" t="n"/>
-      <c r="F31" s="10" t="n"/>
+      <c r="B31" s="14" t="n"/>
+      <c r="C31" s="14" t="n"/>
+      <c r="D31" s="14" t="n"/>
+      <c r="E31" s="14" t="n"/>
+      <c r="F31" s="14" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1380,22 +1441,22 @@
           <t>Paramètres – Police nationale, cycle 12h08 de nuit</t>
         </is>
       </c>
-      <c r="B1" s="10" t="n"/>
-      <c r="C1" s="10" t="n"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Cellules jaunes / texte bleu = à saisir. Le reste se calcule seul.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="n"/>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
+      <c r="A3" s="14" t="n"/>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1415,339 +1476,339 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="16" t="inlineStr">
         <is>
           <t>Année de référence</t>
         </is>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="26" t="n">
         <v>2026</v>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Année civile des droits.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="16" t="inlineStr">
         <is>
           <t>Durée d'une vacation (heures)</t>
         </is>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="22">
         <f>12+8/60</f>
         <v/>
       </c>
-      <c r="C6" s="23" t="inlineStr">
+      <c r="C6" s="27" t="inlineStr">
         <is>
           <t>12h08 = 12,13 h, dont 2 pauses de 20 min (rapport Sénat).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="16" t="inlineStr">
         <is>
           <t>Heures de nuit par vacation</t>
         </is>
       </c>
-      <c r="B7" s="24" t="n">
+      <c r="B7" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="C7" s="23" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>Heures entre 21h et 6h (RGEMPN). 9h si vacation couvre toute la plage.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="16" t="inlineStr">
         <is>
           <t>Quotité de travail</t>
         </is>
       </c>
-      <c r="B8" s="25" t="n">
+      <c r="B8" s="28" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="23" t="inlineStr">
+      <c r="C8" s="27" t="inlineStr">
         <is>
           <t>100 % = temps plein.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="16" t="inlineStr">
         <is>
           <t>CA – jours ouvrés réglementaires</t>
         </is>
       </c>
-      <c r="B9" s="22" t="n">
+      <c r="B9" s="26" t="n">
         <v>25</v>
       </c>
-      <c r="C9" s="23" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>Décret 84-972 : 25 jours ouvrés.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="16" t="inlineStr">
         <is>
           <t>Valeur horaire d'1 jour de CA (h)</t>
         </is>
       </c>
-      <c r="B10" s="24" t="n">
+      <c r="B10" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="C10" s="23" t="inlineStr">
+      <c r="C10" s="27" t="inlineStr">
         <is>
           <t>À vérifier avec ton secrétariat / Géopol.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="16" t="inlineStr">
         <is>
           <t>CA HP – jours CA pris hors 1/05–31/10</t>
         </is>
       </c>
-      <c r="B11" s="22" t="n">
+      <c r="B11" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="23" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>5 à 7 j = 1 j bonus ; 8 j et + = 2 j bonus.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="16" t="inlineStr">
         <is>
           <t>RTC – crédit annuel (heures)</t>
         </is>
       </c>
-      <c r="B12" s="24" t="n">
+      <c r="B12" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="23" t="inlineStr">
+      <c r="C12" s="27" t="inlineStr">
         <is>
           <t>Crédit annuel horaire d'ARTT en régime cyclique (RGEMPN art. 39). Voir Géopol.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="16" t="inlineStr">
         <is>
           <t>CF – nombre de fériés crédités</t>
         </is>
       </c>
-      <c r="B13" s="22" t="n">
+      <c r="B13" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="23" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>Crédit férié annuel, en heures, pour régime cyclique. Voir Géopol.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="16" t="inlineStr">
         <is>
           <t>CF – heures par férié</t>
         </is>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="22">
         <f>B6</f>
         <v/>
       </c>
-      <c r="C14" s="23" t="inlineStr">
+      <c r="C14" s="27" t="inlineStr">
         <is>
           <t>Par défaut = 1 vacation. Modifiable.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="16" t="inlineStr">
         <is>
           <t>HS – heures sup. au compteur (heures)</t>
         </is>
       </c>
-      <c r="B15" s="24" t="n">
+      <c r="B15" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="23" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>Solde HS récupérables. Voir relevé.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>RPS – coef. sur heures de nuit</t>
         </is>
       </c>
-      <c r="B16" s="25" t="n">
+      <c r="B16" s="28" t="n">
         <v>0.1</v>
       </c>
-      <c r="C16" s="23" t="inlineStr">
+      <c r="C16" s="27" t="inlineStr">
         <is>
           <t>0,1 par heure de nuit 21h-6h (0,4 dimanche, non cumulable). Source : RGEMPN.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="16" t="inlineStr">
         <is>
           <t>RPS – vacations de nuit / an</t>
         </is>
       </c>
-      <c r="B17" s="22" t="n">
+      <c r="B17" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="23" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>0 = 140 vacations/an (cycle binaire, rapport Sénat).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="16" t="inlineStr">
         <is>
           <t>CET – solde au 1er janvier (jours)</t>
         </is>
       </c>
-      <c r="B18" s="24" t="n">
+      <c r="B18" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="23" t="inlineStr">
+      <c r="C18" s="27" t="inlineStr">
         <is>
           <t>Repris de ton relevé CET.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>CET – jours versés cette année</t>
         </is>
       </c>
-      <c r="B19" s="24" t="n">
+      <c r="B19" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="C19" s="23" t="inlineStr">
+      <c r="C19" s="27" t="inlineStr">
         <is>
           <t>Ta demande d'alimentation.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>Catégorie (C, B, A)</t>
         </is>
       </c>
-      <c r="B20" s="26" t="inlineStr">
+      <c r="B20" s="29" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C20" s="23" t="inlineStr">
+      <c r="C20" s="27" t="inlineStr">
         <is>
           <t>Pour l'indemnisation CET.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="16" t="inlineStr">
         <is>
           <t>Taux CET catégorie C (€/jour)</t>
         </is>
       </c>
-      <c r="B21" s="27" t="n">
+      <c r="B21" s="30" t="n">
         <v>83</v>
       </c>
-      <c r="C21" s="23" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="16" t="inlineStr">
         <is>
           <t>Taux CET catégorie B (€/jour)</t>
         </is>
       </c>
-      <c r="B22" s="27" t="n">
+      <c r="B22" s="30" t="n">
         <v>100</v>
       </c>
-      <c r="C22" s="23" t="inlineStr">
+      <c r="C22" s="27" t="inlineStr">
         <is>
           <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Taux CET catégorie A (€/jour)</t>
         </is>
       </c>
-      <c r="B23" s="27" t="n">
+      <c r="B23" s="30" t="n">
         <v>150</v>
       </c>
-      <c r="C23" s="23" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="16" t="inlineStr">
         <is>
           <t>Enfants à charge &lt; 16 ans (O/N)</t>
         </is>
       </c>
-      <c r="B24" s="26" t="inlineStr">
+      <c r="B24" s="29" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="C24" s="23" t="inlineStr">
+      <c r="C24" s="27" t="inlineStr">
         <is>
           <t>Pour ASA garde d'enfant.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="16" t="inlineStr">
         <is>
           <t>Élève seul l'enfant ou conjoint sans droit (O/N)</t>
         </is>
       </c>
-      <c r="B25" s="26" t="inlineStr">
+      <c r="B25" s="29" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C25" s="23" t="inlineStr">
+      <c r="C25" s="27" t="inlineStr">
         <is>
           <t>Doublement ASA garde d'enfant.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+      <c r="A26" s="16" t="inlineStr">
         <is>
           <t>Durée d'un jour dans le Tableau (h)</t>
         </is>
       </c>
-      <c r="B26" s="18">
+      <c r="B26" s="22">
         <f>B6</f>
         <v/>
       </c>
-      <c r="C26" s="23" t="inlineStr">
+      <c r="C26" s="27" t="inlineStr">
         <is>
           <t>Par défaut 1 jour = 1 vacation de 12h08. Mets 7 pour des jours ouvrés.</t>
         </is>
@@ -1789,31 +1850,31 @@
           <t>Journal des absences posées</t>
         </is>
       </c>
-      <c r="B1" s="10" t="n"/>
-      <c r="C1" s="10" t="n"/>
-      <c r="D1" s="10" t="n"/>
-      <c r="E1" s="10" t="n"/>
-      <c r="F1" s="10" t="n"/>
+      <c r="B1" s="14" t="n"/>
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="14" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Une ligne par absence. Choisis le type dans la liste. Heures calculées seules.</t>
         </is>
       </c>
-      <c r="B2" s="10" t="n"/>
-      <c r="C2" s="10" t="n"/>
-      <c r="D2" s="10" t="n"/>
-      <c r="E2" s="10" t="n"/>
-      <c r="F2" s="10" t="n"/>
+      <c r="B2" s="14" t="n"/>
+      <c r="C2" s="14" t="n"/>
+      <c r="D2" s="14" t="n"/>
+      <c r="E2" s="14" t="n"/>
+      <c r="F2" s="14" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="10" t="n"/>
-      <c r="B3" s="10" t="n"/>
-      <c r="C3" s="10" t="n"/>
-      <c r="D3" s="10" t="n"/>
-      <c r="E3" s="10" t="n"/>
-      <c r="F3" s="10" t="n"/>
+      <c r="A3" s="14" t="n"/>
+      <c r="B3" s="14" t="n"/>
+      <c r="C3" s="14" t="n"/>
+      <c r="D3" s="14" t="n"/>
+      <c r="E3" s="14" t="n"/>
+      <c r="F3" s="14" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1848,2218 +1909,2218 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="28" t="n">
+      <c r="A5" s="31" t="n">
         <v>46063</v>
       </c>
-      <c r="B5" s="28" t="n">
+      <c r="B5" s="31" t="n">
         <v>46066</v>
       </c>
-      <c r="C5" s="29" t="inlineStr">
+      <c r="C5" s="32" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D5" s="29" t="n">
+      <c r="D5" s="32" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="22">
         <f>IF(D5="","",D5*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F5" s="29" t="inlineStr">
+      <c r="F5" s="32" t="inlineStr">
         <is>
           <t>Exemple – à effacer</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="28" t="n"/>
-      <c r="B6" s="28" t="n"/>
-      <c r="C6" s="29" t="n"/>
-      <c r="D6" s="29" t="n"/>
-      <c r="E6" s="18">
+      <c r="A6" s="31" t="n"/>
+      <c r="B6" s="31" t="n"/>
+      <c r="C6" s="32" t="n"/>
+      <c r="D6" s="32" t="n"/>
+      <c r="E6" s="22">
         <f>IF(D6="","",D6*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F6" s="29" t="n"/>
+      <c r="F6" s="32" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="28" t="n"/>
-      <c r="B7" s="28" t="n"/>
-      <c r="C7" s="29" t="n"/>
-      <c r="D7" s="29" t="n"/>
-      <c r="E7" s="18">
+      <c r="A7" s="31" t="n"/>
+      <c r="B7" s="31" t="n"/>
+      <c r="C7" s="32" t="n"/>
+      <c r="D7" s="32" t="n"/>
+      <c r="E7" s="22">
         <f>IF(D7="","",D7*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F7" s="29" t="n"/>
+      <c r="F7" s="32" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="28" t="n"/>
-      <c r="B8" s="28" t="n"/>
-      <c r="C8" s="29" t="n"/>
-      <c r="D8" s="29" t="n"/>
-      <c r="E8" s="18">
+      <c r="A8" s="31" t="n"/>
+      <c r="B8" s="31" t="n"/>
+      <c r="C8" s="32" t="n"/>
+      <c r="D8" s="32" t="n"/>
+      <c r="E8" s="22">
         <f>IF(D8="","",D8*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F8" s="29" t="n"/>
+      <c r="F8" s="32" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="28" t="n"/>
-      <c r="B9" s="28" t="n"/>
-      <c r="C9" s="29" t="n"/>
-      <c r="D9" s="29" t="n"/>
-      <c r="E9" s="18">
+      <c r="A9" s="31" t="n"/>
+      <c r="B9" s="31" t="n"/>
+      <c r="C9" s="32" t="n"/>
+      <c r="D9" s="32" t="n"/>
+      <c r="E9" s="22">
         <f>IF(D9="","",D9*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F9" s="29" t="n"/>
+      <c r="F9" s="32" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="28" t="n"/>
-      <c r="B10" s="28" t="n"/>
-      <c r="C10" s="29" t="n"/>
-      <c r="D10" s="29" t="n"/>
-      <c r="E10" s="18">
+      <c r="A10" s="31" t="n"/>
+      <c r="B10" s="31" t="n"/>
+      <c r="C10" s="32" t="n"/>
+      <c r="D10" s="32" t="n"/>
+      <c r="E10" s="22">
         <f>IF(D10="","",D10*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F10" s="29" t="n"/>
+      <c r="F10" s="32" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="28" t="n"/>
-      <c r="B11" s="28" t="n"/>
-      <c r="C11" s="29" t="n"/>
-      <c r="D11" s="29" t="n"/>
-      <c r="E11" s="18">
+      <c r="A11" s="31" t="n"/>
+      <c r="B11" s="31" t="n"/>
+      <c r="C11" s="32" t="n"/>
+      <c r="D11" s="32" t="n"/>
+      <c r="E11" s="22">
         <f>IF(D11="","",D11*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F11" s="29" t="n"/>
+      <c r="F11" s="32" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="28" t="n"/>
-      <c r="B12" s="28" t="n"/>
-      <c r="C12" s="29" t="n"/>
-      <c r="D12" s="29" t="n"/>
-      <c r="E12" s="18">
+      <c r="A12" s="31" t="n"/>
+      <c r="B12" s="31" t="n"/>
+      <c r="C12" s="32" t="n"/>
+      <c r="D12" s="32" t="n"/>
+      <c r="E12" s="22">
         <f>IF(D12="","",D12*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F12" s="29" t="n"/>
+      <c r="F12" s="32" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="28" t="n"/>
-      <c r="B13" s="28" t="n"/>
-      <c r="C13" s="29" t="n"/>
-      <c r="D13" s="29" t="n"/>
-      <c r="E13" s="18">
+      <c r="A13" s="31" t="n"/>
+      <c r="B13" s="31" t="n"/>
+      <c r="C13" s="32" t="n"/>
+      <c r="D13" s="32" t="n"/>
+      <c r="E13" s="22">
         <f>IF(D13="","",D13*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F13" s="29" t="n"/>
+      <c r="F13" s="32" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="28" t="n"/>
-      <c r="B14" s="28" t="n"/>
-      <c r="C14" s="29" t="n"/>
-      <c r="D14" s="29" t="n"/>
-      <c r="E14" s="18">
+      <c r="A14" s="31" t="n"/>
+      <c r="B14" s="31" t="n"/>
+      <c r="C14" s="32" t="n"/>
+      <c r="D14" s="32" t="n"/>
+      <c r="E14" s="22">
         <f>IF(D14="","",D14*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F14" s="29" t="n"/>
+      <c r="F14" s="32" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="28" t="n"/>
-      <c r="B15" s="28" t="n"/>
-      <c r="C15" s="29" t="n"/>
-      <c r="D15" s="29" t="n"/>
-      <c r="E15" s="18">
+      <c r="A15" s="31" t="n"/>
+      <c r="B15" s="31" t="n"/>
+      <c r="C15" s="32" t="n"/>
+      <c r="D15" s="32" t="n"/>
+      <c r="E15" s="22">
         <f>IF(D15="","",D15*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F15" s="29" t="n"/>
+      <c r="F15" s="32" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="28" t="n"/>
-      <c r="B16" s="28" t="n"/>
-      <c r="C16" s="29" t="n"/>
-      <c r="D16" s="29" t="n"/>
-      <c r="E16" s="18">
+      <c r="A16" s="31" t="n"/>
+      <c r="B16" s="31" t="n"/>
+      <c r="C16" s="32" t="n"/>
+      <c r="D16" s="32" t="n"/>
+      <c r="E16" s="22">
         <f>IF(D16="","",D16*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F16" s="29" t="n"/>
+      <c r="F16" s="32" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="28" t="n"/>
-      <c r="B17" s="28" t="n"/>
-      <c r="C17" s="29" t="n"/>
-      <c r="D17" s="29" t="n"/>
-      <c r="E17" s="18">
+      <c r="A17" s="31" t="n"/>
+      <c r="B17" s="31" t="n"/>
+      <c r="C17" s="32" t="n"/>
+      <c r="D17" s="32" t="n"/>
+      <c r="E17" s="22">
         <f>IF(D17="","",D17*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F17" s="29" t="n"/>
+      <c r="F17" s="32" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="28" t="n"/>
-      <c r="B18" s="28" t="n"/>
-      <c r="C18" s="29" t="n"/>
-      <c r="D18" s="29" t="n"/>
-      <c r="E18" s="18">
+      <c r="A18" s="31" t="n"/>
+      <c r="B18" s="31" t="n"/>
+      <c r="C18" s="32" t="n"/>
+      <c r="D18" s="32" t="n"/>
+      <c r="E18" s="22">
         <f>IF(D18="","",D18*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F18" s="29" t="n"/>
+      <c r="F18" s="32" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="28" t="n"/>
-      <c r="B19" s="28" t="n"/>
-      <c r="C19" s="29" t="n"/>
-      <c r="D19" s="29" t="n"/>
-      <c r="E19" s="18">
+      <c r="A19" s="31" t="n"/>
+      <c r="B19" s="31" t="n"/>
+      <c r="C19" s="32" t="n"/>
+      <c r="D19" s="32" t="n"/>
+      <c r="E19" s="22">
         <f>IF(D19="","",D19*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F19" s="29" t="n"/>
+      <c r="F19" s="32" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="28" t="n"/>
-      <c r="B20" s="28" t="n"/>
-      <c r="C20" s="29" t="n"/>
-      <c r="D20" s="29" t="n"/>
-      <c r="E20" s="18">
+      <c r="A20" s="31" t="n"/>
+      <c r="B20" s="31" t="n"/>
+      <c r="C20" s="32" t="n"/>
+      <c r="D20" s="32" t="n"/>
+      <c r="E20" s="22">
         <f>IF(D20="","",D20*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F20" s="29" t="n"/>
+      <c r="F20" s="32" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="28" t="n"/>
-      <c r="B21" s="28" t="n"/>
-      <c r="C21" s="29" t="n"/>
-      <c r="D21" s="29" t="n"/>
-      <c r="E21" s="18">
+      <c r="A21" s="31" t="n"/>
+      <c r="B21" s="31" t="n"/>
+      <c r="C21" s="32" t="n"/>
+      <c r="D21" s="32" t="n"/>
+      <c r="E21" s="22">
         <f>IF(D21="","",D21*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F21" s="29" t="n"/>
+      <c r="F21" s="32" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="28" t="n"/>
-      <c r="B22" s="28" t="n"/>
-      <c r="C22" s="29" t="n"/>
-      <c r="D22" s="29" t="n"/>
-      <c r="E22" s="18">
+      <c r="A22" s="31" t="n"/>
+      <c r="B22" s="31" t="n"/>
+      <c r="C22" s="32" t="n"/>
+      <c r="D22" s="32" t="n"/>
+      <c r="E22" s="22">
         <f>IF(D22="","",D22*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F22" s="29" t="n"/>
+      <c r="F22" s="32" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="28" t="n"/>
-      <c r="B23" s="28" t="n"/>
-      <c r="C23" s="29" t="n"/>
-      <c r="D23" s="29" t="n"/>
-      <c r="E23" s="18">
+      <c r="A23" s="31" t="n"/>
+      <c r="B23" s="31" t="n"/>
+      <c r="C23" s="32" t="n"/>
+      <c r="D23" s="32" t="n"/>
+      <c r="E23" s="22">
         <f>IF(D23="","",D23*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F23" s="29" t="n"/>
+      <c r="F23" s="32" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="28" t="n"/>
-      <c r="B24" s="28" t="n"/>
-      <c r="C24" s="29" t="n"/>
-      <c r="D24" s="29" t="n"/>
-      <c r="E24" s="18">
+      <c r="A24" s="31" t="n"/>
+      <c r="B24" s="31" t="n"/>
+      <c r="C24" s="32" t="n"/>
+      <c r="D24" s="32" t="n"/>
+      <c r="E24" s="22">
         <f>IF(D24="","",D24*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F24" s="29" t="n"/>
+      <c r="F24" s="32" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="28" t="n"/>
-      <c r="B25" s="28" t="n"/>
-      <c r="C25" s="29" t="n"/>
-      <c r="D25" s="29" t="n"/>
-      <c r="E25" s="18">
+      <c r="A25" s="31" t="n"/>
+      <c r="B25" s="31" t="n"/>
+      <c r="C25" s="32" t="n"/>
+      <c r="D25" s="32" t="n"/>
+      <c r="E25" s="22">
         <f>IF(D25="","",D25*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F25" s="29" t="n"/>
+      <c r="F25" s="32" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="28" t="n"/>
-      <c r="B26" s="28" t="n"/>
-      <c r="C26" s="29" t="n"/>
-      <c r="D26" s="29" t="n"/>
-      <c r="E26" s="18">
+      <c r="A26" s="31" t="n"/>
+      <c r="B26" s="31" t="n"/>
+      <c r="C26" s="32" t="n"/>
+      <c r="D26" s="32" t="n"/>
+      <c r="E26" s="22">
         <f>IF(D26="","",D26*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F26" s="29" t="n"/>
+      <c r="F26" s="32" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="28" t="n"/>
-      <c r="B27" s="28" t="n"/>
-      <c r="C27" s="29" t="n"/>
-      <c r="D27" s="29" t="n"/>
-      <c r="E27" s="18">
+      <c r="A27" s="31" t="n"/>
+      <c r="B27" s="31" t="n"/>
+      <c r="C27" s="32" t="n"/>
+      <c r="D27" s="32" t="n"/>
+      <c r="E27" s="22">
         <f>IF(D27="","",D27*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F27" s="29" t="n"/>
+      <c r="F27" s="32" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="28" t="n"/>
-      <c r="B28" s="28" t="n"/>
-      <c r="C28" s="29" t="n"/>
-      <c r="D28" s="29" t="n"/>
-      <c r="E28" s="18">
+      <c r="A28" s="31" t="n"/>
+      <c r="B28" s="31" t="n"/>
+      <c r="C28" s="32" t="n"/>
+      <c r="D28" s="32" t="n"/>
+      <c r="E28" s="22">
         <f>IF(D28="","",D28*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F28" s="29" t="n"/>
+      <c r="F28" s="32" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="28" t="n"/>
-      <c r="B29" s="28" t="n"/>
-      <c r="C29" s="29" t="n"/>
-      <c r="D29" s="29" t="n"/>
-      <c r="E29" s="18">
+      <c r="A29" s="31" t="n"/>
+      <c r="B29" s="31" t="n"/>
+      <c r="C29" s="32" t="n"/>
+      <c r="D29" s="32" t="n"/>
+      <c r="E29" s="22">
         <f>IF(D29="","",D29*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F29" s="29" t="n"/>
+      <c r="F29" s="32" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="28" t="n"/>
-      <c r="B30" s="28" t="n"/>
-      <c r="C30" s="29" t="n"/>
-      <c r="D30" s="29" t="n"/>
-      <c r="E30" s="18">
+      <c r="A30" s="31" t="n"/>
+      <c r="B30" s="31" t="n"/>
+      <c r="C30" s="32" t="n"/>
+      <c r="D30" s="32" t="n"/>
+      <c r="E30" s="22">
         <f>IF(D30="","",D30*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F30" s="29" t="n"/>
+      <c r="F30" s="32" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="28" t="n"/>
-      <c r="B31" s="28" t="n"/>
-      <c r="C31" s="29" t="n"/>
-      <c r="D31" s="29" t="n"/>
-      <c r="E31" s="18">
+      <c r="A31" s="31" t="n"/>
+      <c r="B31" s="31" t="n"/>
+      <c r="C31" s="32" t="n"/>
+      <c r="D31" s="32" t="n"/>
+      <c r="E31" s="22">
         <f>IF(D31="","",D31*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F31" s="29" t="n"/>
+      <c r="F31" s="32" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="28" t="n"/>
-      <c r="B32" s="28" t="n"/>
-      <c r="C32" s="29" t="n"/>
-      <c r="D32" s="29" t="n"/>
-      <c r="E32" s="18">
+      <c r="A32" s="31" t="n"/>
+      <c r="B32" s="31" t="n"/>
+      <c r="C32" s="32" t="n"/>
+      <c r="D32" s="32" t="n"/>
+      <c r="E32" s="22">
         <f>IF(D32="","",D32*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F32" s="29" t="n"/>
+      <c r="F32" s="32" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="28" t="n"/>
-      <c r="B33" s="28" t="n"/>
-      <c r="C33" s="29" t="n"/>
-      <c r="D33" s="29" t="n"/>
-      <c r="E33" s="18">
+      <c r="A33" s="31" t="n"/>
+      <c r="B33" s="31" t="n"/>
+      <c r="C33" s="32" t="n"/>
+      <c r="D33" s="32" t="n"/>
+      <c r="E33" s="22">
         <f>IF(D33="","",D33*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F33" s="29" t="n"/>
+      <c r="F33" s="32" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="28" t="n"/>
-      <c r="B34" s="28" t="n"/>
-      <c r="C34" s="29" t="n"/>
-      <c r="D34" s="29" t="n"/>
-      <c r="E34" s="18">
+      <c r="A34" s="31" t="n"/>
+      <c r="B34" s="31" t="n"/>
+      <c r="C34" s="32" t="n"/>
+      <c r="D34" s="32" t="n"/>
+      <c r="E34" s="22">
         <f>IF(D34="","",D34*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F34" s="29" t="n"/>
+      <c r="F34" s="32" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="28" t="n"/>
-      <c r="B35" s="28" t="n"/>
-      <c r="C35" s="29" t="n"/>
-      <c r="D35" s="29" t="n"/>
-      <c r="E35" s="18">
+      <c r="A35" s="31" t="n"/>
+      <c r="B35" s="31" t="n"/>
+      <c r="C35" s="32" t="n"/>
+      <c r="D35" s="32" t="n"/>
+      <c r="E35" s="22">
         <f>IF(D35="","",D35*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F35" s="29" t="n"/>
+      <c r="F35" s="32" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="28" t="n"/>
-      <c r="B36" s="28" t="n"/>
-      <c r="C36" s="29" t="n"/>
-      <c r="D36" s="29" t="n"/>
-      <c r="E36" s="18">
+      <c r="A36" s="31" t="n"/>
+      <c r="B36" s="31" t="n"/>
+      <c r="C36" s="32" t="n"/>
+      <c r="D36" s="32" t="n"/>
+      <c r="E36" s="22">
         <f>IF(D36="","",D36*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F36" s="29" t="n"/>
+      <c r="F36" s="32" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="28" t="n"/>
-      <c r="B37" s="28" t="n"/>
-      <c r="C37" s="29" t="n"/>
-      <c r="D37" s="29" t="n"/>
-      <c r="E37" s="18">
+      <c r="A37" s="31" t="n"/>
+      <c r="B37" s="31" t="n"/>
+      <c r="C37" s="32" t="n"/>
+      <c r="D37" s="32" t="n"/>
+      <c r="E37" s="22">
         <f>IF(D37="","",D37*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F37" s="29" t="n"/>
+      <c r="F37" s="32" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="28" t="n"/>
-      <c r="B38" s="28" t="n"/>
-      <c r="C38" s="29" t="n"/>
-      <c r="D38" s="29" t="n"/>
-      <c r="E38" s="18">
+      <c r="A38" s="31" t="n"/>
+      <c r="B38" s="31" t="n"/>
+      <c r="C38" s="32" t="n"/>
+      <c r="D38" s="32" t="n"/>
+      <c r="E38" s="22">
         <f>IF(D38="","",D38*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F38" s="29" t="n"/>
+      <c r="F38" s="32" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="28" t="n"/>
-      <c r="B39" s="28" t="n"/>
-      <c r="C39" s="29" t="n"/>
-      <c r="D39" s="29" t="n"/>
-      <c r="E39" s="18">
+      <c r="A39" s="31" t="n"/>
+      <c r="B39" s="31" t="n"/>
+      <c r="C39" s="32" t="n"/>
+      <c r="D39" s="32" t="n"/>
+      <c r="E39" s="22">
         <f>IF(D39="","",D39*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F39" s="29" t="n"/>
+      <c r="F39" s="32" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="28" t="n"/>
-      <c r="B40" s="28" t="n"/>
-      <c r="C40" s="29" t="n"/>
-      <c r="D40" s="29" t="n"/>
-      <c r="E40" s="18">
+      <c r="A40" s="31" t="n"/>
+      <c r="B40" s="31" t="n"/>
+      <c r="C40" s="32" t="n"/>
+      <c r="D40" s="32" t="n"/>
+      <c r="E40" s="22">
         <f>IF(D40="","",D40*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F40" s="29" t="n"/>
+      <c r="F40" s="32" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="28" t="n"/>
-      <c r="B41" s="28" t="n"/>
-      <c r="C41" s="29" t="n"/>
-      <c r="D41" s="29" t="n"/>
-      <c r="E41" s="18">
+      <c r="A41" s="31" t="n"/>
+      <c r="B41" s="31" t="n"/>
+      <c r="C41" s="32" t="n"/>
+      <c r="D41" s="32" t="n"/>
+      <c r="E41" s="22">
         <f>IF(D41="","",D41*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F41" s="29" t="n"/>
+      <c r="F41" s="32" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="28" t="n"/>
-      <c r="B42" s="28" t="n"/>
-      <c r="C42" s="29" t="n"/>
-      <c r="D42" s="29" t="n"/>
-      <c r="E42" s="18">
+      <c r="A42" s="31" t="n"/>
+      <c r="B42" s="31" t="n"/>
+      <c r="C42" s="32" t="n"/>
+      <c r="D42" s="32" t="n"/>
+      <c r="E42" s="22">
         <f>IF(D42="","",D42*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F42" s="29" t="n"/>
+      <c r="F42" s="32" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="28" t="n"/>
-      <c r="B43" s="28" t="n"/>
-      <c r="C43" s="29" t="n"/>
-      <c r="D43" s="29" t="n"/>
-      <c r="E43" s="18">
+      <c r="A43" s="31" t="n"/>
+      <c r="B43" s="31" t="n"/>
+      <c r="C43" s="32" t="n"/>
+      <c r="D43" s="32" t="n"/>
+      <c r="E43" s="22">
         <f>IF(D43="","",D43*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F43" s="29" t="n"/>
+      <c r="F43" s="32" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="28" t="n"/>
-      <c r="B44" s="28" t="n"/>
-      <c r="C44" s="29" t="n"/>
-      <c r="D44" s="29" t="n"/>
-      <c r="E44" s="18">
+      <c r="A44" s="31" t="n"/>
+      <c r="B44" s="31" t="n"/>
+      <c r="C44" s="32" t="n"/>
+      <c r="D44" s="32" t="n"/>
+      <c r="E44" s="22">
         <f>IF(D44="","",D44*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F44" s="29" t="n"/>
+      <c r="F44" s="32" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="28" t="n"/>
-      <c r="B45" s="28" t="n"/>
-      <c r="C45" s="29" t="n"/>
-      <c r="D45" s="29" t="n"/>
-      <c r="E45" s="18">
+      <c r="A45" s="31" t="n"/>
+      <c r="B45" s="31" t="n"/>
+      <c r="C45" s="32" t="n"/>
+      <c r="D45" s="32" t="n"/>
+      <c r="E45" s="22">
         <f>IF(D45="","",D45*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F45" s="29" t="n"/>
+      <c r="F45" s="32" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="28" t="n"/>
-      <c r="B46" s="28" t="n"/>
-      <c r="C46" s="29" t="n"/>
-      <c r="D46" s="29" t="n"/>
-      <c r="E46" s="18">
+      <c r="A46" s="31" t="n"/>
+      <c r="B46" s="31" t="n"/>
+      <c r="C46" s="32" t="n"/>
+      <c r="D46" s="32" t="n"/>
+      <c r="E46" s="22">
         <f>IF(D46="","",D46*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F46" s="29" t="n"/>
+      <c r="F46" s="32" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="28" t="n"/>
-      <c r="B47" s="28" t="n"/>
-      <c r="C47" s="29" t="n"/>
-      <c r="D47" s="29" t="n"/>
-      <c r="E47" s="18">
+      <c r="A47" s="31" t="n"/>
+      <c r="B47" s="31" t="n"/>
+      <c r="C47" s="32" t="n"/>
+      <c r="D47" s="32" t="n"/>
+      <c r="E47" s="22">
         <f>IF(D47="","",D47*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F47" s="29" t="n"/>
+      <c r="F47" s="32" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="28" t="n"/>
-      <c r="B48" s="28" t="n"/>
-      <c r="C48" s="29" t="n"/>
-      <c r="D48" s="29" t="n"/>
-      <c r="E48" s="18">
+      <c r="A48" s="31" t="n"/>
+      <c r="B48" s="31" t="n"/>
+      <c r="C48" s="32" t="n"/>
+      <c r="D48" s="32" t="n"/>
+      <c r="E48" s="22">
         <f>IF(D48="","",D48*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F48" s="29" t="n"/>
+      <c r="F48" s="32" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="28" t="n"/>
-      <c r="B49" s="28" t="n"/>
-      <c r="C49" s="29" t="n"/>
-      <c r="D49" s="29" t="n"/>
-      <c r="E49" s="18">
+      <c r="A49" s="31" t="n"/>
+      <c r="B49" s="31" t="n"/>
+      <c r="C49" s="32" t="n"/>
+      <c r="D49" s="32" t="n"/>
+      <c r="E49" s="22">
         <f>IF(D49="","",D49*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F49" s="29" t="n"/>
+      <c r="F49" s="32" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="28" t="n"/>
-      <c r="B50" s="28" t="n"/>
-      <c r="C50" s="29" t="n"/>
-      <c r="D50" s="29" t="n"/>
-      <c r="E50" s="18">
+      <c r="A50" s="31" t="n"/>
+      <c r="B50" s="31" t="n"/>
+      <c r="C50" s="32" t="n"/>
+      <c r="D50" s="32" t="n"/>
+      <c r="E50" s="22">
         <f>IF(D50="","",D50*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F50" s="29" t="n"/>
+      <c r="F50" s="32" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="28" t="n"/>
-      <c r="B51" s="28" t="n"/>
-      <c r="C51" s="29" t="n"/>
-      <c r="D51" s="29" t="n"/>
-      <c r="E51" s="18">
+      <c r="A51" s="31" t="n"/>
+      <c r="B51" s="31" t="n"/>
+      <c r="C51" s="32" t="n"/>
+      <c r="D51" s="32" t="n"/>
+      <c r="E51" s="22">
         <f>IF(D51="","",D51*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F51" s="29" t="n"/>
+      <c r="F51" s="32" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="28" t="n"/>
-      <c r="B52" s="28" t="n"/>
-      <c r="C52" s="29" t="n"/>
-      <c r="D52" s="29" t="n"/>
-      <c r="E52" s="18">
+      <c r="A52" s="31" t="n"/>
+      <c r="B52" s="31" t="n"/>
+      <c r="C52" s="32" t="n"/>
+      <c r="D52" s="32" t="n"/>
+      <c r="E52" s="22">
         <f>IF(D52="","",D52*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F52" s="29" t="n"/>
+      <c r="F52" s="32" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="28" t="n"/>
-      <c r="B53" s="28" t="n"/>
-      <c r="C53" s="29" t="n"/>
-      <c r="D53" s="29" t="n"/>
-      <c r="E53" s="18">
+      <c r="A53" s="31" t="n"/>
+      <c r="B53" s="31" t="n"/>
+      <c r="C53" s="32" t="n"/>
+      <c r="D53" s="32" t="n"/>
+      <c r="E53" s="22">
         <f>IF(D53="","",D53*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F53" s="29" t="n"/>
+      <c r="F53" s="32" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="28" t="n"/>
-      <c r="B54" s="28" t="n"/>
-      <c r="C54" s="29" t="n"/>
-      <c r="D54" s="29" t="n"/>
-      <c r="E54" s="18">
+      <c r="A54" s="31" t="n"/>
+      <c r="B54" s="31" t="n"/>
+      <c r="C54" s="32" t="n"/>
+      <c r="D54" s="32" t="n"/>
+      <c r="E54" s="22">
         <f>IF(D54="","",D54*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F54" s="29" t="n"/>
+      <c r="F54" s="32" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="28" t="n"/>
-      <c r="B55" s="28" t="n"/>
-      <c r="C55" s="29" t="n"/>
-      <c r="D55" s="29" t="n"/>
-      <c r="E55" s="18">
+      <c r="A55" s="31" t="n"/>
+      <c r="B55" s="31" t="n"/>
+      <c r="C55" s="32" t="n"/>
+      <c r="D55" s="32" t="n"/>
+      <c r="E55" s="22">
         <f>IF(D55="","",D55*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F55" s="29" t="n"/>
+      <c r="F55" s="32" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="28" t="n"/>
-      <c r="B56" s="28" t="n"/>
-      <c r="C56" s="29" t="n"/>
-      <c r="D56" s="29" t="n"/>
-      <c r="E56" s="18">
+      <c r="A56" s="31" t="n"/>
+      <c r="B56" s="31" t="n"/>
+      <c r="C56" s="32" t="n"/>
+      <c r="D56" s="32" t="n"/>
+      <c r="E56" s="22">
         <f>IF(D56="","",D56*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F56" s="29" t="n"/>
+      <c r="F56" s="32" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="28" t="n"/>
-      <c r="B57" s="28" t="n"/>
-      <c r="C57" s="29" t="n"/>
-      <c r="D57" s="29" t="n"/>
-      <c r="E57" s="18">
+      <c r="A57" s="31" t="n"/>
+      <c r="B57" s="31" t="n"/>
+      <c r="C57" s="32" t="n"/>
+      <c r="D57" s="32" t="n"/>
+      <c r="E57" s="22">
         <f>IF(D57="","",D57*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F57" s="29" t="n"/>
+      <c r="F57" s="32" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="28" t="n"/>
-      <c r="B58" s="28" t="n"/>
-      <c r="C58" s="29" t="n"/>
-      <c r="D58" s="29" t="n"/>
-      <c r="E58" s="18">
+      <c r="A58" s="31" t="n"/>
+      <c r="B58" s="31" t="n"/>
+      <c r="C58" s="32" t="n"/>
+      <c r="D58" s="32" t="n"/>
+      <c r="E58" s="22">
         <f>IF(D58="","",D58*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F58" s="29" t="n"/>
+      <c r="F58" s="32" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="28" t="n"/>
-      <c r="B59" s="28" t="n"/>
-      <c r="C59" s="29" t="n"/>
-      <c r="D59" s="29" t="n"/>
-      <c r="E59" s="18">
+      <c r="A59" s="31" t="n"/>
+      <c r="B59" s="31" t="n"/>
+      <c r="C59" s="32" t="n"/>
+      <c r="D59" s="32" t="n"/>
+      <c r="E59" s="22">
         <f>IF(D59="","",D59*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F59" s="29" t="n"/>
+      <c r="F59" s="32" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="28" t="n"/>
-      <c r="B60" s="28" t="n"/>
-      <c r="C60" s="29" t="n"/>
-      <c r="D60" s="29" t="n"/>
-      <c r="E60" s="18">
+      <c r="A60" s="31" t="n"/>
+      <c r="B60" s="31" t="n"/>
+      <c r="C60" s="32" t="n"/>
+      <c r="D60" s="32" t="n"/>
+      <c r="E60" s="22">
         <f>IF(D60="","",D60*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F60" s="29" t="n"/>
+      <c r="F60" s="32" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="28" t="n"/>
-      <c r="B61" s="28" t="n"/>
-      <c r="C61" s="29" t="n"/>
-      <c r="D61" s="29" t="n"/>
-      <c r="E61" s="18">
+      <c r="A61" s="31" t="n"/>
+      <c r="B61" s="31" t="n"/>
+      <c r="C61" s="32" t="n"/>
+      <c r="D61" s="32" t="n"/>
+      <c r="E61" s="22">
         <f>IF(D61="","",D61*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F61" s="29" t="n"/>
+      <c r="F61" s="32" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="28" t="n"/>
-      <c r="B62" s="28" t="n"/>
-      <c r="C62" s="29" t="n"/>
-      <c r="D62" s="29" t="n"/>
-      <c r="E62" s="18">
+      <c r="A62" s="31" t="n"/>
+      <c r="B62" s="31" t="n"/>
+      <c r="C62" s="32" t="n"/>
+      <c r="D62" s="32" t="n"/>
+      <c r="E62" s="22">
         <f>IF(D62="","",D62*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F62" s="29" t="n"/>
+      <c r="F62" s="32" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="28" t="n"/>
-      <c r="B63" s="28" t="n"/>
-      <c r="C63" s="29" t="n"/>
-      <c r="D63" s="29" t="n"/>
-      <c r="E63" s="18">
+      <c r="A63" s="31" t="n"/>
+      <c r="B63" s="31" t="n"/>
+      <c r="C63" s="32" t="n"/>
+      <c r="D63" s="32" t="n"/>
+      <c r="E63" s="22">
         <f>IF(D63="","",D63*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F63" s="29" t="n"/>
+      <c r="F63" s="32" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="28" t="n"/>
-      <c r="B64" s="28" t="n"/>
-      <c r="C64" s="29" t="n"/>
-      <c r="D64" s="29" t="n"/>
-      <c r="E64" s="18">
+      <c r="A64" s="31" t="n"/>
+      <c r="B64" s="31" t="n"/>
+      <c r="C64" s="32" t="n"/>
+      <c r="D64" s="32" t="n"/>
+      <c r="E64" s="22">
         <f>IF(D64="","",D64*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F64" s="29" t="n"/>
+      <c r="F64" s="32" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="28" t="n"/>
-      <c r="B65" s="28" t="n"/>
-      <c r="C65" s="29" t="n"/>
-      <c r="D65" s="29" t="n"/>
-      <c r="E65" s="18">
+      <c r="A65" s="31" t="n"/>
+      <c r="B65" s="31" t="n"/>
+      <c r="C65" s="32" t="n"/>
+      <c r="D65" s="32" t="n"/>
+      <c r="E65" s="22">
         <f>IF(D65="","",D65*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F65" s="29" t="n"/>
+      <c r="F65" s="32" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="28" t="n"/>
-      <c r="B66" s="28" t="n"/>
-      <c r="C66" s="29" t="n"/>
-      <c r="D66" s="29" t="n"/>
-      <c r="E66" s="18">
+      <c r="A66" s="31" t="n"/>
+      <c r="B66" s="31" t="n"/>
+      <c r="C66" s="32" t="n"/>
+      <c r="D66" s="32" t="n"/>
+      <c r="E66" s="22">
         <f>IF(D66="","",D66*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F66" s="29" t="n"/>
+      <c r="F66" s="32" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="28" t="n"/>
-      <c r="B67" s="28" t="n"/>
-      <c r="C67" s="29" t="n"/>
-      <c r="D67" s="29" t="n"/>
-      <c r="E67" s="18">
+      <c r="A67" s="31" t="n"/>
+      <c r="B67" s="31" t="n"/>
+      <c r="C67" s="32" t="n"/>
+      <c r="D67" s="32" t="n"/>
+      <c r="E67" s="22">
         <f>IF(D67="","",D67*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F67" s="29" t="n"/>
+      <c r="F67" s="32" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="28" t="n"/>
-      <c r="B68" s="28" t="n"/>
-      <c r="C68" s="29" t="n"/>
-      <c r="D68" s="29" t="n"/>
-      <c r="E68" s="18">
+      <c r="A68" s="31" t="n"/>
+      <c r="B68" s="31" t="n"/>
+      <c r="C68" s="32" t="n"/>
+      <c r="D68" s="32" t="n"/>
+      <c r="E68" s="22">
         <f>IF(D68="","",D68*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F68" s="29" t="n"/>
+      <c r="F68" s="32" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="28" t="n"/>
-      <c r="B69" s="28" t="n"/>
-      <c r="C69" s="29" t="n"/>
-      <c r="D69" s="29" t="n"/>
-      <c r="E69" s="18">
+      <c r="A69" s="31" t="n"/>
+      <c r="B69" s="31" t="n"/>
+      <c r="C69" s="32" t="n"/>
+      <c r="D69" s="32" t="n"/>
+      <c r="E69" s="22">
         <f>IF(D69="","",D69*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F69" s="29" t="n"/>
+      <c r="F69" s="32" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="28" t="n"/>
-      <c r="B70" s="28" t="n"/>
-      <c r="C70" s="29" t="n"/>
-      <c r="D70" s="29" t="n"/>
-      <c r="E70" s="18">
+      <c r="A70" s="31" t="n"/>
+      <c r="B70" s="31" t="n"/>
+      <c r="C70" s="32" t="n"/>
+      <c r="D70" s="32" t="n"/>
+      <c r="E70" s="22">
         <f>IF(D70="","",D70*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F70" s="29" t="n"/>
+      <c r="F70" s="32" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="28" t="n"/>
-      <c r="B71" s="28" t="n"/>
-      <c r="C71" s="29" t="n"/>
-      <c r="D71" s="29" t="n"/>
-      <c r="E71" s="18">
+      <c r="A71" s="31" t="n"/>
+      <c r="B71" s="31" t="n"/>
+      <c r="C71" s="32" t="n"/>
+      <c r="D71" s="32" t="n"/>
+      <c r="E71" s="22">
         <f>IF(D71="","",D71*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F71" s="29" t="n"/>
+      <c r="F71" s="32" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="28" t="n"/>
-      <c r="B72" s="28" t="n"/>
-      <c r="C72" s="29" t="n"/>
-      <c r="D72" s="29" t="n"/>
-      <c r="E72" s="18">
+      <c r="A72" s="31" t="n"/>
+      <c r="B72" s="31" t="n"/>
+      <c r="C72" s="32" t="n"/>
+      <c r="D72" s="32" t="n"/>
+      <c r="E72" s="22">
         <f>IF(D72="","",D72*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F72" s="29" t="n"/>
+      <c r="F72" s="32" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="28" t="n"/>
-      <c r="B73" s="28" t="n"/>
-      <c r="C73" s="29" t="n"/>
-      <c r="D73" s="29" t="n"/>
-      <c r="E73" s="18">
+      <c r="A73" s="31" t="n"/>
+      <c r="B73" s="31" t="n"/>
+      <c r="C73" s="32" t="n"/>
+      <c r="D73" s="32" t="n"/>
+      <c r="E73" s="22">
         <f>IF(D73="","",D73*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F73" s="29" t="n"/>
+      <c r="F73" s="32" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="28" t="n"/>
-      <c r="B74" s="28" t="n"/>
-      <c r="C74" s="29" t="n"/>
-      <c r="D74" s="29" t="n"/>
-      <c r="E74" s="18">
+      <c r="A74" s="31" t="n"/>
+      <c r="B74" s="31" t="n"/>
+      <c r="C74" s="32" t="n"/>
+      <c r="D74" s="32" t="n"/>
+      <c r="E74" s="22">
         <f>IF(D74="","",D74*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F74" s="29" t="n"/>
+      <c r="F74" s="32" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="28" t="n"/>
-      <c r="B75" s="28" t="n"/>
-      <c r="C75" s="29" t="n"/>
-      <c r="D75" s="29" t="n"/>
-      <c r="E75" s="18">
+      <c r="A75" s="31" t="n"/>
+      <c r="B75" s="31" t="n"/>
+      <c r="C75" s="32" t="n"/>
+      <c r="D75" s="32" t="n"/>
+      <c r="E75" s="22">
         <f>IF(D75="","",D75*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F75" s="29" t="n"/>
+      <c r="F75" s="32" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="28" t="n"/>
-      <c r="B76" s="28" t="n"/>
-      <c r="C76" s="29" t="n"/>
-      <c r="D76" s="29" t="n"/>
-      <c r="E76" s="18">
+      <c r="A76" s="31" t="n"/>
+      <c r="B76" s="31" t="n"/>
+      <c r="C76" s="32" t="n"/>
+      <c r="D76" s="32" t="n"/>
+      <c r="E76" s="22">
         <f>IF(D76="","",D76*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F76" s="29" t="n"/>
+      <c r="F76" s="32" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="28" t="n"/>
-      <c r="B77" s="28" t="n"/>
-      <c r="C77" s="29" t="n"/>
-      <c r="D77" s="29" t="n"/>
-      <c r="E77" s="18">
+      <c r="A77" s="31" t="n"/>
+      <c r="B77" s="31" t="n"/>
+      <c r="C77" s="32" t="n"/>
+      <c r="D77" s="32" t="n"/>
+      <c r="E77" s="22">
         <f>IF(D77="","",D77*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F77" s="29" t="n"/>
+      <c r="F77" s="32" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="28" t="n"/>
-      <c r="B78" s="28" t="n"/>
-      <c r="C78" s="29" t="n"/>
-      <c r="D78" s="29" t="n"/>
-      <c r="E78" s="18">
+      <c r="A78" s="31" t="n"/>
+      <c r="B78" s="31" t="n"/>
+      <c r="C78" s="32" t="n"/>
+      <c r="D78" s="32" t="n"/>
+      <c r="E78" s="22">
         <f>IF(D78="","",D78*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F78" s="29" t="n"/>
+      <c r="F78" s="32" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="28" t="n"/>
-      <c r="B79" s="28" t="n"/>
-      <c r="C79" s="29" t="n"/>
-      <c r="D79" s="29" t="n"/>
-      <c r="E79" s="18">
+      <c r="A79" s="31" t="n"/>
+      <c r="B79" s="31" t="n"/>
+      <c r="C79" s="32" t="n"/>
+      <c r="D79" s="32" t="n"/>
+      <c r="E79" s="22">
         <f>IF(D79="","",D79*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F79" s="29" t="n"/>
+      <c r="F79" s="32" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="28" t="n"/>
-      <c r="B80" s="28" t="n"/>
-      <c r="C80" s="29" t="n"/>
-      <c r="D80" s="29" t="n"/>
-      <c r="E80" s="18">
+      <c r="A80" s="31" t="n"/>
+      <c r="B80" s="31" t="n"/>
+      <c r="C80" s="32" t="n"/>
+      <c r="D80" s="32" t="n"/>
+      <c r="E80" s="22">
         <f>IF(D80="","",D80*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F80" s="29" t="n"/>
+      <c r="F80" s="32" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="28" t="n"/>
-      <c r="B81" s="28" t="n"/>
-      <c r="C81" s="29" t="n"/>
-      <c r="D81" s="29" t="n"/>
-      <c r="E81" s="18">
+      <c r="A81" s="31" t="n"/>
+      <c r="B81" s="31" t="n"/>
+      <c r="C81" s="32" t="n"/>
+      <c r="D81" s="32" t="n"/>
+      <c r="E81" s="22">
         <f>IF(D81="","",D81*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F81" s="29" t="n"/>
+      <c r="F81" s="32" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="28" t="n"/>
-      <c r="B82" s="28" t="n"/>
-      <c r="C82" s="29" t="n"/>
-      <c r="D82" s="29" t="n"/>
-      <c r="E82" s="18">
+      <c r="A82" s="31" t="n"/>
+      <c r="B82" s="31" t="n"/>
+      <c r="C82" s="32" t="n"/>
+      <c r="D82" s="32" t="n"/>
+      <c r="E82" s="22">
         <f>IF(D82="","",D82*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F82" s="29" t="n"/>
+      <c r="F82" s="32" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="28" t="n"/>
-      <c r="B83" s="28" t="n"/>
-      <c r="C83" s="29" t="n"/>
-      <c r="D83" s="29" t="n"/>
-      <c r="E83" s="18">
+      <c r="A83" s="31" t="n"/>
+      <c r="B83" s="31" t="n"/>
+      <c r="C83" s="32" t="n"/>
+      <c r="D83" s="32" t="n"/>
+      <c r="E83" s="22">
         <f>IF(D83="","",D83*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F83" s="29" t="n"/>
+      <c r="F83" s="32" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="28" t="n"/>
-      <c r="B84" s="28" t="n"/>
-      <c r="C84" s="29" t="n"/>
-      <c r="D84" s="29" t="n"/>
-      <c r="E84" s="18">
+      <c r="A84" s="31" t="n"/>
+      <c r="B84" s="31" t="n"/>
+      <c r="C84" s="32" t="n"/>
+      <c r="D84" s="32" t="n"/>
+      <c r="E84" s="22">
         <f>IF(D84="","",D84*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F84" s="29" t="n"/>
+      <c r="F84" s="32" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="28" t="n"/>
-      <c r="B85" s="28" t="n"/>
-      <c r="C85" s="29" t="n"/>
-      <c r="D85" s="29" t="n"/>
-      <c r="E85" s="18">
+      <c r="A85" s="31" t="n"/>
+      <c r="B85" s="31" t="n"/>
+      <c r="C85" s="32" t="n"/>
+      <c r="D85" s="32" t="n"/>
+      <c r="E85" s="22">
         <f>IF(D85="","",D85*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F85" s="29" t="n"/>
+      <c r="F85" s="32" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="28" t="n"/>
-      <c r="B86" s="28" t="n"/>
-      <c r="C86" s="29" t="n"/>
-      <c r="D86" s="29" t="n"/>
-      <c r="E86" s="18">
+      <c r="A86" s="31" t="n"/>
+      <c r="B86" s="31" t="n"/>
+      <c r="C86" s="32" t="n"/>
+      <c r="D86" s="32" t="n"/>
+      <c r="E86" s="22">
         <f>IF(D86="","",D86*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F86" s="29" t="n"/>
+      <c r="F86" s="32" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="28" t="n"/>
-      <c r="B87" s="28" t="n"/>
-      <c r="C87" s="29" t="n"/>
-      <c r="D87" s="29" t="n"/>
-      <c r="E87" s="18">
+      <c r="A87" s="31" t="n"/>
+      <c r="B87" s="31" t="n"/>
+      <c r="C87" s="32" t="n"/>
+      <c r="D87" s="32" t="n"/>
+      <c r="E87" s="22">
         <f>IF(D87="","",D87*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F87" s="29" t="n"/>
+      <c r="F87" s="32" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="28" t="n"/>
-      <c r="B88" s="28" t="n"/>
-      <c r="C88" s="29" t="n"/>
-      <c r="D88" s="29" t="n"/>
-      <c r="E88" s="18">
+      <c r="A88" s="31" t="n"/>
+      <c r="B88" s="31" t="n"/>
+      <c r="C88" s="32" t="n"/>
+      <c r="D88" s="32" t="n"/>
+      <c r="E88" s="22">
         <f>IF(D88="","",D88*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F88" s="29" t="n"/>
+      <c r="F88" s="32" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="28" t="n"/>
-      <c r="B89" s="28" t="n"/>
-      <c r="C89" s="29" t="n"/>
-      <c r="D89" s="29" t="n"/>
-      <c r="E89" s="18">
+      <c r="A89" s="31" t="n"/>
+      <c r="B89" s="31" t="n"/>
+      <c r="C89" s="32" t="n"/>
+      <c r="D89" s="32" t="n"/>
+      <c r="E89" s="22">
         <f>IF(D89="","",D89*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F89" s="29" t="n"/>
+      <c r="F89" s="32" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="28" t="n"/>
-      <c r="B90" s="28" t="n"/>
-      <c r="C90" s="29" t="n"/>
-      <c r="D90" s="29" t="n"/>
-      <c r="E90" s="18">
+      <c r="A90" s="31" t="n"/>
+      <c r="B90" s="31" t="n"/>
+      <c r="C90" s="32" t="n"/>
+      <c r="D90" s="32" t="n"/>
+      <c r="E90" s="22">
         <f>IF(D90="","",D90*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F90" s="29" t="n"/>
+      <c r="F90" s="32" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="28" t="n"/>
-      <c r="B91" s="28" t="n"/>
-      <c r="C91" s="29" t="n"/>
-      <c r="D91" s="29" t="n"/>
-      <c r="E91" s="18">
+      <c r="A91" s="31" t="n"/>
+      <c r="B91" s="31" t="n"/>
+      <c r="C91" s="32" t="n"/>
+      <c r="D91" s="32" t="n"/>
+      <c r="E91" s="22">
         <f>IF(D91="","",D91*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F91" s="29" t="n"/>
+      <c r="F91" s="32" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="28" t="n"/>
-      <c r="B92" s="28" t="n"/>
-      <c r="C92" s="29" t="n"/>
-      <c r="D92" s="29" t="n"/>
-      <c r="E92" s="18">
+      <c r="A92" s="31" t="n"/>
+      <c r="B92" s="31" t="n"/>
+      <c r="C92" s="32" t="n"/>
+      <c r="D92" s="32" t="n"/>
+      <c r="E92" s="22">
         <f>IF(D92="","",D92*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F92" s="29" t="n"/>
+      <c r="F92" s="32" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="28" t="n"/>
-      <c r="B93" s="28" t="n"/>
-      <c r="C93" s="29" t="n"/>
-      <c r="D93" s="29" t="n"/>
-      <c r="E93" s="18">
+      <c r="A93" s="31" t="n"/>
+      <c r="B93" s="31" t="n"/>
+      <c r="C93" s="32" t="n"/>
+      <c r="D93" s="32" t="n"/>
+      <c r="E93" s="22">
         <f>IF(D93="","",D93*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F93" s="29" t="n"/>
+      <c r="F93" s="32" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="28" t="n"/>
-      <c r="B94" s="28" t="n"/>
-      <c r="C94" s="29" t="n"/>
-      <c r="D94" s="29" t="n"/>
-      <c r="E94" s="18">
+      <c r="A94" s="31" t="n"/>
+      <c r="B94" s="31" t="n"/>
+      <c r="C94" s="32" t="n"/>
+      <c r="D94" s="32" t="n"/>
+      <c r="E94" s="22">
         <f>IF(D94="","",D94*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F94" s="29" t="n"/>
+      <c r="F94" s="32" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="28" t="n"/>
-      <c r="B95" s="28" t="n"/>
-      <c r="C95" s="29" t="n"/>
-      <c r="D95" s="29" t="n"/>
-      <c r="E95" s="18">
+      <c r="A95" s="31" t="n"/>
+      <c r="B95" s="31" t="n"/>
+      <c r="C95" s="32" t="n"/>
+      <c r="D95" s="32" t="n"/>
+      <c r="E95" s="22">
         <f>IF(D95="","",D95*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F95" s="29" t="n"/>
+      <c r="F95" s="32" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="28" t="n"/>
-      <c r="B96" s="28" t="n"/>
-      <c r="C96" s="29" t="n"/>
-      <c r="D96" s="29" t="n"/>
-      <c r="E96" s="18">
+      <c r="A96" s="31" t="n"/>
+      <c r="B96" s="31" t="n"/>
+      <c r="C96" s="32" t="n"/>
+      <c r="D96" s="32" t="n"/>
+      <c r="E96" s="22">
         <f>IF(D96="","",D96*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F96" s="29" t="n"/>
+      <c r="F96" s="32" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="28" t="n"/>
-      <c r="B97" s="28" t="n"/>
-      <c r="C97" s="29" t="n"/>
-      <c r="D97" s="29" t="n"/>
-      <c r="E97" s="18">
+      <c r="A97" s="31" t="n"/>
+      <c r="B97" s="31" t="n"/>
+      <c r="C97" s="32" t="n"/>
+      <c r="D97" s="32" t="n"/>
+      <c r="E97" s="22">
         <f>IF(D97="","",D97*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F97" s="29" t="n"/>
+      <c r="F97" s="32" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="28" t="n"/>
-      <c r="B98" s="28" t="n"/>
-      <c r="C98" s="29" t="n"/>
-      <c r="D98" s="29" t="n"/>
-      <c r="E98" s="18">
+      <c r="A98" s="31" t="n"/>
+      <c r="B98" s="31" t="n"/>
+      <c r="C98" s="32" t="n"/>
+      <c r="D98" s="32" t="n"/>
+      <c r="E98" s="22">
         <f>IF(D98="","",D98*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F98" s="29" t="n"/>
+      <c r="F98" s="32" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="28" t="n"/>
-      <c r="B99" s="28" t="n"/>
-      <c r="C99" s="29" t="n"/>
-      <c r="D99" s="29" t="n"/>
-      <c r="E99" s="18">
+      <c r="A99" s="31" t="n"/>
+      <c r="B99" s="31" t="n"/>
+      <c r="C99" s="32" t="n"/>
+      <c r="D99" s="32" t="n"/>
+      <c r="E99" s="22">
         <f>IF(D99="","",D99*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F99" s="29" t="n"/>
+      <c r="F99" s="32" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="28" t="n"/>
-      <c r="B100" s="28" t="n"/>
-      <c r="C100" s="29" t="n"/>
-      <c r="D100" s="29" t="n"/>
-      <c r="E100" s="18">
+      <c r="A100" s="31" t="n"/>
+      <c r="B100" s="31" t="n"/>
+      <c r="C100" s="32" t="n"/>
+      <c r="D100" s="32" t="n"/>
+      <c r="E100" s="22">
         <f>IF(D100="","",D100*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F100" s="29" t="n"/>
+      <c r="F100" s="32" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="28" t="n"/>
-      <c r="B101" s="28" t="n"/>
-      <c r="C101" s="29" t="n"/>
-      <c r="D101" s="29" t="n"/>
-      <c r="E101" s="18">
+      <c r="A101" s="31" t="n"/>
+      <c r="B101" s="31" t="n"/>
+      <c r="C101" s="32" t="n"/>
+      <c r="D101" s="32" t="n"/>
+      <c r="E101" s="22">
         <f>IF(D101="","",D101*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F101" s="29" t="n"/>
+      <c r="F101" s="32" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="28" t="n"/>
-      <c r="B102" s="28" t="n"/>
-      <c r="C102" s="29" t="n"/>
-      <c r="D102" s="29" t="n"/>
-      <c r="E102" s="18">
+      <c r="A102" s="31" t="n"/>
+      <c r="B102" s="31" t="n"/>
+      <c r="C102" s="32" t="n"/>
+      <c r="D102" s="32" t="n"/>
+      <c r="E102" s="22">
         <f>IF(D102="","",D102*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F102" s="29" t="n"/>
+      <c r="F102" s="32" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="28" t="n"/>
-      <c r="B103" s="28" t="n"/>
-      <c r="C103" s="29" t="n"/>
-      <c r="D103" s="29" t="n"/>
-      <c r="E103" s="18">
+      <c r="A103" s="31" t="n"/>
+      <c r="B103" s="31" t="n"/>
+      <c r="C103" s="32" t="n"/>
+      <c r="D103" s="32" t="n"/>
+      <c r="E103" s="22">
         <f>IF(D103="","",D103*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F103" s="29" t="n"/>
+      <c r="F103" s="32" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="28" t="n"/>
-      <c r="B104" s="28" t="n"/>
-      <c r="C104" s="29" t="n"/>
-      <c r="D104" s="29" t="n"/>
-      <c r="E104" s="18">
+      <c r="A104" s="31" t="n"/>
+      <c r="B104" s="31" t="n"/>
+      <c r="C104" s="32" t="n"/>
+      <c r="D104" s="32" t="n"/>
+      <c r="E104" s="22">
         <f>IF(D104="","",D104*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F104" s="29" t="n"/>
+      <c r="F104" s="32" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="28" t="n"/>
-      <c r="B105" s="28" t="n"/>
-      <c r="C105" s="29" t="n"/>
-      <c r="D105" s="29" t="n"/>
-      <c r="E105" s="18">
+      <c r="A105" s="31" t="n"/>
+      <c r="B105" s="31" t="n"/>
+      <c r="C105" s="32" t="n"/>
+      <c r="D105" s="32" t="n"/>
+      <c r="E105" s="22">
         <f>IF(D105="","",D105*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F105" s="29" t="n"/>
+      <c r="F105" s="32" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="28" t="n"/>
-      <c r="B106" s="28" t="n"/>
-      <c r="C106" s="29" t="n"/>
-      <c r="D106" s="29" t="n"/>
-      <c r="E106" s="18">
+      <c r="A106" s="31" t="n"/>
+      <c r="B106" s="31" t="n"/>
+      <c r="C106" s="32" t="n"/>
+      <c r="D106" s="32" t="n"/>
+      <c r="E106" s="22">
         <f>IF(D106="","",D106*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F106" s="29" t="n"/>
+      <c r="F106" s="32" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="28" t="n"/>
-      <c r="B107" s="28" t="n"/>
-      <c r="C107" s="29" t="n"/>
-      <c r="D107" s="29" t="n"/>
-      <c r="E107" s="18">
+      <c r="A107" s="31" t="n"/>
+      <c r="B107" s="31" t="n"/>
+      <c r="C107" s="32" t="n"/>
+      <c r="D107" s="32" t="n"/>
+      <c r="E107" s="22">
         <f>IF(D107="","",D107*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F107" s="29" t="n"/>
+      <c r="F107" s="32" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="28" t="n"/>
-      <c r="B108" s="28" t="n"/>
-      <c r="C108" s="29" t="n"/>
-      <c r="D108" s="29" t="n"/>
-      <c r="E108" s="18">
+      <c r="A108" s="31" t="n"/>
+      <c r="B108" s="31" t="n"/>
+      <c r="C108" s="32" t="n"/>
+      <c r="D108" s="32" t="n"/>
+      <c r="E108" s="22">
         <f>IF(D108="","",D108*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F108" s="29" t="n"/>
+      <c r="F108" s="32" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="28" t="n"/>
-      <c r="B109" s="28" t="n"/>
-      <c r="C109" s="29" t="n"/>
-      <c r="D109" s="29" t="n"/>
-      <c r="E109" s="18">
+      <c r="A109" s="31" t="n"/>
+      <c r="B109" s="31" t="n"/>
+      <c r="C109" s="32" t="n"/>
+      <c r="D109" s="32" t="n"/>
+      <c r="E109" s="22">
         <f>IF(D109="","",D109*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F109" s="29" t="n"/>
+      <c r="F109" s="32" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="28" t="n"/>
-      <c r="B110" s="28" t="n"/>
-      <c r="C110" s="29" t="n"/>
-      <c r="D110" s="29" t="n"/>
-      <c r="E110" s="18">
+      <c r="A110" s="31" t="n"/>
+      <c r="B110" s="31" t="n"/>
+      <c r="C110" s="32" t="n"/>
+      <c r="D110" s="32" t="n"/>
+      <c r="E110" s="22">
         <f>IF(D110="","",D110*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F110" s="29" t="n"/>
+      <c r="F110" s="32" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="28" t="n"/>
-      <c r="B111" s="28" t="n"/>
-      <c r="C111" s="29" t="n"/>
-      <c r="D111" s="29" t="n"/>
-      <c r="E111" s="18">
+      <c r="A111" s="31" t="n"/>
+      <c r="B111" s="31" t="n"/>
+      <c r="C111" s="32" t="n"/>
+      <c r="D111" s="32" t="n"/>
+      <c r="E111" s="22">
         <f>IF(D111="","",D111*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F111" s="29" t="n"/>
+      <c r="F111" s="32" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="28" t="n"/>
-      <c r="B112" s="28" t="n"/>
-      <c r="C112" s="29" t="n"/>
-      <c r="D112" s="29" t="n"/>
-      <c r="E112" s="18">
+      <c r="A112" s="31" t="n"/>
+      <c r="B112" s="31" t="n"/>
+      <c r="C112" s="32" t="n"/>
+      <c r="D112" s="32" t="n"/>
+      <c r="E112" s="22">
         <f>IF(D112="","",D112*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F112" s="29" t="n"/>
+      <c r="F112" s="32" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="28" t="n"/>
-      <c r="B113" s="28" t="n"/>
-      <c r="C113" s="29" t="n"/>
-      <c r="D113" s="29" t="n"/>
-      <c r="E113" s="18">
+      <c r="A113" s="31" t="n"/>
+      <c r="B113" s="31" t="n"/>
+      <c r="C113" s="32" t="n"/>
+      <c r="D113" s="32" t="n"/>
+      <c r="E113" s="22">
         <f>IF(D113="","",D113*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F113" s="29" t="n"/>
+      <c r="F113" s="32" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="28" t="n"/>
-      <c r="B114" s="28" t="n"/>
-      <c r="C114" s="29" t="n"/>
-      <c r="D114" s="29" t="n"/>
-      <c r="E114" s="18">
+      <c r="A114" s="31" t="n"/>
+      <c r="B114" s="31" t="n"/>
+      <c r="C114" s="32" t="n"/>
+      <c r="D114" s="32" t="n"/>
+      <c r="E114" s="22">
         <f>IF(D114="","",D114*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F114" s="29" t="n"/>
+      <c r="F114" s="32" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="28" t="n"/>
-      <c r="B115" s="28" t="n"/>
-      <c r="C115" s="29" t="n"/>
-      <c r="D115" s="29" t="n"/>
-      <c r="E115" s="18">
+      <c r="A115" s="31" t="n"/>
+      <c r="B115" s="31" t="n"/>
+      <c r="C115" s="32" t="n"/>
+      <c r="D115" s="32" t="n"/>
+      <c r="E115" s="22">
         <f>IF(D115="","",D115*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F115" s="29" t="n"/>
+      <c r="F115" s="32" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="28" t="n"/>
-      <c r="B116" s="28" t="n"/>
-      <c r="C116" s="29" t="n"/>
-      <c r="D116" s="29" t="n"/>
-      <c r="E116" s="18">
+      <c r="A116" s="31" t="n"/>
+      <c r="B116" s="31" t="n"/>
+      <c r="C116" s="32" t="n"/>
+      <c r="D116" s="32" t="n"/>
+      <c r="E116" s="22">
         <f>IF(D116="","",D116*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F116" s="29" t="n"/>
+      <c r="F116" s="32" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="28" t="n"/>
-      <c r="B117" s="28" t="n"/>
-      <c r="C117" s="29" t="n"/>
-      <c r="D117" s="29" t="n"/>
-      <c r="E117" s="18">
+      <c r="A117" s="31" t="n"/>
+      <c r="B117" s="31" t="n"/>
+      <c r="C117" s="32" t="n"/>
+      <c r="D117" s="32" t="n"/>
+      <c r="E117" s="22">
         <f>IF(D117="","",D117*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F117" s="29" t="n"/>
+      <c r="F117" s="32" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="28" t="n"/>
-      <c r="B118" s="28" t="n"/>
-      <c r="C118" s="29" t="n"/>
-      <c r="D118" s="29" t="n"/>
-      <c r="E118" s="18">
+      <c r="A118" s="31" t="n"/>
+      <c r="B118" s="31" t="n"/>
+      <c r="C118" s="32" t="n"/>
+      <c r="D118" s="32" t="n"/>
+      <c r="E118" s="22">
         <f>IF(D118="","",D118*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F118" s="29" t="n"/>
+      <c r="F118" s="32" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="28" t="n"/>
-      <c r="B119" s="28" t="n"/>
-      <c r="C119" s="29" t="n"/>
-      <c r="D119" s="29" t="n"/>
-      <c r="E119" s="18">
+      <c r="A119" s="31" t="n"/>
+      <c r="B119" s="31" t="n"/>
+      <c r="C119" s="32" t="n"/>
+      <c r="D119" s="32" t="n"/>
+      <c r="E119" s="22">
         <f>IF(D119="","",D119*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F119" s="29" t="n"/>
+      <c r="F119" s="32" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="28" t="n"/>
-      <c r="B120" s="28" t="n"/>
-      <c r="C120" s="29" t="n"/>
-      <c r="D120" s="29" t="n"/>
-      <c r="E120" s="18">
+      <c r="A120" s="31" t="n"/>
+      <c r="B120" s="31" t="n"/>
+      <c r="C120" s="32" t="n"/>
+      <c r="D120" s="32" t="n"/>
+      <c r="E120" s="22">
         <f>IF(D120="","",D120*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F120" s="29" t="n"/>
+      <c r="F120" s="32" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="28" t="n"/>
-      <c r="B121" s="28" t="n"/>
-      <c r="C121" s="29" t="n"/>
-      <c r="D121" s="29" t="n"/>
-      <c r="E121" s="18">
+      <c r="A121" s="31" t="n"/>
+      <c r="B121" s="31" t="n"/>
+      <c r="C121" s="32" t="n"/>
+      <c r="D121" s="32" t="n"/>
+      <c r="E121" s="22">
         <f>IF(D121="","",D121*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F121" s="29" t="n"/>
+      <c r="F121" s="32" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="28" t="n"/>
-      <c r="B122" s="28" t="n"/>
-      <c r="C122" s="29" t="n"/>
-      <c r="D122" s="29" t="n"/>
-      <c r="E122" s="18">
+      <c r="A122" s="31" t="n"/>
+      <c r="B122" s="31" t="n"/>
+      <c r="C122" s="32" t="n"/>
+      <c r="D122" s="32" t="n"/>
+      <c r="E122" s="22">
         <f>IF(D122="","",D122*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F122" s="29" t="n"/>
+      <c r="F122" s="32" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="28" t="n"/>
-      <c r="B123" s="28" t="n"/>
-      <c r="C123" s="29" t="n"/>
-      <c r="D123" s="29" t="n"/>
-      <c r="E123" s="18">
+      <c r="A123" s="31" t="n"/>
+      <c r="B123" s="31" t="n"/>
+      <c r="C123" s="32" t="n"/>
+      <c r="D123" s="32" t="n"/>
+      <c r="E123" s="22">
         <f>IF(D123="","",D123*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F123" s="29" t="n"/>
+      <c r="F123" s="32" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="28" t="n"/>
-      <c r="B124" s="28" t="n"/>
-      <c r="C124" s="29" t="n"/>
-      <c r="D124" s="29" t="n"/>
-      <c r="E124" s="18">
+      <c r="A124" s="31" t="n"/>
+      <c r="B124" s="31" t="n"/>
+      <c r="C124" s="32" t="n"/>
+      <c r="D124" s="32" t="n"/>
+      <c r="E124" s="22">
         <f>IF(D124="","",D124*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F124" s="29" t="n"/>
+      <c r="F124" s="32" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="28" t="n"/>
-      <c r="B125" s="28" t="n"/>
-      <c r="C125" s="29" t="n"/>
-      <c r="D125" s="29" t="n"/>
-      <c r="E125" s="18">
+      <c r="A125" s="31" t="n"/>
+      <c r="B125" s="31" t="n"/>
+      <c r="C125" s="32" t="n"/>
+      <c r="D125" s="32" t="n"/>
+      <c r="E125" s="22">
         <f>IF(D125="","",D125*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F125" s="29" t="n"/>
+      <c r="F125" s="32" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="28" t="n"/>
-      <c r="B126" s="28" t="n"/>
-      <c r="C126" s="29" t="n"/>
-      <c r="D126" s="29" t="n"/>
-      <c r="E126" s="18">
+      <c r="A126" s="31" t="n"/>
+      <c r="B126" s="31" t="n"/>
+      <c r="C126" s="32" t="n"/>
+      <c r="D126" s="32" t="n"/>
+      <c r="E126" s="22">
         <f>IF(D126="","",D126*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F126" s="29" t="n"/>
+      <c r="F126" s="32" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="28" t="n"/>
-      <c r="B127" s="28" t="n"/>
-      <c r="C127" s="29" t="n"/>
-      <c r="D127" s="29" t="n"/>
-      <c r="E127" s="18">
+      <c r="A127" s="31" t="n"/>
+      <c r="B127" s="31" t="n"/>
+      <c r="C127" s="32" t="n"/>
+      <c r="D127" s="32" t="n"/>
+      <c r="E127" s="22">
         <f>IF(D127="","",D127*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F127" s="29" t="n"/>
+      <c r="F127" s="32" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="28" t="n"/>
-      <c r="B128" s="28" t="n"/>
-      <c r="C128" s="29" t="n"/>
-      <c r="D128" s="29" t="n"/>
-      <c r="E128" s="18">
+      <c r="A128" s="31" t="n"/>
+      <c r="B128" s="31" t="n"/>
+      <c r="C128" s="32" t="n"/>
+      <c r="D128" s="32" t="n"/>
+      <c r="E128" s="22">
         <f>IF(D128="","",D128*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F128" s="29" t="n"/>
+      <c r="F128" s="32" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="28" t="n"/>
-      <c r="B129" s="28" t="n"/>
-      <c r="C129" s="29" t="n"/>
-      <c r="D129" s="29" t="n"/>
-      <c r="E129" s="18">
+      <c r="A129" s="31" t="n"/>
+      <c r="B129" s="31" t="n"/>
+      <c r="C129" s="32" t="n"/>
+      <c r="D129" s="32" t="n"/>
+      <c r="E129" s="22">
         <f>IF(D129="","",D129*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F129" s="29" t="n"/>
+      <c r="F129" s="32" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="28" t="n"/>
-      <c r="B130" s="28" t="n"/>
-      <c r="C130" s="29" t="n"/>
-      <c r="D130" s="29" t="n"/>
-      <c r="E130" s="18">
+      <c r="A130" s="31" t="n"/>
+      <c r="B130" s="31" t="n"/>
+      <c r="C130" s="32" t="n"/>
+      <c r="D130" s="32" t="n"/>
+      <c r="E130" s="22">
         <f>IF(D130="","",D130*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F130" s="29" t="n"/>
+      <c r="F130" s="32" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="28" t="n"/>
-      <c r="B131" s="28" t="n"/>
-      <c r="C131" s="29" t="n"/>
-      <c r="D131" s="29" t="n"/>
-      <c r="E131" s="18">
+      <c r="A131" s="31" t="n"/>
+      <c r="B131" s="31" t="n"/>
+      <c r="C131" s="32" t="n"/>
+      <c r="D131" s="32" t="n"/>
+      <c r="E131" s="22">
         <f>IF(D131="","",D131*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F131" s="29" t="n"/>
+      <c r="F131" s="32" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="28" t="n"/>
-      <c r="B132" s="28" t="n"/>
-      <c r="C132" s="29" t="n"/>
-      <c r="D132" s="29" t="n"/>
-      <c r="E132" s="18">
+      <c r="A132" s="31" t="n"/>
+      <c r="B132" s="31" t="n"/>
+      <c r="C132" s="32" t="n"/>
+      <c r="D132" s="32" t="n"/>
+      <c r="E132" s="22">
         <f>IF(D132="","",D132*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F132" s="29" t="n"/>
+      <c r="F132" s="32" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="28" t="n"/>
-      <c r="B133" s="28" t="n"/>
-      <c r="C133" s="29" t="n"/>
-      <c r="D133" s="29" t="n"/>
-      <c r="E133" s="18">
+      <c r="A133" s="31" t="n"/>
+      <c r="B133" s="31" t="n"/>
+      <c r="C133" s="32" t="n"/>
+      <c r="D133" s="32" t="n"/>
+      <c r="E133" s="22">
         <f>IF(D133="","",D133*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F133" s="29" t="n"/>
+      <c r="F133" s="32" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="28" t="n"/>
-      <c r="B134" s="28" t="n"/>
-      <c r="C134" s="29" t="n"/>
-      <c r="D134" s="29" t="n"/>
-      <c r="E134" s="18">
+      <c r="A134" s="31" t="n"/>
+      <c r="B134" s="31" t="n"/>
+      <c r="C134" s="32" t="n"/>
+      <c r="D134" s="32" t="n"/>
+      <c r="E134" s="22">
         <f>IF(D134="","",D134*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F134" s="29" t="n"/>
+      <c r="F134" s="32" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="28" t="n"/>
-      <c r="B135" s="28" t="n"/>
-      <c r="C135" s="29" t="n"/>
-      <c r="D135" s="29" t="n"/>
-      <c r="E135" s="18">
+      <c r="A135" s="31" t="n"/>
+      <c r="B135" s="31" t="n"/>
+      <c r="C135" s="32" t="n"/>
+      <c r="D135" s="32" t="n"/>
+      <c r="E135" s="22">
         <f>IF(D135="","",D135*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F135" s="29" t="n"/>
+      <c r="F135" s="32" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="28" t="n"/>
-      <c r="B136" s="28" t="n"/>
-      <c r="C136" s="29" t="n"/>
-      <c r="D136" s="29" t="n"/>
-      <c r="E136" s="18">
+      <c r="A136" s="31" t="n"/>
+      <c r="B136" s="31" t="n"/>
+      <c r="C136" s="32" t="n"/>
+      <c r="D136" s="32" t="n"/>
+      <c r="E136" s="22">
         <f>IF(D136="","",D136*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F136" s="29" t="n"/>
+      <c r="F136" s="32" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="28" t="n"/>
-      <c r="B137" s="28" t="n"/>
-      <c r="C137" s="29" t="n"/>
-      <c r="D137" s="29" t="n"/>
-      <c r="E137" s="18">
+      <c r="A137" s="31" t="n"/>
+      <c r="B137" s="31" t="n"/>
+      <c r="C137" s="32" t="n"/>
+      <c r="D137" s="32" t="n"/>
+      <c r="E137" s="22">
         <f>IF(D137="","",D137*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F137" s="29" t="n"/>
+      <c r="F137" s="32" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="28" t="n"/>
-      <c r="B138" s="28" t="n"/>
-      <c r="C138" s="29" t="n"/>
-      <c r="D138" s="29" t="n"/>
-      <c r="E138" s="18">
+      <c r="A138" s="31" t="n"/>
+      <c r="B138" s="31" t="n"/>
+      <c r="C138" s="32" t="n"/>
+      <c r="D138" s="32" t="n"/>
+      <c r="E138" s="22">
         <f>IF(D138="","",D138*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F138" s="29" t="n"/>
+      <c r="F138" s="32" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="28" t="n"/>
-      <c r="B139" s="28" t="n"/>
-      <c r="C139" s="29" t="n"/>
-      <c r="D139" s="29" t="n"/>
-      <c r="E139" s="18">
+      <c r="A139" s="31" t="n"/>
+      <c r="B139" s="31" t="n"/>
+      <c r="C139" s="32" t="n"/>
+      <c r="D139" s="32" t="n"/>
+      <c r="E139" s="22">
         <f>IF(D139="","",D139*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F139" s="29" t="n"/>
+      <c r="F139" s="32" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="28" t="n"/>
-      <c r="B140" s="28" t="n"/>
-      <c r="C140" s="29" t="n"/>
-      <c r="D140" s="29" t="n"/>
-      <c r="E140" s="18">
+      <c r="A140" s="31" t="n"/>
+      <c r="B140" s="31" t="n"/>
+      <c r="C140" s="32" t="n"/>
+      <c r="D140" s="32" t="n"/>
+      <c r="E140" s="22">
         <f>IF(D140="","",D140*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F140" s="29" t="n"/>
+      <c r="F140" s="32" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="28" t="n"/>
-      <c r="B141" s="28" t="n"/>
-      <c r="C141" s="29" t="n"/>
-      <c r="D141" s="29" t="n"/>
-      <c r="E141" s="18">
+      <c r="A141" s="31" t="n"/>
+      <c r="B141" s="31" t="n"/>
+      <c r="C141" s="32" t="n"/>
+      <c r="D141" s="32" t="n"/>
+      <c r="E141" s="22">
         <f>IF(D141="","",D141*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F141" s="29" t="n"/>
+      <c r="F141" s="32" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="28" t="n"/>
-      <c r="B142" s="28" t="n"/>
-      <c r="C142" s="29" t="n"/>
-      <c r="D142" s="29" t="n"/>
-      <c r="E142" s="18">
+      <c r="A142" s="31" t="n"/>
+      <c r="B142" s="31" t="n"/>
+      <c r="C142" s="32" t="n"/>
+      <c r="D142" s="32" t="n"/>
+      <c r="E142" s="22">
         <f>IF(D142="","",D142*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F142" s="29" t="n"/>
+      <c r="F142" s="32" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="28" t="n"/>
-      <c r="B143" s="28" t="n"/>
-      <c r="C143" s="29" t="n"/>
-      <c r="D143" s="29" t="n"/>
-      <c r="E143" s="18">
+      <c r="A143" s="31" t="n"/>
+      <c r="B143" s="31" t="n"/>
+      <c r="C143" s="32" t="n"/>
+      <c r="D143" s="32" t="n"/>
+      <c r="E143" s="22">
         <f>IF(D143="","",D143*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F143" s="29" t="n"/>
+      <c r="F143" s="32" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="28" t="n"/>
-      <c r="B144" s="28" t="n"/>
-      <c r="C144" s="29" t="n"/>
-      <c r="D144" s="29" t="n"/>
-      <c r="E144" s="18">
+      <c r="A144" s="31" t="n"/>
+      <c r="B144" s="31" t="n"/>
+      <c r="C144" s="32" t="n"/>
+      <c r="D144" s="32" t="n"/>
+      <c r="E144" s="22">
         <f>IF(D144="","",D144*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F144" s="29" t="n"/>
+      <c r="F144" s="32" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="28" t="n"/>
-      <c r="B145" s="28" t="n"/>
-      <c r="C145" s="29" t="n"/>
-      <c r="D145" s="29" t="n"/>
-      <c r="E145" s="18">
+      <c r="A145" s="31" t="n"/>
+      <c r="B145" s="31" t="n"/>
+      <c r="C145" s="32" t="n"/>
+      <c r="D145" s="32" t="n"/>
+      <c r="E145" s="22">
         <f>IF(D145="","",D145*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F145" s="29" t="n"/>
+      <c r="F145" s="32" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="28" t="n"/>
-      <c r="B146" s="28" t="n"/>
-      <c r="C146" s="29" t="n"/>
-      <c r="D146" s="29" t="n"/>
-      <c r="E146" s="18">
+      <c r="A146" s="31" t="n"/>
+      <c r="B146" s="31" t="n"/>
+      <c r="C146" s="32" t="n"/>
+      <c r="D146" s="32" t="n"/>
+      <c r="E146" s="22">
         <f>IF(D146="","",D146*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F146" s="29" t="n"/>
+      <c r="F146" s="32" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="28" t="n"/>
-      <c r="B147" s="28" t="n"/>
-      <c r="C147" s="29" t="n"/>
-      <c r="D147" s="29" t="n"/>
-      <c r="E147" s="18">
+      <c r="A147" s="31" t="n"/>
+      <c r="B147" s="31" t="n"/>
+      <c r="C147" s="32" t="n"/>
+      <c r="D147" s="32" t="n"/>
+      <c r="E147" s="22">
         <f>IF(D147="","",D147*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F147" s="29" t="n"/>
+      <c r="F147" s="32" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="28" t="n"/>
-      <c r="B148" s="28" t="n"/>
-      <c r="C148" s="29" t="n"/>
-      <c r="D148" s="29" t="n"/>
-      <c r="E148" s="18">
+      <c r="A148" s="31" t="n"/>
+      <c r="B148" s="31" t="n"/>
+      <c r="C148" s="32" t="n"/>
+      <c r="D148" s="32" t="n"/>
+      <c r="E148" s="22">
         <f>IF(D148="","",D148*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F148" s="29" t="n"/>
+      <c r="F148" s="32" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="28" t="n"/>
-      <c r="B149" s="28" t="n"/>
-      <c r="C149" s="29" t="n"/>
-      <c r="D149" s="29" t="n"/>
-      <c r="E149" s="18">
+      <c r="A149" s="31" t="n"/>
+      <c r="B149" s="31" t="n"/>
+      <c r="C149" s="32" t="n"/>
+      <c r="D149" s="32" t="n"/>
+      <c r="E149" s="22">
         <f>IF(D149="","",D149*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F149" s="29" t="n"/>
+      <c r="F149" s="32" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="28" t="n"/>
-      <c r="B150" s="28" t="n"/>
-      <c r="C150" s="29" t="n"/>
-      <c r="D150" s="29" t="n"/>
-      <c r="E150" s="18">
+      <c r="A150" s="31" t="n"/>
+      <c r="B150" s="31" t="n"/>
+      <c r="C150" s="32" t="n"/>
+      <c r="D150" s="32" t="n"/>
+      <c r="E150" s="22">
         <f>IF(D150="","",D150*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F150" s="29" t="n"/>
+      <c r="F150" s="32" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="28" t="n"/>
-      <c r="B151" s="28" t="n"/>
-      <c r="C151" s="29" t="n"/>
-      <c r="D151" s="29" t="n"/>
-      <c r="E151" s="18">
+      <c r="A151" s="31" t="n"/>
+      <c r="B151" s="31" t="n"/>
+      <c r="C151" s="32" t="n"/>
+      <c r="D151" s="32" t="n"/>
+      <c r="E151" s="22">
         <f>IF(D151="","",D151*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F151" s="29" t="n"/>
+      <c r="F151" s="32" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="28" t="n"/>
-      <c r="B152" s="28" t="n"/>
-      <c r="C152" s="29" t="n"/>
-      <c r="D152" s="29" t="n"/>
-      <c r="E152" s="18">
+      <c r="A152" s="31" t="n"/>
+      <c r="B152" s="31" t="n"/>
+      <c r="C152" s="32" t="n"/>
+      <c r="D152" s="32" t="n"/>
+      <c r="E152" s="22">
         <f>IF(D152="","",D152*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F152" s="29" t="n"/>
+      <c r="F152" s="32" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="28" t="n"/>
-      <c r="B153" s="28" t="n"/>
-      <c r="C153" s="29" t="n"/>
-      <c r="D153" s="29" t="n"/>
-      <c r="E153" s="18">
+      <c r="A153" s="31" t="n"/>
+      <c r="B153" s="31" t="n"/>
+      <c r="C153" s="32" t="n"/>
+      <c r="D153" s="32" t="n"/>
+      <c r="E153" s="22">
         <f>IF(D153="","",D153*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F153" s="29" t="n"/>
+      <c r="F153" s="32" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="28" t="n"/>
-      <c r="B154" s="28" t="n"/>
-      <c r="C154" s="29" t="n"/>
-      <c r="D154" s="29" t="n"/>
-      <c r="E154" s="18">
+      <c r="A154" s="31" t="n"/>
+      <c r="B154" s="31" t="n"/>
+      <c r="C154" s="32" t="n"/>
+      <c r="D154" s="32" t="n"/>
+      <c r="E154" s="22">
         <f>IF(D154="","",D154*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F154" s="29" t="n"/>
+      <c r="F154" s="32" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="28" t="n"/>
-      <c r="B155" s="28" t="n"/>
-      <c r="C155" s="29" t="n"/>
-      <c r="D155" s="29" t="n"/>
-      <c r="E155" s="18">
+      <c r="A155" s="31" t="n"/>
+      <c r="B155" s="31" t="n"/>
+      <c r="C155" s="32" t="n"/>
+      <c r="D155" s="32" t="n"/>
+      <c r="E155" s="22">
         <f>IF(D155="","",D155*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F155" s="29" t="n"/>
+      <c r="F155" s="32" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="28" t="n"/>
-      <c r="B156" s="28" t="n"/>
-      <c r="C156" s="29" t="n"/>
-      <c r="D156" s="29" t="n"/>
-      <c r="E156" s="18">
+      <c r="A156" s="31" t="n"/>
+      <c r="B156" s="31" t="n"/>
+      <c r="C156" s="32" t="n"/>
+      <c r="D156" s="32" t="n"/>
+      <c r="E156" s="22">
         <f>IF(D156="","",D156*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F156" s="29" t="n"/>
+      <c r="F156" s="32" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="28" t="n"/>
-      <c r="B157" s="28" t="n"/>
-      <c r="C157" s="29" t="n"/>
-      <c r="D157" s="29" t="n"/>
-      <c r="E157" s="18">
+      <c r="A157" s="31" t="n"/>
+      <c r="B157" s="31" t="n"/>
+      <c r="C157" s="32" t="n"/>
+      <c r="D157" s="32" t="n"/>
+      <c r="E157" s="22">
         <f>IF(D157="","",D157*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F157" s="29" t="n"/>
+      <c r="F157" s="32" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="28" t="n"/>
-      <c r="B158" s="28" t="n"/>
-      <c r="C158" s="29" t="n"/>
-      <c r="D158" s="29" t="n"/>
-      <c r="E158" s="18">
+      <c r="A158" s="31" t="n"/>
+      <c r="B158" s="31" t="n"/>
+      <c r="C158" s="32" t="n"/>
+      <c r="D158" s="32" t="n"/>
+      <c r="E158" s="22">
         <f>IF(D158="","",D158*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F158" s="29" t="n"/>
+      <c r="F158" s="32" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="28" t="n"/>
-      <c r="B159" s="28" t="n"/>
-      <c r="C159" s="29" t="n"/>
-      <c r="D159" s="29" t="n"/>
-      <c r="E159" s="18">
+      <c r="A159" s="31" t="n"/>
+      <c r="B159" s="31" t="n"/>
+      <c r="C159" s="32" t="n"/>
+      <c r="D159" s="32" t="n"/>
+      <c r="E159" s="22">
         <f>IF(D159="","",D159*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F159" s="29" t="n"/>
+      <c r="F159" s="32" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="28" t="n"/>
-      <c r="B160" s="28" t="n"/>
-      <c r="C160" s="29" t="n"/>
-      <c r="D160" s="29" t="n"/>
-      <c r="E160" s="18">
+      <c r="A160" s="31" t="n"/>
+      <c r="B160" s="31" t="n"/>
+      <c r="C160" s="32" t="n"/>
+      <c r="D160" s="32" t="n"/>
+      <c r="E160" s="22">
         <f>IF(D160="","",D160*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F160" s="29" t="n"/>
+      <c r="F160" s="32" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="28" t="n"/>
-      <c r="B161" s="28" t="n"/>
-      <c r="C161" s="29" t="n"/>
-      <c r="D161" s="29" t="n"/>
-      <c r="E161" s="18">
+      <c r="A161" s="31" t="n"/>
+      <c r="B161" s="31" t="n"/>
+      <c r="C161" s="32" t="n"/>
+      <c r="D161" s="32" t="n"/>
+      <c r="E161" s="22">
         <f>IF(D161="","",D161*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F161" s="29" t="n"/>
+      <c r="F161" s="32" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="28" t="n"/>
-      <c r="B162" s="28" t="n"/>
-      <c r="C162" s="29" t="n"/>
-      <c r="D162" s="29" t="n"/>
-      <c r="E162" s="18">
+      <c r="A162" s="31" t="n"/>
+      <c r="B162" s="31" t="n"/>
+      <c r="C162" s="32" t="n"/>
+      <c r="D162" s="32" t="n"/>
+      <c r="E162" s="22">
         <f>IF(D162="","",D162*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F162" s="29" t="n"/>
+      <c r="F162" s="32" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="28" t="n"/>
-      <c r="B163" s="28" t="n"/>
-      <c r="C163" s="29" t="n"/>
-      <c r="D163" s="29" t="n"/>
-      <c r="E163" s="18">
+      <c r="A163" s="31" t="n"/>
+      <c r="B163" s="31" t="n"/>
+      <c r="C163" s="32" t="n"/>
+      <c r="D163" s="32" t="n"/>
+      <c r="E163" s="22">
         <f>IF(D163="","",D163*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F163" s="29" t="n"/>
+      <c r="F163" s="32" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="28" t="n"/>
-      <c r="B164" s="28" t="n"/>
-      <c r="C164" s="29" t="n"/>
-      <c r="D164" s="29" t="n"/>
-      <c r="E164" s="18">
+      <c r="A164" s="31" t="n"/>
+      <c r="B164" s="31" t="n"/>
+      <c r="C164" s="32" t="n"/>
+      <c r="D164" s="32" t="n"/>
+      <c r="E164" s="22">
         <f>IF(D164="","",D164*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F164" s="29" t="n"/>
+      <c r="F164" s="32" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="28" t="n"/>
-      <c r="B165" s="28" t="n"/>
-      <c r="C165" s="29" t="n"/>
-      <c r="D165" s="29" t="n"/>
-      <c r="E165" s="18">
+      <c r="A165" s="31" t="n"/>
+      <c r="B165" s="31" t="n"/>
+      <c r="C165" s="32" t="n"/>
+      <c r="D165" s="32" t="n"/>
+      <c r="E165" s="22">
         <f>IF(D165="","",D165*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F165" s="29" t="n"/>
+      <c r="F165" s="32" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="28" t="n"/>
-      <c r="B166" s="28" t="n"/>
-      <c r="C166" s="29" t="n"/>
-      <c r="D166" s="29" t="n"/>
-      <c r="E166" s="18">
+      <c r="A166" s="31" t="n"/>
+      <c r="B166" s="31" t="n"/>
+      <c r="C166" s="32" t="n"/>
+      <c r="D166" s="32" t="n"/>
+      <c r="E166" s="22">
         <f>IF(D166="","",D166*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F166" s="29" t="n"/>
+      <c r="F166" s="32" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="28" t="n"/>
-      <c r="B167" s="28" t="n"/>
-      <c r="C167" s="29" t="n"/>
-      <c r="D167" s="29" t="n"/>
-      <c r="E167" s="18">
+      <c r="A167" s="31" t="n"/>
+      <c r="B167" s="31" t="n"/>
+      <c r="C167" s="32" t="n"/>
+      <c r="D167" s="32" t="n"/>
+      <c r="E167" s="22">
         <f>IF(D167="","",D167*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F167" s="29" t="n"/>
+      <c r="F167" s="32" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="28" t="n"/>
-      <c r="B168" s="28" t="n"/>
-      <c r="C168" s="29" t="n"/>
-      <c r="D168" s="29" t="n"/>
-      <c r="E168" s="18">
+      <c r="A168" s="31" t="n"/>
+      <c r="B168" s="31" t="n"/>
+      <c r="C168" s="32" t="n"/>
+      <c r="D168" s="32" t="n"/>
+      <c r="E168" s="22">
         <f>IF(D168="","",D168*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F168" s="29" t="n"/>
+      <c r="F168" s="32" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" s="28" t="n"/>
-      <c r="B169" s="28" t="n"/>
-      <c r="C169" s="29" t="n"/>
-      <c r="D169" s="29" t="n"/>
-      <c r="E169" s="18">
+      <c r="A169" s="31" t="n"/>
+      <c r="B169" s="31" t="n"/>
+      <c r="C169" s="32" t="n"/>
+      <c r="D169" s="32" t="n"/>
+      <c r="E169" s="22">
         <f>IF(D169="","",D169*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F169" s="29" t="n"/>
+      <c r="F169" s="32" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="28" t="n"/>
-      <c r="B170" s="28" t="n"/>
-      <c r="C170" s="29" t="n"/>
-      <c r="D170" s="29" t="n"/>
-      <c r="E170" s="18">
+      <c r="A170" s="31" t="n"/>
+      <c r="B170" s="31" t="n"/>
+      <c r="C170" s="32" t="n"/>
+      <c r="D170" s="32" t="n"/>
+      <c r="E170" s="22">
         <f>IF(D170="","",D170*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F170" s="29" t="n"/>
+      <c r="F170" s="32" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="28" t="n"/>
-      <c r="B171" s="28" t="n"/>
-      <c r="C171" s="29" t="n"/>
-      <c r="D171" s="29" t="n"/>
-      <c r="E171" s="18">
+      <c r="A171" s="31" t="n"/>
+      <c r="B171" s="31" t="n"/>
+      <c r="C171" s="32" t="n"/>
+      <c r="D171" s="32" t="n"/>
+      <c r="E171" s="22">
         <f>IF(D171="","",D171*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F171" s="29" t="n"/>
+      <c r="F171" s="32" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="28" t="n"/>
-      <c r="B172" s="28" t="n"/>
-      <c r="C172" s="29" t="n"/>
-      <c r="D172" s="29" t="n"/>
-      <c r="E172" s="18">
+      <c r="A172" s="31" t="n"/>
+      <c r="B172" s="31" t="n"/>
+      <c r="C172" s="32" t="n"/>
+      <c r="D172" s="32" t="n"/>
+      <c r="E172" s="22">
         <f>IF(D172="","",D172*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F172" s="29" t="n"/>
+      <c r="F172" s="32" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" s="28" t="n"/>
-      <c r="B173" s="28" t="n"/>
-      <c r="C173" s="29" t="n"/>
-      <c r="D173" s="29" t="n"/>
-      <c r="E173" s="18">
+      <c r="A173" s="31" t="n"/>
+      <c r="B173" s="31" t="n"/>
+      <c r="C173" s="32" t="n"/>
+      <c r="D173" s="32" t="n"/>
+      <c r="E173" s="22">
         <f>IF(D173="","",D173*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F173" s="29" t="n"/>
+      <c r="F173" s="32" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="28" t="n"/>
-      <c r="B174" s="28" t="n"/>
-      <c r="C174" s="29" t="n"/>
-      <c r="D174" s="29" t="n"/>
-      <c r="E174" s="18">
+      <c r="A174" s="31" t="n"/>
+      <c r="B174" s="31" t="n"/>
+      <c r="C174" s="32" t="n"/>
+      <c r="D174" s="32" t="n"/>
+      <c r="E174" s="22">
         <f>IF(D174="","",D174*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F174" s="29" t="n"/>
+      <c r="F174" s="32" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="28" t="n"/>
-      <c r="B175" s="28" t="n"/>
-      <c r="C175" s="29" t="n"/>
-      <c r="D175" s="29" t="n"/>
-      <c r="E175" s="18">
+      <c r="A175" s="31" t="n"/>
+      <c r="B175" s="31" t="n"/>
+      <c r="C175" s="32" t="n"/>
+      <c r="D175" s="32" t="n"/>
+      <c r="E175" s="22">
         <f>IF(D175="","",D175*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F175" s="29" t="n"/>
+      <c r="F175" s="32" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" s="28" t="n"/>
-      <c r="B176" s="28" t="n"/>
-      <c r="C176" s="29" t="n"/>
-      <c r="D176" s="29" t="n"/>
-      <c r="E176" s="18">
+      <c r="A176" s="31" t="n"/>
+      <c r="B176" s="31" t="n"/>
+      <c r="C176" s="32" t="n"/>
+      <c r="D176" s="32" t="n"/>
+      <c r="E176" s="22">
         <f>IF(D176="","",D176*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F176" s="29" t="n"/>
+      <c r="F176" s="32" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="28" t="n"/>
-      <c r="B177" s="28" t="n"/>
-      <c r="C177" s="29" t="n"/>
-      <c r="D177" s="29" t="n"/>
-      <c r="E177" s="18">
+      <c r="A177" s="31" t="n"/>
+      <c r="B177" s="31" t="n"/>
+      <c r="C177" s="32" t="n"/>
+      <c r="D177" s="32" t="n"/>
+      <c r="E177" s="22">
         <f>IF(D177="","",D177*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F177" s="29" t="n"/>
+      <c r="F177" s="32" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="28" t="n"/>
-      <c r="B178" s="28" t="n"/>
-      <c r="C178" s="29" t="n"/>
-      <c r="D178" s="29" t="n"/>
-      <c r="E178" s="18">
+      <c r="A178" s="31" t="n"/>
+      <c r="B178" s="31" t="n"/>
+      <c r="C178" s="32" t="n"/>
+      <c r="D178" s="32" t="n"/>
+      <c r="E178" s="22">
         <f>IF(D178="","",D178*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F178" s="29" t="n"/>
+      <c r="F178" s="32" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" s="28" t="n"/>
-      <c r="B179" s="28" t="n"/>
-      <c r="C179" s="29" t="n"/>
-      <c r="D179" s="29" t="n"/>
-      <c r="E179" s="18">
+      <c r="A179" s="31" t="n"/>
+      <c r="B179" s="31" t="n"/>
+      <c r="C179" s="32" t="n"/>
+      <c r="D179" s="32" t="n"/>
+      <c r="E179" s="22">
         <f>IF(D179="","",D179*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F179" s="29" t="n"/>
+      <c r="F179" s="32" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" s="28" t="n"/>
-      <c r="B180" s="28" t="n"/>
-      <c r="C180" s="29" t="n"/>
-      <c r="D180" s="29" t="n"/>
-      <c r="E180" s="18">
+      <c r="A180" s="31" t="n"/>
+      <c r="B180" s="31" t="n"/>
+      <c r="C180" s="32" t="n"/>
+      <c r="D180" s="32" t="n"/>
+      <c r="E180" s="22">
         <f>IF(D180="","",D180*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F180" s="29" t="n"/>
+      <c r="F180" s="32" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="28" t="n"/>
-      <c r="B181" s="28" t="n"/>
-      <c r="C181" s="29" t="n"/>
-      <c r="D181" s="29" t="n"/>
-      <c r="E181" s="18">
+      <c r="A181" s="31" t="n"/>
+      <c r="B181" s="31" t="n"/>
+      <c r="C181" s="32" t="n"/>
+      <c r="D181" s="32" t="n"/>
+      <c r="E181" s="22">
         <f>IF(D181="","",D181*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F181" s="29" t="n"/>
+      <c r="F181" s="32" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="28" t="n"/>
-      <c r="B182" s="28" t="n"/>
-      <c r="C182" s="29" t="n"/>
-      <c r="D182" s="29" t="n"/>
-      <c r="E182" s="18">
+      <c r="A182" s="31" t="n"/>
+      <c r="B182" s="31" t="n"/>
+      <c r="C182" s="32" t="n"/>
+      <c r="D182" s="32" t="n"/>
+      <c r="E182" s="22">
         <f>IF(D182="","",D182*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F182" s="29" t="n"/>
+      <c r="F182" s="32" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="28" t="n"/>
-      <c r="B183" s="28" t="n"/>
-      <c r="C183" s="29" t="n"/>
-      <c r="D183" s="29" t="n"/>
-      <c r="E183" s="18">
+      <c r="A183" s="31" t="n"/>
+      <c r="B183" s="31" t="n"/>
+      <c r="C183" s="32" t="n"/>
+      <c r="D183" s="32" t="n"/>
+      <c r="E183" s="22">
         <f>IF(D183="","",D183*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F183" s="29" t="n"/>
+      <c r="F183" s="32" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="28" t="n"/>
-      <c r="B184" s="28" t="n"/>
-      <c r="C184" s="29" t="n"/>
-      <c r="D184" s="29" t="n"/>
-      <c r="E184" s="18">
+      <c r="A184" s="31" t="n"/>
+      <c r="B184" s="31" t="n"/>
+      <c r="C184" s="32" t="n"/>
+      <c r="D184" s="32" t="n"/>
+      <c r="E184" s="22">
         <f>IF(D184="","",D184*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F184" s="29" t="n"/>
+      <c r="F184" s="32" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="28" t="n"/>
-      <c r="B185" s="28" t="n"/>
-      <c r="C185" s="29" t="n"/>
-      <c r="D185" s="29" t="n"/>
-      <c r="E185" s="18">
+      <c r="A185" s="31" t="n"/>
+      <c r="B185" s="31" t="n"/>
+      <c r="C185" s="32" t="n"/>
+      <c r="D185" s="32" t="n"/>
+      <c r="E185" s="22">
         <f>IF(D185="","",D185*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F185" s="29" t="n"/>
+      <c r="F185" s="32" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="28" t="n"/>
-      <c r="B186" s="28" t="n"/>
-      <c r="C186" s="29" t="n"/>
-      <c r="D186" s="29" t="n"/>
-      <c r="E186" s="18">
+      <c r="A186" s="31" t="n"/>
+      <c r="B186" s="31" t="n"/>
+      <c r="C186" s="32" t="n"/>
+      <c r="D186" s="32" t="n"/>
+      <c r="E186" s="22">
         <f>IF(D186="","",D186*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F186" s="29" t="n"/>
+      <c r="F186" s="32" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" s="28" t="n"/>
-      <c r="B187" s="28" t="n"/>
-      <c r="C187" s="29" t="n"/>
-      <c r="D187" s="29" t="n"/>
-      <c r="E187" s="18">
+      <c r="A187" s="31" t="n"/>
+      <c r="B187" s="31" t="n"/>
+      <c r="C187" s="32" t="n"/>
+      <c r="D187" s="32" t="n"/>
+      <c r="E187" s="22">
         <f>IF(D187="","",D187*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F187" s="29" t="n"/>
+      <c r="F187" s="32" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" s="28" t="n"/>
-      <c r="B188" s="28" t="n"/>
-      <c r="C188" s="29" t="n"/>
-      <c r="D188" s="29" t="n"/>
-      <c r="E188" s="18">
+      <c r="A188" s="31" t="n"/>
+      <c r="B188" s="31" t="n"/>
+      <c r="C188" s="32" t="n"/>
+      <c r="D188" s="32" t="n"/>
+      <c r="E188" s="22">
         <f>IF(D188="","",D188*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F188" s="29" t="n"/>
+      <c r="F188" s="32" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" s="28" t="n"/>
-      <c r="B189" s="28" t="n"/>
-      <c r="C189" s="29" t="n"/>
-      <c r="D189" s="29" t="n"/>
-      <c r="E189" s="18">
+      <c r="A189" s="31" t="n"/>
+      <c r="B189" s="31" t="n"/>
+      <c r="C189" s="32" t="n"/>
+      <c r="D189" s="32" t="n"/>
+      <c r="E189" s="22">
         <f>IF(D189="","",D189*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F189" s="29" t="n"/>
+      <c r="F189" s="32" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" s="28" t="n"/>
-      <c r="B190" s="28" t="n"/>
-      <c r="C190" s="29" t="n"/>
-      <c r="D190" s="29" t="n"/>
-      <c r="E190" s="18">
+      <c r="A190" s="31" t="n"/>
+      <c r="B190" s="31" t="n"/>
+      <c r="C190" s="32" t="n"/>
+      <c r="D190" s="32" t="n"/>
+      <c r="E190" s="22">
         <f>IF(D190="","",D190*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F190" s="29" t="n"/>
+      <c r="F190" s="32" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="28" t="n"/>
-      <c r="B191" s="28" t="n"/>
-      <c r="C191" s="29" t="n"/>
-      <c r="D191" s="29" t="n"/>
-      <c r="E191" s="18">
+      <c r="A191" s="31" t="n"/>
+      <c r="B191" s="31" t="n"/>
+      <c r="C191" s="32" t="n"/>
+      <c r="D191" s="32" t="n"/>
+      <c r="E191" s="22">
         <f>IF(D191="","",D191*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F191" s="29" t="n"/>
+      <c r="F191" s="32" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="28" t="n"/>
-      <c r="B192" s="28" t="n"/>
-      <c r="C192" s="29" t="n"/>
-      <c r="D192" s="29" t="n"/>
-      <c r="E192" s="18">
+      <c r="A192" s="31" t="n"/>
+      <c r="B192" s="31" t="n"/>
+      <c r="C192" s="32" t="n"/>
+      <c r="D192" s="32" t="n"/>
+      <c r="E192" s="22">
         <f>IF(D192="","",D192*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F192" s="29" t="n"/>
+      <c r="F192" s="32" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="28" t="n"/>
-      <c r="B193" s="28" t="n"/>
-      <c r="C193" s="29" t="n"/>
-      <c r="D193" s="29" t="n"/>
-      <c r="E193" s="18">
+      <c r="A193" s="31" t="n"/>
+      <c r="B193" s="31" t="n"/>
+      <c r="C193" s="32" t="n"/>
+      <c r="D193" s="32" t="n"/>
+      <c r="E193" s="22">
         <f>IF(D193="","",D193*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F193" s="29" t="n"/>
+      <c r="F193" s="32" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="28" t="n"/>
-      <c r="B194" s="28" t="n"/>
-      <c r="C194" s="29" t="n"/>
-      <c r="D194" s="29" t="n"/>
-      <c r="E194" s="18">
+      <c r="A194" s="31" t="n"/>
+      <c r="B194" s="31" t="n"/>
+      <c r="C194" s="32" t="n"/>
+      <c r="D194" s="32" t="n"/>
+      <c r="E194" s="22">
         <f>IF(D194="","",D194*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F194" s="29" t="n"/>
+      <c r="F194" s="32" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="28" t="n"/>
-      <c r="B195" s="28" t="n"/>
-      <c r="C195" s="29" t="n"/>
-      <c r="D195" s="29" t="n"/>
-      <c r="E195" s="18">
+      <c r="A195" s="31" t="n"/>
+      <c r="B195" s="31" t="n"/>
+      <c r="C195" s="32" t="n"/>
+      <c r="D195" s="32" t="n"/>
+      <c r="E195" s="22">
         <f>IF(D195="","",D195*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F195" s="29" t="n"/>
+      <c r="F195" s="32" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="28" t="n"/>
-      <c r="B196" s="28" t="n"/>
-      <c r="C196" s="29" t="n"/>
-      <c r="D196" s="29" t="n"/>
-      <c r="E196" s="18">
+      <c r="A196" s="31" t="n"/>
+      <c r="B196" s="31" t="n"/>
+      <c r="C196" s="32" t="n"/>
+      <c r="D196" s="32" t="n"/>
+      <c r="E196" s="22">
         <f>IF(D196="","",D196*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F196" s="29" t="n"/>
+      <c r="F196" s="32" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="28" t="n"/>
-      <c r="B197" s="28" t="n"/>
-      <c r="C197" s="29" t="n"/>
-      <c r="D197" s="29" t="n"/>
-      <c r="E197" s="18">
+      <c r="A197" s="31" t="n"/>
+      <c r="B197" s="31" t="n"/>
+      <c r="C197" s="32" t="n"/>
+      <c r="D197" s="32" t="n"/>
+      <c r="E197" s="22">
         <f>IF(D197="","",D197*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F197" s="29" t="n"/>
+      <c r="F197" s="32" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="28" t="n"/>
-      <c r="B198" s="28" t="n"/>
-      <c r="C198" s="29" t="n"/>
-      <c r="D198" s="29" t="n"/>
-      <c r="E198" s="18">
+      <c r="A198" s="31" t="n"/>
+      <c r="B198" s="31" t="n"/>
+      <c r="C198" s="32" t="n"/>
+      <c r="D198" s="32" t="n"/>
+      <c r="E198" s="22">
         <f>IF(D198="","",D198*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F198" s="29" t="n"/>
+      <c r="F198" s="32" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" s="28" t="n"/>
-      <c r="B199" s="28" t="n"/>
-      <c r="C199" s="29" t="n"/>
-      <c r="D199" s="29" t="n"/>
-      <c r="E199" s="18">
+      <c r="A199" s="31" t="n"/>
+      <c r="B199" s="31" t="n"/>
+      <c r="C199" s="32" t="n"/>
+      <c r="D199" s="32" t="n"/>
+      <c r="E199" s="22">
         <f>IF(D199="","",D199*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F199" s="29" t="n"/>
+      <c r="F199" s="32" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="28" t="n"/>
-      <c r="B200" s="28" t="n"/>
-      <c r="C200" s="29" t="n"/>
-      <c r="D200" s="29" t="n"/>
-      <c r="E200" s="18">
+      <c r="A200" s="31" t="n"/>
+      <c r="B200" s="31" t="n"/>
+      <c r="C200" s="32" t="n"/>
+      <c r="D200" s="32" t="n"/>
+      <c r="E200" s="22">
         <f>IF(D200="","",D200*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F200" s="29" t="n"/>
+      <c r="F200" s="32" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" s="28" t="n"/>
-      <c r="B201" s="28" t="n"/>
-      <c r="C201" s="29" t="n"/>
-      <c r="D201" s="29" t="n"/>
-      <c r="E201" s="18">
+      <c r="A201" s="31" t="n"/>
+      <c r="B201" s="31" t="n"/>
+      <c r="C201" s="32" t="n"/>
+      <c r="D201" s="32" t="n"/>
+      <c r="E201" s="22">
         <f>IF(D201="","",D201*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F201" s="29" t="n"/>
+      <c r="F201" s="32" t="n"/>
     </row>
     <row r="202">
-      <c r="A202" s="28" t="n"/>
-      <c r="B202" s="28" t="n"/>
-      <c r="C202" s="29" t="n"/>
-      <c r="D202" s="29" t="n"/>
-      <c r="E202" s="18">
+      <c r="A202" s="31" t="n"/>
+      <c r="B202" s="31" t="n"/>
+      <c r="C202" s="32" t="n"/>
+      <c r="D202" s="32" t="n"/>
+      <c r="E202" s="22">
         <f>IF(D202="","",D202*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F202" s="29" t="n"/>
+      <c r="F202" s="32" t="n"/>
     </row>
     <row r="203">
-      <c r="A203" s="28" t="n"/>
-      <c r="B203" s="28" t="n"/>
-      <c r="C203" s="29" t="n"/>
-      <c r="D203" s="29" t="n"/>
-      <c r="E203" s="18">
+      <c r="A203" s="31" t="n"/>
+      <c r="B203" s="31" t="n"/>
+      <c r="C203" s="32" t="n"/>
+      <c r="D203" s="32" t="n"/>
+      <c r="E203" s="22">
         <f>IF(D203="","",D203*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F203" s="29" t="n"/>
+      <c r="F203" s="32" t="n"/>
     </row>
     <row r="204">
-      <c r="A204" s="28" t="n"/>
-      <c r="B204" s="28" t="n"/>
-      <c r="C204" s="29" t="n"/>
-      <c r="D204" s="29" t="n"/>
-      <c r="E204" s="18">
+      <c r="A204" s="31" t="n"/>
+      <c r="B204" s="31" t="n"/>
+      <c r="C204" s="32" t="n"/>
+      <c r="D204" s="32" t="n"/>
+      <c r="E204" s="22">
         <f>IF(D204="","",D204*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F204" s="29" t="n"/>
+      <c r="F204" s="32" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Tableau simple : actuel en jours modifiable
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1LRXK2yXR6W5viD25HWb5
</commit_message>
<xml_diff>
--- a/conges/conges_police_12h08.xlsx
+++ b/conges/conges_police_12h08.xlsx
@@ -155,10 +155,10 @@
     <xf numFmtId="166" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -618,10 +618,10 @@
         <f>B4/$B$15</f>
         <v/>
       </c>
-      <c r="D4" s="7" t="n">
+      <c r="D4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" s="7">
         <f>C4-D4</f>
         <v/>
       </c>
@@ -639,10 +639,10 @@
         <f>B5/$B$15</f>
         <v/>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E5" s="6">
+      <c r="E5" s="7">
         <f>C5-D5</f>
         <v/>
       </c>
@@ -660,10 +660,10 @@
         <f>B6/$B$15</f>
         <v/>
       </c>
-      <c r="D6" s="7" t="n">
+      <c r="D6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="7">
         <f>C6-D6</f>
         <v/>
       </c>
@@ -681,10 +681,10 @@
         <f>B7/$B$15</f>
         <v/>
       </c>
-      <c r="D7" s="7" t="n">
+      <c r="D7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="6">
+      <c r="E7" s="7">
         <f>C7-D7</f>
         <v/>
       </c>
@@ -702,10 +702,10 @@
         <f>B8/$B$15</f>
         <v/>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="6">
+      <c r="E8" s="7">
         <f>C8-D8</f>
         <v/>
       </c>
@@ -723,10 +723,10 @@
         <f>B9/$B$15</f>
         <v/>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="6">
+      <c r="E9" s="7">
         <f>C9-D9</f>
         <v/>
       </c>
@@ -744,10 +744,10 @@
         <f>B10/$B$15</f>
         <v/>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="6">
+      <c r="E10" s="7">
         <f>C10-D10</f>
         <v/>
       </c>
@@ -778,7 +778,7 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>Cases jaunes : tape l'actuel en heures et le pris en jours. Le reste se calcule seul.</t>
+          <t>Cases jaunes : tu peux écrire dedans. Actuel (jours) se calcule depuis les heures si tu n'y touches pas.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Tableau simple : saisie en heures ou en jours avec conversion auto
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1LRXK2yXR6W5viD25HWb5
</commit_message>
<xml_diff>
--- a/conges/conges_police_12h08.xlsx
+++ b/conges/conges_police_12h08.xlsx
@@ -95,7 +95,7 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -115,6 +115,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -144,7 +149,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -158,7 +163,10 @@
     <xf numFmtId="167" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="167" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="12" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -557,14 +565,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -586,20 +596,30 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
+          <t>Tape en heures</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>ou tape en jours</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
           <t>Actuel (heures)</t>
         </is>
       </c>
-      <c r="C3" s="3" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Actuel (jours)</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Pris (jours)</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Restant (jours)</t>
         </is>
@@ -611,18 +631,21 @@
           <t>CA</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="5" t="n"/>
+      <c r="C4" s="6" t="n"/>
+      <c r="D4" s="7">
+        <f>IF(B4&lt;&gt;"",B4,IF(C4&lt;&gt;"",C4*$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="E4" s="8">
+        <f>IF(C4&lt;&gt;"",C4,IF(B4&lt;&gt;"",B4/$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="F4" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C4" s="6">
-        <f>B4/$B$15</f>
-        <v/>
-      </c>
-      <c r="D4" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E4" s="7">
-        <f>C4-D4</f>
+      <c r="G4" s="8">
+        <f>E4-F4</f>
         <v/>
       </c>
     </row>
@@ -632,18 +655,21 @@
           <t>CA HP</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="5" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="7">
+        <f>IF(B5&lt;&gt;"",B5,IF(C5&lt;&gt;"",C5*$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="E5" s="8">
+        <f>IF(C5&lt;&gt;"",C5,IF(B5&lt;&gt;"",B5/$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="F5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C5" s="6">
-        <f>B5/$B$15</f>
-        <v/>
-      </c>
-      <c r="D5" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E5" s="7">
-        <f>C5-D5</f>
+      <c r="G5" s="8">
+        <f>E5-F5</f>
         <v/>
       </c>
     </row>
@@ -653,18 +679,21 @@
           <t>RTC</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="5" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="7">
+        <f>IF(B6&lt;&gt;"",B6,IF(C6&lt;&gt;"",C6*$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="E6" s="8">
+        <f>IF(C6&lt;&gt;"",C6,IF(B6&lt;&gt;"",B6/$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="F6" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C6" s="6">
-        <f>B6/$B$15</f>
-        <v/>
-      </c>
-      <c r="D6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="7">
-        <f>C6-D6</f>
+      <c r="G6" s="8">
+        <f>E6-F6</f>
         <v/>
       </c>
     </row>
@@ -674,18 +703,21 @@
           <t>CET</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="7">
+        <f>IF(B7&lt;&gt;"",B7,IF(C7&lt;&gt;"",C7*$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="E7" s="8">
+        <f>IF(C7&lt;&gt;"",C7,IF(B7&lt;&gt;"",B7/$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="F7" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C7" s="6">
-        <f>B7/$B$15</f>
-        <v/>
-      </c>
-      <c r="D7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E7" s="7">
-        <f>C7-D7</f>
+      <c r="G7" s="8">
+        <f>E7-F7</f>
         <v/>
       </c>
     </row>
@@ -695,18 +727,21 @@
           <t>CF</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="5" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="7">
+        <f>IF(B8&lt;&gt;"",B8,IF(C8&lt;&gt;"",C8*$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="E8" s="8">
+        <f>IF(C8&lt;&gt;"",C8,IF(B8&lt;&gt;"",B8/$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="F8" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C8" s="6">
-        <f>B8/$B$15</f>
-        <v/>
-      </c>
-      <c r="D8" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E8" s="7">
-        <f>C8-D8</f>
+      <c r="G8" s="8">
+        <f>E8-F8</f>
         <v/>
       </c>
     </row>
@@ -716,18 +751,21 @@
           <t>HS</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="5" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="7">
+        <f>IF(B9&lt;&gt;"",B9,IF(C9&lt;&gt;"",C9*$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="E9" s="8">
+        <f>IF(C9&lt;&gt;"",C9,IF(B9&lt;&gt;"",B9/$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="F9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C9" s="6">
-        <f>B9/$B$15</f>
-        <v/>
-      </c>
-      <c r="D9" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E9" s="7">
-        <f>C9-D9</f>
+      <c r="G9" s="8">
+        <f>E9-F9</f>
         <v/>
       </c>
     </row>
@@ -737,69 +775,74 @@
           <t>RPS</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="5" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="7">
+        <f>IF(B10&lt;&gt;"",B10,IF(C10&lt;&gt;"",C10*$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="E10" s="8">
+        <f>IF(C10&lt;&gt;"",C10,IF(B10&lt;&gt;"",B10/$B$15,0))</f>
+        <v/>
+      </c>
+      <c r="F10" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="C10" s="6">
-        <f>B10/$B$15</f>
-        <v/>
-      </c>
-      <c r="D10" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E10" s="7">
-        <f>C10-D10</f>
+      <c r="G10" s="8">
+        <f>E10-F10</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="9" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="9">
-        <f>SUM(B4:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="10">
-        <f>SUM(C4:C10)</f>
-        <v/>
-      </c>
+      <c r="B11" s="10" t="n"/>
+      <c r="C11" s="11" t="n"/>
       <c r="D11" s="10">
         <f>SUM(D4:D10)</f>
         <v/>
       </c>
-      <c r="E11" s="10">
+      <c r="E11" s="11">
         <f>SUM(E4:E10)</f>
         <v/>
       </c>
+      <c r="F11" s="11">
+        <f>SUM(F4:F10)</f>
+        <v/>
+      </c>
+      <c r="G11" s="11">
+        <f>SUM(G4:G10)</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
-        <is>
-          <t>Cases jaunes : tu peux écrire dedans. Actuel (jours) se calcule depuis les heures si tu n'y touches pas.</t>
+      <c r="A13" s="12" t="inlineStr">
+        <is>
+          <t>Cases jaunes : tape en heures OU en jours. L'autre unité se calcule seule dans les colonnes grises.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="13" t="inlineStr">
         <is>
           <t>1 jour =</t>
         </is>
       </c>
-      <c r="B15" s="13">
+      <c r="B15" s="14">
         <f>12+8/60</f>
         <v/>
       </c>
-      <c r="C15" s="11" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>heures (12h08). Mets 7 pour un jour ouvré.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="11" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Les autres onglets sont une aide au calcul, facultative.</t>
         </is>
@@ -833,31 +876,31 @@
           <t>Mes droits à congés – récapitulatif</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
+      <c r="B1" s="15" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="15" t="n"/>
+      <c r="E1" s="15" t="n"/>
+      <c r="F1" s="15" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Tout se calcule depuis Parametres et Suivi. Ne rien saisir ici.</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="n"/>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="14" t="n"/>
+      <c r="A3" s="15" t="n"/>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -892,244 +935,244 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>CA – Congés annuels</t>
         </is>
       </c>
-      <c r="B5" s="17">
+      <c r="B5" s="18">
         <f>Parametres!$B$9*Parametres!$B$10*Parametres!$B$8</f>
         <v/>
       </c>
-      <c r="C5" s="17">
+      <c r="C5" s="18">
         <f>SUMIF(Suivi!$C$5:$C$204,"CA",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D5" s="18">
+      <c r="D5" s="19">
         <f>B5-C5</f>
         <v/>
       </c>
-      <c r="E5" s="17">
+      <c r="E5" s="18">
         <f>D5/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F5" s="16" t="inlineStr">
+      <c r="F5" s="17" t="inlineStr">
         <is>
           <t>25 j ouvrés × valeur horaire × quotité.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>CA HP – Hors période</t>
         </is>
       </c>
-      <c r="B6" s="17">
+      <c r="B6" s="18">
         <f>IF(Parametres!$B$11&gt;=8,2,IF(Parametres!$B$11&gt;=5,1,0))*Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C6" s="17">
+      <c r="C6" s="18">
         <f>SUMIF(Suivi!$C$5:$C$204,"CA HP",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D6" s="18">
+      <c r="D6" s="19">
         <f>B6-C6</f>
         <v/>
       </c>
-      <c r="E6" s="17">
+      <c r="E6" s="18">
         <f>D6/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F6" s="16" t="inlineStr">
+      <c r="F6" s="17" t="inlineStr">
         <is>
           <t>Bonus : 1 j si 5-7 j CA hors mai-oct ; 2 j si 8 et +.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>RTC</t>
         </is>
       </c>
-      <c r="B7" s="17">
+      <c r="B7" s="18">
         <f>Parametres!$B$12</f>
         <v/>
       </c>
-      <c r="C7" s="17">
+      <c r="C7" s="18">
         <f>SUMIF(Suivi!$C$5:$C$204,"RTC",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D7" s="18">
+      <c r="D7" s="19">
         <f>B7-C7</f>
         <v/>
       </c>
-      <c r="E7" s="17">
+      <c r="E7" s="18">
         <f>D7/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F7" s="16" t="inlineStr">
+      <c r="F7" s="17" t="inlineStr">
         <is>
           <t>Crédit saisi dans Parametres.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>CET – Compte épargne-temps</t>
         </is>
       </c>
-      <c r="B8" s="17">
+      <c r="B8" s="18">
         <f>(Parametres!$B$18+Parametres!$B$19)*Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C8" s="17">
+      <c r="C8" s="18">
         <f>SUMIF(Suivi!$C$5:$C$204,"CET",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D8" s="18">
+      <c r="D8" s="19">
         <f>B8-C8</f>
         <v/>
       </c>
-      <c r="E8" s="17">
+      <c r="E8" s="18">
         <f>D8/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F8" s="16" t="inlineStr">
+      <c r="F8" s="17" t="inlineStr">
         <is>
           <t>Solde 1er janvier + jours versés.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>CF – Crédit férié</t>
         </is>
       </c>
-      <c r="B9" s="17">
+      <c r="B9" s="18">
         <f>Parametres!$B$13*Parametres!$B$14</f>
         <v/>
       </c>
-      <c r="C9" s="17">
+      <c r="C9" s="18">
         <f>SUMIF(Suivi!$C$5:$C$204,"CF",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D9" s="18">
+      <c r="D9" s="19">
         <f>B9-C9</f>
         <v/>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="18">
         <f>D9/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F9" s="16" t="inlineStr">
+      <c r="F9" s="17" t="inlineStr">
         <is>
           <t>Nb fériés × heures par férié.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>HS – Heures supplémentaires</t>
         </is>
       </c>
-      <c r="B10" s="17">
+      <c r="B10" s="18">
         <f>Parametres!$B$15</f>
         <v/>
       </c>
-      <c r="C10" s="17">
+      <c r="C10" s="18">
         <f>SUMIF(Suivi!$C$5:$C$204,"HS",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D10" s="18">
+      <c r="D10" s="19">
         <f>B10-C10</f>
         <v/>
       </c>
-      <c r="E10" s="17">
+      <c r="E10" s="18">
         <f>D10/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F10" s="16" t="inlineStr">
+      <c r="F10" s="17" t="inlineStr">
         <is>
           <t>Compteur HS récupérables.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>RPS – Repos pénibilité nuit</t>
         </is>
       </c>
-      <c r="B11" s="17">
+      <c r="B11" s="18">
         <f>IF(Parametres!$B$17&gt;0,Parametres!$B$17,ROUND(140*Parametres!$B$8,0))*Parametres!$B$7*Parametres!$B$16</f>
         <v/>
       </c>
-      <c r="C11" s="17">
+      <c r="C11" s="18">
         <f>SUMIF(Suivi!$C$5:$C$204,"RPS",Suivi!$E$5:$E$204)</f>
         <v/>
       </c>
-      <c r="D11" s="18">
+      <c r="D11" s="19">
         <f>B11-C11</f>
         <v/>
       </c>
-      <c r="E11" s="17">
+      <c r="E11" s="18">
         <f>D11/Parametres!$B$6</f>
         <v/>
       </c>
-      <c r="F11" s="16" t="inlineStr">
+      <c r="F11" s="17" t="inlineStr">
         <is>
           <t>Vacations nuit × heures nuit × coef.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="19" t="inlineStr">
+      <c r="A12" s="20" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="20">
+      <c r="B12" s="21">
         <f>SUM(B5:B11)</f>
         <v/>
       </c>
-      <c r="C12" s="20">
+      <c r="C12" s="21">
         <f>SUM(C5:C11)</f>
         <v/>
       </c>
-      <c r="D12" s="20">
+      <c r="D12" s="21">
         <f>SUM(D5:D11)</f>
         <v/>
       </c>
-      <c r="E12" s="20">
+      <c r="E12" s="21">
         <f>SUM(E5:E11)</f>
         <v/>
       </c>
-      <c r="F12" s="19" t="n"/>
+      <c r="F12" s="20" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="n"/>
-      <c r="B13" s="14" t="n"/>
-      <c r="C13" s="14" t="n"/>
-      <c r="D13" s="14" t="n"/>
-      <c r="E13" s="14" t="n"/>
-      <c r="F13" s="14" t="n"/>
+      <c r="A13" s="15" t="n"/>
+      <c r="B13" s="15" t="n"/>
+      <c r="C13" s="15" t="n"/>
+      <c r="D13" s="15" t="n"/>
+      <c r="E13" s="15" t="n"/>
+      <c r="F13" s="15" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>CET – détail</t>
         </is>
       </c>
-      <c r="B14" s="14" t="n"/>
-      <c r="C14" s="14" t="n"/>
-      <c r="D14" s="14" t="n"/>
-      <c r="E14" s="14" t="n"/>
-      <c r="F14" s="14" t="n"/>
+      <c r="B14" s="15" t="n"/>
+      <c r="C14" s="15" t="n"/>
+      <c r="D14" s="15" t="n"/>
+      <c r="E14" s="15" t="n"/>
+      <c r="F14" s="15" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
@@ -1152,134 +1195,134 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>Jours CA pris dans l'année</t>
         </is>
       </c>
-      <c r="B16" s="22">
+      <c r="B16" s="23">
         <f>C5/Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C16" s="14" t="n"/>
-      <c r="D16" s="14" t="n"/>
-      <c r="E16" s="14" t="n"/>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="C16" s="15" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="15" t="n"/>
+      <c r="F16" s="15" t="inlineStr">
         <is>
           <t>Depuis Suivi.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>Jours épargnables max</t>
         </is>
       </c>
-      <c r="B17" s="22">
+      <c r="B17" s="23">
         <f>MAX(0,MIN((B5+B6-C5-C6)/Parametres!$B$10,(B5+B6)/Parametres!$B$10-20))</f>
         <v/>
       </c>
-      <c r="C17" s="14" t="n"/>
-      <c r="D17" s="14" t="n"/>
-      <c r="E17" s="14" t="n"/>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="C17" s="15" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="15" t="n"/>
+      <c r="F17" s="15" t="inlineStr">
         <is>
           <t>20 j de CA obligatoires. Le reliquat est épargnable.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>Solde CET restant (jours)</t>
         </is>
       </c>
-      <c r="B18" s="22">
+      <c r="B18" s="23">
         <f>D8/Parametres!$B$10</f>
         <v/>
       </c>
-      <c r="C18" s="14" t="n"/>
-      <c r="D18" s="14" t="n"/>
-      <c r="E18" s="14" t="n"/>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="C18" s="15" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="15" t="n"/>
+      <c r="F18" s="15" t="inlineStr">
         <is>
           <t>Plafond 60 jours.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>Alerte plafond</t>
         </is>
       </c>
-      <c r="B19" s="22">
+      <c r="B19" s="23">
         <f>IF(B18&gt;60,"Plafond 60 j dépassé","OK")</f>
         <v/>
       </c>
-      <c r="C19" s="14" t="n"/>
-      <c r="D19" s="14" t="n"/>
-      <c r="E19" s="14" t="n"/>
-      <c r="F19" s="14" t="inlineStr"/>
+      <c r="C19" s="15" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="15" t="n"/>
+      <c r="F19" s="15" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Jours indemnisables (au-delà de 15)</t>
         </is>
       </c>
-      <c r="B20" s="22">
+      <c r="B20" s="23">
         <f>MAX(0,MIN(B18,60)-15)</f>
         <v/>
       </c>
-      <c r="C20" s="14" t="n"/>
-      <c r="D20" s="14" t="n"/>
-      <c r="E20" s="14" t="n"/>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="C20" s="15" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="15" t="n"/>
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>Option possible au-delà de 15 j.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Valeur si indemnisés (€)</t>
         </is>
       </c>
-      <c r="B21" s="23">
+      <c r="B21" s="24">
         <f>B20*IF(Parametres!$B$20="A",Parametres!$B$23,IF(Parametres!$B$20="B",Parametres!$B$22,Parametres!$B$21))</f>
         <v/>
       </c>
-      <c r="C21" s="14" t="n"/>
-      <c r="D21" s="14" t="n"/>
-      <c r="E21" s="14" t="n"/>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="C21" s="15" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="15" t="n"/>
+      <c r="F21" s="15" t="inlineStr">
         <is>
           <t>Montant brut selon catégorie.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="14" t="n"/>
-      <c r="B22" s="14" t="n"/>
-      <c r="C22" s="14" t="n"/>
-      <c r="D22" s="14" t="n"/>
-      <c r="E22" s="14" t="n"/>
-      <c r="F22" s="14" t="n"/>
+      <c r="A22" s="15" t="n"/>
+      <c r="B22" s="15" t="n"/>
+      <c r="C22" s="15" t="n"/>
+      <c r="D22" s="15" t="n"/>
+      <c r="E22" s="15" t="n"/>
+      <c r="F22" s="15" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="21" t="inlineStr">
+      <c r="A23" s="22" t="inlineStr">
         <is>
           <t>ASA – Autorisations spéciales d'absence (hors compteur)</t>
         </is>
       </c>
-      <c r="B23" s="14" t="n"/>
-      <c r="C23" s="14" t="n"/>
-      <c r="D23" s="14" t="n"/>
-      <c r="E23" s="14" t="n"/>
-      <c r="F23" s="14" t="n"/>
+      <c r="B23" s="15" t="n"/>
+      <c r="C23" s="15" t="n"/>
+      <c r="D23" s="15" t="n"/>
+      <c r="E23" s="15" t="n"/>
+      <c r="F23" s="15" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
@@ -1302,119 +1345,119 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Garde d'enfant malade</t>
         </is>
       </c>
-      <c r="B25" s="24">
+      <c r="B25" s="25">
         <f>IF(Parametres!$B$24="O",IF(Parametres!$B$25="O",12,6)*Parametres!$B$8,0)</f>
         <v/>
       </c>
-      <c r="C25" s="14" t="n"/>
-      <c r="D25" s="14" t="n"/>
-      <c r="E25" s="14" t="n"/>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="C25" s="15" t="n"/>
+      <c r="D25" s="15" t="n"/>
+      <c r="E25" s="15" t="n"/>
+      <c r="F25" s="15" t="inlineStr">
         <is>
           <t>6 j/an ; 12 j si seul ou conjoint sans droit. À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Mariage / PACS de l'agent</t>
         </is>
       </c>
-      <c r="B26" s="24" t="n">
+      <c r="B26" s="25" t="n">
         <v>5</v>
       </c>
-      <c r="C26" s="14" t="n"/>
-      <c r="D26" s="14" t="n"/>
-      <c r="E26" s="14" t="n"/>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="C26" s="15" t="n"/>
+      <c r="D26" s="15" t="n"/>
+      <c r="E26" s="15" t="n"/>
+      <c r="F26" s="15" t="inlineStr">
         <is>
           <t>Barème FP. À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="16" t="inlineStr">
+      <c r="A27" s="17" t="inlineStr">
         <is>
           <t>Décès conjoint / parent / enfant</t>
         </is>
       </c>
-      <c r="B27" s="24" t="n">
+      <c r="B27" s="25" t="n">
         <v>3</v>
       </c>
-      <c r="C27" s="14" t="n"/>
-      <c r="D27" s="14" t="n"/>
-      <c r="E27" s="14" t="n"/>
-      <c r="F27" s="14" t="inlineStr">
+      <c r="C27" s="15" t="n"/>
+      <c r="D27" s="15" t="n"/>
+      <c r="E27" s="15" t="n"/>
+      <c r="F27" s="15" t="inlineStr">
         <is>
           <t>Barème FP. Enfant : régime renforcé.</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="16" t="inlineStr">
+      <c r="A28" s="17" t="inlineStr">
         <is>
           <t>Naissance / adoption</t>
         </is>
       </c>
-      <c r="B28" s="24" t="inlineStr">
+      <c r="B28" s="25" t="inlineStr">
         <is>
           <t>Voir RH</t>
         </is>
       </c>
-      <c r="C28" s="14" t="n"/>
-      <c r="D28" s="14" t="n"/>
-      <c r="E28" s="14" t="n"/>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="C28" s="15" t="n"/>
+      <c r="D28" s="15" t="n"/>
+      <c r="E28" s="15" t="n"/>
+      <c r="F28" s="15" t="inlineStr">
         <is>
           <t>Congé naissance 3 j + paternité 25 j.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="16" t="inlineStr">
+      <c r="A29" s="17" t="inlineStr">
         <is>
           <t>Déménagement</t>
         </is>
       </c>
-      <c r="B29" s="24" t="inlineStr">
+      <c r="B29" s="25" t="inlineStr">
         <is>
           <t>Voir RH</t>
         </is>
       </c>
-      <c r="C29" s="14" t="n"/>
-      <c r="D29" s="14" t="n"/>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="14" t="inlineStr">
+      <c r="C29" s="15" t="n"/>
+      <c r="D29" s="15" t="n"/>
+      <c r="E29" s="15" t="n"/>
+      <c r="F29" s="15" t="inlineStr">
         <is>
           <t>Selon note de service.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="14" t="n"/>
-      <c r="B30" s="14" t="n"/>
-      <c r="C30" s="14" t="n"/>
-      <c r="D30" s="14" t="n"/>
-      <c r="E30" s="14" t="n"/>
-      <c r="F30" s="14" t="n"/>
+      <c r="A30" s="15" t="n"/>
+      <c r="B30" s="15" t="n"/>
+      <c r="C30" s="15" t="n"/>
+      <c r="D30" s="15" t="n"/>
+      <c r="E30" s="15" t="n"/>
+      <c r="F30" s="15" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="25" t="inlineStr">
+      <c r="A31" s="26" t="inlineStr">
         <is>
           <t>Les montants et barèmes sont indicatifs. Vérifie avec ton secrétariat / Géopol et ta note de service locale.</t>
         </is>
       </c>
-      <c r="B31" s="14" t="n"/>
-      <c r="C31" s="14" t="n"/>
-      <c r="D31" s="14" t="n"/>
-      <c r="E31" s="14" t="n"/>
-      <c r="F31" s="14" t="n"/>
+      <c r="B31" s="15" t="n"/>
+      <c r="C31" s="15" t="n"/>
+      <c r="D31" s="15" t="n"/>
+      <c r="E31" s="15" t="n"/>
+      <c r="F31" s="15" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1441,22 +1484,22 @@
           <t>Paramètres – Police nationale, cycle 12h08 de nuit</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
+      <c r="B1" s="15" t="n"/>
+      <c r="C1" s="15" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Cellules jaunes / texte bleu = à saisir. Le reste se calcule seul.</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="n"/>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
+      <c r="A3" s="15" t="n"/>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1476,339 +1519,339 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="16" t="inlineStr">
+      <c r="A5" s="17" t="inlineStr">
         <is>
           <t>Année de référence</t>
         </is>
       </c>
-      <c r="B5" s="26" t="n">
+      <c r="B5" s="27" t="n">
         <v>2026</v>
       </c>
-      <c r="C5" s="27" t="inlineStr">
+      <c r="C5" s="28" t="inlineStr">
         <is>
           <t>Année civile des droits.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="16" t="inlineStr">
+      <c r="A6" s="17" t="inlineStr">
         <is>
           <t>Durée d'une vacation (heures)</t>
         </is>
       </c>
-      <c r="B6" s="22">
+      <c r="B6" s="23">
         <f>12+8/60</f>
         <v/>
       </c>
-      <c r="C6" s="27" t="inlineStr">
+      <c r="C6" s="28" t="inlineStr">
         <is>
           <t>12h08 = 12,13 h, dont 2 pauses de 20 min (rapport Sénat).</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="16" t="inlineStr">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Heures de nuit par vacation</t>
         </is>
       </c>
-      <c r="B7" s="13" t="n">
+      <c r="B7" s="14" t="n">
         <v>9</v>
       </c>
-      <c r="C7" s="27" t="inlineStr">
+      <c r="C7" s="28" t="inlineStr">
         <is>
           <t>Heures entre 21h et 6h (RGEMPN). 9h si vacation couvre toute la plage.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="16" t="inlineStr">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Quotité de travail</t>
         </is>
       </c>
-      <c r="B8" s="28" t="n">
+      <c r="B8" s="29" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="27" t="inlineStr">
+      <c r="C8" s="28" t="inlineStr">
         <is>
           <t>100 % = temps plein.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="16" t="inlineStr">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>CA – jours ouvrés réglementaires</t>
         </is>
       </c>
-      <c r="B9" s="26" t="n">
+      <c r="B9" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="C9" s="27" t="inlineStr">
+      <c r="C9" s="28" t="inlineStr">
         <is>
           <t>Décret 84-972 : 25 jours ouvrés.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="16" t="inlineStr">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>Valeur horaire d'1 jour de CA (h)</t>
         </is>
       </c>
-      <c r="B10" s="13" t="n">
+      <c r="B10" s="14" t="n">
         <v>7</v>
       </c>
-      <c r="C10" s="27" t="inlineStr">
+      <c r="C10" s="28" t="inlineStr">
         <is>
           <t>À vérifier avec ton secrétariat / Géopol.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="16" t="inlineStr">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>CA HP – jours CA pris hors 1/05–31/10</t>
         </is>
       </c>
-      <c r="B11" s="26" t="n">
+      <c r="B11" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C11" s="27" t="inlineStr">
+      <c r="C11" s="28" t="inlineStr">
         <is>
           <t>5 à 7 j = 1 j bonus ; 8 j et + = 2 j bonus.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="16" t="inlineStr">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>RTC – crédit annuel (heures)</t>
         </is>
       </c>
-      <c r="B12" s="13" t="n">
+      <c r="B12" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C12" s="27" t="inlineStr">
+      <c r="C12" s="28" t="inlineStr">
         <is>
           <t>Crédit annuel horaire d'ARTT en régime cyclique (RGEMPN art. 39). Voir Géopol.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="16" t="inlineStr">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>CF – nombre de fériés crédités</t>
         </is>
       </c>
-      <c r="B13" s="26" t="n">
+      <c r="B13" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C13" s="27" t="inlineStr">
+      <c r="C13" s="28" t="inlineStr">
         <is>
           <t>Crédit férié annuel, en heures, pour régime cyclique. Voir Géopol.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="16" t="inlineStr">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>CF – heures par férié</t>
         </is>
       </c>
-      <c r="B14" s="22">
+      <c r="B14" s="23">
         <f>B6</f>
         <v/>
       </c>
-      <c r="C14" s="27" t="inlineStr">
+      <c r="C14" s="28" t="inlineStr">
         <is>
           <t>Par défaut = 1 vacation. Modifiable.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="16" t="inlineStr">
+      <c r="A15" s="17" t="inlineStr">
         <is>
           <t>HS – heures sup. au compteur (heures)</t>
         </is>
       </c>
-      <c r="B15" s="13" t="n">
+      <c r="B15" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C15" s="27" t="inlineStr">
+      <c r="C15" s="28" t="inlineStr">
         <is>
           <t>Solde HS récupérables. Voir relevé.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="16" t="inlineStr">
+      <c r="A16" s="17" t="inlineStr">
         <is>
           <t>RPS – coef. sur heures de nuit</t>
         </is>
       </c>
-      <c r="B16" s="28" t="n">
+      <c r="B16" s="29" t="n">
         <v>0.1</v>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C16" s="28" t="inlineStr">
         <is>
           <t>0,1 par heure de nuit 21h-6h (0,4 dimanche, non cumulable). Source : RGEMPN.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="16" t="inlineStr">
+      <c r="A17" s="17" t="inlineStr">
         <is>
           <t>RPS – vacations de nuit / an</t>
         </is>
       </c>
-      <c r="B17" s="26" t="n">
+      <c r="B17" s="27" t="n">
         <v>0</v>
       </c>
-      <c r="C17" s="27" t="inlineStr">
+      <c r="C17" s="28" t="inlineStr">
         <is>
           <t>0 = 140 vacations/an (cycle binaire, rapport Sénat).</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="16" t="inlineStr">
+      <c r="A18" s="17" t="inlineStr">
         <is>
           <t>CET – solde au 1er janvier (jours)</t>
         </is>
       </c>
-      <c r="B18" s="13" t="n">
+      <c r="B18" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C18" s="27" t="inlineStr">
+      <c r="C18" s="28" t="inlineStr">
         <is>
           <t>Repris de ton relevé CET.</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="16" t="inlineStr">
+      <c r="A19" s="17" t="inlineStr">
         <is>
           <t>CET – jours versés cette année</t>
         </is>
       </c>
-      <c r="B19" s="13" t="n">
+      <c r="B19" s="14" t="n">
         <v>0</v>
       </c>
-      <c r="C19" s="27" t="inlineStr">
+      <c r="C19" s="28" t="inlineStr">
         <is>
           <t>Ta demande d'alimentation.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="16" t="inlineStr">
+      <c r="A20" s="17" t="inlineStr">
         <is>
           <t>Catégorie (C, B, A)</t>
         </is>
       </c>
-      <c r="B20" s="29" t="inlineStr">
+      <c r="B20" s="30" t="inlineStr">
         <is>
           <t>B</t>
         </is>
       </c>
-      <c r="C20" s="27" t="inlineStr">
+      <c r="C20" s="28" t="inlineStr">
         <is>
           <t>Pour l'indemnisation CET.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="16" t="inlineStr">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Taux CET catégorie C (€/jour)</t>
         </is>
       </c>
-      <c r="B21" s="30" t="n">
+      <c r="B21" s="31" t="n">
         <v>83</v>
       </c>
-      <c r="C21" s="27" t="inlineStr">
+      <c r="C21" s="28" t="inlineStr">
         <is>
           <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="16" t="inlineStr">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Taux CET catégorie B (€/jour)</t>
         </is>
       </c>
-      <c r="B22" s="30" t="n">
+      <c r="B22" s="31" t="n">
         <v>100</v>
       </c>
-      <c r="C22" s="27" t="inlineStr">
+      <c r="C22" s="28" t="inlineStr">
         <is>
           <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="16" t="inlineStr">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Taux CET catégorie A (€/jour)</t>
         </is>
       </c>
-      <c r="B23" s="30" t="n">
+      <c r="B23" s="31" t="n">
         <v>150</v>
       </c>
-      <c r="C23" s="27" t="inlineStr">
+      <c r="C23" s="28" t="inlineStr">
         <is>
           <t>À vérifier.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="16" t="inlineStr">
+      <c r="A24" s="17" t="inlineStr">
         <is>
           <t>Enfants à charge &lt; 16 ans (O/N)</t>
         </is>
       </c>
-      <c r="B24" s="29" t="inlineStr">
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t>O</t>
         </is>
       </c>
-      <c r="C24" s="27" t="inlineStr">
+      <c r="C24" s="28" t="inlineStr">
         <is>
           <t>Pour ASA garde d'enfant.</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="16" t="inlineStr">
+      <c r="A25" s="17" t="inlineStr">
         <is>
           <t>Élève seul l'enfant ou conjoint sans droit (O/N)</t>
         </is>
       </c>
-      <c r="B25" s="29" t="inlineStr">
+      <c r="B25" s="30" t="inlineStr">
         <is>
           <t>N</t>
         </is>
       </c>
-      <c r="C25" s="27" t="inlineStr">
+      <c r="C25" s="28" t="inlineStr">
         <is>
           <t>Doublement ASA garde d'enfant.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="16" t="inlineStr">
+      <c r="A26" s="17" t="inlineStr">
         <is>
           <t>Durée d'un jour dans le Tableau (h)</t>
         </is>
       </c>
-      <c r="B26" s="22">
+      <c r="B26" s="23">
         <f>B6</f>
         <v/>
       </c>
-      <c r="C26" s="27" t="inlineStr">
+      <c r="C26" s="28" t="inlineStr">
         <is>
           <t>Par défaut 1 jour = 1 vacation de 12h08. Mets 7 pour des jours ouvrés.</t>
         </is>
@@ -1850,31 +1893,31 @@
           <t>Journal des absences posées</t>
         </is>
       </c>
-      <c r="B1" s="14" t="n"/>
-      <c r="C1" s="14" t="n"/>
-      <c r="D1" s="14" t="n"/>
-      <c r="E1" s="14" t="n"/>
-      <c r="F1" s="14" t="n"/>
+      <c r="B1" s="15" t="n"/>
+      <c r="C1" s="15" t="n"/>
+      <c r="D1" s="15" t="n"/>
+      <c r="E1" s="15" t="n"/>
+      <c r="F1" s="15" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" s="15" t="inlineStr">
+      <c r="A2" s="16" t="inlineStr">
         <is>
           <t>Une ligne par absence. Choisis le type dans la liste. Heures calculées seules.</t>
         </is>
       </c>
-      <c r="B2" s="14" t="n"/>
-      <c r="C2" s="14" t="n"/>
-      <c r="D2" s="14" t="n"/>
-      <c r="E2" s="14" t="n"/>
-      <c r="F2" s="14" t="n"/>
+      <c r="B2" s="15" t="n"/>
+      <c r="C2" s="15" t="n"/>
+      <c r="D2" s="15" t="n"/>
+      <c r="E2" s="15" t="n"/>
+      <c r="F2" s="15" t="n"/>
     </row>
     <row r="3">
-      <c r="A3" s="14" t="n"/>
-      <c r="B3" s="14" t="n"/>
-      <c r="C3" s="14" t="n"/>
-      <c r="D3" s="14" t="n"/>
-      <c r="E3" s="14" t="n"/>
-      <c r="F3" s="14" t="n"/>
+      <c r="A3" s="15" t="n"/>
+      <c r="B3" s="15" t="n"/>
+      <c r="C3" s="15" t="n"/>
+      <c r="D3" s="15" t="n"/>
+      <c r="E3" s="15" t="n"/>
+      <c r="F3" s="15" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1909,2218 +1952,2218 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="31" t="n">
+      <c r="A5" s="32" t="n">
         <v>46063</v>
       </c>
-      <c r="B5" s="31" t="n">
+      <c r="B5" s="32" t="n">
         <v>46066</v>
       </c>
-      <c r="C5" s="32" t="inlineStr">
+      <c r="C5" s="33" t="inlineStr">
         <is>
           <t>CA</t>
         </is>
       </c>
-      <c r="D5" s="32" t="n">
+      <c r="D5" s="33" t="n">
         <v>2</v>
       </c>
-      <c r="E5" s="22">
+      <c r="E5" s="23">
         <f>IF(D5="","",D5*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F5" s="32" t="inlineStr">
+      <c r="F5" s="33" t="inlineStr">
         <is>
           <t>Exemple – à effacer</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="31" t="n"/>
-      <c r="B6" s="31" t="n"/>
-      <c r="C6" s="32" t="n"/>
-      <c r="D6" s="32" t="n"/>
-      <c r="E6" s="22">
+      <c r="A6" s="32" t="n"/>
+      <c r="B6" s="32" t="n"/>
+      <c r="C6" s="33" t="n"/>
+      <c r="D6" s="33" t="n"/>
+      <c r="E6" s="23">
         <f>IF(D6="","",D6*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F6" s="32" t="n"/>
+      <c r="F6" s="33" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="31" t="n"/>
-      <c r="B7" s="31" t="n"/>
-      <c r="C7" s="32" t="n"/>
-      <c r="D7" s="32" t="n"/>
-      <c r="E7" s="22">
+      <c r="A7" s="32" t="n"/>
+      <c r="B7" s="32" t="n"/>
+      <c r="C7" s="33" t="n"/>
+      <c r="D7" s="33" t="n"/>
+      <c r="E7" s="23">
         <f>IF(D7="","",D7*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F7" s="32" t="n"/>
+      <c r="F7" s="33" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="31" t="n"/>
-      <c r="B8" s="31" t="n"/>
-      <c r="C8" s="32" t="n"/>
-      <c r="D8" s="32" t="n"/>
-      <c r="E8" s="22">
+      <c r="A8" s="32" t="n"/>
+      <c r="B8" s="32" t="n"/>
+      <c r="C8" s="33" t="n"/>
+      <c r="D8" s="33" t="n"/>
+      <c r="E8" s="23">
         <f>IF(D8="","",D8*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F8" s="32" t="n"/>
+      <c r="F8" s="33" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="31" t="n"/>
-      <c r="B9" s="31" t="n"/>
-      <c r="C9" s="32" t="n"/>
-      <c r="D9" s="32" t="n"/>
-      <c r="E9" s="22">
+      <c r="A9" s="32" t="n"/>
+      <c r="B9" s="32" t="n"/>
+      <c r="C9" s="33" t="n"/>
+      <c r="D9" s="33" t="n"/>
+      <c r="E9" s="23">
         <f>IF(D9="","",D9*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F9" s="32" t="n"/>
+      <c r="F9" s="33" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="31" t="n"/>
-      <c r="B10" s="31" t="n"/>
-      <c r="C10" s="32" t="n"/>
-      <c r="D10" s="32" t="n"/>
-      <c r="E10" s="22">
+      <c r="A10" s="32" t="n"/>
+      <c r="B10" s="32" t="n"/>
+      <c r="C10" s="33" t="n"/>
+      <c r="D10" s="33" t="n"/>
+      <c r="E10" s="23">
         <f>IF(D10="","",D10*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F10" s="32" t="n"/>
+      <c r="F10" s="33" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="31" t="n"/>
-      <c r="B11" s="31" t="n"/>
-      <c r="C11" s="32" t="n"/>
-      <c r="D11" s="32" t="n"/>
-      <c r="E11" s="22">
+      <c r="A11" s="32" t="n"/>
+      <c r="B11" s="32" t="n"/>
+      <c r="C11" s="33" t="n"/>
+      <c r="D11" s="33" t="n"/>
+      <c r="E11" s="23">
         <f>IF(D11="","",D11*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F11" s="32" t="n"/>
+      <c r="F11" s="33" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="31" t="n"/>
-      <c r="B12" s="31" t="n"/>
-      <c r="C12" s="32" t="n"/>
-      <c r="D12" s="32" t="n"/>
-      <c r="E12" s="22">
+      <c r="A12" s="32" t="n"/>
+      <c r="B12" s="32" t="n"/>
+      <c r="C12" s="33" t="n"/>
+      <c r="D12" s="33" t="n"/>
+      <c r="E12" s="23">
         <f>IF(D12="","",D12*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F12" s="32" t="n"/>
+      <c r="F12" s="33" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="31" t="n"/>
-      <c r="B13" s="31" t="n"/>
-      <c r="C13" s="32" t="n"/>
-      <c r="D13" s="32" t="n"/>
-      <c r="E13" s="22">
+      <c r="A13" s="32" t="n"/>
+      <c r="B13" s="32" t="n"/>
+      <c r="C13" s="33" t="n"/>
+      <c r="D13" s="33" t="n"/>
+      <c r="E13" s="23">
         <f>IF(D13="","",D13*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F13" s="32" t="n"/>
+      <c r="F13" s="33" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="31" t="n"/>
-      <c r="B14" s="31" t="n"/>
-      <c r="C14" s="32" t="n"/>
-      <c r="D14" s="32" t="n"/>
-      <c r="E14" s="22">
+      <c r="A14" s="32" t="n"/>
+      <c r="B14" s="32" t="n"/>
+      <c r="C14" s="33" t="n"/>
+      <c r="D14" s="33" t="n"/>
+      <c r="E14" s="23">
         <f>IF(D14="","",D14*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F14" s="32" t="n"/>
+      <c r="F14" s="33" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="31" t="n"/>
-      <c r="B15" s="31" t="n"/>
-      <c r="C15" s="32" t="n"/>
-      <c r="D15" s="32" t="n"/>
-      <c r="E15" s="22">
+      <c r="A15" s="32" t="n"/>
+      <c r="B15" s="32" t="n"/>
+      <c r="C15" s="33" t="n"/>
+      <c r="D15" s="33" t="n"/>
+      <c r="E15" s="23">
         <f>IF(D15="","",D15*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F15" s="32" t="n"/>
+      <c r="F15" s="33" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="31" t="n"/>
-      <c r="B16" s="31" t="n"/>
-      <c r="C16" s="32" t="n"/>
-      <c r="D16" s="32" t="n"/>
-      <c r="E16" s="22">
+      <c r="A16" s="32" t="n"/>
+      <c r="B16" s="32" t="n"/>
+      <c r="C16" s="33" t="n"/>
+      <c r="D16" s="33" t="n"/>
+      <c r="E16" s="23">
         <f>IF(D16="","",D16*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F16" s="32" t="n"/>
+      <c r="F16" s="33" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="31" t="n"/>
-      <c r="B17" s="31" t="n"/>
-      <c r="C17" s="32" t="n"/>
-      <c r="D17" s="32" t="n"/>
-      <c r="E17" s="22">
+      <c r="A17" s="32" t="n"/>
+      <c r="B17" s="32" t="n"/>
+      <c r="C17" s="33" t="n"/>
+      <c r="D17" s="33" t="n"/>
+      <c r="E17" s="23">
         <f>IF(D17="","",D17*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F17" s="32" t="n"/>
+      <c r="F17" s="33" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="31" t="n"/>
-      <c r="B18" s="31" t="n"/>
-      <c r="C18" s="32" t="n"/>
-      <c r="D18" s="32" t="n"/>
-      <c r="E18" s="22">
+      <c r="A18" s="32" t="n"/>
+      <c r="B18" s="32" t="n"/>
+      <c r="C18" s="33" t="n"/>
+      <c r="D18" s="33" t="n"/>
+      <c r="E18" s="23">
         <f>IF(D18="","",D18*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F18" s="32" t="n"/>
+      <c r="F18" s="33" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="31" t="n"/>
-      <c r="B19" s="31" t="n"/>
-      <c r="C19" s="32" t="n"/>
-      <c r="D19" s="32" t="n"/>
-      <c r="E19" s="22">
+      <c r="A19" s="32" t="n"/>
+      <c r="B19" s="32" t="n"/>
+      <c r="C19" s="33" t="n"/>
+      <c r="D19" s="33" t="n"/>
+      <c r="E19" s="23">
         <f>IF(D19="","",D19*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F19" s="32" t="n"/>
+      <c r="F19" s="33" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="31" t="n"/>
-      <c r="B20" s="31" t="n"/>
-      <c r="C20" s="32" t="n"/>
-      <c r="D20" s="32" t="n"/>
-      <c r="E20" s="22">
+      <c r="A20" s="32" t="n"/>
+      <c r="B20" s="32" t="n"/>
+      <c r="C20" s="33" t="n"/>
+      <c r="D20" s="33" t="n"/>
+      <c r="E20" s="23">
         <f>IF(D20="","",D20*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F20" s="32" t="n"/>
+      <c r="F20" s="33" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="31" t="n"/>
-      <c r="B21" s="31" t="n"/>
-      <c r="C21" s="32" t="n"/>
-      <c r="D21" s="32" t="n"/>
-      <c r="E21" s="22">
+      <c r="A21" s="32" t="n"/>
+      <c r="B21" s="32" t="n"/>
+      <c r="C21" s="33" t="n"/>
+      <c r="D21" s="33" t="n"/>
+      <c r="E21" s="23">
         <f>IF(D21="","",D21*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F21" s="32" t="n"/>
+      <c r="F21" s="33" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="31" t="n"/>
-      <c r="B22" s="31" t="n"/>
-      <c r="C22" s="32" t="n"/>
-      <c r="D22" s="32" t="n"/>
-      <c r="E22" s="22">
+      <c r="A22" s="32" t="n"/>
+      <c r="B22" s="32" t="n"/>
+      <c r="C22" s="33" t="n"/>
+      <c r="D22" s="33" t="n"/>
+      <c r="E22" s="23">
         <f>IF(D22="","",D22*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F22" s="32" t="n"/>
+      <c r="F22" s="33" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="31" t="n"/>
-      <c r="B23" s="31" t="n"/>
-      <c r="C23" s="32" t="n"/>
-      <c r="D23" s="32" t="n"/>
-      <c r="E23" s="22">
+      <c r="A23" s="32" t="n"/>
+      <c r="B23" s="32" t="n"/>
+      <c r="C23" s="33" t="n"/>
+      <c r="D23" s="33" t="n"/>
+      <c r="E23" s="23">
         <f>IF(D23="","",D23*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F23" s="32" t="n"/>
+      <c r="F23" s="33" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="31" t="n"/>
-      <c r="B24" s="31" t="n"/>
-      <c r="C24" s="32" t="n"/>
-      <c r="D24" s="32" t="n"/>
-      <c r="E24" s="22">
+      <c r="A24" s="32" t="n"/>
+      <c r="B24" s="32" t="n"/>
+      <c r="C24" s="33" t="n"/>
+      <c r="D24" s="33" t="n"/>
+      <c r="E24" s="23">
         <f>IF(D24="","",D24*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F24" s="32" t="n"/>
+      <c r="F24" s="33" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="31" t="n"/>
-      <c r="B25" s="31" t="n"/>
-      <c r="C25" s="32" t="n"/>
-      <c r="D25" s="32" t="n"/>
-      <c r="E25" s="22">
+      <c r="A25" s="32" t="n"/>
+      <c r="B25" s="32" t="n"/>
+      <c r="C25" s="33" t="n"/>
+      <c r="D25" s="33" t="n"/>
+      <c r="E25" s="23">
         <f>IF(D25="","",D25*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F25" s="32" t="n"/>
+      <c r="F25" s="33" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="31" t="n"/>
-      <c r="B26" s="31" t="n"/>
-      <c r="C26" s="32" t="n"/>
-      <c r="D26" s="32" t="n"/>
-      <c r="E26" s="22">
+      <c r="A26" s="32" t="n"/>
+      <c r="B26" s="32" t="n"/>
+      <c r="C26" s="33" t="n"/>
+      <c r="D26" s="33" t="n"/>
+      <c r="E26" s="23">
         <f>IF(D26="","",D26*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F26" s="32" t="n"/>
+      <c r="F26" s="33" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="31" t="n"/>
-      <c r="B27" s="31" t="n"/>
-      <c r="C27" s="32" t="n"/>
-      <c r="D27" s="32" t="n"/>
-      <c r="E27" s="22">
+      <c r="A27" s="32" t="n"/>
+      <c r="B27" s="32" t="n"/>
+      <c r="C27" s="33" t="n"/>
+      <c r="D27" s="33" t="n"/>
+      <c r="E27" s="23">
         <f>IF(D27="","",D27*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F27" s="32" t="n"/>
+      <c r="F27" s="33" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="31" t="n"/>
-      <c r="B28" s="31" t="n"/>
-      <c r="C28" s="32" t="n"/>
-      <c r="D28" s="32" t="n"/>
-      <c r="E28" s="22">
+      <c r="A28" s="32" t="n"/>
+      <c r="B28" s="32" t="n"/>
+      <c r="C28" s="33" t="n"/>
+      <c r="D28" s="33" t="n"/>
+      <c r="E28" s="23">
         <f>IF(D28="","",D28*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F28" s="32" t="n"/>
+      <c r="F28" s="33" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="31" t="n"/>
-      <c r="B29" s="31" t="n"/>
-      <c r="C29" s="32" t="n"/>
-      <c r="D29" s="32" t="n"/>
-      <c r="E29" s="22">
+      <c r="A29" s="32" t="n"/>
+      <c r="B29" s="32" t="n"/>
+      <c r="C29" s="33" t="n"/>
+      <c r="D29" s="33" t="n"/>
+      <c r="E29" s="23">
         <f>IF(D29="","",D29*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F29" s="32" t="n"/>
+      <c r="F29" s="33" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="31" t="n"/>
-      <c r="B30" s="31" t="n"/>
-      <c r="C30" s="32" t="n"/>
-      <c r="D30" s="32" t="n"/>
-      <c r="E30" s="22">
+      <c r="A30" s="32" t="n"/>
+      <c r="B30" s="32" t="n"/>
+      <c r="C30" s="33" t="n"/>
+      <c r="D30" s="33" t="n"/>
+      <c r="E30" s="23">
         <f>IF(D30="","",D30*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F30" s="32" t="n"/>
+      <c r="F30" s="33" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="31" t="n"/>
-      <c r="B31" s="31" t="n"/>
-      <c r="C31" s="32" t="n"/>
-      <c r="D31" s="32" t="n"/>
-      <c r="E31" s="22">
+      <c r="A31" s="32" t="n"/>
+      <c r="B31" s="32" t="n"/>
+      <c r="C31" s="33" t="n"/>
+      <c r="D31" s="33" t="n"/>
+      <c r="E31" s="23">
         <f>IF(D31="","",D31*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F31" s="32" t="n"/>
+      <c r="F31" s="33" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="31" t="n"/>
-      <c r="B32" s="31" t="n"/>
-      <c r="C32" s="32" t="n"/>
-      <c r="D32" s="32" t="n"/>
-      <c r="E32" s="22">
+      <c r="A32" s="32" t="n"/>
+      <c r="B32" s="32" t="n"/>
+      <c r="C32" s="33" t="n"/>
+      <c r="D32" s="33" t="n"/>
+      <c r="E32" s="23">
         <f>IF(D32="","",D32*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F32" s="32" t="n"/>
+      <c r="F32" s="33" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="31" t="n"/>
-      <c r="B33" s="31" t="n"/>
-      <c r="C33" s="32" t="n"/>
-      <c r="D33" s="32" t="n"/>
-      <c r="E33" s="22">
+      <c r="A33" s="32" t="n"/>
+      <c r="B33" s="32" t="n"/>
+      <c r="C33" s="33" t="n"/>
+      <c r="D33" s="33" t="n"/>
+      <c r="E33" s="23">
         <f>IF(D33="","",D33*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F33" s="32" t="n"/>
+      <c r="F33" s="33" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="31" t="n"/>
-      <c r="B34" s="31" t="n"/>
-      <c r="C34" s="32" t="n"/>
-      <c r="D34" s="32" t="n"/>
-      <c r="E34" s="22">
+      <c r="A34" s="32" t="n"/>
+      <c r="B34" s="32" t="n"/>
+      <c r="C34" s="33" t="n"/>
+      <c r="D34" s="33" t="n"/>
+      <c r="E34" s="23">
         <f>IF(D34="","",D34*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F34" s="32" t="n"/>
+      <c r="F34" s="33" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="31" t="n"/>
-      <c r="B35" s="31" t="n"/>
-      <c r="C35" s="32" t="n"/>
-      <c r="D35" s="32" t="n"/>
-      <c r="E35" s="22">
+      <c r="A35" s="32" t="n"/>
+      <c r="B35" s="32" t="n"/>
+      <c r="C35" s="33" t="n"/>
+      <c r="D35" s="33" t="n"/>
+      <c r="E35" s="23">
         <f>IF(D35="","",D35*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F35" s="32" t="n"/>
+      <c r="F35" s="33" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="31" t="n"/>
-      <c r="B36" s="31" t="n"/>
-      <c r="C36" s="32" t="n"/>
-      <c r="D36" s="32" t="n"/>
-      <c r="E36" s="22">
+      <c r="A36" s="32" t="n"/>
+      <c r="B36" s="32" t="n"/>
+      <c r="C36" s="33" t="n"/>
+      <c r="D36" s="33" t="n"/>
+      <c r="E36" s="23">
         <f>IF(D36="","",D36*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F36" s="32" t="n"/>
+      <c r="F36" s="33" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="31" t="n"/>
-      <c r="B37" s="31" t="n"/>
-      <c r="C37" s="32" t="n"/>
-      <c r="D37" s="32" t="n"/>
-      <c r="E37" s="22">
+      <c r="A37" s="32" t="n"/>
+      <c r="B37" s="32" t="n"/>
+      <c r="C37" s="33" t="n"/>
+      <c r="D37" s="33" t="n"/>
+      <c r="E37" s="23">
         <f>IF(D37="","",D37*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F37" s="32" t="n"/>
+      <c r="F37" s="33" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="31" t="n"/>
-      <c r="B38" s="31" t="n"/>
-      <c r="C38" s="32" t="n"/>
-      <c r="D38" s="32" t="n"/>
-      <c r="E38" s="22">
+      <c r="A38" s="32" t="n"/>
+      <c r="B38" s="32" t="n"/>
+      <c r="C38" s="33" t="n"/>
+      <c r="D38" s="33" t="n"/>
+      <c r="E38" s="23">
         <f>IF(D38="","",D38*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F38" s="32" t="n"/>
+      <c r="F38" s="33" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="31" t="n"/>
-      <c r="B39" s="31" t="n"/>
-      <c r="C39" s="32" t="n"/>
-      <c r="D39" s="32" t="n"/>
-      <c r="E39" s="22">
+      <c r="A39" s="32" t="n"/>
+      <c r="B39" s="32" t="n"/>
+      <c r="C39" s="33" t="n"/>
+      <c r="D39" s="33" t="n"/>
+      <c r="E39" s="23">
         <f>IF(D39="","",D39*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F39" s="32" t="n"/>
+      <c r="F39" s="33" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="31" t="n"/>
-      <c r="B40" s="31" t="n"/>
-      <c r="C40" s="32" t="n"/>
-      <c r="D40" s="32" t="n"/>
-      <c r="E40" s="22">
+      <c r="A40" s="32" t="n"/>
+      <c r="B40" s="32" t="n"/>
+      <c r="C40" s="33" t="n"/>
+      <c r="D40" s="33" t="n"/>
+      <c r="E40" s="23">
         <f>IF(D40="","",D40*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F40" s="32" t="n"/>
+      <c r="F40" s="33" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="31" t="n"/>
-      <c r="B41" s="31" t="n"/>
-      <c r="C41" s="32" t="n"/>
-      <c r="D41" s="32" t="n"/>
-      <c r="E41" s="22">
+      <c r="A41" s="32" t="n"/>
+      <c r="B41" s="32" t="n"/>
+      <c r="C41" s="33" t="n"/>
+      <c r="D41" s="33" t="n"/>
+      <c r="E41" s="23">
         <f>IF(D41="","",D41*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F41" s="32" t="n"/>
+      <c r="F41" s="33" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="31" t="n"/>
-      <c r="B42" s="31" t="n"/>
-      <c r="C42" s="32" t="n"/>
-      <c r="D42" s="32" t="n"/>
-      <c r="E42" s="22">
+      <c r="A42" s="32" t="n"/>
+      <c r="B42" s="32" t="n"/>
+      <c r="C42" s="33" t="n"/>
+      <c r="D42" s="33" t="n"/>
+      <c r="E42" s="23">
         <f>IF(D42="","",D42*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F42" s="32" t="n"/>
+      <c r="F42" s="33" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="31" t="n"/>
-      <c r="B43" s="31" t="n"/>
-      <c r="C43" s="32" t="n"/>
-      <c r="D43" s="32" t="n"/>
-      <c r="E43" s="22">
+      <c r="A43" s="32" t="n"/>
+      <c r="B43" s="32" t="n"/>
+      <c r="C43" s="33" t="n"/>
+      <c r="D43" s="33" t="n"/>
+      <c r="E43" s="23">
         <f>IF(D43="","",D43*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F43" s="32" t="n"/>
+      <c r="F43" s="33" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="31" t="n"/>
-      <c r="B44" s="31" t="n"/>
-      <c r="C44" s="32" t="n"/>
-      <c r="D44" s="32" t="n"/>
-      <c r="E44" s="22">
+      <c r="A44" s="32" t="n"/>
+      <c r="B44" s="32" t="n"/>
+      <c r="C44" s="33" t="n"/>
+      <c r="D44" s="33" t="n"/>
+      <c r="E44" s="23">
         <f>IF(D44="","",D44*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F44" s="32" t="n"/>
+      <c r="F44" s="33" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="31" t="n"/>
-      <c r="B45" s="31" t="n"/>
-      <c r="C45" s="32" t="n"/>
-      <c r="D45" s="32" t="n"/>
-      <c r="E45" s="22">
+      <c r="A45" s="32" t="n"/>
+      <c r="B45" s="32" t="n"/>
+      <c r="C45" s="33" t="n"/>
+      <c r="D45" s="33" t="n"/>
+      <c r="E45" s="23">
         <f>IF(D45="","",D45*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F45" s="32" t="n"/>
+      <c r="F45" s="33" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="31" t="n"/>
-      <c r="B46" s="31" t="n"/>
-      <c r="C46" s="32" t="n"/>
-      <c r="D46" s="32" t="n"/>
-      <c r="E46" s="22">
+      <c r="A46" s="32" t="n"/>
+      <c r="B46" s="32" t="n"/>
+      <c r="C46" s="33" t="n"/>
+      <c r="D46" s="33" t="n"/>
+      <c r="E46" s="23">
         <f>IF(D46="","",D46*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F46" s="32" t="n"/>
+      <c r="F46" s="33" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="31" t="n"/>
-      <c r="B47" s="31" t="n"/>
-      <c r="C47" s="32" t="n"/>
-      <c r="D47" s="32" t="n"/>
-      <c r="E47" s="22">
+      <c r="A47" s="32" t="n"/>
+      <c r="B47" s="32" t="n"/>
+      <c r="C47" s="33" t="n"/>
+      <c r="D47" s="33" t="n"/>
+      <c r="E47" s="23">
         <f>IF(D47="","",D47*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F47" s="32" t="n"/>
+      <c r="F47" s="33" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="31" t="n"/>
-      <c r="B48" s="31" t="n"/>
-      <c r="C48" s="32" t="n"/>
-      <c r="D48" s="32" t="n"/>
-      <c r="E48" s="22">
+      <c r="A48" s="32" t="n"/>
+      <c r="B48" s="32" t="n"/>
+      <c r="C48" s="33" t="n"/>
+      <c r="D48" s="33" t="n"/>
+      <c r="E48" s="23">
         <f>IF(D48="","",D48*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F48" s="32" t="n"/>
+      <c r="F48" s="33" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="31" t="n"/>
-      <c r="B49" s="31" t="n"/>
-      <c r="C49" s="32" t="n"/>
-      <c r="D49" s="32" t="n"/>
-      <c r="E49" s="22">
+      <c r="A49" s="32" t="n"/>
+      <c r="B49" s="32" t="n"/>
+      <c r="C49" s="33" t="n"/>
+      <c r="D49" s="33" t="n"/>
+      <c r="E49" s="23">
         <f>IF(D49="","",D49*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F49" s="32" t="n"/>
+      <c r="F49" s="33" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="31" t="n"/>
-      <c r="B50" s="31" t="n"/>
-      <c r="C50" s="32" t="n"/>
-      <c r="D50" s="32" t="n"/>
-      <c r="E50" s="22">
+      <c r="A50" s="32" t="n"/>
+      <c r="B50" s="32" t="n"/>
+      <c r="C50" s="33" t="n"/>
+      <c r="D50" s="33" t="n"/>
+      <c r="E50" s="23">
         <f>IF(D50="","",D50*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F50" s="32" t="n"/>
+      <c r="F50" s="33" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="31" t="n"/>
-      <c r="B51" s="31" t="n"/>
-      <c r="C51" s="32" t="n"/>
-      <c r="D51" s="32" t="n"/>
-      <c r="E51" s="22">
+      <c r="A51" s="32" t="n"/>
+      <c r="B51" s="32" t="n"/>
+      <c r="C51" s="33" t="n"/>
+      <c r="D51" s="33" t="n"/>
+      <c r="E51" s="23">
         <f>IF(D51="","",D51*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F51" s="32" t="n"/>
+      <c r="F51" s="33" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="31" t="n"/>
-      <c r="B52" s="31" t="n"/>
-      <c r="C52" s="32" t="n"/>
-      <c r="D52" s="32" t="n"/>
-      <c r="E52" s="22">
+      <c r="A52" s="32" t="n"/>
+      <c r="B52" s="32" t="n"/>
+      <c r="C52" s="33" t="n"/>
+      <c r="D52" s="33" t="n"/>
+      <c r="E52" s="23">
         <f>IF(D52="","",D52*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F52" s="32" t="n"/>
+      <c r="F52" s="33" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="31" t="n"/>
-      <c r="B53" s="31" t="n"/>
-      <c r="C53" s="32" t="n"/>
-      <c r="D53" s="32" t="n"/>
-      <c r="E53" s="22">
+      <c r="A53" s="32" t="n"/>
+      <c r="B53" s="32" t="n"/>
+      <c r="C53" s="33" t="n"/>
+      <c r="D53" s="33" t="n"/>
+      <c r="E53" s="23">
         <f>IF(D53="","",D53*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F53" s="32" t="n"/>
+      <c r="F53" s="33" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="31" t="n"/>
-      <c r="B54" s="31" t="n"/>
-      <c r="C54" s="32" t="n"/>
-      <c r="D54" s="32" t="n"/>
-      <c r="E54" s="22">
+      <c r="A54" s="32" t="n"/>
+      <c r="B54" s="32" t="n"/>
+      <c r="C54" s="33" t="n"/>
+      <c r="D54" s="33" t="n"/>
+      <c r="E54" s="23">
         <f>IF(D54="","",D54*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F54" s="32" t="n"/>
+      <c r="F54" s="33" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="31" t="n"/>
-      <c r="B55" s="31" t="n"/>
-      <c r="C55" s="32" t="n"/>
-      <c r="D55" s="32" t="n"/>
-      <c r="E55" s="22">
+      <c r="A55" s="32" t="n"/>
+      <c r="B55" s="32" t="n"/>
+      <c r="C55" s="33" t="n"/>
+      <c r="D55" s="33" t="n"/>
+      <c r="E55" s="23">
         <f>IF(D55="","",D55*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F55" s="32" t="n"/>
+      <c r="F55" s="33" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="31" t="n"/>
-      <c r="B56" s="31" t="n"/>
-      <c r="C56" s="32" t="n"/>
-      <c r="D56" s="32" t="n"/>
-      <c r="E56" s="22">
+      <c r="A56" s="32" t="n"/>
+      <c r="B56" s="32" t="n"/>
+      <c r="C56" s="33" t="n"/>
+      <c r="D56" s="33" t="n"/>
+      <c r="E56" s="23">
         <f>IF(D56="","",D56*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F56" s="32" t="n"/>
+      <c r="F56" s="33" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="31" t="n"/>
-      <c r="B57" s="31" t="n"/>
-      <c r="C57" s="32" t="n"/>
-      <c r="D57" s="32" t="n"/>
-      <c r="E57" s="22">
+      <c r="A57" s="32" t="n"/>
+      <c r="B57" s="32" t="n"/>
+      <c r="C57" s="33" t="n"/>
+      <c r="D57" s="33" t="n"/>
+      <c r="E57" s="23">
         <f>IF(D57="","",D57*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F57" s="32" t="n"/>
+      <c r="F57" s="33" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="31" t="n"/>
-      <c r="B58" s="31" t="n"/>
-      <c r="C58" s="32" t="n"/>
-      <c r="D58" s="32" t="n"/>
-      <c r="E58" s="22">
+      <c r="A58" s="32" t="n"/>
+      <c r="B58" s="32" t="n"/>
+      <c r="C58" s="33" t="n"/>
+      <c r="D58" s="33" t="n"/>
+      <c r="E58" s="23">
         <f>IF(D58="","",D58*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F58" s="32" t="n"/>
+      <c r="F58" s="33" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="31" t="n"/>
-      <c r="B59" s="31" t="n"/>
-      <c r="C59" s="32" t="n"/>
-      <c r="D59" s="32" t="n"/>
-      <c r="E59" s="22">
+      <c r="A59" s="32" t="n"/>
+      <c r="B59" s="32" t="n"/>
+      <c r="C59" s="33" t="n"/>
+      <c r="D59" s="33" t="n"/>
+      <c r="E59" s="23">
         <f>IF(D59="","",D59*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F59" s="32" t="n"/>
+      <c r="F59" s="33" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="31" t="n"/>
-      <c r="B60" s="31" t="n"/>
-      <c r="C60" s="32" t="n"/>
-      <c r="D60" s="32" t="n"/>
-      <c r="E60" s="22">
+      <c r="A60" s="32" t="n"/>
+      <c r="B60" s="32" t="n"/>
+      <c r="C60" s="33" t="n"/>
+      <c r="D60" s="33" t="n"/>
+      <c r="E60" s="23">
         <f>IF(D60="","",D60*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F60" s="32" t="n"/>
+      <c r="F60" s="33" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="31" t="n"/>
-      <c r="B61" s="31" t="n"/>
-      <c r="C61" s="32" t="n"/>
-      <c r="D61" s="32" t="n"/>
-      <c r="E61" s="22">
+      <c r="A61" s="32" t="n"/>
+      <c r="B61" s="32" t="n"/>
+      <c r="C61" s="33" t="n"/>
+      <c r="D61" s="33" t="n"/>
+      <c r="E61" s="23">
         <f>IF(D61="","",D61*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F61" s="32" t="n"/>
+      <c r="F61" s="33" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="31" t="n"/>
-      <c r="B62" s="31" t="n"/>
-      <c r="C62" s="32" t="n"/>
-      <c r="D62" s="32" t="n"/>
-      <c r="E62" s="22">
+      <c r="A62" s="32" t="n"/>
+      <c r="B62" s="32" t="n"/>
+      <c r="C62" s="33" t="n"/>
+      <c r="D62" s="33" t="n"/>
+      <c r="E62" s="23">
         <f>IF(D62="","",D62*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F62" s="32" t="n"/>
+      <c r="F62" s="33" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="31" t="n"/>
-      <c r="B63" s="31" t="n"/>
-      <c r="C63" s="32" t="n"/>
-      <c r="D63" s="32" t="n"/>
-      <c r="E63" s="22">
+      <c r="A63" s="32" t="n"/>
+      <c r="B63" s="32" t="n"/>
+      <c r="C63" s="33" t="n"/>
+      <c r="D63" s="33" t="n"/>
+      <c r="E63" s="23">
         <f>IF(D63="","",D63*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F63" s="32" t="n"/>
+      <c r="F63" s="33" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="31" t="n"/>
-      <c r="B64" s="31" t="n"/>
-      <c r="C64" s="32" t="n"/>
-      <c r="D64" s="32" t="n"/>
-      <c r="E64" s="22">
+      <c r="A64" s="32" t="n"/>
+      <c r="B64" s="32" t="n"/>
+      <c r="C64" s="33" t="n"/>
+      <c r="D64" s="33" t="n"/>
+      <c r="E64" s="23">
         <f>IF(D64="","",D64*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F64" s="32" t="n"/>
+      <c r="F64" s="33" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="31" t="n"/>
-      <c r="B65" s="31" t="n"/>
-      <c r="C65" s="32" t="n"/>
-      <c r="D65" s="32" t="n"/>
-      <c r="E65" s="22">
+      <c r="A65" s="32" t="n"/>
+      <c r="B65" s="32" t="n"/>
+      <c r="C65" s="33" t="n"/>
+      <c r="D65" s="33" t="n"/>
+      <c r="E65" s="23">
         <f>IF(D65="","",D65*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F65" s="32" t="n"/>
+      <c r="F65" s="33" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="31" t="n"/>
-      <c r="B66" s="31" t="n"/>
-      <c r="C66" s="32" t="n"/>
-      <c r="D66" s="32" t="n"/>
-      <c r="E66" s="22">
+      <c r="A66" s="32" t="n"/>
+      <c r="B66" s="32" t="n"/>
+      <c r="C66" s="33" t="n"/>
+      <c r="D66" s="33" t="n"/>
+      <c r="E66" s="23">
         <f>IF(D66="","",D66*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F66" s="32" t="n"/>
+      <c r="F66" s="33" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="31" t="n"/>
-      <c r="B67" s="31" t="n"/>
-      <c r="C67" s="32" t="n"/>
-      <c r="D67" s="32" t="n"/>
-      <c r="E67" s="22">
+      <c r="A67" s="32" t="n"/>
+      <c r="B67" s="32" t="n"/>
+      <c r="C67" s="33" t="n"/>
+      <c r="D67" s="33" t="n"/>
+      <c r="E67" s="23">
         <f>IF(D67="","",D67*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F67" s="32" t="n"/>
+      <c r="F67" s="33" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="31" t="n"/>
-      <c r="B68" s="31" t="n"/>
-      <c r="C68" s="32" t="n"/>
-      <c r="D68" s="32" t="n"/>
-      <c r="E68" s="22">
+      <c r="A68" s="32" t="n"/>
+      <c r="B68" s="32" t="n"/>
+      <c r="C68" s="33" t="n"/>
+      <c r="D68" s="33" t="n"/>
+      <c r="E68" s="23">
         <f>IF(D68="","",D68*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F68" s="32" t="n"/>
+      <c r="F68" s="33" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="31" t="n"/>
-      <c r="B69" s="31" t="n"/>
-      <c r="C69" s="32" t="n"/>
-      <c r="D69" s="32" t="n"/>
-      <c r="E69" s="22">
+      <c r="A69" s="32" t="n"/>
+      <c r="B69" s="32" t="n"/>
+      <c r="C69" s="33" t="n"/>
+      <c r="D69" s="33" t="n"/>
+      <c r="E69" s="23">
         <f>IF(D69="","",D69*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F69" s="32" t="n"/>
+      <c r="F69" s="33" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="31" t="n"/>
-      <c r="B70" s="31" t="n"/>
-      <c r="C70" s="32" t="n"/>
-      <c r="D70" s="32" t="n"/>
-      <c r="E70" s="22">
+      <c r="A70" s="32" t="n"/>
+      <c r="B70" s="32" t="n"/>
+      <c r="C70" s="33" t="n"/>
+      <c r="D70" s="33" t="n"/>
+      <c r="E70" s="23">
         <f>IF(D70="","",D70*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F70" s="32" t="n"/>
+      <c r="F70" s="33" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="31" t="n"/>
-      <c r="B71" s="31" t="n"/>
-      <c r="C71" s="32" t="n"/>
-      <c r="D71" s="32" t="n"/>
-      <c r="E71" s="22">
+      <c r="A71" s="32" t="n"/>
+      <c r="B71" s="32" t="n"/>
+      <c r="C71" s="33" t="n"/>
+      <c r="D71" s="33" t="n"/>
+      <c r="E71" s="23">
         <f>IF(D71="","",D71*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F71" s="32" t="n"/>
+      <c r="F71" s="33" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="31" t="n"/>
-      <c r="B72" s="31" t="n"/>
-      <c r="C72" s="32" t="n"/>
-      <c r="D72" s="32" t="n"/>
-      <c r="E72" s="22">
+      <c r="A72" s="32" t="n"/>
+      <c r="B72" s="32" t="n"/>
+      <c r="C72" s="33" t="n"/>
+      <c r="D72" s="33" t="n"/>
+      <c r="E72" s="23">
         <f>IF(D72="","",D72*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F72" s="32" t="n"/>
+      <c r="F72" s="33" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="31" t="n"/>
-      <c r="B73" s="31" t="n"/>
-      <c r="C73" s="32" t="n"/>
-      <c r="D73" s="32" t="n"/>
-      <c r="E73" s="22">
+      <c r="A73" s="32" t="n"/>
+      <c r="B73" s="32" t="n"/>
+      <c r="C73" s="33" t="n"/>
+      <c r="D73" s="33" t="n"/>
+      <c r="E73" s="23">
         <f>IF(D73="","",D73*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F73" s="32" t="n"/>
+      <c r="F73" s="33" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="31" t="n"/>
-      <c r="B74" s="31" t="n"/>
-      <c r="C74" s="32" t="n"/>
-      <c r="D74" s="32" t="n"/>
-      <c r="E74" s="22">
+      <c r="A74" s="32" t="n"/>
+      <c r="B74" s="32" t="n"/>
+      <c r="C74" s="33" t="n"/>
+      <c r="D74" s="33" t="n"/>
+      <c r="E74" s="23">
         <f>IF(D74="","",D74*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F74" s="32" t="n"/>
+      <c r="F74" s="33" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="31" t="n"/>
-      <c r="B75" s="31" t="n"/>
-      <c r="C75" s="32" t="n"/>
-      <c r="D75" s="32" t="n"/>
-      <c r="E75" s="22">
+      <c r="A75" s="32" t="n"/>
+      <c r="B75" s="32" t="n"/>
+      <c r="C75" s="33" t="n"/>
+      <c r="D75" s="33" t="n"/>
+      <c r="E75" s="23">
         <f>IF(D75="","",D75*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F75" s="32" t="n"/>
+      <c r="F75" s="33" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="31" t="n"/>
-      <c r="B76" s="31" t="n"/>
-      <c r="C76" s="32" t="n"/>
-      <c r="D76" s="32" t="n"/>
-      <c r="E76" s="22">
+      <c r="A76" s="32" t="n"/>
+      <c r="B76" s="32" t="n"/>
+      <c r="C76" s="33" t="n"/>
+      <c r="D76" s="33" t="n"/>
+      <c r="E76" s="23">
         <f>IF(D76="","",D76*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F76" s="32" t="n"/>
+      <c r="F76" s="33" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="31" t="n"/>
-      <c r="B77" s="31" t="n"/>
-      <c r="C77" s="32" t="n"/>
-      <c r="D77" s="32" t="n"/>
-      <c r="E77" s="22">
+      <c r="A77" s="32" t="n"/>
+      <c r="B77" s="32" t="n"/>
+      <c r="C77" s="33" t="n"/>
+      <c r="D77" s="33" t="n"/>
+      <c r="E77" s="23">
         <f>IF(D77="","",D77*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F77" s="32" t="n"/>
+      <c r="F77" s="33" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="31" t="n"/>
-      <c r="B78" s="31" t="n"/>
-      <c r="C78" s="32" t="n"/>
-      <c r="D78" s="32" t="n"/>
-      <c r="E78" s="22">
+      <c r="A78" s="32" t="n"/>
+      <c r="B78" s="32" t="n"/>
+      <c r="C78" s="33" t="n"/>
+      <c r="D78" s="33" t="n"/>
+      <c r="E78" s="23">
         <f>IF(D78="","",D78*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F78" s="32" t="n"/>
+      <c r="F78" s="33" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="31" t="n"/>
-      <c r="B79" s="31" t="n"/>
-      <c r="C79" s="32" t="n"/>
-      <c r="D79" s="32" t="n"/>
-      <c r="E79" s="22">
+      <c r="A79" s="32" t="n"/>
+      <c r="B79" s="32" t="n"/>
+      <c r="C79" s="33" t="n"/>
+      <c r="D79" s="33" t="n"/>
+      <c r="E79" s="23">
         <f>IF(D79="","",D79*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F79" s="32" t="n"/>
+      <c r="F79" s="33" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="31" t="n"/>
-      <c r="B80" s="31" t="n"/>
-      <c r="C80" s="32" t="n"/>
-      <c r="D80" s="32" t="n"/>
-      <c r="E80" s="22">
+      <c r="A80" s="32" t="n"/>
+      <c r="B80" s="32" t="n"/>
+      <c r="C80" s="33" t="n"/>
+      <c r="D80" s="33" t="n"/>
+      <c r="E80" s="23">
         <f>IF(D80="","",D80*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F80" s="32" t="n"/>
+      <c r="F80" s="33" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="31" t="n"/>
-      <c r="B81" s="31" t="n"/>
-      <c r="C81" s="32" t="n"/>
-      <c r="D81" s="32" t="n"/>
-      <c r="E81" s="22">
+      <c r="A81" s="32" t="n"/>
+      <c r="B81" s="32" t="n"/>
+      <c r="C81" s="33" t="n"/>
+      <c r="D81" s="33" t="n"/>
+      <c r="E81" s="23">
         <f>IF(D81="","",D81*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F81" s="32" t="n"/>
+      <c r="F81" s="33" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="31" t="n"/>
-      <c r="B82" s="31" t="n"/>
-      <c r="C82" s="32" t="n"/>
-      <c r="D82" s="32" t="n"/>
-      <c r="E82" s="22">
+      <c r="A82" s="32" t="n"/>
+      <c r="B82" s="32" t="n"/>
+      <c r="C82" s="33" t="n"/>
+      <c r="D82" s="33" t="n"/>
+      <c r="E82" s="23">
         <f>IF(D82="","",D82*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F82" s="32" t="n"/>
+      <c r="F82" s="33" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="31" t="n"/>
-      <c r="B83" s="31" t="n"/>
-      <c r="C83" s="32" t="n"/>
-      <c r="D83" s="32" t="n"/>
-      <c r="E83" s="22">
+      <c r="A83" s="32" t="n"/>
+      <c r="B83" s="32" t="n"/>
+      <c r="C83" s="33" t="n"/>
+      <c r="D83" s="33" t="n"/>
+      <c r="E83" s="23">
         <f>IF(D83="","",D83*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F83" s="32" t="n"/>
+      <c r="F83" s="33" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="31" t="n"/>
-      <c r="B84" s="31" t="n"/>
-      <c r="C84" s="32" t="n"/>
-      <c r="D84" s="32" t="n"/>
-      <c r="E84" s="22">
+      <c r="A84" s="32" t="n"/>
+      <c r="B84" s="32" t="n"/>
+      <c r="C84" s="33" t="n"/>
+      <c r="D84" s="33" t="n"/>
+      <c r="E84" s="23">
         <f>IF(D84="","",D84*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F84" s="32" t="n"/>
+      <c r="F84" s="33" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="31" t="n"/>
-      <c r="B85" s="31" t="n"/>
-      <c r="C85" s="32" t="n"/>
-      <c r="D85" s="32" t="n"/>
-      <c r="E85" s="22">
+      <c r="A85" s="32" t="n"/>
+      <c r="B85" s="32" t="n"/>
+      <c r="C85" s="33" t="n"/>
+      <c r="D85" s="33" t="n"/>
+      <c r="E85" s="23">
         <f>IF(D85="","",D85*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F85" s="32" t="n"/>
+      <c r="F85" s="33" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="31" t="n"/>
-      <c r="B86" s="31" t="n"/>
-      <c r="C86" s="32" t="n"/>
-      <c r="D86" s="32" t="n"/>
-      <c r="E86" s="22">
+      <c r="A86" s="32" t="n"/>
+      <c r="B86" s="32" t="n"/>
+      <c r="C86" s="33" t="n"/>
+      <c r="D86" s="33" t="n"/>
+      <c r="E86" s="23">
         <f>IF(D86="","",D86*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F86" s="32" t="n"/>
+      <c r="F86" s="33" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="31" t="n"/>
-      <c r="B87" s="31" t="n"/>
-      <c r="C87" s="32" t="n"/>
-      <c r="D87" s="32" t="n"/>
-      <c r="E87" s="22">
+      <c r="A87" s="32" t="n"/>
+      <c r="B87" s="32" t="n"/>
+      <c r="C87" s="33" t="n"/>
+      <c r="D87" s="33" t="n"/>
+      <c r="E87" s="23">
         <f>IF(D87="","",D87*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F87" s="32" t="n"/>
+      <c r="F87" s="33" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="31" t="n"/>
-      <c r="B88" s="31" t="n"/>
-      <c r="C88" s="32" t="n"/>
-      <c r="D88" s="32" t="n"/>
-      <c r="E88" s="22">
+      <c r="A88" s="32" t="n"/>
+      <c r="B88" s="32" t="n"/>
+      <c r="C88" s="33" t="n"/>
+      <c r="D88" s="33" t="n"/>
+      <c r="E88" s="23">
         <f>IF(D88="","",D88*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F88" s="32" t="n"/>
+      <c r="F88" s="33" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="31" t="n"/>
-      <c r="B89" s="31" t="n"/>
-      <c r="C89" s="32" t="n"/>
-      <c r="D89" s="32" t="n"/>
-      <c r="E89" s="22">
+      <c r="A89" s="32" t="n"/>
+      <c r="B89" s="32" t="n"/>
+      <c r="C89" s="33" t="n"/>
+      <c r="D89" s="33" t="n"/>
+      <c r="E89" s="23">
         <f>IF(D89="","",D89*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F89" s="32" t="n"/>
+      <c r="F89" s="33" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="31" t="n"/>
-      <c r="B90" s="31" t="n"/>
-      <c r="C90" s="32" t="n"/>
-      <c r="D90" s="32" t="n"/>
-      <c r="E90" s="22">
+      <c r="A90" s="32" t="n"/>
+      <c r="B90" s="32" t="n"/>
+      <c r="C90" s="33" t="n"/>
+      <c r="D90" s="33" t="n"/>
+      <c r="E90" s="23">
         <f>IF(D90="","",D90*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F90" s="32" t="n"/>
+      <c r="F90" s="33" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="31" t="n"/>
-      <c r="B91" s="31" t="n"/>
-      <c r="C91" s="32" t="n"/>
-      <c r="D91" s="32" t="n"/>
-      <c r="E91" s="22">
+      <c r="A91" s="32" t="n"/>
+      <c r="B91" s="32" t="n"/>
+      <c r="C91" s="33" t="n"/>
+      <c r="D91" s="33" t="n"/>
+      <c r="E91" s="23">
         <f>IF(D91="","",D91*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F91" s="32" t="n"/>
+      <c r="F91" s="33" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="31" t="n"/>
-      <c r="B92" s="31" t="n"/>
-      <c r="C92" s="32" t="n"/>
-      <c r="D92" s="32" t="n"/>
-      <c r="E92" s="22">
+      <c r="A92" s="32" t="n"/>
+      <c r="B92" s="32" t="n"/>
+      <c r="C92" s="33" t="n"/>
+      <c r="D92" s="33" t="n"/>
+      <c r="E92" s="23">
         <f>IF(D92="","",D92*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F92" s="32" t="n"/>
+      <c r="F92" s="33" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="31" t="n"/>
-      <c r="B93" s="31" t="n"/>
-      <c r="C93" s="32" t="n"/>
-      <c r="D93" s="32" t="n"/>
-      <c r="E93" s="22">
+      <c r="A93" s="32" t="n"/>
+      <c r="B93" s="32" t="n"/>
+      <c r="C93" s="33" t="n"/>
+      <c r="D93" s="33" t="n"/>
+      <c r="E93" s="23">
         <f>IF(D93="","",D93*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F93" s="32" t="n"/>
+      <c r="F93" s="33" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="31" t="n"/>
-      <c r="B94" s="31" t="n"/>
-      <c r="C94" s="32" t="n"/>
-      <c r="D94" s="32" t="n"/>
-      <c r="E94" s="22">
+      <c r="A94" s="32" t="n"/>
+      <c r="B94" s="32" t="n"/>
+      <c r="C94" s="33" t="n"/>
+      <c r="D94" s="33" t="n"/>
+      <c r="E94" s="23">
         <f>IF(D94="","",D94*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F94" s="32" t="n"/>
+      <c r="F94" s="33" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="31" t="n"/>
-      <c r="B95" s="31" t="n"/>
-      <c r="C95" s="32" t="n"/>
-      <c r="D95" s="32" t="n"/>
-      <c r="E95" s="22">
+      <c r="A95" s="32" t="n"/>
+      <c r="B95" s="32" t="n"/>
+      <c r="C95" s="33" t="n"/>
+      <c r="D95" s="33" t="n"/>
+      <c r="E95" s="23">
         <f>IF(D95="","",D95*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F95" s="32" t="n"/>
+      <c r="F95" s="33" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="31" t="n"/>
-      <c r="B96" s="31" t="n"/>
-      <c r="C96" s="32" t="n"/>
-      <c r="D96" s="32" t="n"/>
-      <c r="E96" s="22">
+      <c r="A96" s="32" t="n"/>
+      <c r="B96" s="32" t="n"/>
+      <c r="C96" s="33" t="n"/>
+      <c r="D96" s="33" t="n"/>
+      <c r="E96" s="23">
         <f>IF(D96="","",D96*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F96" s="32" t="n"/>
+      <c r="F96" s="33" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="31" t="n"/>
-      <c r="B97" s="31" t="n"/>
-      <c r="C97" s="32" t="n"/>
-      <c r="D97" s="32" t="n"/>
-      <c r="E97" s="22">
+      <c r="A97" s="32" t="n"/>
+      <c r="B97" s="32" t="n"/>
+      <c r="C97" s="33" t="n"/>
+      <c r="D97" s="33" t="n"/>
+      <c r="E97" s="23">
         <f>IF(D97="","",D97*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F97" s="32" t="n"/>
+      <c r="F97" s="33" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="31" t="n"/>
-      <c r="B98" s="31" t="n"/>
-      <c r="C98" s="32" t="n"/>
-      <c r="D98" s="32" t="n"/>
-      <c r="E98" s="22">
+      <c r="A98" s="32" t="n"/>
+      <c r="B98" s="32" t="n"/>
+      <c r="C98" s="33" t="n"/>
+      <c r="D98" s="33" t="n"/>
+      <c r="E98" s="23">
         <f>IF(D98="","",D98*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F98" s="32" t="n"/>
+      <c r="F98" s="33" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="31" t="n"/>
-      <c r="B99" s="31" t="n"/>
-      <c r="C99" s="32" t="n"/>
-      <c r="D99" s="32" t="n"/>
-      <c r="E99" s="22">
+      <c r="A99" s="32" t="n"/>
+      <c r="B99" s="32" t="n"/>
+      <c r="C99" s="33" t="n"/>
+      <c r="D99" s="33" t="n"/>
+      <c r="E99" s="23">
         <f>IF(D99="","",D99*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F99" s="32" t="n"/>
+      <c r="F99" s="33" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="31" t="n"/>
-      <c r="B100" s="31" t="n"/>
-      <c r="C100" s="32" t="n"/>
-      <c r="D100" s="32" t="n"/>
-      <c r="E100" s="22">
+      <c r="A100" s="32" t="n"/>
+      <c r="B100" s="32" t="n"/>
+      <c r="C100" s="33" t="n"/>
+      <c r="D100" s="33" t="n"/>
+      <c r="E100" s="23">
         <f>IF(D100="","",D100*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F100" s="32" t="n"/>
+      <c r="F100" s="33" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="31" t="n"/>
-      <c r="B101" s="31" t="n"/>
-      <c r="C101" s="32" t="n"/>
-      <c r="D101" s="32" t="n"/>
-      <c r="E101" s="22">
+      <c r="A101" s="32" t="n"/>
+      <c r="B101" s="32" t="n"/>
+      <c r="C101" s="33" t="n"/>
+      <c r="D101" s="33" t="n"/>
+      <c r="E101" s="23">
         <f>IF(D101="","",D101*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F101" s="32" t="n"/>
+      <c r="F101" s="33" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="31" t="n"/>
-      <c r="B102" s="31" t="n"/>
-      <c r="C102" s="32" t="n"/>
-      <c r="D102" s="32" t="n"/>
-      <c r="E102" s="22">
+      <c r="A102" s="32" t="n"/>
+      <c r="B102" s="32" t="n"/>
+      <c r="C102" s="33" t="n"/>
+      <c r="D102" s="33" t="n"/>
+      <c r="E102" s="23">
         <f>IF(D102="","",D102*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F102" s="32" t="n"/>
+      <c r="F102" s="33" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="31" t="n"/>
-      <c r="B103" s="31" t="n"/>
-      <c r="C103" s="32" t="n"/>
-      <c r="D103" s="32" t="n"/>
-      <c r="E103" s="22">
+      <c r="A103" s="32" t="n"/>
+      <c r="B103" s="32" t="n"/>
+      <c r="C103" s="33" t="n"/>
+      <c r="D103" s="33" t="n"/>
+      <c r="E103" s="23">
         <f>IF(D103="","",D103*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F103" s="32" t="n"/>
+      <c r="F103" s="33" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="31" t="n"/>
-      <c r="B104" s="31" t="n"/>
-      <c r="C104" s="32" t="n"/>
-      <c r="D104" s="32" t="n"/>
-      <c r="E104" s="22">
+      <c r="A104" s="32" t="n"/>
+      <c r="B104" s="32" t="n"/>
+      <c r="C104" s="33" t="n"/>
+      <c r="D104" s="33" t="n"/>
+      <c r="E104" s="23">
         <f>IF(D104="","",D104*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F104" s="32" t="n"/>
+      <c r="F104" s="33" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="31" t="n"/>
-      <c r="B105" s="31" t="n"/>
-      <c r="C105" s="32" t="n"/>
-      <c r="D105" s="32" t="n"/>
-      <c r="E105" s="22">
+      <c r="A105" s="32" t="n"/>
+      <c r="B105" s="32" t="n"/>
+      <c r="C105" s="33" t="n"/>
+      <c r="D105" s="33" t="n"/>
+      <c r="E105" s="23">
         <f>IF(D105="","",D105*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F105" s="32" t="n"/>
+      <c r="F105" s="33" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="31" t="n"/>
-      <c r="B106" s="31" t="n"/>
-      <c r="C106" s="32" t="n"/>
-      <c r="D106" s="32" t="n"/>
-      <c r="E106" s="22">
+      <c r="A106" s="32" t="n"/>
+      <c r="B106" s="32" t="n"/>
+      <c r="C106" s="33" t="n"/>
+      <c r="D106" s="33" t="n"/>
+      <c r="E106" s="23">
         <f>IF(D106="","",D106*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F106" s="32" t="n"/>
+      <c r="F106" s="33" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="31" t="n"/>
-      <c r="B107" s="31" t="n"/>
-      <c r="C107" s="32" t="n"/>
-      <c r="D107" s="32" t="n"/>
-      <c r="E107" s="22">
+      <c r="A107" s="32" t="n"/>
+      <c r="B107" s="32" t="n"/>
+      <c r="C107" s="33" t="n"/>
+      <c r="D107" s="33" t="n"/>
+      <c r="E107" s="23">
         <f>IF(D107="","",D107*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F107" s="32" t="n"/>
+      <c r="F107" s="33" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="31" t="n"/>
-      <c r="B108" s="31" t="n"/>
-      <c r="C108" s="32" t="n"/>
-      <c r="D108" s="32" t="n"/>
-      <c r="E108" s="22">
+      <c r="A108" s="32" t="n"/>
+      <c r="B108" s="32" t="n"/>
+      <c r="C108" s="33" t="n"/>
+      <c r="D108" s="33" t="n"/>
+      <c r="E108" s="23">
         <f>IF(D108="","",D108*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F108" s="32" t="n"/>
+      <c r="F108" s="33" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="31" t="n"/>
-      <c r="B109" s="31" t="n"/>
-      <c r="C109" s="32" t="n"/>
-      <c r="D109" s="32" t="n"/>
-      <c r="E109" s="22">
+      <c r="A109" s="32" t="n"/>
+      <c r="B109" s="32" t="n"/>
+      <c r="C109" s="33" t="n"/>
+      <c r="D109" s="33" t="n"/>
+      <c r="E109" s="23">
         <f>IF(D109="","",D109*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F109" s="32" t="n"/>
+      <c r="F109" s="33" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="31" t="n"/>
-      <c r="B110" s="31" t="n"/>
-      <c r="C110" s="32" t="n"/>
-      <c r="D110" s="32" t="n"/>
-      <c r="E110" s="22">
+      <c r="A110" s="32" t="n"/>
+      <c r="B110" s="32" t="n"/>
+      <c r="C110" s="33" t="n"/>
+      <c r="D110" s="33" t="n"/>
+      <c r="E110" s="23">
         <f>IF(D110="","",D110*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F110" s="32" t="n"/>
+      <c r="F110" s="33" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="31" t="n"/>
-      <c r="B111" s="31" t="n"/>
-      <c r="C111" s="32" t="n"/>
-      <c r="D111" s="32" t="n"/>
-      <c r="E111" s="22">
+      <c r="A111" s="32" t="n"/>
+      <c r="B111" s="32" t="n"/>
+      <c r="C111" s="33" t="n"/>
+      <c r="D111" s="33" t="n"/>
+      <c r="E111" s="23">
         <f>IF(D111="","",D111*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F111" s="32" t="n"/>
+      <c r="F111" s="33" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="31" t="n"/>
-      <c r="B112" s="31" t="n"/>
-      <c r="C112" s="32" t="n"/>
-      <c r="D112" s="32" t="n"/>
-      <c r="E112" s="22">
+      <c r="A112" s="32" t="n"/>
+      <c r="B112" s="32" t="n"/>
+      <c r="C112" s="33" t="n"/>
+      <c r="D112" s="33" t="n"/>
+      <c r="E112" s="23">
         <f>IF(D112="","",D112*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F112" s="32" t="n"/>
+      <c r="F112" s="33" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="31" t="n"/>
-      <c r="B113" s="31" t="n"/>
-      <c r="C113" s="32" t="n"/>
-      <c r="D113" s="32" t="n"/>
-      <c r="E113" s="22">
+      <c r="A113" s="32" t="n"/>
+      <c r="B113" s="32" t="n"/>
+      <c r="C113" s="33" t="n"/>
+      <c r="D113" s="33" t="n"/>
+      <c r="E113" s="23">
         <f>IF(D113="","",D113*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F113" s="32" t="n"/>
+      <c r="F113" s="33" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="31" t="n"/>
-      <c r="B114" s="31" t="n"/>
-      <c r="C114" s="32" t="n"/>
-      <c r="D114" s="32" t="n"/>
-      <c r="E114" s="22">
+      <c r="A114" s="32" t="n"/>
+      <c r="B114" s="32" t="n"/>
+      <c r="C114" s="33" t="n"/>
+      <c r="D114" s="33" t="n"/>
+      <c r="E114" s="23">
         <f>IF(D114="","",D114*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F114" s="32" t="n"/>
+      <c r="F114" s="33" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="31" t="n"/>
-      <c r="B115" s="31" t="n"/>
-      <c r="C115" s="32" t="n"/>
-      <c r="D115" s="32" t="n"/>
-      <c r="E115" s="22">
+      <c r="A115" s="32" t="n"/>
+      <c r="B115" s="32" t="n"/>
+      <c r="C115" s="33" t="n"/>
+      <c r="D115" s="33" t="n"/>
+      <c r="E115" s="23">
         <f>IF(D115="","",D115*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F115" s="32" t="n"/>
+      <c r="F115" s="33" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="31" t="n"/>
-      <c r="B116" s="31" t="n"/>
-      <c r="C116" s="32" t="n"/>
-      <c r="D116" s="32" t="n"/>
-      <c r="E116" s="22">
+      <c r="A116" s="32" t="n"/>
+      <c r="B116" s="32" t="n"/>
+      <c r="C116" s="33" t="n"/>
+      <c r="D116" s="33" t="n"/>
+      <c r="E116" s="23">
         <f>IF(D116="","",D116*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F116" s="32" t="n"/>
+      <c r="F116" s="33" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="31" t="n"/>
-      <c r="B117" s="31" t="n"/>
-      <c r="C117" s="32" t="n"/>
-      <c r="D117" s="32" t="n"/>
-      <c r="E117" s="22">
+      <c r="A117" s="32" t="n"/>
+      <c r="B117" s="32" t="n"/>
+      <c r="C117" s="33" t="n"/>
+      <c r="D117" s="33" t="n"/>
+      <c r="E117" s="23">
         <f>IF(D117="","",D117*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F117" s="32" t="n"/>
+      <c r="F117" s="33" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="31" t="n"/>
-      <c r="B118" s="31" t="n"/>
-      <c r="C118" s="32" t="n"/>
-      <c r="D118" s="32" t="n"/>
-      <c r="E118" s="22">
+      <c r="A118" s="32" t="n"/>
+      <c r="B118" s="32" t="n"/>
+      <c r="C118" s="33" t="n"/>
+      <c r="D118" s="33" t="n"/>
+      <c r="E118" s="23">
         <f>IF(D118="","",D118*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F118" s="32" t="n"/>
+      <c r="F118" s="33" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="31" t="n"/>
-      <c r="B119" s="31" t="n"/>
-      <c r="C119" s="32" t="n"/>
-      <c r="D119" s="32" t="n"/>
-      <c r="E119" s="22">
+      <c r="A119" s="32" t="n"/>
+      <c r="B119" s="32" t="n"/>
+      <c r="C119" s="33" t="n"/>
+      <c r="D119" s="33" t="n"/>
+      <c r="E119" s="23">
         <f>IF(D119="","",D119*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F119" s="32" t="n"/>
+      <c r="F119" s="33" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="31" t="n"/>
-      <c r="B120" s="31" t="n"/>
-      <c r="C120" s="32" t="n"/>
-      <c r="D120" s="32" t="n"/>
-      <c r="E120" s="22">
+      <c r="A120" s="32" t="n"/>
+      <c r="B120" s="32" t="n"/>
+      <c r="C120" s="33" t="n"/>
+      <c r="D120" s="33" t="n"/>
+      <c r="E120" s="23">
         <f>IF(D120="","",D120*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F120" s="32" t="n"/>
+      <c r="F120" s="33" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="31" t="n"/>
-      <c r="B121" s="31" t="n"/>
-      <c r="C121" s="32" t="n"/>
-      <c r="D121" s="32" t="n"/>
-      <c r="E121" s="22">
+      <c r="A121" s="32" t="n"/>
+      <c r="B121" s="32" t="n"/>
+      <c r="C121" s="33" t="n"/>
+      <c r="D121" s="33" t="n"/>
+      <c r="E121" s="23">
         <f>IF(D121="","",D121*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F121" s="32" t="n"/>
+      <c r="F121" s="33" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="31" t="n"/>
-      <c r="B122" s="31" t="n"/>
-      <c r="C122" s="32" t="n"/>
-      <c r="D122" s="32" t="n"/>
-      <c r="E122" s="22">
+      <c r="A122" s="32" t="n"/>
+      <c r="B122" s="32" t="n"/>
+      <c r="C122" s="33" t="n"/>
+      <c r="D122" s="33" t="n"/>
+      <c r="E122" s="23">
         <f>IF(D122="","",D122*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F122" s="32" t="n"/>
+      <c r="F122" s="33" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="31" t="n"/>
-      <c r="B123" s="31" t="n"/>
-      <c r="C123" s="32" t="n"/>
-      <c r="D123" s="32" t="n"/>
-      <c r="E123" s="22">
+      <c r="A123" s="32" t="n"/>
+      <c r="B123" s="32" t="n"/>
+      <c r="C123" s="33" t="n"/>
+      <c r="D123" s="33" t="n"/>
+      <c r="E123" s="23">
         <f>IF(D123="","",D123*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F123" s="32" t="n"/>
+      <c r="F123" s="33" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="31" t="n"/>
-      <c r="B124" s="31" t="n"/>
-      <c r="C124" s="32" t="n"/>
-      <c r="D124" s="32" t="n"/>
-      <c r="E124" s="22">
+      <c r="A124" s="32" t="n"/>
+      <c r="B124" s="32" t="n"/>
+      <c r="C124" s="33" t="n"/>
+      <c r="D124" s="33" t="n"/>
+      <c r="E124" s="23">
         <f>IF(D124="","",D124*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F124" s="32" t="n"/>
+      <c r="F124" s="33" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="31" t="n"/>
-      <c r="B125" s="31" t="n"/>
-      <c r="C125" s="32" t="n"/>
-      <c r="D125" s="32" t="n"/>
-      <c r="E125" s="22">
+      <c r="A125" s="32" t="n"/>
+      <c r="B125" s="32" t="n"/>
+      <c r="C125" s="33" t="n"/>
+      <c r="D125" s="33" t="n"/>
+      <c r="E125" s="23">
         <f>IF(D125="","",D125*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F125" s="32" t="n"/>
+      <c r="F125" s="33" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="31" t="n"/>
-      <c r="B126" s="31" t="n"/>
-      <c r="C126" s="32" t="n"/>
-      <c r="D126" s="32" t="n"/>
-      <c r="E126" s="22">
+      <c r="A126" s="32" t="n"/>
+      <c r="B126" s="32" t="n"/>
+      <c r="C126" s="33" t="n"/>
+      <c r="D126" s="33" t="n"/>
+      <c r="E126" s="23">
         <f>IF(D126="","",D126*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F126" s="32" t="n"/>
+      <c r="F126" s="33" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="31" t="n"/>
-      <c r="B127" s="31" t="n"/>
-      <c r="C127" s="32" t="n"/>
-      <c r="D127" s="32" t="n"/>
-      <c r="E127" s="22">
+      <c r="A127" s="32" t="n"/>
+      <c r="B127" s="32" t="n"/>
+      <c r="C127" s="33" t="n"/>
+      <c r="D127" s="33" t="n"/>
+      <c r="E127" s="23">
         <f>IF(D127="","",D127*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F127" s="32" t="n"/>
+      <c r="F127" s="33" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="31" t="n"/>
-      <c r="B128" s="31" t="n"/>
-      <c r="C128" s="32" t="n"/>
-      <c r="D128" s="32" t="n"/>
-      <c r="E128" s="22">
+      <c r="A128" s="32" t="n"/>
+      <c r="B128" s="32" t="n"/>
+      <c r="C128" s="33" t="n"/>
+      <c r="D128" s="33" t="n"/>
+      <c r="E128" s="23">
         <f>IF(D128="","",D128*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F128" s="32" t="n"/>
+      <c r="F128" s="33" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="31" t="n"/>
-      <c r="B129" s="31" t="n"/>
-      <c r="C129" s="32" t="n"/>
-      <c r="D129" s="32" t="n"/>
-      <c r="E129" s="22">
+      <c r="A129" s="32" t="n"/>
+      <c r="B129" s="32" t="n"/>
+      <c r="C129" s="33" t="n"/>
+      <c r="D129" s="33" t="n"/>
+      <c r="E129" s="23">
         <f>IF(D129="","",D129*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F129" s="32" t="n"/>
+      <c r="F129" s="33" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="31" t="n"/>
-      <c r="B130" s="31" t="n"/>
-      <c r="C130" s="32" t="n"/>
-      <c r="D130" s="32" t="n"/>
-      <c r="E130" s="22">
+      <c r="A130" s="32" t="n"/>
+      <c r="B130" s="32" t="n"/>
+      <c r="C130" s="33" t="n"/>
+      <c r="D130" s="33" t="n"/>
+      <c r="E130" s="23">
         <f>IF(D130="","",D130*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F130" s="32" t="n"/>
+      <c r="F130" s="33" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="31" t="n"/>
-      <c r="B131" s="31" t="n"/>
-      <c r="C131" s="32" t="n"/>
-      <c r="D131" s="32" t="n"/>
-      <c r="E131" s="22">
+      <c r="A131" s="32" t="n"/>
+      <c r="B131" s="32" t="n"/>
+      <c r="C131" s="33" t="n"/>
+      <c r="D131" s="33" t="n"/>
+      <c r="E131" s="23">
         <f>IF(D131="","",D131*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F131" s="32" t="n"/>
+      <c r="F131" s="33" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="31" t="n"/>
-      <c r="B132" s="31" t="n"/>
-      <c r="C132" s="32" t="n"/>
-      <c r="D132" s="32" t="n"/>
-      <c r="E132" s="22">
+      <c r="A132" s="32" t="n"/>
+      <c r="B132" s="32" t="n"/>
+      <c r="C132" s="33" t="n"/>
+      <c r="D132" s="33" t="n"/>
+      <c r="E132" s="23">
         <f>IF(D132="","",D132*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F132" s="32" t="n"/>
+      <c r="F132" s="33" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="31" t="n"/>
-      <c r="B133" s="31" t="n"/>
-      <c r="C133" s="32" t="n"/>
-      <c r="D133" s="32" t="n"/>
-      <c r="E133" s="22">
+      <c r="A133" s="32" t="n"/>
+      <c r="B133" s="32" t="n"/>
+      <c r="C133" s="33" t="n"/>
+      <c r="D133" s="33" t="n"/>
+      <c r="E133" s="23">
         <f>IF(D133="","",D133*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F133" s="32" t="n"/>
+      <c r="F133" s="33" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="31" t="n"/>
-      <c r="B134" s="31" t="n"/>
-      <c r="C134" s="32" t="n"/>
-      <c r="D134" s="32" t="n"/>
-      <c r="E134" s="22">
+      <c r="A134" s="32" t="n"/>
+      <c r="B134" s="32" t="n"/>
+      <c r="C134" s="33" t="n"/>
+      <c r="D134" s="33" t="n"/>
+      <c r="E134" s="23">
         <f>IF(D134="","",D134*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F134" s="32" t="n"/>
+      <c r="F134" s="33" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="31" t="n"/>
-      <c r="B135" s="31" t="n"/>
-      <c r="C135" s="32" t="n"/>
-      <c r="D135" s="32" t="n"/>
-      <c r="E135" s="22">
+      <c r="A135" s="32" t="n"/>
+      <c r="B135" s="32" t="n"/>
+      <c r="C135" s="33" t="n"/>
+      <c r="D135" s="33" t="n"/>
+      <c r="E135" s="23">
         <f>IF(D135="","",D135*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F135" s="32" t="n"/>
+      <c r="F135" s="33" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="31" t="n"/>
-      <c r="B136" s="31" t="n"/>
-      <c r="C136" s="32" t="n"/>
-      <c r="D136" s="32" t="n"/>
-      <c r="E136" s="22">
+      <c r="A136" s="32" t="n"/>
+      <c r="B136" s="32" t="n"/>
+      <c r="C136" s="33" t="n"/>
+      <c r="D136" s="33" t="n"/>
+      <c r="E136" s="23">
         <f>IF(D136="","",D136*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F136" s="32" t="n"/>
+      <c r="F136" s="33" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="31" t="n"/>
-      <c r="B137" s="31" t="n"/>
-      <c r="C137" s="32" t="n"/>
-      <c r="D137" s="32" t="n"/>
-      <c r="E137" s="22">
+      <c r="A137" s="32" t="n"/>
+      <c r="B137" s="32" t="n"/>
+      <c r="C137" s="33" t="n"/>
+      <c r="D137" s="33" t="n"/>
+      <c r="E137" s="23">
         <f>IF(D137="","",D137*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F137" s="32" t="n"/>
+      <c r="F137" s="33" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="31" t="n"/>
-      <c r="B138" s="31" t="n"/>
-      <c r="C138" s="32" t="n"/>
-      <c r="D138" s="32" t="n"/>
-      <c r="E138" s="22">
+      <c r="A138" s="32" t="n"/>
+      <c r="B138" s="32" t="n"/>
+      <c r="C138" s="33" t="n"/>
+      <c r="D138" s="33" t="n"/>
+      <c r="E138" s="23">
         <f>IF(D138="","",D138*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F138" s="32" t="n"/>
+      <c r="F138" s="33" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="31" t="n"/>
-      <c r="B139" s="31" t="n"/>
-      <c r="C139" s="32" t="n"/>
-      <c r="D139" s="32" t="n"/>
-      <c r="E139" s="22">
+      <c r="A139" s="32" t="n"/>
+      <c r="B139" s="32" t="n"/>
+      <c r="C139" s="33" t="n"/>
+      <c r="D139" s="33" t="n"/>
+      <c r="E139" s="23">
         <f>IF(D139="","",D139*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F139" s="32" t="n"/>
+      <c r="F139" s="33" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="31" t="n"/>
-      <c r="B140" s="31" t="n"/>
-      <c r="C140" s="32" t="n"/>
-      <c r="D140" s="32" t="n"/>
-      <c r="E140" s="22">
+      <c r="A140" s="32" t="n"/>
+      <c r="B140" s="32" t="n"/>
+      <c r="C140" s="33" t="n"/>
+      <c r="D140" s="33" t="n"/>
+      <c r="E140" s="23">
         <f>IF(D140="","",D140*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F140" s="32" t="n"/>
+      <c r="F140" s="33" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="31" t="n"/>
-      <c r="B141" s="31" t="n"/>
-      <c r="C141" s="32" t="n"/>
-      <c r="D141" s="32" t="n"/>
-      <c r="E141" s="22">
+      <c r="A141" s="32" t="n"/>
+      <c r="B141" s="32" t="n"/>
+      <c r="C141" s="33" t="n"/>
+      <c r="D141" s="33" t="n"/>
+      <c r="E141" s="23">
         <f>IF(D141="","",D141*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F141" s="32" t="n"/>
+      <c r="F141" s="33" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="31" t="n"/>
-      <c r="B142" s="31" t="n"/>
-      <c r="C142" s="32" t="n"/>
-      <c r="D142" s="32" t="n"/>
-      <c r="E142" s="22">
+      <c r="A142" s="32" t="n"/>
+      <c r="B142" s="32" t="n"/>
+      <c r="C142" s="33" t="n"/>
+      <c r="D142" s="33" t="n"/>
+      <c r="E142" s="23">
         <f>IF(D142="","",D142*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F142" s="32" t="n"/>
+      <c r="F142" s="33" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="31" t="n"/>
-      <c r="B143" s="31" t="n"/>
-      <c r="C143" s="32" t="n"/>
-      <c r="D143" s="32" t="n"/>
-      <c r="E143" s="22">
+      <c r="A143" s="32" t="n"/>
+      <c r="B143" s="32" t="n"/>
+      <c r="C143" s="33" t="n"/>
+      <c r="D143" s="33" t="n"/>
+      <c r="E143" s="23">
         <f>IF(D143="","",D143*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F143" s="32" t="n"/>
+      <c r="F143" s="33" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="31" t="n"/>
-      <c r="B144" s="31" t="n"/>
-      <c r="C144" s="32" t="n"/>
-      <c r="D144" s="32" t="n"/>
-      <c r="E144" s="22">
+      <c r="A144" s="32" t="n"/>
+      <c r="B144" s="32" t="n"/>
+      <c r="C144" s="33" t="n"/>
+      <c r="D144" s="33" t="n"/>
+      <c r="E144" s="23">
         <f>IF(D144="","",D144*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F144" s="32" t="n"/>
+      <c r="F144" s="33" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="31" t="n"/>
-      <c r="B145" s="31" t="n"/>
-      <c r="C145" s="32" t="n"/>
-      <c r="D145" s="32" t="n"/>
-      <c r="E145" s="22">
+      <c r="A145" s="32" t="n"/>
+      <c r="B145" s="32" t="n"/>
+      <c r="C145" s="33" t="n"/>
+      <c r="D145" s="33" t="n"/>
+      <c r="E145" s="23">
         <f>IF(D145="","",D145*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F145" s="32" t="n"/>
+      <c r="F145" s="33" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="31" t="n"/>
-      <c r="B146" s="31" t="n"/>
-      <c r="C146" s="32" t="n"/>
-      <c r="D146" s="32" t="n"/>
-      <c r="E146" s="22">
+      <c r="A146" s="32" t="n"/>
+      <c r="B146" s="32" t="n"/>
+      <c r="C146" s="33" t="n"/>
+      <c r="D146" s="33" t="n"/>
+      <c r="E146" s="23">
         <f>IF(D146="","",D146*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F146" s="32" t="n"/>
+      <c r="F146" s="33" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="31" t="n"/>
-      <c r="B147" s="31" t="n"/>
-      <c r="C147" s="32" t="n"/>
-      <c r="D147" s="32" t="n"/>
-      <c r="E147" s="22">
+      <c r="A147" s="32" t="n"/>
+      <c r="B147" s="32" t="n"/>
+      <c r="C147" s="33" t="n"/>
+      <c r="D147" s="33" t="n"/>
+      <c r="E147" s="23">
         <f>IF(D147="","",D147*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F147" s="32" t="n"/>
+      <c r="F147" s="33" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="31" t="n"/>
-      <c r="B148" s="31" t="n"/>
-      <c r="C148" s="32" t="n"/>
-      <c r="D148" s="32" t="n"/>
-      <c r="E148" s="22">
+      <c r="A148" s="32" t="n"/>
+      <c r="B148" s="32" t="n"/>
+      <c r="C148" s="33" t="n"/>
+      <c r="D148" s="33" t="n"/>
+      <c r="E148" s="23">
         <f>IF(D148="","",D148*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F148" s="32" t="n"/>
+      <c r="F148" s="33" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="31" t="n"/>
-      <c r="B149" s="31" t="n"/>
-      <c r="C149" s="32" t="n"/>
-      <c r="D149" s="32" t="n"/>
-      <c r="E149" s="22">
+      <c r="A149" s="32" t="n"/>
+      <c r="B149" s="32" t="n"/>
+      <c r="C149" s="33" t="n"/>
+      <c r="D149" s="33" t="n"/>
+      <c r="E149" s="23">
         <f>IF(D149="","",D149*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F149" s="32" t="n"/>
+      <c r="F149" s="33" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="31" t="n"/>
-      <c r="B150" s="31" t="n"/>
-      <c r="C150" s="32" t="n"/>
-      <c r="D150" s="32" t="n"/>
-      <c r="E150" s="22">
+      <c r="A150" s="32" t="n"/>
+      <c r="B150" s="32" t="n"/>
+      <c r="C150" s="33" t="n"/>
+      <c r="D150" s="33" t="n"/>
+      <c r="E150" s="23">
         <f>IF(D150="","",D150*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F150" s="32" t="n"/>
+      <c r="F150" s="33" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="31" t="n"/>
-      <c r="B151" s="31" t="n"/>
-      <c r="C151" s="32" t="n"/>
-      <c r="D151" s="32" t="n"/>
-      <c r="E151" s="22">
+      <c r="A151" s="32" t="n"/>
+      <c r="B151" s="32" t="n"/>
+      <c r="C151" s="33" t="n"/>
+      <c r="D151" s="33" t="n"/>
+      <c r="E151" s="23">
         <f>IF(D151="","",D151*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F151" s="32" t="n"/>
+      <c r="F151" s="33" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="31" t="n"/>
-      <c r="B152" s="31" t="n"/>
-      <c r="C152" s="32" t="n"/>
-      <c r="D152" s="32" t="n"/>
-      <c r="E152" s="22">
+      <c r="A152" s="32" t="n"/>
+      <c r="B152" s="32" t="n"/>
+      <c r="C152" s="33" t="n"/>
+      <c r="D152" s="33" t="n"/>
+      <c r="E152" s="23">
         <f>IF(D152="","",D152*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F152" s="32" t="n"/>
+      <c r="F152" s="33" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="31" t="n"/>
-      <c r="B153" s="31" t="n"/>
-      <c r="C153" s="32" t="n"/>
-      <c r="D153" s="32" t="n"/>
-      <c r="E153" s="22">
+      <c r="A153" s="32" t="n"/>
+      <c r="B153" s="32" t="n"/>
+      <c r="C153" s="33" t="n"/>
+      <c r="D153" s="33" t="n"/>
+      <c r="E153" s="23">
         <f>IF(D153="","",D153*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F153" s="32" t="n"/>
+      <c r="F153" s="33" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="31" t="n"/>
-      <c r="B154" s="31" t="n"/>
-      <c r="C154" s="32" t="n"/>
-      <c r="D154" s="32" t="n"/>
-      <c r="E154" s="22">
+      <c r="A154" s="32" t="n"/>
+      <c r="B154" s="32" t="n"/>
+      <c r="C154" s="33" t="n"/>
+      <c r="D154" s="33" t="n"/>
+      <c r="E154" s="23">
         <f>IF(D154="","",D154*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F154" s="32" t="n"/>
+      <c r="F154" s="33" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="31" t="n"/>
-      <c r="B155" s="31" t="n"/>
-      <c r="C155" s="32" t="n"/>
-      <c r="D155" s="32" t="n"/>
-      <c r="E155" s="22">
+      <c r="A155" s="32" t="n"/>
+      <c r="B155" s="32" t="n"/>
+      <c r="C155" s="33" t="n"/>
+      <c r="D155" s="33" t="n"/>
+      <c r="E155" s="23">
         <f>IF(D155="","",D155*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F155" s="32" t="n"/>
+      <c r="F155" s="33" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="31" t="n"/>
-      <c r="B156" s="31" t="n"/>
-      <c r="C156" s="32" t="n"/>
-      <c r="D156" s="32" t="n"/>
-      <c r="E156" s="22">
+      <c r="A156" s="32" t="n"/>
+      <c r="B156" s="32" t="n"/>
+      <c r="C156" s="33" t="n"/>
+      <c r="D156" s="33" t="n"/>
+      <c r="E156" s="23">
         <f>IF(D156="","",D156*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F156" s="32" t="n"/>
+      <c r="F156" s="33" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="31" t="n"/>
-      <c r="B157" s="31" t="n"/>
-      <c r="C157" s="32" t="n"/>
-      <c r="D157" s="32" t="n"/>
-      <c r="E157" s="22">
+      <c r="A157" s="32" t="n"/>
+      <c r="B157" s="32" t="n"/>
+      <c r="C157" s="33" t="n"/>
+      <c r="D157" s="33" t="n"/>
+      <c r="E157" s="23">
         <f>IF(D157="","",D157*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F157" s="32" t="n"/>
+      <c r="F157" s="33" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="31" t="n"/>
-      <c r="B158" s="31" t="n"/>
-      <c r="C158" s="32" t="n"/>
-      <c r="D158" s="32" t="n"/>
-      <c r="E158" s="22">
+      <c r="A158" s="32" t="n"/>
+      <c r="B158" s="32" t="n"/>
+      <c r="C158" s="33" t="n"/>
+      <c r="D158" s="33" t="n"/>
+      <c r="E158" s="23">
         <f>IF(D158="","",D158*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F158" s="32" t="n"/>
+      <c r="F158" s="33" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="31" t="n"/>
-      <c r="B159" s="31" t="n"/>
-      <c r="C159" s="32" t="n"/>
-      <c r="D159" s="32" t="n"/>
-      <c r="E159" s="22">
+      <c r="A159" s="32" t="n"/>
+      <c r="B159" s="32" t="n"/>
+      <c r="C159" s="33" t="n"/>
+      <c r="D159" s="33" t="n"/>
+      <c r="E159" s="23">
         <f>IF(D159="","",D159*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F159" s="32" t="n"/>
+      <c r="F159" s="33" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="31" t="n"/>
-      <c r="B160" s="31" t="n"/>
-      <c r="C160" s="32" t="n"/>
-      <c r="D160" s="32" t="n"/>
-      <c r="E160" s="22">
+      <c r="A160" s="32" t="n"/>
+      <c r="B160" s="32" t="n"/>
+      <c r="C160" s="33" t="n"/>
+      <c r="D160" s="33" t="n"/>
+      <c r="E160" s="23">
         <f>IF(D160="","",D160*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F160" s="32" t="n"/>
+      <c r="F160" s="33" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="31" t="n"/>
-      <c r="B161" s="31" t="n"/>
-      <c r="C161" s="32" t="n"/>
-      <c r="D161" s="32" t="n"/>
-      <c r="E161" s="22">
+      <c r="A161" s="32" t="n"/>
+      <c r="B161" s="32" t="n"/>
+      <c r="C161" s="33" t="n"/>
+      <c r="D161" s="33" t="n"/>
+      <c r="E161" s="23">
         <f>IF(D161="","",D161*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F161" s="32" t="n"/>
+      <c r="F161" s="33" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="31" t="n"/>
-      <c r="B162" s="31" t="n"/>
-      <c r="C162" s="32" t="n"/>
-      <c r="D162" s="32" t="n"/>
-      <c r="E162" s="22">
+      <c r="A162" s="32" t="n"/>
+      <c r="B162" s="32" t="n"/>
+      <c r="C162" s="33" t="n"/>
+      <c r="D162" s="33" t="n"/>
+      <c r="E162" s="23">
         <f>IF(D162="","",D162*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F162" s="32" t="n"/>
+      <c r="F162" s="33" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="31" t="n"/>
-      <c r="B163" s="31" t="n"/>
-      <c r="C163" s="32" t="n"/>
-      <c r="D163" s="32" t="n"/>
-      <c r="E163" s="22">
+      <c r="A163" s="32" t="n"/>
+      <c r="B163" s="32" t="n"/>
+      <c r="C163" s="33" t="n"/>
+      <c r="D163" s="33" t="n"/>
+      <c r="E163" s="23">
         <f>IF(D163="","",D163*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F163" s="32" t="n"/>
+      <c r="F163" s="33" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="31" t="n"/>
-      <c r="B164" s="31" t="n"/>
-      <c r="C164" s="32" t="n"/>
-      <c r="D164" s="32" t="n"/>
-      <c r="E164" s="22">
+      <c r="A164" s="32" t="n"/>
+      <c r="B164" s="32" t="n"/>
+      <c r="C164" s="33" t="n"/>
+      <c r="D164" s="33" t="n"/>
+      <c r="E164" s="23">
         <f>IF(D164="","",D164*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F164" s="32" t="n"/>
+      <c r="F164" s="33" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="31" t="n"/>
-      <c r="B165" s="31" t="n"/>
-      <c r="C165" s="32" t="n"/>
-      <c r="D165" s="32" t="n"/>
-      <c r="E165" s="22">
+      <c r="A165" s="32" t="n"/>
+      <c r="B165" s="32" t="n"/>
+      <c r="C165" s="33" t="n"/>
+      <c r="D165" s="33" t="n"/>
+      <c r="E165" s="23">
         <f>IF(D165="","",D165*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F165" s="32" t="n"/>
+      <c r="F165" s="33" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="31" t="n"/>
-      <c r="B166" s="31" t="n"/>
-      <c r="C166" s="32" t="n"/>
-      <c r="D166" s="32" t="n"/>
-      <c r="E166" s="22">
+      <c r="A166" s="32" t="n"/>
+      <c r="B166" s="32" t="n"/>
+      <c r="C166" s="33" t="n"/>
+      <c r="D166" s="33" t="n"/>
+      <c r="E166" s="23">
         <f>IF(D166="","",D166*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F166" s="32" t="n"/>
+      <c r="F166" s="33" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="31" t="n"/>
-      <c r="B167" s="31" t="n"/>
-      <c r="C167" s="32" t="n"/>
-      <c r="D167" s="32" t="n"/>
-      <c r="E167" s="22">
+      <c r="A167" s="32" t="n"/>
+      <c r="B167" s="32" t="n"/>
+      <c r="C167" s="33" t="n"/>
+      <c r="D167" s="33" t="n"/>
+      <c r="E167" s="23">
         <f>IF(D167="","",D167*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F167" s="32" t="n"/>
+      <c r="F167" s="33" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="31" t="n"/>
-      <c r="B168" s="31" t="n"/>
-      <c r="C168" s="32" t="n"/>
-      <c r="D168" s="32" t="n"/>
-      <c r="E168" s="22">
+      <c r="A168" s="32" t="n"/>
+      <c r="B168" s="32" t="n"/>
+      <c r="C168" s="33" t="n"/>
+      <c r="D168" s="33" t="n"/>
+      <c r="E168" s="23">
         <f>IF(D168="","",D168*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F168" s="32" t="n"/>
+      <c r="F168" s="33" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" s="31" t="n"/>
-      <c r="B169" s="31" t="n"/>
-      <c r="C169" s="32" t="n"/>
-      <c r="D169" s="32" t="n"/>
-      <c r="E169" s="22">
+      <c r="A169" s="32" t="n"/>
+      <c r="B169" s="32" t="n"/>
+      <c r="C169" s="33" t="n"/>
+      <c r="D169" s="33" t="n"/>
+      <c r="E169" s="23">
         <f>IF(D169="","",D169*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F169" s="32" t="n"/>
+      <c r="F169" s="33" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="31" t="n"/>
-      <c r="B170" s="31" t="n"/>
-      <c r="C170" s="32" t="n"/>
-      <c r="D170" s="32" t="n"/>
-      <c r="E170" s="22">
+      <c r="A170" s="32" t="n"/>
+      <c r="B170" s="32" t="n"/>
+      <c r="C170" s="33" t="n"/>
+      <c r="D170" s="33" t="n"/>
+      <c r="E170" s="23">
         <f>IF(D170="","",D170*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F170" s="32" t="n"/>
+      <c r="F170" s="33" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="31" t="n"/>
-      <c r="B171" s="31" t="n"/>
-      <c r="C171" s="32" t="n"/>
-      <c r="D171" s="32" t="n"/>
-      <c r="E171" s="22">
+      <c r="A171" s="32" t="n"/>
+      <c r="B171" s="32" t="n"/>
+      <c r="C171" s="33" t="n"/>
+      <c r="D171" s="33" t="n"/>
+      <c r="E171" s="23">
         <f>IF(D171="","",D171*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F171" s="32" t="n"/>
+      <c r="F171" s="33" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="31" t="n"/>
-      <c r="B172" s="31" t="n"/>
-      <c r="C172" s="32" t="n"/>
-      <c r="D172" s="32" t="n"/>
-      <c r="E172" s="22">
+      <c r="A172" s="32" t="n"/>
+      <c r="B172" s="32" t="n"/>
+      <c r="C172" s="33" t="n"/>
+      <c r="D172" s="33" t="n"/>
+      <c r="E172" s="23">
         <f>IF(D172="","",D172*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F172" s="32" t="n"/>
+      <c r="F172" s="33" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" s="31" t="n"/>
-      <c r="B173" s="31" t="n"/>
-      <c r="C173" s="32" t="n"/>
-      <c r="D173" s="32" t="n"/>
-      <c r="E173" s="22">
+      <c r="A173" s="32" t="n"/>
+      <c r="B173" s="32" t="n"/>
+      <c r="C173" s="33" t="n"/>
+      <c r="D173" s="33" t="n"/>
+      <c r="E173" s="23">
         <f>IF(D173="","",D173*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F173" s="32" t="n"/>
+      <c r="F173" s="33" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="31" t="n"/>
-      <c r="B174" s="31" t="n"/>
-      <c r="C174" s="32" t="n"/>
-      <c r="D174" s="32" t="n"/>
-      <c r="E174" s="22">
+      <c r="A174" s="32" t="n"/>
+      <c r="B174" s="32" t="n"/>
+      <c r="C174" s="33" t="n"/>
+      <c r="D174" s="33" t="n"/>
+      <c r="E174" s="23">
         <f>IF(D174="","",D174*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F174" s="32" t="n"/>
+      <c r="F174" s="33" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="31" t="n"/>
-      <c r="B175" s="31" t="n"/>
-      <c r="C175" s="32" t="n"/>
-      <c r="D175" s="32" t="n"/>
-      <c r="E175" s="22">
+      <c r="A175" s="32" t="n"/>
+      <c r="B175" s="32" t="n"/>
+      <c r="C175" s="33" t="n"/>
+      <c r="D175" s="33" t="n"/>
+      <c r="E175" s="23">
         <f>IF(D175="","",D175*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F175" s="32" t="n"/>
+      <c r="F175" s="33" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" s="31" t="n"/>
-      <c r="B176" s="31" t="n"/>
-      <c r="C176" s="32" t="n"/>
-      <c r="D176" s="32" t="n"/>
-      <c r="E176" s="22">
+      <c r="A176" s="32" t="n"/>
+      <c r="B176" s="32" t="n"/>
+      <c r="C176" s="33" t="n"/>
+      <c r="D176" s="33" t="n"/>
+      <c r="E176" s="23">
         <f>IF(D176="","",D176*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F176" s="32" t="n"/>
+      <c r="F176" s="33" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="31" t="n"/>
-      <c r="B177" s="31" t="n"/>
-      <c r="C177" s="32" t="n"/>
-      <c r="D177" s="32" t="n"/>
-      <c r="E177" s="22">
+      <c r="A177" s="32" t="n"/>
+      <c r="B177" s="32" t="n"/>
+      <c r="C177" s="33" t="n"/>
+      <c r="D177" s="33" t="n"/>
+      <c r="E177" s="23">
         <f>IF(D177="","",D177*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F177" s="32" t="n"/>
+      <c r="F177" s="33" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="31" t="n"/>
-      <c r="B178" s="31" t="n"/>
-      <c r="C178" s="32" t="n"/>
-      <c r="D178" s="32" t="n"/>
-      <c r="E178" s="22">
+      <c r="A178" s="32" t="n"/>
+      <c r="B178" s="32" t="n"/>
+      <c r="C178" s="33" t="n"/>
+      <c r="D178" s="33" t="n"/>
+      <c r="E178" s="23">
         <f>IF(D178="","",D178*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F178" s="32" t="n"/>
+      <c r="F178" s="33" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" s="31" t="n"/>
-      <c r="B179" s="31" t="n"/>
-      <c r="C179" s="32" t="n"/>
-      <c r="D179" s="32" t="n"/>
-      <c r="E179" s="22">
+      <c r="A179" s="32" t="n"/>
+      <c r="B179" s="32" t="n"/>
+      <c r="C179" s="33" t="n"/>
+      <c r="D179" s="33" t="n"/>
+      <c r="E179" s="23">
         <f>IF(D179="","",D179*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F179" s="32" t="n"/>
+      <c r="F179" s="33" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" s="31" t="n"/>
-      <c r="B180" s="31" t="n"/>
-      <c r="C180" s="32" t="n"/>
-      <c r="D180" s="32" t="n"/>
-      <c r="E180" s="22">
+      <c r="A180" s="32" t="n"/>
+      <c r="B180" s="32" t="n"/>
+      <c r="C180" s="33" t="n"/>
+      <c r="D180" s="33" t="n"/>
+      <c r="E180" s="23">
         <f>IF(D180="","",D180*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F180" s="32" t="n"/>
+      <c r="F180" s="33" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="31" t="n"/>
-      <c r="B181" s="31" t="n"/>
-      <c r="C181" s="32" t="n"/>
-      <c r="D181" s="32" t="n"/>
-      <c r="E181" s="22">
+      <c r="A181" s="32" t="n"/>
+      <c r="B181" s="32" t="n"/>
+      <c r="C181" s="33" t="n"/>
+      <c r="D181" s="33" t="n"/>
+      <c r="E181" s="23">
         <f>IF(D181="","",D181*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F181" s="32" t="n"/>
+      <c r="F181" s="33" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="31" t="n"/>
-      <c r="B182" s="31" t="n"/>
-      <c r="C182" s="32" t="n"/>
-      <c r="D182" s="32" t="n"/>
-      <c r="E182" s="22">
+      <c r="A182" s="32" t="n"/>
+      <c r="B182" s="32" t="n"/>
+      <c r="C182" s="33" t="n"/>
+      <c r="D182" s="33" t="n"/>
+      <c r="E182" s="23">
         <f>IF(D182="","",D182*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F182" s="32" t="n"/>
+      <c r="F182" s="33" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="31" t="n"/>
-      <c r="B183" s="31" t="n"/>
-      <c r="C183" s="32" t="n"/>
-      <c r="D183" s="32" t="n"/>
-      <c r="E183" s="22">
+      <c r="A183" s="32" t="n"/>
+      <c r="B183" s="32" t="n"/>
+      <c r="C183" s="33" t="n"/>
+      <c r="D183" s="33" t="n"/>
+      <c r="E183" s="23">
         <f>IF(D183="","",D183*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F183" s="32" t="n"/>
+      <c r="F183" s="33" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="31" t="n"/>
-      <c r="B184" s="31" t="n"/>
-      <c r="C184" s="32" t="n"/>
-      <c r="D184" s="32" t="n"/>
-      <c r="E184" s="22">
+      <c r="A184" s="32" t="n"/>
+      <c r="B184" s="32" t="n"/>
+      <c r="C184" s="33" t="n"/>
+      <c r="D184" s="33" t="n"/>
+      <c r="E184" s="23">
         <f>IF(D184="","",D184*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F184" s="32" t="n"/>
+      <c r="F184" s="33" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="31" t="n"/>
-      <c r="B185" s="31" t="n"/>
-      <c r="C185" s="32" t="n"/>
-      <c r="D185" s="32" t="n"/>
-      <c r="E185" s="22">
+      <c r="A185" s="32" t="n"/>
+      <c r="B185" s="32" t="n"/>
+      <c r="C185" s="33" t="n"/>
+      <c r="D185" s="33" t="n"/>
+      <c r="E185" s="23">
         <f>IF(D185="","",D185*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F185" s="32" t="n"/>
+      <c r="F185" s="33" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="31" t="n"/>
-      <c r="B186" s="31" t="n"/>
-      <c r="C186" s="32" t="n"/>
-      <c r="D186" s="32" t="n"/>
-      <c r="E186" s="22">
+      <c r="A186" s="32" t="n"/>
+      <c r="B186" s="32" t="n"/>
+      <c r="C186" s="33" t="n"/>
+      <c r="D186" s="33" t="n"/>
+      <c r="E186" s="23">
         <f>IF(D186="","",D186*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F186" s="32" t="n"/>
+      <c r="F186" s="33" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" s="31" t="n"/>
-      <c r="B187" s="31" t="n"/>
-      <c r="C187" s="32" t="n"/>
-      <c r="D187" s="32" t="n"/>
-      <c r="E187" s="22">
+      <c r="A187" s="32" t="n"/>
+      <c r="B187" s="32" t="n"/>
+      <c r="C187" s="33" t="n"/>
+      <c r="D187" s="33" t="n"/>
+      <c r="E187" s="23">
         <f>IF(D187="","",D187*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F187" s="32" t="n"/>
+      <c r="F187" s="33" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" s="31" t="n"/>
-      <c r="B188" s="31" t="n"/>
-      <c r="C188" s="32" t="n"/>
-      <c r="D188" s="32" t="n"/>
-      <c r="E188" s="22">
+      <c r="A188" s="32" t="n"/>
+      <c r="B188" s="32" t="n"/>
+      <c r="C188" s="33" t="n"/>
+      <c r="D188" s="33" t="n"/>
+      <c r="E188" s="23">
         <f>IF(D188="","",D188*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F188" s="32" t="n"/>
+      <c r="F188" s="33" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" s="31" t="n"/>
-      <c r="B189" s="31" t="n"/>
-      <c r="C189" s="32" t="n"/>
-      <c r="D189" s="32" t="n"/>
-      <c r="E189" s="22">
+      <c r="A189" s="32" t="n"/>
+      <c r="B189" s="32" t="n"/>
+      <c r="C189" s="33" t="n"/>
+      <c r="D189" s="33" t="n"/>
+      <c r="E189" s="23">
         <f>IF(D189="","",D189*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F189" s="32" t="n"/>
+      <c r="F189" s="33" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" s="31" t="n"/>
-      <c r="B190" s="31" t="n"/>
-      <c r="C190" s="32" t="n"/>
-      <c r="D190" s="32" t="n"/>
-      <c r="E190" s="22">
+      <c r="A190" s="32" t="n"/>
+      <c r="B190" s="32" t="n"/>
+      <c r="C190" s="33" t="n"/>
+      <c r="D190" s="33" t="n"/>
+      <c r="E190" s="23">
         <f>IF(D190="","",D190*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F190" s="32" t="n"/>
+      <c r="F190" s="33" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="31" t="n"/>
-      <c r="B191" s="31" t="n"/>
-      <c r="C191" s="32" t="n"/>
-      <c r="D191" s="32" t="n"/>
-      <c r="E191" s="22">
+      <c r="A191" s="32" t="n"/>
+      <c r="B191" s="32" t="n"/>
+      <c r="C191" s="33" t="n"/>
+      <c r="D191" s="33" t="n"/>
+      <c r="E191" s="23">
         <f>IF(D191="","",D191*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F191" s="32" t="n"/>
+      <c r="F191" s="33" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="31" t="n"/>
-      <c r="B192" s="31" t="n"/>
-      <c r="C192" s="32" t="n"/>
-      <c r="D192" s="32" t="n"/>
-      <c r="E192" s="22">
+      <c r="A192" s="32" t="n"/>
+      <c r="B192" s="32" t="n"/>
+      <c r="C192" s="33" t="n"/>
+      <c r="D192" s="33" t="n"/>
+      <c r="E192" s="23">
         <f>IF(D192="","",D192*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F192" s="32" t="n"/>
+      <c r="F192" s="33" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="31" t="n"/>
-      <c r="B193" s="31" t="n"/>
-      <c r="C193" s="32" t="n"/>
-      <c r="D193" s="32" t="n"/>
-      <c r="E193" s="22">
+      <c r="A193" s="32" t="n"/>
+      <c r="B193" s="32" t="n"/>
+      <c r="C193" s="33" t="n"/>
+      <c r="D193" s="33" t="n"/>
+      <c r="E193" s="23">
         <f>IF(D193="","",D193*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F193" s="32" t="n"/>
+      <c r="F193" s="33" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="31" t="n"/>
-      <c r="B194" s="31" t="n"/>
-      <c r="C194" s="32" t="n"/>
-      <c r="D194" s="32" t="n"/>
-      <c r="E194" s="22">
+      <c r="A194" s="32" t="n"/>
+      <c r="B194" s="32" t="n"/>
+      <c r="C194" s="33" t="n"/>
+      <c r="D194" s="33" t="n"/>
+      <c r="E194" s="23">
         <f>IF(D194="","",D194*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F194" s="32" t="n"/>
+      <c r="F194" s="33" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="31" t="n"/>
-      <c r="B195" s="31" t="n"/>
-      <c r="C195" s="32" t="n"/>
-      <c r="D195" s="32" t="n"/>
-      <c r="E195" s="22">
+      <c r="A195" s="32" t="n"/>
+      <c r="B195" s="32" t="n"/>
+      <c r="C195" s="33" t="n"/>
+      <c r="D195" s="33" t="n"/>
+      <c r="E195" s="23">
         <f>IF(D195="","",D195*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F195" s="32" t="n"/>
+      <c r="F195" s="33" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="31" t="n"/>
-      <c r="B196" s="31" t="n"/>
-      <c r="C196" s="32" t="n"/>
-      <c r="D196" s="32" t="n"/>
-      <c r="E196" s="22">
+      <c r="A196" s="32" t="n"/>
+      <c r="B196" s="32" t="n"/>
+      <c r="C196" s="33" t="n"/>
+      <c r="D196" s="33" t="n"/>
+      <c r="E196" s="23">
         <f>IF(D196="","",D196*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F196" s="32" t="n"/>
+      <c r="F196" s="33" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="31" t="n"/>
-      <c r="B197" s="31" t="n"/>
-      <c r="C197" s="32" t="n"/>
-      <c r="D197" s="32" t="n"/>
-      <c r="E197" s="22">
+      <c r="A197" s="32" t="n"/>
+      <c r="B197" s="32" t="n"/>
+      <c r="C197" s="33" t="n"/>
+      <c r="D197" s="33" t="n"/>
+      <c r="E197" s="23">
         <f>IF(D197="","",D197*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F197" s="32" t="n"/>
+      <c r="F197" s="33" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="31" t="n"/>
-      <c r="B198" s="31" t="n"/>
-      <c r="C198" s="32" t="n"/>
-      <c r="D198" s="32" t="n"/>
-      <c r="E198" s="22">
+      <c r="A198" s="32" t="n"/>
+      <c r="B198" s="32" t="n"/>
+      <c r="C198" s="33" t="n"/>
+      <c r="D198" s="33" t="n"/>
+      <c r="E198" s="23">
         <f>IF(D198="","",D198*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F198" s="32" t="n"/>
+      <c r="F198" s="33" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" s="31" t="n"/>
-      <c r="B199" s="31" t="n"/>
-      <c r="C199" s="32" t="n"/>
-      <c r="D199" s="32" t="n"/>
-      <c r="E199" s="22">
+      <c r="A199" s="32" t="n"/>
+      <c r="B199" s="32" t="n"/>
+      <c r="C199" s="33" t="n"/>
+      <c r="D199" s="33" t="n"/>
+      <c r="E199" s="23">
         <f>IF(D199="","",D199*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F199" s="32" t="n"/>
+      <c r="F199" s="33" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="31" t="n"/>
-      <c r="B200" s="31" t="n"/>
-      <c r="C200" s="32" t="n"/>
-      <c r="D200" s="32" t="n"/>
-      <c r="E200" s="22">
+      <c r="A200" s="32" t="n"/>
+      <c r="B200" s="32" t="n"/>
+      <c r="C200" s="33" t="n"/>
+      <c r="D200" s="33" t="n"/>
+      <c r="E200" s="23">
         <f>IF(D200="","",D200*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F200" s="32" t="n"/>
+      <c r="F200" s="33" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" s="31" t="n"/>
-      <c r="B201" s="31" t="n"/>
-      <c r="C201" s="32" t="n"/>
-      <c r="D201" s="32" t="n"/>
-      <c r="E201" s="22">
+      <c r="A201" s="32" t="n"/>
+      <c r="B201" s="32" t="n"/>
+      <c r="C201" s="33" t="n"/>
+      <c r="D201" s="33" t="n"/>
+      <c r="E201" s="23">
         <f>IF(D201="","",D201*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F201" s="32" t="n"/>
+      <c r="F201" s="33" t="n"/>
     </row>
     <row r="202">
-      <c r="A202" s="31" t="n"/>
-      <c r="B202" s="31" t="n"/>
-      <c r="C202" s="32" t="n"/>
-      <c r="D202" s="32" t="n"/>
-      <c r="E202" s="22">
+      <c r="A202" s="32" t="n"/>
+      <c r="B202" s="32" t="n"/>
+      <c r="C202" s="33" t="n"/>
+      <c r="D202" s="33" t="n"/>
+      <c r="E202" s="23">
         <f>IF(D202="","",D202*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F202" s="32" t="n"/>
+      <c r="F202" s="33" t="n"/>
     </row>
     <row r="203">
-      <c r="A203" s="31" t="n"/>
-      <c r="B203" s="31" t="n"/>
-      <c r="C203" s="32" t="n"/>
-      <c r="D203" s="32" t="n"/>
-      <c r="E203" s="22">
+      <c r="A203" s="32" t="n"/>
+      <c r="B203" s="32" t="n"/>
+      <c r="C203" s="33" t="n"/>
+      <c r="D203" s="33" t="n"/>
+      <c r="E203" s="23">
         <f>IF(D203="","",D203*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F203" s="32" t="n"/>
+      <c r="F203" s="33" t="n"/>
     </row>
     <row r="204">
-      <c r="A204" s="31" t="n"/>
-      <c r="B204" s="31" t="n"/>
-      <c r="C204" s="32" t="n"/>
-      <c r="D204" s="32" t="n"/>
-      <c r="E204" s="22">
+      <c r="A204" s="32" t="n"/>
+      <c r="B204" s="32" t="n"/>
+      <c r="C204" s="33" t="n"/>
+      <c r="D204" s="33" t="n"/>
+      <c r="E204" s="23">
         <f>IF(D204="","",D204*Parametres!$B$6)</f>
         <v/>
       </c>
-      <c r="F204" s="32" t="n"/>
+      <c r="F204" s="33" t="n"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
Planning : jours travaillés en clair, repos en foncé
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01A1LRXK2yXR6W5viD25HWb5
</commit_message>
<xml_diff>
--- a/conges/conges_police_12h08.xlsx
+++ b/conges/conges_police_12h08.xlsx
@@ -280,7 +280,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
   </cellStyles>
-  <dxfs count="3">
+  <dxfs count="4">
     <dxf>
       <font>
         <name val="Arial"/>
@@ -307,9 +307,26 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00FFFFFF"/>
+      </font>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="00BFBFBF"/>
+          <fgColor rgb="00404040"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <name val="Arial"/>
+        <b val="1"/>
+        <color rgb="00375623"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="00E2F0D9"/>
         </patternFill>
       </fill>
     </dxf>
@@ -1449,14 +1466,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -1472,9 +1489,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -1965,14 +1987,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -1988,9 +2010,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -2481,14 +2508,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -2504,9 +2531,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -2997,14 +3029,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -3020,9 +3052,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -3513,14 +3550,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -3536,9 +3573,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -4029,14 +4071,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -4052,9 +4094,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -4545,14 +4592,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -4568,9 +4615,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -8415,14 +8467,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -8438,9 +8490,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -8931,14 +8988,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -8954,9 +9011,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -9447,14 +9509,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -9470,9 +9532,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -9963,14 +10030,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -9986,9 +10053,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
@@ -10479,14 +10551,14 @@
     <row r="8">
       <c r="A8" s="12" t="inlineStr">
         <is>
-          <t>Lignes grises = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
+          <t>Clair = jour travaillé, tu peux poser. Foncé = repos du cycle. Tape ou choisis ton code sur la ligne « Moi » (CA, CA HP, RTC, CET, CF, HS, RPS, ASA).</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="12" t="inlineStr">
         <is>
-          <t>Seuls les codes posés sur un jour travaillé sont déduits du Tableau.</t>
+          <t>Seuls les codes posés sur un jour clair sont déduits du Tableau.</t>
         </is>
       </c>
     </row>
@@ -10502,9 +10574,14 @@
       <formula>OR(B$6="RTC",B$6="CF",B$6="HS",B$6="ASA")</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B5:AF6">
+  <conditionalFormatting sqref="B3:AF6">
     <cfRule type="expression" priority="3" dxfId="2">
       <formula>B$5="R"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B5:AF6">
+    <cfRule type="expression" priority="4" dxfId="3">
+      <formula>B$5="T"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">

</xml_diff>